<commit_message>
Add Kathmandu Metropolitan City municipal officer interview as NPL_4
- Codes the KTM Municipal Office interview (Kathmandu Metropolitan City
  Solid Waste Management Office, 23 June) from the guideline notes and
  full verbatim transcript.
- Flags and excludes a Q3a bullet block that appears to describe a
  different, unrelated multi-city (Kathmandu/Pokhara) private/NGO
  recycling operation with a Bhaktapur awareness campaign and UNDP
  training - inconsistent with a single-city municipal government's own
  operations - documented in the Notes field for transparency.
- Adds full Coding_Explanations entries for every coded value in NPL_4.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to three interview sources from the 'Plastic Pollution Governance in Nepal' project. Column names and order in 'Coded_Data' follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to four interview sources from the 'Plastic Pollution Governance in Nepal' project. Column names and order in 'Coded_Data' follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -508,72 +508,79 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. NPL_4 - Kathmandu Metropolitan City (KMC), Solid Waste Management Office - unnamed municipal officer(s), Kathmandu (23 June). Coded from both the interview guideline notes and the full verbatim transcript. Note: the Q3a bullet notes in the source document describing a multi-city (Kathmandu/Pokhara) dry-waste operation with UNDP training and a Bhaktapur awareness campaign appear to belong to a different, unrelated interview accidentally included in the same file, and were excluded from this row's coding (see the 'Notes' cell for NPL_4 in Coded_Data for detail).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix (one row per interview, one column per codebook variable, including a free-hand 'Notes' column) with the coded values.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix (one row per interview, one column per codebook variable, including a free-hand 'Notes' column) with the coded values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation used to justify every non-NA code in Coded_Data (one row per Interview x Variable).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way). 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no for all three interviews, since each explicitly states extended producer responsibility does not yet exist in Nepal).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way). 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no for all three interviews, since each explicitly states extended producer responsibility does not yet exist in Nepal).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Note on source material: a block of longer, polished paragraph-style quotes appeared under the RSCT question list in the original material, but the content and first-person phrasing ("we have... directives...", "Department of Environment is regularly monitoring...") match the Department of Environment notes and transcript almost verbatim. These paragraphs were therefore treated as additional corroborating evidence for the DoE interview (NPL_1), not for RSCT (NPL_3), and coded accordingly.</t>
         </is>
@@ -1760,7 +1767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ4"/>
+  <dimension ref="A1:CQ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3768,6 +3775,483 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>visual pollution (described as "the biggest problem"), drainage/sewer blockage, riverbank and roadside litter, open dumping (due to lack of land for proper storage/sorting), microplastics, wildlife (plastics found in animal excreta), tourism (visual pollution affecting the city's image)</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>rivers and riverbanks, drainage/sewer systems, wildlife (plastic found in excreta), the visual/tourism image of Kathmandu, and neighbouring communities near landfill/transfer sites who bear the burden of other municipalities' waste</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>plastic manufacturers who keep producing bags below 40 microns despite the ban, and importers bringing banned bags/plastic flowers in from neighbouring countries; residents who oppose siting any waste/recovery facility near their homes (NIMBY-style "public opposition"); and, to a lesser degree, consumers who keep choosing cheap single-use plastic out of convenience despite being aware of its harms</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City's own solid waste management office (formalising private-sector partnerships across seven clusters, drafting new regulations, planning micron-threshold increases); DoCoRecyclers (the NGO partner collecting/processing recyclables in Cluster 7); UNDP (technical/financial partner for mechanised recovery and storage systems); and department stores that have voluntarily stopped giving out plastic bags</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AE5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AL5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA5" s="5" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="BB5" s="5" t="inlineStr">
+        <is>
+          <t>As an autonomous local government, Kathmandu Metropolitan City drafts its own regulations (e.g. the new solid waste management regulation enabling formal cluster-based partnerships with private actors) and independently negotiates MoUs/terms with private and NGO partners (e.g. the DoCoRecyclers agreement in Cluster 7, the UNDP MoU for mechanised recovery/storage), showing considerable discretion in how it organises implementation.</t>
+        </is>
+      </c>
+      <c r="BC5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI5" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ5" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BK5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BL5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW5" s="5" t="inlineStr">
+        <is>
+          <t>"Plastic bags below 40 microns have already been banned in Kathmandu Metropolitan City, and also nationally... But on the ground, the reality is very different. Plastics below 40 microns are still widely available, and plastic flowers are commonly found. The main issue lies in implementation... enforcement is weak"; "there's been no full assessment [of the micron ban]... it's not fully operational"; "we also try to ban the single use of plastic, but it's very hard for us to achieve that goal."</t>
+        </is>
+      </c>
+      <c r="BX5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CA5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CJ5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM5" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP5" s="5" t="inlineStr">
+        <is>
+          <t>When asked directly, the interviewee initially said no specific tradition came to mind, but then described "lobti" - leaf plates used at some Kathmandu community festivals instead of plastic plates. Effective at cutting plastic use at large gatherings, but costly (~20 rupees/piece vs. much cheaper plastic), so currently only used by wealthier groups; the interviewee agreed government subsidies for producers of such alternatives could help scale this practice.</t>
+        </is>
+      </c>
+      <c r="CQ5" s="5" t="inlineStr">
+        <is>
+          <t>Affiliation: Kathmandu Metropolitan City (KMC), Solid Waste Management Office/Department (municipal/local government level). Interviewee name(s) not given; the transcript suggests at least two KMC staff were present ("our ma'am has answered..."). Location: Kathmandu. Interview date: 23 June (year not stated on this document, but consistent with the other Nepal interviews conducted around 21-23 June 2025). Coded from both the interview guideline notes and the full verbatim transcript. Data-quality note: the bullet list under Q3a ("2017; dry waste management...situated in Kathmandu and Pokhara...UNDP skill development training in Pokhara, 400 participants... Awareness campaigns Bhaktapur... research on policy framework in collaboration with a UK university") describes a multi-city private/NGO recycling and research operation, not Kathmandu Metropolitan City's own government office (a single-city municipal authority would not itself be based in Pokhara or run a campaign in Bhaktapur, a separate metropolitan city). This content appears to belong to a different interview accidentally included in the same document and was therefore excluded from this row's coding; the coding instead relies on the content that is clearly attributable to the Kathmandu Metropolitan City office (Q3b onward in the notes, and the full PEGO/KTM Municipal Office transcript).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3779,7 +4263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E156"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8001,6 +8485,1653 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>The interviewee(s) work for Kathmandu Metropolitan City's Solid Waste Management Office, a municipal/local government body; coded as loc_government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>"Most of the people are very well aware about the impact of plastic pollution... they know about the microplastic, they know about the harmful impact... Still, they choose to use the plastic because it is very convenient." Unlike other Nepal interviews, this respondent explicitly says awareness is already high and the barrier is convenience/habit, not ignorance - hence coded 'no' (lack of awareness was not identified as the problem).</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>"Most of the plastic is multi-layer plastic, which is thrown riverside, bank of the river, corridor, drainage"; "visible litter" is a recurring theme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>"They don't have the habit of taking the cloth bag wherever we go" and continued preference for cheap single-use plastic over costlier reusable alternatives (e.g. leaf plates) reflect ongoing excessive single-use consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>"Multi-layer plastic has no value and is often left behind"; "cherry picking" by collectors (Q3b notes) means only valuable plastics get collected/recycled, leaving low-value plastic unmanaged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>Extensive description of structural waste-management gaps: no space to sort/store waste in the city, waste has to be trucked to a landfill in another district, and "lack of infrastructure to manage, collect, recycle" (Q3b notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>"The plastics are so much cheaper"; leaf plates (lobti) "cost 20rs per piece, that is very costly" and are only used by wealthier groups - explicit statement that affordable alternatives are lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>"Lack of the land, we cannot separate, collect [or store] in storage" - segregation is explicitly hampered by space constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Problem_import</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>"Plastic companies continue to produce bags below 40 microns, and we also import such plastic products - including plastic flowers - from neighboring countries" - explicit statement that imports undermine the existing ban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>visual pollution (described as "the biggest problem"), drainage/sewer blockage, riverbank and roadside litter, open dumping (due to lack of land for proper storage/sorting), microplastics, wildlife (plastics found in animal excreta), tourism (visual pollution affecting the city's image)</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>"The biggest problem is visual pollution"; "due to the plastic problem, all the drainage is blockage"; plastic thrown "riverside, bank of the river"; microplastics and plastics "in the excreta of wildlife" (per research cited by the interviewee); visual pollution linked to tourism and lifestyle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>rivers and riverbanks, drainage/sewer systems, wildlife (plastic found in excreta), the visual/tourism image of Kathmandu, and neighbouring communities near landfill/transfer sites who bear the burden of other municipalities' waste</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>Rivers/riverbanks and drainage systems (blocked and littered), wildlife (plastic found in excreta), the city's visual/tourism appeal, and neighbouring districts/communities that host the Bancharedanda landfill or the Dakshinkali debris-dumping site without being responsible for managing them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>plastic manufacturers who keep producing bags below 40 microns despite the ban, and importers bringing banned bags/plastic flowers in from neighbouring countries; residents who oppose siting any waste/recovery facility near their homes (NIMBY-style "public opposition"); and, to a lesser degree, consumers who keep choosing cheap single-use plastic out of convenience despite being aware of its harms</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>"Plastic companies... are still producing the plastic that is less than 40 micron" and imported plastic bags/flowers "from neighboring countries" undermine the ban; "public opposition" to siting any recovery facility nearby ("no one wants waste on their side"); and consumers who "still choose to use plastic because it's convenient" despite being aware of the harms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City's own solid waste management office (formalising private-sector partnerships across seven clusters, drafting new regulations, planning micron-threshold increases); DoCoRecyclers (the NGO partner collecting/processing recyclables in Cluster 7); UNDP (technical/financial partner for mechanised recovery and storage systems); and department stores that have voluntarily stopped giving out plastic bags</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City's own office (drafting new solid waste regulation, formalising 7 cluster-based private-sector partnerships, planning micron increases and subsidies); DoCoRecyclers (the NGO partner in Cluster 7); UNDP (MoU for mechanised plastic recovery/storage); and department stores that "no longer provide plastic bags".</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>"Uncertain which Department should look after" plastic waste at the national level (Q5 notes); "lack of coordination of the stakeholders" (Q3b notes); "no clear coordination with local communities".</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>"If land is under the jurisdiction of the national government, it will be very difficult for the local government to reach out to that land"; explicit call for "better coordination with both the national and provincial government."</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>"Gov Nepal; uncertain which Department should look after" plastic waste (Q5 notes) - explicit statement of unclear institutional ownership at the national level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>The Ministry of Forest and Environment has drafted a national policy (under revision) and the Department of Environment is named; central government's help is also invoked for land identification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>"The central or provincial governments could help us identify suitable locations within the city or valley for plastic recovery and management facilities" - explicit responsibility role assigned to provincial government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>"The Solid Waste Management Act of 2068 clearly assigns the responsibility for managing solid waste to the local level... our office and the metropolitan city are responsible for managing plastic waste."</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>DoCoRecyclers and other registered private actors now formally collect and process recyclable waste in KMC's seven clusters under signed MoUs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>DoCoRecyclers is explicitly described as "a local NGO" that collects recyclable waste under an MoU with the municipality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>Land needed for waste facilities "is under the jurisdiction of the national government" making it "very difficult for the local government to reach out to that land"; the national policy revision remains stalled/unclear ("I do not know exactly").</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>The interviewee acknowledges enforcement gaps under the municipality's own remit: "there's been no full assessment [of the ban]"; "we also try to ban the single use of plastic, but it's very hard for us to achieve that goal."</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D180" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>"Cherry picking" by collectors (Q3b notes) - only valuable plastics are collected, leaving low-value/multi-layer plastic behind to accumulate in rivers/dumpsites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>"Public opposition" to hosting any waste facility nearby ("no one wants waste on their side"); continued convenience-driven plastic use despite awareness of harms; "people are not taking it very seriously" (Q3b notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D182" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>"Plastic companies, they are still producing the plastic that is less than 40 micron"; plastic bags and plastic flowers "also being imported from neighboring countries" despite the ban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>"Implementing partners/monitoring should [be] the municipality -&gt; they should be made accountable" (Q9 notes) - the municipality itself is named as a target for accountability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D184" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>"As young as you can catch them; waste management should be in the education system" (Q10 follow-up) - explicit call to target children/students through the curriculum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>"Waste managers" explicitly listed as a target group for future policy (Q9 notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D186" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>"Focus reduce plastic consumers" (Q9 notes); consumers/shoppers targeted via cloth-bag requirements at department stores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>Tied to the same call to embed waste management "in the education system", implicating schools as a target for future policy/curriculum change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D188" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>"Producers (EPR)" explicitly listed as a target group (Q9 notes); plastic industry also targeted for micron-threshold subsidies to encourage compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City both formulates its own local rules ("we can have our own legal code and formulate our own rules and regulations", e.g. the new solid waste management regulation - role 1) and directly manages implementation (cluster-based MoUs, transfer stations, subsidy planning - role 2), so both are coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>As an autonomous local government, Kathmandu Metropolitan City drafts its own regulations (e.g. the new solid waste management regulation enabling formal cluster-based partnerships with private actors) and independently negotiates MoUs/terms with private and NGO partners (e.g. the DoCoRecyclers agreement in Cluster 7, the UNDP MoU for mechanised recovery/storage), showing considerable discretion in how it organises implementation.</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>"Kathmandu Metropolitan City is a local government, so we can create our own laws and regulations. We also manage our own facilities"; the cluster-based MoU with DoCoRecyclers (negotiated terms, payment amount) further shows discretion in implementation design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>"There is no assessment of [the micron ban]... fully not [in] operation[al]" - explicit statement that current measures are not being monitored/evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>Q10 notes call for "collection chains; recycling facilities -&gt; financing" and the interview highlights ongoing reliance on donor/partner funding (UNDP, DoCoRecyclers' annual payment) to sustain and expand operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>"There's been no full assessment" of the effectiveness of the micron increases; "even if we increase it to 100 microns, we're unsure if that would be beneficial" - explicit knowledge/evaluation gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>"Land is the biggest challenge... lack of infrastructure to manage, collect, recycle"; "we lack... technology and recycling infrastructure"; no space within the city for a transfer station or material recovery facility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>"Technology transfer, do not reinvent the wheel" (Q10 notes) signals a technical/knowledge capacity gap that external partners are expected to help fill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B196" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D196" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E196" s="5" t="inlineStr">
+        <is>
+          <t>"On paper, the legal provisions are very well-written. But in practice, enforcement is weak"; plastic companies and importers continue supplying banned products despite the rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>"First policy EPR" is listed among future/needed solutions (Q8), and "EPR should be introduced" (Q6 notes) - both frame EPR as not yet in place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B198" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>Pol_import</t>
+        </is>
+      </c>
+      <c r="D198" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E198" s="5" t="inlineStr">
+        <is>
+          <t>No dedicated import-control mechanism is described; instead the interviewee states banned bags/flowers "are also being imported from neighboring countries" unchecked, indicating the absence of an effective import regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>"Plastic bags below 40 microns have already been banned in Kathmandu Metropolitan City, and also nationally. Plastic flowers have also been banned."</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B200" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D200" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E200" s="5" t="inlineStr">
+        <is>
+          <t>"If you visit department stores... you'll notice they no longer provide plastic bags. Shoppers have to buy cloth bags. Our office also produces and occasionally distributes cloth bags."</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D201" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>DoCoRecyclers "collect recyclable waste from that cluster and transport it to our Deku transfer station" under a formal, ongoing MoU with the municipality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B202" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D202" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E202" s="5" t="inlineStr">
+        <is>
+          <t>Extensive existing collection system: city divided into 7 clusters by ward, MoUs with registered private actors, waste transported to Bancharedanda landfill, debris collection arrangement with Dakshinkali Municipality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D203" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>"On the ground, the reality is very different"; "the main issue lies in implementation... enforcement is weak"; "there's been no full assessment" of the micron-threshold policy; "it's very hard for us to achieve that goal" (regarding the single-use plastic ban).</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D204" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>"There is the need of a body, guiding governing body"; "important missing link is implementing body" (Q6 notes) - explicit call for establishing/clarifying a lead implementing agency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D205" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>Tied to the same call for a guiding/implementing body, plus the explicit proposal that municipalities "should be made accountable" (Q9 notes) as part of a clearer division of roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>Sol_epr</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>"First policy EPR" listed as the top future policy priority (Q8 notes); "producers (EPR)" named as a target group (Q9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>"As young as you can catch them; waste management should be in the education system; Reduce ignorance" (Q10 follow-up) calls for future awareness/education efforts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D208" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>"Processing treatment/recycling" listed as a needed future policy focus (Q8 notes); "policies to export recycling produces" (Q10 notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D209" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>"Waste management should be in the education system" (Q10 follow-up) - explicit proposed solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D210" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="inlineStr">
+        <is>
+          <t>"Technology transfer, do not reinvent the wheel" (Q10 notes) proposes building capacity via external knowledge/technology transfer rather than developing everything from scratch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C211" s="5" t="inlineStr">
+        <is>
+          <t>Sol_ban</t>
+        </is>
+      </c>
+      <c r="D211" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>Plan to progressively raise the minimum plastic thickness standard ("we plan to increase it to 75 microns - possibly [beyond]... previously it was 20 microns, then upgraded to 40, and now the goal is 75 microns") as a strengthened ban/standard going forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C212" s="5" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D212" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="inlineStr">
+        <is>
+          <t>"Subsidies should be provided to the plastic industry, especially to increase plastic thickness"; "government subsidizing companies producing alternatives" endorsed as "perhaps" a good opportunity; Q10 notes call for "financing" for collection chains and recycling facilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B213" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C213" s="5" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D213" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>"If we get the land, we can [establish an] MRF... recycle"; call for national/provincial government help "to identify suitable locations... for plastic recovery and management facilities"; UNDP MoU for "mechanized plastic recovery and storage systems."</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B214" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C214" s="5" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D214" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E214" s="5" t="inlineStr">
+        <is>
+          <t>"Government subsidizing companies producing alternatives is a good opportunity - Yes, perhaps", discussed in relation to scaling up leaf-plate (lobti) style alternatives that are currently too expensive for widespread use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B215" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C215" s="5" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D215" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E215" s="5" t="inlineStr">
+        <is>
+          <t>"Regular field inspections are needed" - explicit proposed enforcement solution to address the currently weak enforcement of the micron ban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B216" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C216" s="5" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D216" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E216" s="5" t="inlineStr">
+        <is>
+          <t>Tied to the same call for "regular field inspections" and the acknowledged lack of assessment of policy effectiveness, implying a need for stronger ongoing monitoring going forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B217" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C217" s="5" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D217" s="5" t="inlineStr">
+        <is>
+          <t>When asked directly, the interviewee initially said no specific tradition came to mind, but then described "lobti" - leaf plates used at some Kathmandu community festivals instead of plastic plates. Effective at cutting plastic use at large gatherings, but costly (~20 rupees/piece vs. much cheaper plastic), so currently only used by wealthier groups; the interviewee agreed government subsidies for producers of such alternatives could help scale this practice.</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>When first asked directly about traditional practices (in a Bhutan-comparison framing), the interviewee said "No." But later, when the question was revisited, described "lobti" - leaf plates used in some Kathmandu community festivals instead of plastic ones - as an existing, if underused and costly (20 rupees/piece), alternative practice.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-verify NPL_4 actor grids/NPF/effectiveness columns against codebook
- Strict re-check of NPF_victims/villains/hero, Res_/Cul_/Tar_ actor
  grids, Actor_role, Discretion, Capacity, Pol_effectiveness and
  Pol_effectiveness_example for the KTM Municipal Office interview
  (NPL_4) against the codebook definitions.
- Adds Res_private_companies = yes: department stores already
  voluntarily discontinuing single-use plastic bags is direct evidence
  of private companies exercising responsibility, which was missed in
  the initial pass.
- All other requested columns confirmed consistent with the codebook
  and interview evidence; no further changes needed.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -3933,7 +3933,7 @@
       </c>
       <c r="AF5" s="5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AG5" s="5" t="inlineStr">
@@ -4263,7 +4263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E217"/>
+  <dimension ref="A1:E218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="C178" s="5" t="inlineStr">
         <is>
-          <t>Cul_nat_government</t>
+          <t>Res_private_companies</t>
         </is>
       </c>
       <c r="D178" s="5" t="inlineStr">
@@ -9075,7 +9075,7 @@
       </c>
       <c r="E178" s="5" t="inlineStr">
         <is>
-          <t>Land needed for waste facilities "is under the jurisdiction of the national government" making it "very difficult for the local government to reach out to that land"; the national policy revision remains stalled/unclear ("I do not know exactly").</t>
+          <t>"If you visit department stores in our city... you'll notice they no longer provide plastic bags. Shoppers have to buy cloth bags" - private retail companies already exercising responsibility by voluntarily discontinuing single-use plastic bags.</t>
         </is>
       </c>
     </row>
@@ -9092,7 +9092,7 @@
       </c>
       <c r="C179" s="5" t="inlineStr">
         <is>
-          <t>Cul_loc_government</t>
+          <t>Cul_nat_government</t>
         </is>
       </c>
       <c r="D179" s="5" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>The interviewee acknowledges enforcement gaps under the municipality's own remit: "there's been no full assessment [of the ban]"; "we also try to ban the single use of plastic, but it's very hard for us to achieve that goal."</t>
+          <t>Land needed for waste facilities "is under the jurisdiction of the national government" making it "very difficult for the local government to reach out to that land"; the national policy revision remains stalled/unclear ("I do not know exactly").</t>
         </is>
       </c>
     </row>
@@ -9119,7 +9119,7 @@
       </c>
       <c r="C180" s="5" t="inlineStr">
         <is>
-          <t>Cul_private_sector</t>
+          <t>Cul_loc_government</t>
         </is>
       </c>
       <c r="D180" s="5" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
-          <t>"Cherry picking" by collectors (Q3b notes) - only valuable plastics are collected, leaving low-value/multi-layer plastic behind to accumulate in rivers/dumpsites.</t>
+          <t>The interviewee acknowledges enforcement gaps under the municipality's own remit: "there's been no full assessment [of the ban]"; "we also try to ban the single use of plastic, but it's very hard for us to achieve that goal."</t>
         </is>
       </c>
     </row>
@@ -9146,7 +9146,7 @@
       </c>
       <c r="C181" s="5" t="inlineStr">
         <is>
-          <t>Cul_households</t>
+          <t>Cul_private_sector</t>
         </is>
       </c>
       <c r="D181" s="5" t="inlineStr">
@@ -9156,7 +9156,7 @@
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>"Public opposition" to hosting any waste facility nearby ("no one wants waste on their side"); continued convenience-driven plastic use despite awareness of harms; "people are not taking it very seriously" (Q3b notes).</t>
+          <t>"Cherry picking" by collectors (Q3b notes) - only valuable plastics are collected, leaving low-value/multi-layer plastic behind to accumulate in rivers/dumpsites.</t>
         </is>
       </c>
     </row>
@@ -9173,7 +9173,7 @@
       </c>
       <c r="C182" s="5" t="inlineStr">
         <is>
-          <t>Cul_private_companies</t>
+          <t>Cul_households</t>
         </is>
       </c>
       <c r="D182" s="5" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="E182" s="5" t="inlineStr">
         <is>
-          <t>"Plastic companies, they are still producing the plastic that is less than 40 micron"; plastic bags and plastic flowers "also being imported from neighboring countries" despite the ban.</t>
+          <t>"Public opposition" to hosting any waste facility nearby ("no one wants waste on their side"); continued convenience-driven plastic use despite awareness of harms; "people are not taking it very seriously" (Q3b notes).</t>
         </is>
       </c>
     </row>
@@ -9200,7 +9200,7 @@
       </c>
       <c r="C183" s="5" t="inlineStr">
         <is>
-          <t>Tar_loc_government</t>
+          <t>Cul_private_companies</t>
         </is>
       </c>
       <c r="D183" s="5" t="inlineStr">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>"Implementing partners/monitoring should [be] the municipality -&gt; they should be made accountable" (Q9 notes) - the municipality itself is named as a target for accountability.</t>
+          <t>"Plastic companies, they are still producing the plastic that is less than 40 micron"; plastic bags and plastic flowers "also being imported from neighboring countries" despite the ban.</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="C184" s="5" t="inlineStr">
         <is>
-          <t>Tar_students</t>
+          <t>Tar_loc_government</t>
         </is>
       </c>
       <c r="D184" s="5" t="inlineStr">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
-          <t>"As young as you can catch them; waste management should be in the education system" (Q10 follow-up) - explicit call to target children/students through the curriculum.</t>
+          <t>"Implementing partners/monitoring should [be] the municipality -&gt; they should be made accountable" (Q9 notes) - the municipality itself is named as a target for accountability.</t>
         </is>
       </c>
     </row>
@@ -9254,7 +9254,7 @@
       </c>
       <c r="C185" s="5" t="inlineStr">
         <is>
-          <t>Tar_private_sector</t>
+          <t>Tar_students</t>
         </is>
       </c>
       <c r="D185" s="5" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
-          <t>"Waste managers" explicitly listed as a target group for future policy (Q9 notes).</t>
+          <t>"As young as you can catch them; waste management should be in the education system" (Q10 follow-up) - explicit call to target children/students through the curriculum.</t>
         </is>
       </c>
     </row>
@@ -9281,7 +9281,7 @@
       </c>
       <c r="C186" s="5" t="inlineStr">
         <is>
-          <t>Tar_households</t>
+          <t>Tar_private_sector</t>
         </is>
       </c>
       <c r="D186" s="5" t="inlineStr">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="E186" s="5" t="inlineStr">
         <is>
-          <t>"Focus reduce plastic consumers" (Q9 notes); consumers/shoppers targeted via cloth-bag requirements at department stores.</t>
+          <t>"Waste managers" explicitly listed as a target group for future policy (Q9 notes).</t>
         </is>
       </c>
     </row>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>Tar_edu_institutions</t>
+          <t>Tar_households</t>
         </is>
       </c>
       <c r="D187" s="5" t="inlineStr">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
-          <t>Tied to the same call to embed waste management "in the education system", implicating schools as a target for future policy/curriculum change.</t>
+          <t>"Focus reduce plastic consumers" (Q9 notes); consumers/shoppers targeted via cloth-bag requirements at department stores.</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9335,7 @@
       </c>
       <c r="C188" s="5" t="inlineStr">
         <is>
-          <t>Tar_private_companies</t>
+          <t>Tar_edu_institutions</t>
         </is>
       </c>
       <c r="D188" s="5" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="E188" s="5" t="inlineStr">
         <is>
-          <t>"Producers (EPR)" explicitly listed as a target group (Q9 notes); plastic industry also targeted for micron-threshold subsidies to encourage compliance.</t>
+          <t>Tied to the same call to embed waste management "in the education system", implicating schools as a target for future policy/curriculum change.</t>
         </is>
       </c>
     </row>
@@ -9362,17 +9362,17 @@
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>Actor_role</t>
+          <t>Tar_private_companies</t>
         </is>
       </c>
       <c r="D189" s="5" t="inlineStr">
         <is>
-          <t>1,2</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>Kathmandu Metropolitan City both formulates its own local rules ("we can have our own legal code and formulate our own rules and regulations", e.g. the new solid waste management regulation - role 1) and directly manages implementation (cluster-based MoUs, transfer stations, subsidy planning - role 2), so both are coded.</t>
+          <t>"Producers (EPR)" explicitly listed as a target group (Q9 notes); plastic industry also targeted for micron-threshold subsidies to encourage compliance.</t>
         </is>
       </c>
     </row>
@@ -9389,17 +9389,17 @@
       </c>
       <c r="C190" s="5" t="inlineStr">
         <is>
-          <t>Discretion</t>
+          <t>Actor_role</t>
         </is>
       </c>
       <c r="D190" s="5" t="inlineStr">
         <is>
-          <t>As an autonomous local government, Kathmandu Metropolitan City drafts its own regulations (e.g. the new solid waste management regulation enabling formal cluster-based partnerships with private actors) and independently negotiates MoUs/terms with private and NGO partners (e.g. the DoCoRecyclers agreement in Cluster 7, the UNDP MoU for mechanised recovery/storage), showing considerable discretion in how it organises implementation.</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="E190" s="5" t="inlineStr">
         <is>
-          <t>"Kathmandu Metropolitan City is a local government, so we can create our own laws and regulations. We also manage our own facilities"; the cluster-based MoU with DoCoRecyclers (negotiated terms, payment amount) further shows discretion in implementation design.</t>
+          <t>Kathmandu Metropolitan City both formulates its own local rules ("we can have our own legal code and formulate our own rules and regulations", e.g. the new solid waste management regulation - role 1) and directly manages implementation (cluster-based MoUs, transfer stations, subsidy planning - role 2), so both are coded.</t>
         </is>
       </c>
     </row>
@@ -9416,17 +9416,17 @@
       </c>
       <c r="C191" s="5" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Discretion</t>
         </is>
       </c>
       <c r="D191" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>As an autonomous local government, Kathmandu Metropolitan City drafts its own regulations (e.g. the new solid waste management regulation enabling formal cluster-based partnerships with private actors) and independently negotiates MoUs/terms with private and NGO partners (e.g. the DoCoRecyclers agreement in Cluster 7, the UNDP MoU for mechanised recovery/storage), showing considerable discretion in how it organises implementation.</t>
         </is>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
-          <t>"There is no assessment of [the micron ban]... fully not [in] operation[al]" - explicit statement that current measures are not being monitored/evaluated.</t>
+          <t>"Kathmandu Metropolitan City is a local government, so we can create our own laws and regulations. We also manage our own facilities"; the cluster-based MoU with DoCoRecyclers (negotiated terms, payment amount) further shows discretion in implementation design.</t>
         </is>
       </c>
     </row>
@@ -9443,7 +9443,7 @@
       </c>
       <c r="C192" s="5" t="inlineStr">
         <is>
-          <t>Financial_resources</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="D192" s="5" t="inlineStr">
@@ -9453,7 +9453,7 @@
       </c>
       <c r="E192" s="5" t="inlineStr">
         <is>
-          <t>Q10 notes call for "collection chains; recycling facilities -&gt; financing" and the interview highlights ongoing reliance on donor/partner funding (UNDP, DoCoRecyclers' annual payment) to sustain and expand operations.</t>
+          <t>"There is no assessment of [the micron ban]... fully not [in] operation[al]" - explicit statement that current measures are not being monitored/evaluated.</t>
         </is>
       </c>
     </row>
@@ -9470,7 +9470,7 @@
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Financial_resources</t>
         </is>
       </c>
       <c r="D193" s="5" t="inlineStr">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="E193" s="5" t="inlineStr">
         <is>
-          <t>"There's been no full assessment" of the effectiveness of the micron increases; "even if we increase it to 100 microns, we're unsure if that would be beneficial" - explicit knowledge/evaluation gap.</t>
+          <t>Q10 notes call for "collection chains; recycling facilities -&gt; financing" and the interview highlights ongoing reliance on donor/partner funding (UNDP, DoCoRecyclers' annual payment) to sustain and expand operations.</t>
         </is>
       </c>
     </row>
@@ -9497,7 +9497,7 @@
       </c>
       <c r="C194" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D194" s="5" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="E194" s="5" t="inlineStr">
         <is>
-          <t>"Land is the biggest challenge... lack of infrastructure to manage, collect, recycle"; "we lack... technology and recycling infrastructure"; no space within the city for a transfer station or material recovery facility.</t>
+          <t>"There's been no full assessment" of the effectiveness of the micron increases; "even if we increase it to 100 microns, we're unsure if that would be beneficial" - explicit knowledge/evaluation gap.</t>
         </is>
       </c>
     </row>
@@ -9524,7 +9524,7 @@
       </c>
       <c r="C195" s="5" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D195" s="5" t="inlineStr">
@@ -9534,7 +9534,7 @@
       </c>
       <c r="E195" s="5" t="inlineStr">
         <is>
-          <t>"Technology transfer, do not reinvent the wheel" (Q10 notes) signals a technical/knowledge capacity gap that external partners are expected to help fill.</t>
+          <t>"Land is the biggest challenge... lack of infrastructure to manage, collect, recycle"; "we lack... technology and recycling infrastructure"; no space within the city for a transfer station or material recovery facility.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
       </c>
       <c r="C196" s="5" t="inlineStr">
         <is>
-          <t>Enforcement</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="D196" s="5" t="inlineStr">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="E196" s="5" t="inlineStr">
         <is>
-          <t>"On paper, the legal provisions are very well-written. But in practice, enforcement is weak"; plastic companies and importers continue supplying banned products despite the rules.</t>
+          <t>"Technology transfer, do not reinvent the wheel" (Q10 notes) signals a technical/knowledge capacity gap that external partners are expected to help fill.</t>
         </is>
       </c>
     </row>
@@ -9578,17 +9578,17 @@
       </c>
       <c r="C197" s="5" t="inlineStr">
         <is>
-          <t>Pol_epr</t>
+          <t>Enforcement</t>
         </is>
       </c>
       <c r="D197" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
         <is>
-          <t>"First policy EPR" is listed among future/needed solutions (Q8), and "EPR should be introduced" (Q6 notes) - both frame EPR as not yet in place.</t>
+          <t>"On paper, the legal provisions are very well-written. But in practice, enforcement is weak"; plastic companies and importers continue supplying banned products despite the rules.</t>
         </is>
       </c>
     </row>
@@ -9605,7 +9605,7 @@
       </c>
       <c r="C198" s="5" t="inlineStr">
         <is>
-          <t>Pol_import</t>
+          <t>Pol_epr</t>
         </is>
       </c>
       <c r="D198" s="5" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="E198" s="5" t="inlineStr">
         <is>
-          <t>No dedicated import-control mechanism is described; instead the interviewee states banned bags/flowers "are also being imported from neighboring countries" unchecked, indicating the absence of an effective import regulation.</t>
+          <t>"First policy EPR" is listed among future/needed solutions (Q8), and "EPR should be introduced" (Q6 notes) - both frame EPR as not yet in place.</t>
         </is>
       </c>
     </row>
@@ -9632,17 +9632,17 @@
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
-          <t>Pol_ban</t>
+          <t>Pol_import</t>
         </is>
       </c>
       <c r="D199" s="5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
         <is>
-          <t>"Plastic bags below 40 microns have already been banned in Kathmandu Metropolitan City, and also nationally. Plastic flowers have also been banned."</t>
+          <t>No dedicated import-control mechanism is described; instead the interviewee states banned bags/flowers "are also being imported from neighboring countries" unchecked, indicating the absence of an effective import regulation.</t>
         </is>
       </c>
     </row>
@@ -9659,7 +9659,7 @@
       </c>
       <c r="C200" s="5" t="inlineStr">
         <is>
-          <t>Pol_subsitutes</t>
+          <t>Pol_ban</t>
         </is>
       </c>
       <c r="D200" s="5" t="inlineStr">
@@ -9669,7 +9669,7 @@
       </c>
       <c r="E200" s="5" t="inlineStr">
         <is>
-          <t>"If you visit department stores... you'll notice they no longer provide plastic bags. Shoppers have to buy cloth bags. Our office also produces and occasionally distributes cloth bags."</t>
+          <t>"Plastic bags below 40 microns have already been banned in Kathmandu Metropolitan City, and also nationally. Plastic flowers have also been banned."</t>
         </is>
       </c>
     </row>
@@ -9686,7 +9686,7 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>Pol_recycling</t>
+          <t>Pol_subsitutes</t>
         </is>
       </c>
       <c r="D201" s="5" t="inlineStr">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="E201" s="5" t="inlineStr">
         <is>
-          <t>DoCoRecyclers "collect recyclable waste from that cluster and transport it to our Deku transfer station" under a formal, ongoing MoU with the municipality.</t>
+          <t>"If you visit department stores... you'll notice they no longer provide plastic bags. Shoppers have to buy cloth bags. Our office also produces and occasionally distributes cloth bags."</t>
         </is>
       </c>
     </row>
@@ -9713,7 +9713,7 @@
       </c>
       <c r="C202" s="5" t="inlineStr">
         <is>
-          <t>Pol_waste_collection</t>
+          <t>Pol_recycling</t>
         </is>
       </c>
       <c r="D202" s="5" t="inlineStr">
@@ -9723,7 +9723,7 @@
       </c>
       <c r="E202" s="5" t="inlineStr">
         <is>
-          <t>Extensive existing collection system: city divided into 7 clusters by ward, MoUs with registered private actors, waste transported to Bancharedanda landfill, debris collection arrangement with Dakshinkali Municipality.</t>
+          <t>DoCoRecyclers "collect recyclable waste from that cluster and transport it to our Deku transfer station" under a formal, ongoing MoU with the municipality.</t>
         </is>
       </c>
     </row>
@@ -9740,7 +9740,7 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>Pol_effectiveness</t>
+          <t>Pol_waste_collection</t>
         </is>
       </c>
       <c r="D203" s="5" t="inlineStr">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="E203" s="5" t="inlineStr">
         <is>
-          <t>"On the ground, the reality is very different"; "the main issue lies in implementation... enforcement is weak"; "there's been no full assessment" of the micron-threshold policy; "it's very hard for us to achieve that goal" (regarding the single-use plastic ban).</t>
+          <t>Extensive existing collection system: city divided into 7 clusters by ward, MoUs with registered private actors, waste transported to Bancharedanda landfill, debris collection arrangement with Dakshinkali Municipality.</t>
         </is>
       </c>
     </row>
@@ -9767,7 +9767,7 @@
       </c>
       <c r="C204" s="5" t="inlineStr">
         <is>
-          <t>Sol_lead_agency</t>
+          <t>Pol_effectiveness</t>
         </is>
       </c>
       <c r="D204" s="5" t="inlineStr">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="E204" s="5" t="inlineStr">
         <is>
-          <t>"There is the need of a body, guiding governing body"; "important missing link is implementing body" (Q6 notes) - explicit call for establishing/clarifying a lead implementing agency.</t>
+          <t>"On the ground, the reality is very different"; "the main issue lies in implementation... enforcement is weak"; "there's been no full assessment" of the micron-threshold policy; "it's very hard for us to achieve that goal" (regarding the single-use plastic ban).</t>
         </is>
       </c>
     </row>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>Sol_responsibilities</t>
+          <t>Sol_lead_agency</t>
         </is>
       </c>
       <c r="D205" s="5" t="inlineStr">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="E205" s="5" t="inlineStr">
         <is>
-          <t>Tied to the same call for a guiding/implementing body, plus the explicit proposal that municipalities "should be made accountable" (Q9 notes) as part of a clearer division of roles.</t>
+          <t>"There is the need of a body, guiding governing body"; "important missing link is implementing body" (Q6 notes) - explicit call for establishing/clarifying a lead implementing agency.</t>
         </is>
       </c>
     </row>
@@ -9821,7 +9821,7 @@
       </c>
       <c r="C206" s="5" t="inlineStr">
         <is>
-          <t>Sol_epr</t>
+          <t>Sol_responsibilities</t>
         </is>
       </c>
       <c r="D206" s="5" t="inlineStr">
@@ -9831,7 +9831,7 @@
       </c>
       <c r="E206" s="5" t="inlineStr">
         <is>
-          <t>"First policy EPR" listed as the top future policy priority (Q8 notes); "producers (EPR)" named as a target group (Q9).</t>
+          <t>Tied to the same call for a guiding/implementing body, plus the explicit proposal that municipalities "should be made accountable" (Q9 notes) as part of a clearer division of roles.</t>
         </is>
       </c>
     </row>
@@ -9848,7 +9848,7 @@
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>Sol_awareness</t>
+          <t>Sol_epr</t>
         </is>
       </c>
       <c r="D207" s="5" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="E207" s="5" t="inlineStr">
         <is>
-          <t>"As young as you can catch them; waste management should be in the education system; Reduce ignorance" (Q10 follow-up) calls for future awareness/education efforts.</t>
+          <t>"First policy EPR" listed as the top future policy priority (Q8 notes); "producers (EPR)" named as a target group (Q9).</t>
         </is>
       </c>
     </row>
@@ -9875,7 +9875,7 @@
       </c>
       <c r="C208" s="5" t="inlineStr">
         <is>
-          <t>Sol_recycling</t>
+          <t>Sol_awareness</t>
         </is>
       </c>
       <c r="D208" s="5" t="inlineStr">
@@ -9885,7 +9885,7 @@
       </c>
       <c r="E208" s="5" t="inlineStr">
         <is>
-          <t>"Processing treatment/recycling" listed as a needed future policy focus (Q8 notes); "policies to export recycling produces" (Q10 notes).</t>
+          <t>"As young as you can catch them; waste management should be in the education system; Reduce ignorance" (Q10 follow-up) calls for future awareness/education efforts.</t>
         </is>
       </c>
     </row>
@@ -9902,7 +9902,7 @@
       </c>
       <c r="C209" s="5" t="inlineStr">
         <is>
-          <t>Sol_education</t>
+          <t>Sol_recycling</t>
         </is>
       </c>
       <c r="D209" s="5" t="inlineStr">
@@ -9912,7 +9912,7 @@
       </c>
       <c r="E209" s="5" t="inlineStr">
         <is>
-          <t>"Waste management should be in the education system" (Q10 follow-up) - explicit proposed solution.</t>
+          <t>"Processing treatment/recycling" listed as a needed future policy focus (Q8 notes); "policies to export recycling produces" (Q10 notes).</t>
         </is>
       </c>
     </row>
@@ -9929,7 +9929,7 @@
       </c>
       <c r="C210" s="5" t="inlineStr">
         <is>
-          <t>Sol_capacity</t>
+          <t>Sol_education</t>
         </is>
       </c>
       <c r="D210" s="5" t="inlineStr">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="E210" s="5" t="inlineStr">
         <is>
-          <t>"Technology transfer, do not reinvent the wheel" (Q10 notes) proposes building capacity via external knowledge/technology transfer rather than developing everything from scratch.</t>
+          <t>"Waste management should be in the education system" (Q10 follow-up) - explicit proposed solution.</t>
         </is>
       </c>
     </row>
@@ -9956,7 +9956,7 @@
       </c>
       <c r="C211" s="5" t="inlineStr">
         <is>
-          <t>Sol_ban</t>
+          <t>Sol_capacity</t>
         </is>
       </c>
       <c r="D211" s="5" t="inlineStr">
@@ -9966,7 +9966,7 @@
       </c>
       <c r="E211" s="5" t="inlineStr">
         <is>
-          <t>Plan to progressively raise the minimum plastic thickness standard ("we plan to increase it to 75 microns - possibly [beyond]... previously it was 20 microns, then upgraded to 40, and now the goal is 75 microns") as a strengthened ban/standard going forward.</t>
+          <t>"Technology transfer, do not reinvent the wheel" (Q10 notes) proposes building capacity via external knowledge/technology transfer rather than developing everything from scratch.</t>
         </is>
       </c>
     </row>
@@ -9983,7 +9983,7 @@
       </c>
       <c r="C212" s="5" t="inlineStr">
         <is>
-          <t>Sol_finance</t>
+          <t>Sol_ban</t>
         </is>
       </c>
       <c r="D212" s="5" t="inlineStr">
@@ -9993,7 +9993,7 @@
       </c>
       <c r="E212" s="5" t="inlineStr">
         <is>
-          <t>"Subsidies should be provided to the plastic industry, especially to increase plastic thickness"; "government subsidizing companies producing alternatives" endorsed as "perhaps" a good opportunity; Q10 notes call for "financing" for collection chains and recycling facilities.</t>
+          <t>Plan to progressively raise the minimum plastic thickness standard ("we plan to increase it to 75 microns - possibly [beyond]... previously it was 20 microns, then upgraded to 40, and now the goal is 75 microns") as a strengthened ban/standard going forward.</t>
         </is>
       </c>
     </row>
@@ -10010,7 +10010,7 @@
       </c>
       <c r="C213" s="5" t="inlineStr">
         <is>
-          <t>Sol_infrastructure</t>
+          <t>Sol_finance</t>
         </is>
       </c>
       <c r="D213" s="5" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="E213" s="5" t="inlineStr">
         <is>
-          <t>"If we get the land, we can [establish an] MRF... recycle"; call for national/provincial government help "to identify suitable locations... for plastic recovery and management facilities"; UNDP MoU for "mechanized plastic recovery and storage systems."</t>
+          <t>"Subsidies should be provided to the plastic industry, especially to increase plastic thickness"; "government subsidizing companies producing alternatives" endorsed as "perhaps" a good opportunity; Q10 notes call for "financing" for collection chains and recycling facilities.</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10037,7 @@
       </c>
       <c r="C214" s="5" t="inlineStr">
         <is>
-          <t>Sol_subsitutes</t>
+          <t>Sol_infrastructure</t>
         </is>
       </c>
       <c r="D214" s="5" t="inlineStr">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="E214" s="5" t="inlineStr">
         <is>
-          <t>"Government subsidizing companies producing alternatives is a good opportunity - Yes, perhaps", discussed in relation to scaling up leaf-plate (lobti) style alternatives that are currently too expensive for widespread use.</t>
+          <t>"If we get the land, we can [establish an] MRF... recycle"; call for national/provincial government help "to identify suitable locations... for plastic recovery and management facilities"; UNDP MoU for "mechanized plastic recovery and storage systems."</t>
         </is>
       </c>
     </row>
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C215" s="5" t="inlineStr">
         <is>
-          <t>Sol_enforcement</t>
+          <t>Sol_subsitutes</t>
         </is>
       </c>
       <c r="D215" s="5" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="E215" s="5" t="inlineStr">
         <is>
-          <t>"Regular field inspections are needed" - explicit proposed enforcement solution to address the currently weak enforcement of the micron ban.</t>
+          <t>"Government subsidizing companies producing alternatives is a good opportunity - Yes, perhaps", discussed in relation to scaling up leaf-plate (lobti) style alternatives that are currently too expensive for widespread use.</t>
         </is>
       </c>
     </row>
@@ -10091,7 +10091,7 @@
       </c>
       <c r="C216" s="5" t="inlineStr">
         <is>
-          <t>Sol_monitoring</t>
+          <t>Sol_enforcement</t>
         </is>
       </c>
       <c r="D216" s="5" t="inlineStr">
@@ -10101,7 +10101,7 @@
       </c>
       <c r="E216" s="5" t="inlineStr">
         <is>
-          <t>Tied to the same call for "regular field inspections" and the acknowledged lack of assessment of policy effectiveness, implying a need for stronger ongoing monitoring going forward.</t>
+          <t>"Regular field inspections are needed" - explicit proposed enforcement solution to address the currently weak enforcement of the micron ban.</t>
         </is>
       </c>
     </row>
@@ -10118,15 +10118,42 @@
       </c>
       <c r="C217" s="5" t="inlineStr">
         <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D217" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>Tied to the same call for "regular field inspections" and the acknowledged lack of assessment of policy effectiveness, implying a need for stronger ongoing monitoring going forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="5" t="inlineStr">
+        <is>
+          <t>NPL_4</t>
+        </is>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (KMC), Solid Waste Management Office - Municipality Officer(s), Kathmandu (23 June)</t>
+        </is>
+      </c>
+      <c r="C218" s="5" t="inlineStr">
+        <is>
           <t>Traditions to build on (free-hand)</t>
         </is>
       </c>
-      <c r="D217" s="5" t="inlineStr">
+      <c r="D218" s="5" t="inlineStr">
         <is>
           <t>When asked directly, the interviewee initially said no specific tradition came to mind, but then described "lobti" - leaf plates used at some Kathmandu community festivals instead of plastic plates. Effective at cutting plastic use at large gatherings, but costly (~20 rupees/piece vs. much cheaper plastic), so currently only used by wealthier groups; the interviewee agreed government subsidies for producers of such alternatives could help scale this practice.</t>
         </is>
       </c>
-      <c r="E217" s="5" t="inlineStr">
+      <c r="E218" s="5" t="inlineStr">
         <is>
           <t>When first asked directly about traditional practices (in a Bhutan-comparison framing), the interviewee said "No." But later, when the question was revisited, described "lobti" - leaf plates used in some Kathmandu community festivals instead of plastic ones - as an existing, if underused and costly (20 rupees/piece), alternative practice.</t>
         </is>

</xml_diff>

<commit_message>
Code NPL_9 Dhulikhel ward office interview
Add Dhulikhel Municipality ward-level interview (Ward Head and staff)
as NPL_9 from full notes and transcript. Codes street-level local
government perspectives on weak implementation, no source segregation,
municipal waste contracting, cloth-bag campaigns, Tol Sudhar Samiti,
and Ward No. 2 agricultural/health impacts from the Ward No. 8 dumping
site. NPF victims, villains and hero documented as implied.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -62,44 +62,50 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD9A2"/>
-        <bgColor rgb="00EBD9A2"/>
+        <fgColor rgb="00EBD3A2"/>
+        <bgColor rgb="00EBD3A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EBA2"/>
-        <bgColor rgb="00C6EBA2"/>
+        <fgColor rgb="00D3EBA2"/>
+        <bgColor rgb="00D3EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBB4"/>
-        <bgColor rgb="00A2EBB4"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBD3"/>
+        <bgColor rgb="00A2EBD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2B4EB"/>
-        <bgColor rgb="00A2B4EB"/>
+        <fgColor rgb="00A2D3EB"/>
+        <bgColor rgb="00A2D3EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6A2EB"/>
-        <bgColor rgb="00C6A2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D9"/>
-        <bgColor rgb="00EBA2D9"/>
+        <fgColor rgb="00D3A2EB"/>
+        <bgColor rgb="00D3A2EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2D3"/>
+        <bgColor rgb="00EBA2D3"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -168,6 +174,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -535,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -554,7 +563,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_8, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_9, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -625,82 +634,89 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  9. NPL_9 - Dhulikhel Municipality Ward Office, Ward Head + ward staff (E, Deep, F), Dhulikhel. Master list label: Ward no. 1; transcript focal ward: Ward No. 2. Interviewers: Ram Devi (Kathmandu University) and PEGO team. Coded from both the interview guideline notes and the full verbatim transcript.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_8, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_9, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_8) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_9) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1887,7 +1903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ9"/>
+  <dimension ref="A1:CQ10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6280,6 +6296,483 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>agriculture (plastic in farmlands, severely affected farmland fertility in Ward No. 2), rivers and canals (blockages), health (plastic bottles; open syringes along Panchkhal stream; medical/hazardous waste mismanagement), lower settlements (dumping-site runoff due to topography), lifestyle (everything packaged in plastic)</t>
+        </is>
+      </c>
+      <c r="P10" s="14" t="inlineStr">
+        <is>
+          <t>farmers and residents of Wards No. 2 and 3 (most affected by the Ward No. 8 dumping site; farmland fertility loss); lower settlements downstream of the dumping site; the general public/households (health risks from plastic use and waste, including syringe scavenging); rivers and agricultural environments in Ward No. 2</t>
+        </is>
+      </c>
+      <c r="Q10" s="14" t="inlineStr">
+        <is>
+          <t>the general public/households (lack of awareness, casual plastic use, not following syringe-collection guidance); factories (resisted the micron-thickness ban, no follow-through); hotels, shops and restaurants (prioritised quick profits over cloth-bag and anti-plastic-container campaigns); the municipality (collects annual cleaning taxes but weak execution; no segregation in collection vehicles; unclear allocation of funds across 12 wards); people who collect syringes and other waste materials to sell</t>
+        </is>
+      </c>
+      <c r="R10" s="14" t="inlineStr">
+        <is>
+          <t>the ward office as first contact point and coordinator (Tol Sudhar Samiti pilot projects, Environment Day rallies, awareness activities with limited ward funds); Dhulikhel Hospital/nursing college (cloth-bag campaign — ~1,000 bags to hotels/shops); former ETPC NGO (household waste collection); Tribhuvan University (market-area development collaboration); researchers/universities invited to support awareness and continue efforts</t>
+        </is>
+      </c>
+      <c r="S10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AW10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AX10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA10" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BB10" s="14" t="inlineStr">
+        <is>
+          <t>The ward can coordinate grassroots activities through Tol Sudhar Samiti (~100–150 households per committee), run awareness activities from limited ward funds, act as first contact for NGO/researcher collaborations, and report problems to the municipality — but has no separate waste-management budget, no authority over municipal collection trucks, and no manpower or materials to segregate or manage waste independently.</t>
+        </is>
+      </c>
+      <c r="BC10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI10" s="14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BP10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BS10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW10" s="14" t="inlineStr">
+        <is>
+          <t>"Policies exist only on paper; they are not implemented"; "The local government collects annual cleaning taxes from us yearly, but there's no effective execution"; "The government tried to make a rule but couldn't enforce it" (micron ban introduced ~3–4 years ago but factories resisted); "No, everything collected in the vehicles goes together" — no source segregation in practice.</t>
+        </is>
+      </c>
+      <c r="BX10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI10" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CN10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO10" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP10" s="14" t="inlineStr">
+        <is>
+          <t>Baskets made from paper or bamboo; meat wrapped in straw bundles; large reusable cloth bags for carrying goods; earlier practice of carrying items in reusable bags before plastic became common.</t>
+        </is>
+      </c>
+      <c r="CQ10" s="14" t="inlineStr">
+        <is>
+          <t>Master list label: "9. Dhulikhel Ward no.1", affiliation: Dhulikhel Municipality - Ward No. 1. However, the transcript consistently identifies the respondents' focal ward as Ward No. 2 (e.g. plastic in farmlands and rivers in Ward No. 2; Wards 2 and 3 most affected by dumping site in Ward No. 8). Interviewees: Ward Head (name not given), E, Deep and F (ward/municipal staff; exact roles not fully identified). Interviewers: Ram Devi (Kathmandu University researcher) and PEGO project team. Location: Dhulikhel. Coded from both the interview guideline notes and the full verbatim transcript. NPF fields: victims, villains and hero are not named using explicit NPF narrative labels but are clearly implied (see Coding_Explanations). Hospital collaboration refers to Dhulikhel Hospital; ETPC = Environment Tourism Committee (former NGO).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6291,7 +6784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E622"/>
+  <dimension ref="A1:E701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23095,6 +23588,2139 @@
         </is>
       </c>
     </row>
+    <row r="623">
+      <c r="A623" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B623" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C623" s="14" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D623" s="14" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="E623" s="14" t="inlineStr">
+        <is>
+          <t>Interview conducted at the Dhulikhel Municipality ward office with the Ward Head and ward/municipal staff — coded as loc_government (ward-level local government).</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B624" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C624" s="14" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D624" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E624" s="14" t="inlineStr">
+        <is>
+          <t>"People don't understand, they just collect and store waste, unaware of the consequences"; "People treat plastic casually"; "The biggest challenge is education. Until the community itself becomes aware, no matter how many programs we run, it won't work."</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B625" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C625" s="14" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D625" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E625" s="14" t="inlineStr">
+        <is>
+          <t>"Policies exist only on paper; they are not implemented"; ward lacks authority and resources to act on national/municipal rules; "some matters fall under higher authorities, we haven't been able to act effectively."</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B626" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C626" s="14" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D626" s="14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E626" s="14" t="inlineStr">
+        <is>
+          <t>"It's a major problem"; "Plastic is creating severe problems here"; "Plastic has become a serious issue regarding waste"; "Plastic has severely affected farmland fertility."</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B627" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C627" s="14" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D627" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E627" s="14" t="inlineStr">
+        <is>
+          <t>Open syringes found along the Panchkhal stream; waste dumped at one site; dumping-site runoff affecting lower settlements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B628" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C628" s="14" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D628" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E628" s="14" t="inlineStr">
+        <is>
+          <t>"Everything now comes packaged in plastic"; "Plastic is convenient and cheap for just 1 rupee"; even if households avoid bringing plastic home, food products always arrive in plastic packaging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B629" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C629" s="14" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D629" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E629" s="14" t="inlineStr">
+        <is>
+          <t>Former ETPC NGO collected household waste but could not sustain operations; no systematic recycling at ward level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B630" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C630" s="14" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D630" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E630" s="14" t="inlineStr">
+        <is>
+          <t>"The implementation aspect is weak"; waste collected twice a week and dumped at one site; ward tried hospital collaboration but "couldn't succeed"; no ward-level systematic framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B631" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C631" s="14" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D631" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E631" s="14" t="inlineStr">
+        <is>
+          <t>"There's no monitoring of what kind of plastic is being produced or used"; factories resisted the micron ban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B632" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C632" s="14" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D632" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E632" s="14" t="inlineStr">
+        <is>
+          <t>"We don't have affordable alternatives"; without alternatives "it's difficult to stop its use."</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B633" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C633" s="14" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D633" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E633" s="14" t="inlineStr">
+        <is>
+          <t>"No, everything collected in the vehicles goes together"; "Exactly" — no source segregation; "Some segregation happens later, but not properly."</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B634" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C634" s="14" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D634" s="14" t="inlineStr">
+        <is>
+          <t>agriculture (plastic in farmlands, severely affected farmland fertility in Ward No. 2), rivers and canals (blockages), health (plastic bottles; open syringes along Panchkhal stream; medical/hazardous waste mismanagement), lower settlements (dumping-site runoff due to topography), lifestyle (everything packaged in plastic)</t>
+        </is>
+      </c>
+      <c r="E634" s="14" t="inlineStr">
+        <is>
+          <t>Plastic in Ward No. 2 farmlands and rivers; canal blockages; farmland fertility loss; health concerns (plastic bottles; syringes); dumping-site runoff to lower settlements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B635" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C635" s="14" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D635" s="14" t="inlineStr">
+        <is>
+          <t>farmers and residents of Wards No. 2 and 3 (most affected by the Ward No. 8 dumping site; farmland fertility loss); lower settlements downstream of the dumping site; the general public/households (health risks from plastic use and waste, including syringe scavenging); rivers and agricultural environments in Ward No. 2</t>
+        </is>
+      </c>
+      <c r="E635" s="14" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: farmers and residents of Wards 2 and 3 (dumping site in Ward 8); lower settlements affected by runoff; households/public facing health risks; rivers and agricultural land in Ward No. 2. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B636" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C636" s="14" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D636" s="14" t="inlineStr">
+        <is>
+          <t>the general public/households (lack of awareness, casual plastic use, not following syringe-collection guidance); factories (resisted the micron-thickness ban, no follow-through); hotels, shops and restaurants (prioritised quick profits over cloth-bag and anti-plastic-container campaigns); the municipality (collects annual cleaning taxes but weak execution; no segregation in collection vehicles; unclear allocation of funds across 12 wards); people who collect syringes and other waste materials to sell</t>
+        </is>
+      </c>
+      <c r="E636" s="14" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: unaware/casual public; factories resisting the ban; profit-prioritising hotels/restaurants/shops; municipality with weak implementation; syringe scavengers. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B637" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C637" s="14" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D637" s="14" t="inlineStr">
+        <is>
+          <t>the ward office as first contact point and coordinator (Tol Sudhar Samiti pilot projects, Environment Day rallies, awareness activities with limited ward funds); Dhulikhel Hospital/nursing college (cloth-bag campaign — ~1,000 bags to hotels/shops); former ETPC NGO (household waste collection); Tribhuvan University (market-area development collaboration); researchers/universities invited to support awareness and continue efforts</t>
+        </is>
+      </c>
+      <c r="E637" s="14" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: ward office (coordination, awareness, Tol Sudhar Samiti); hospital/nursing-college cloth-bag campaign; ETPC; Tribhuvan University; researchers. Ward partly positions itself and partners as problem-solvers despite limited capacity. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B638" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C638" s="14" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D638" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E638" s="14" t="inlineStr">
+        <is>
+          <t>Ward coordinated with nursing college and Dhulikhel Hospital (cloth bags), ETPC (waste collection), Tol Sudhar Samiti (grassroots), Tribhuvan University (market development), and welcomes researcher collaboration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B639" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C639" s="14" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D639" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E639" s="14" t="inlineStr">
+        <is>
+          <t>Waste management contracted at municipality level; ward reports problems to municipality but has no separate budget or authority; "difficult to control from the ward level alone."</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B640" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C640" s="14" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D640" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E640" s="14" t="inlineStr">
+        <is>
+          <t>Ward says plastic management is within its responsibility but matters fall under higher authorities; residents pay municipal cleaning fees but "we don't know exactly how funds are distributed among the 12 wards."</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B641" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C641" s="14" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D641" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E641" s="14" t="inlineStr">
+        <is>
+          <t>National/municipal rules on micron-thickness bans cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B642" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C642" s="14" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D642" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E642" s="14" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B643" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C643" s="14" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D643" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E643" s="14" t="inlineStr">
+        <is>
+          <t>Municipality contracts waste management to a company, collects revenue and manages disposal; ward reports problems upward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B644" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C644" s="14" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D644" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E644" s="14" t="inlineStr">
+        <is>
+          <t>NA - students not named as responsible actors (nursing college is an institution, coded under Res_edu_institutions).</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B645" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C645" s="14" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D645" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E645" s="14" t="inlineStr">
+        <is>
+          <t>Waste-management company contracted by municipality; private companies proposed to collect household waste for a fee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B646" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C646" s="14" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D646" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E646" s="14" t="inlineStr">
+        <is>
+          <t>ETPC formerly collected waste; Tol Sudhar Samiti operates under ward guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B647" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C647" s="14" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D647" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E647" s="14" t="inlineStr">
+        <is>
+          <t>Researchers (Kathmandu University team) and Tribhuvan University collaboration welcomed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B648" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C648" s="14" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D648" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E648" s="14" t="inlineStr">
+        <is>
+          <t>"Plastic originates from households"; households should separate waste at home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B649" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C649" s="14" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D649" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E649" s="14" t="inlineStr">
+        <is>
+          <t>Nursing college partnered on cloth-bag distribution; Tribhuvan University coordinating on market-area development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B650" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C650" s="14" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D650" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E650" s="14" t="inlineStr">
+        <is>
+          <t>Hotels, shops and restaurants targeted in anti-plastic campaigns; businesses generate plastic waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B651" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C651" s="14" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D651" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E651" s="14" t="inlineStr">
+        <is>
+          <t>"The government tried to make a rule but couldn't enforce it"; policies exist on paper only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B652" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C652" s="14" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D652" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E652" s="14" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B653" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C653" s="14" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D653" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E653" s="14" t="inlineStr">
+        <is>
+          <t>Municipality collects annual cleaning taxes but "there's no effective execution"; unclear fund allocation to wards; collection vehicles mix all waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B654" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C654" s="14" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D654" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E654" s="14" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B655" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C655" s="14" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D655" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E655" s="14" t="inlineStr">
+        <is>
+          <t>NA - private waste contractor not blamed; private collection proposed as solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B656" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C656" s="14" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D656" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E656" s="14" t="inlineStr">
+        <is>
+          <t>NA - NGOs not blamed (ETPC lacked resources).</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B657" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C657" s="14" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D657" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E657" s="14" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B658" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C658" s="14" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D658" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E658" s="14" t="inlineStr">
+        <is>
+          <t>Public lacks awareness; people store waste without understanding consequences; historically throw waste expecting municipality to clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B659" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C659" s="14" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D659" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E659" s="14" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B660" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C660" s="14" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D660" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E660" s="14" t="inlineStr">
+        <is>
+          <t>Restaurants continued serving food in plastic containers; businesses "prioritized quick profits"; campaigns could not continue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B661" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C661" s="14" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D661" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E661" s="14" t="inlineStr">
+        <is>
+          <t>Strict policy enforcement of micron ban cited as one of three essentials alongside awareness and resources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B662" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C662" s="14" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D662" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E662" s="14" t="inlineStr">
+        <is>
+          <t>NA - not named as target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B663" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C663" s="14" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D663" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E663" s="14" t="inlineStr">
+        <is>
+          <t>Deep argues ward should implement rules like road building; municipality must improve execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B664" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C664" s="14" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D664" s="14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E664" s="14" t="inlineStr">
+        <is>
+          <t>NA - not named as target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B665" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C665" s="14" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D665" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E665" s="14" t="inlineStr">
+        <is>
+          <t>Private companies could collect segregated waste from households for a fee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B666" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C666" s="14" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D666" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E666" s="14" t="inlineStr">
+        <is>
+          <t>Tol Sudhar Samiti and NGOs suggested for pilot projects and awareness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B667" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C667" s="14" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D667" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E667" s="14" t="inlineStr">
+        <is>
+          <t>Researchers invited to support and continue ward efforts after the study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B668" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C668" s="14" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D668" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E668" s="14" t="inlineStr">
+        <is>
+          <t>Awareness and household source segregation emphasised as essential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B669" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C669" s="14" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D669" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E669" s="14" t="inlineStr">
+        <is>
+          <t>Nursing college involved in distribution campaign; TU collaboration planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B670" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C670" s="14" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D670" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E670" s="14" t="inlineStr">
+        <is>
+          <t>Hotels, shops and restaurants were direct targets of the cloth-bag and anti-plastic-container campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B671" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C671" s="14" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D671" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E671" s="14" t="inlineStr">
+        <is>
+          <t>Ward Head and staff describe grassroots coordination, Tol Sudhar Samiti guidance, awareness rallies and reporting to the municipality — typical street-level/local implementer role (3), not national policy formulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B672" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C672" s="14" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D672" s="14" t="inlineStr">
+        <is>
+          <t>The ward can coordinate grassroots activities through Tol Sudhar Samiti (~100–150 households per committee), run awareness activities from limited ward funds, act as first contact for NGO/researcher collaborations, and report problems to the municipality — but has no separate waste-management budget, no authority over municipal collection trucks, and no manpower or materials to segregate or manage waste independently.</t>
+        </is>
+      </c>
+      <c r="E672" s="14" t="inlineStr">
+        <is>
+          <t>Ward can run awareness with limited funds and coordinate pilots through Tol Sudhar Samiti, but cannot control municipal trucks, segregation, dumping-site location (Ward 8) or waste-contractor operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B673" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C673" s="14" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D673" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E673" s="14" t="inlineStr">
+        <is>
+          <t>"There's no monitoring of what kind of plastic is being produced or used"; ban not enforced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B674" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C674" s="14" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D674" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E674" s="14" t="inlineStr">
+        <is>
+          <t>Ward receives no separate waste-management budget; lacks resources and manpower despite residents paying municipal cleaning fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B675" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C675" s="14" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D675" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E675" s="14" t="inlineStr">
+        <is>
+          <t>Ward Head requests researcher suggestions to improve waste management; TU collaboration discussed; researchers welcomed to continue efforts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B676" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C676" s="14" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D676" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E676" s="14" t="inlineStr">
+        <is>
+          <t>Ward has no own dumping site (site in Ward No. 8); topography causes runoff affecting Wards 2 and 3; hospital lacks own dumping site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B677" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C677" s="14" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D677" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E677" s="14" t="inlineStr">
+        <is>
+          <t>"The ward lacks both resources and manpower"; no right, manpower or materials to manage waste separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B678" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C678" s="14" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D678" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E678" s="14" t="inlineStr">
+        <is>
+          <t>Micron ban and municipal rules not enforced; factories resisted; ward lacks authority to enforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B679" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C679" s="14" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D679" s="14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E679" s="14" t="inlineStr">
+        <is>
+          <t>Extended producer responsibility not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B680" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C680" s="14" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D680" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E680" s="14" t="inlineStr">
+        <is>
+          <t>Environment Day rallies; cloth-bag campaign with nursing college; syringe-collection awareness ~8–10 years ago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B681" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C681" s="14" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D681" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E681" s="14" t="inlineStr">
+        <is>
+          <t>"The biggest challenge is education"; awareness essential for long-term control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B682" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C682" s="14" t="inlineStr">
+        <is>
+          <t>Pol_tax</t>
+        </is>
+      </c>
+      <c r="D682" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E682" s="14" t="inlineStr">
+        <is>
+          <t>Annual cleaning taxes/fees collected by the municipality from residents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B683" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C683" s="14" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D683" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E683" s="14" t="inlineStr">
+        <is>
+          <t>Plastics below a certain micron thickness banned (~3–4 years ago; 40 microns referenced in discussion).</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B684" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C684" s="14" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D684" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E684" s="14" t="inlineStr">
+        <is>
+          <t>Cloth-bag distribution campaign (~1,000 bags to hotels and shops).</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B685" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C685" s="14" t="inlineStr">
+        <is>
+          <t>Pol_clean_up</t>
+        </is>
+      </c>
+      <c r="D685" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E685" s="14" t="inlineStr">
+        <is>
+          <t>Environment Day observed with rallies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B686" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C686" s="14" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D686" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E686" s="14" t="inlineStr">
+        <is>
+          <t>Household waste collected twice a week by municipal contractor and dumped at one site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B687" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C687" s="14" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D687" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E687" s="14" t="inlineStr">
+        <is>
+          <t>Implementation weak; policies on paper; ban not enforced; no segregation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B688" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C688" s="14" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D688" s="14" t="inlineStr">
+        <is>
+          <t>"Policies exist only on paper; they are not implemented"; "The local government collects annual cleaning taxes from us yearly, but there's no effective execution"; "The government tried to make a rule but couldn't enforce it" (micron ban introduced ~3–4 years ago but factories resisted); "No, everything collected in the vehicles goes together" — no source segregation in practice.</t>
+        </is>
+      </c>
+      <c r="E688" s="14" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B689" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C689" s="14" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D689" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E689" s="14" t="inlineStr">
+        <is>
+          <t>Ward as first contact point for collaborations; Tol Sudhar Samiti for neighbourhood pilots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B690" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C690" s="14" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D690" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E690" s="14" t="inlineStr">
+        <is>
+          <t>Three essentials: public awareness, proper resources, strict policy enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B691" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C691" s="14" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D691" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E691" s="14" t="inlineStr">
+        <is>
+          <t>Awareness campaigns, Environment Day, cloth-bag distribution, researcher-supported awareness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B692" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C692" s="14" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D692" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E692" s="14" t="inlineStr">
+        <is>
+          <t>Household source segregation and separate bins/cloth bags proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B693" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C693" s="14" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D693" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E693" s="14" t="inlineStr">
+        <is>
+          <t>Community education emphasised as prerequisite for any programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B694" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C694" s="14" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D694" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E694" s="14" t="inlineStr">
+        <is>
+          <t>Technical and resource support needed for ward and municipal implementers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B695" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C695" s="14" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D695" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E695" s="14" t="inlineStr">
+        <is>
+          <t>Ward funds used for awareness; calls for clearer municipal budget allocation; private collection for a fee proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B696" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C696" s="14" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D696" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E696" s="14" t="inlineStr">
+        <is>
+          <t>Separate bins at household level; ward lacks own disposal site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B697" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C697" s="14" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D697" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E697" s="14" t="inlineStr">
+        <is>
+          <t>Cloth bags, bamboo/paper baskets, straw bundles for meat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B698" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C698" s="14" t="inlineStr">
+        <is>
+          <t>Sol_clean_up</t>
+        </is>
+      </c>
+      <c r="D698" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E698" s="14" t="inlineStr">
+        <is>
+          <t>Environment Day rallies; small-scale ward activities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B699" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C699" s="14" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D699" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E699" s="14" t="inlineStr">
+        <is>
+          <t>Strict policy enforcement named as essential alongside awareness and resources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B700" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C700" s="14" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D700" s="14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E700" s="14" t="inlineStr">
+        <is>
+          <t>Implied need to monitor plastic production and usage (currently absent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="14" t="inlineStr">
+        <is>
+          <t>NPL_9</t>
+        </is>
+      </c>
+      <c r="B701" s="14" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality Ward Office - Ward Head + ward staff (E, Deep, F), Dhulikhel (Ward No. 2 per transcript; master list: Ward no. 1)</t>
+        </is>
+      </c>
+      <c r="C701" s="14" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D701" s="14" t="inlineStr">
+        <is>
+          <t>Baskets made from paper or bamboo; meat wrapped in straw bundles; large reusable cloth bags for carrying goods; earlier practice of carrying items in reusable bags before plastic became common.</t>
+        </is>
+      </c>
+      <c r="E701" s="14" t="inlineStr">
+        <is>
+          <t>Bamboo/paper baskets, straw-wrapped meat, large reusable cloth bags — pre-plastic carrying practices.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Code NPL_10 Dhulikhel ward chairman interview
Add long-serving Dhulikhel ward chairman (32 years, five terms) as
NPL_10 from verbatim transcript. Codes weak federal-local coordination,
door-to-door container programme failures, Sunday plastic collection,
transfer-station planning in Ward No. 3, and implied NPF framing.

Exclude structured theme notes at top of source file (Bio-Camp, Plast
Foundation, EPR policy bullets) as they do not appear in this transcript.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -62,50 +62,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD3A2"/>
-        <bgColor rgb="00EBD3A2"/>
+        <fgColor rgb="00EBCEA2"/>
+        <bgColor rgb="00EBCEA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3EBA2"/>
-        <bgColor rgb="00D3EBA2"/>
+        <fgColor rgb="00DCEBA2"/>
+        <bgColor rgb="00DCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA2"/>
-        <bgColor rgb="00A2EBA2"/>
+        <fgColor rgb="00B1EBA2"/>
+        <bgColor rgb="00B1EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD3"/>
-        <bgColor rgb="00A2EBD3"/>
+        <fgColor rgb="00A2EBBF"/>
+        <bgColor rgb="00A2EBBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D3EB"/>
-        <bgColor rgb="00A2D3EB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A2EB"/>
-        <bgColor rgb="00A2A2EB"/>
+        <fgColor rgb="00A2BFEB"/>
+        <bgColor rgb="00A2BFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3A2EB"/>
-        <bgColor rgb="00D3A2EB"/>
+        <fgColor rgb="00B1A2EB"/>
+        <bgColor rgb="00B1A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D3"/>
-        <bgColor rgb="00EBA2D3"/>
+        <fgColor rgb="00DCA2EB"/>
+        <bgColor rgb="00DCA2EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2CE"/>
+        <bgColor rgb="00EBA2CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -135,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -177,6 +183,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -544,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -563,7 +572,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_9, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_10, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -641,82 +650,89 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  10. NPL_10 - Dhulikhel Municipality Ward Chairman (32 years, five terms), Dhulikhel. Master list label: Ward no. 7; transcript focal ward: Ward No. 3 (Thakuri village transfer-station planning). Interviewers: Ram Devi (Kathmandu University), Deep and F. Coded from the verbatim transcript; structured theme notes at the top of the source file (Bio-Camp, Plast Foundation, EPR policy content) excluded as they do not appear in this transcript.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_9, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_10, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_9) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_10) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
-    </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1903,7 +1919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ10"/>
+  <dimension ref="A1:CQ11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6773,6 +6789,483 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O11" s="15" t="inlineStr">
+        <is>
+          <t>rivers and riverbanks (Panchkhal area; Bagmati waste through pipelines; "no good river in Nepal"), smell affecting residents daily (including near the ward chairman's house), ecosystem described as "already destroyed", dust and visual pollution ("everywhere is dusty"), tourism/national image (embarrassment compared with Switzerland), waste still reaching rivers despite collection efforts</t>
+        </is>
+      </c>
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>local residents and downstream communities (daily smell, Panchkhal negative impacts); rivers and the broader environment/ecosystem; Nepal's national image ("people call Nepal a beautiful country, like Switzerland, but everywhere is dusty")</t>
+        </is>
+      </c>
+      <c r="Q11" s="15" t="inlineStr">
+        <is>
+          <t>households/residents who leave plastic outside despite distributed containers, throw waste in forests, and fail to cooperate with segregation; the central/federal government ("big gap" with local government, slow progress, no master plans, draft act not reaching wards); pervasive plastic use in food packaging and single-use items without affordable systemic alternatives</t>
+        </is>
+      </c>
+      <c r="R11" s="15" t="inlineStr">
+        <is>
+          <t>the ward chairman personally (model zero-waste household behaviour, picks up litter, organic diet); Dhulikhel Municipality (segregating plastic and composting organic waste, transfer-station/landfill plan passed, contracting waste collection); Bhutan cited as an awareness example; researchers to find plastic alternatives; 2–4 workers separating recyclables at the dumping/refining site; international donors on Bagmati (World Bank, ADB)</t>
+        </is>
+      </c>
+      <c r="S11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AX11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA11" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BB11" s="15" t="inlineStr">
+        <is>
+          <t>As elected ward chairman (32 years, five terms) he supervises dumping sites, ran door-to-door container programmes, coordinates directly with the municipality on contractor arrangements, and requests land from the Nepal government — but has no formal ward-level waste-management staff, no separate ward budget (municipality contracts fund collection), and processing-company agreements were terminated.</t>
+        </is>
+      </c>
+      <c r="BC11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI11" s="15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BS11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW11" s="15" t="inlineStr">
+        <is>
+          <t>Door-to-door household containers "wasn't enough" because people left plastic outside; processing-company agreements "were terminated"; despite Sunday plastic collection and refining (Rs 10–15/kg), "even if there's a collection problem here, it still ends up in the river"; "now there's a big gap between the local and federal governments — they keep making plans and talking, but progress is very slow."</t>
+        </is>
+      </c>
+      <c r="BX11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI11" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CN11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO11" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP11" s="15" t="inlineStr">
+        <is>
+          <t>Baskets made from natural materials; paper bags used for vegetables; cloth bags encouraged; biodegradable vs. non-biodegradable household separation promoted in recent 1–2 year efforts.</t>
+        </is>
+      </c>
+      <c r="CQ11" s="15" t="inlineStr">
+        <is>
+          <t>Master list label: "10. Dhulikhel Ward no.7", affiliation: Dhulikhel Municipality - Ward No. 7. Transcript identifies Ward No. 3 (land-ownership request, transfer-station planning in Thakuri village) and Panchkhal-area impacts. Interviewee: Ward Chairman/Ward Head (name not given), 32 years as ward chairman (five terms). Also present: Ram Devi (Kathmandu University), Deep and F. Location: Dhulikhel. Coded primarily from the full verbatim transcript. DATA-QUALITY NOTE: the structured theme notes at the top of the source document (Bio-Camp pilot, Plast Foundation Nepal, Solid Waste Management Association, EPR nationwide, microplastics in fertilisers, Environmental Protection Act without plastics policy, etc.) do not appear in this ward-head transcript and were excluded as likely belonging to a different interview accidentally bundled in the same file. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6784,7 +7277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E701"/>
+  <dimension ref="A1:E781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -25721,6 +26214,2166 @@
         </is>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B702" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C702" s="15" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D702" s="15" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="E702" s="15" t="inlineStr">
+        <is>
+          <t>Interview with the Dhulikhel Municipality ward chairman/ward head — coded as loc_government (ward-level elected local government).</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B703" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C703" s="15" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D703" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E703" s="15" t="inlineStr">
+        <is>
+          <t>Households left plastic outside despite distributed containers ("they made bags and throw"); waste thrown in forests; awareness improving but cooperation insufficient; Deep: "people won't change as long as they aren't penalized."</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B704" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C704" s="15" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D704" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E704" s="15" t="inlineStr">
+        <is>
+          <t>"Big gap between the local and federal governments"; draft Waste Management Act on webpage but ward "hasn't reached that stage yet"; "there are no master plans made"; central government slow while municipality must act.</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B705" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C705" s="15" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D705" s="15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E705" s="15" t="inlineStr">
+        <is>
+          <t>"Plastic is a very harmful material"; pollution "spread everywhere"; "the ecosystem is already destroyed"; rivers embarrass Nepal internationally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B706" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C706" s="15" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D706" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E706" s="15" t="inlineStr">
+        <is>
+          <t>Plastic spread everywhere; riverbanks covered ~20–30 years of dumping; sweepers collect and dump at open sites; waste thrown in forests despite highway cleaning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B707" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C707" s="15" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D707" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E707" s="15" t="inlineStr">
+        <is>
+          <t>"Plastic is used everywhere, in food packaging, drinking glasses, etc."; fast-food packaging plastics need alternatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B708" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C708" s="15" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D708" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E708" s="15" t="inlineStr">
+        <is>
+          <t>Some refining at Rs 10–15/kg and on-site separation by 2–4 workers, but processing-company agreements terminated; collection still ends in rivers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B709" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C709" s="15" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D709" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E709" s="15" t="inlineStr">
+        <is>
+          <t>20–30 years of dumping; daily smell near residences; waste from Banepa and Okharpauwa; contractor system but gaps remain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B710" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C710" s="15" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D710" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E710" s="15" t="inlineStr">
+        <is>
+          <t>"We also need alternatives to plastic, like the plastic used in fast food packaging"; ward encourages cloth bags and natural materials but systemic alternatives lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B711" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C711" s="15" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D711" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E711" s="15" t="inlineStr">
+        <is>
+          <t>Sunday plastic collection exists but household implementation weak; door-to-door container programme insufficient; Deep proposes separate collection days per waste type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B712" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C712" s="15" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D712" s="15" t="inlineStr">
+        <is>
+          <t>rivers and riverbanks (Panchkhal area; Bagmati waste through pipelines; "no good river in Nepal"), smell affecting residents daily (including near the ward chairman's house), ecosystem described as "already destroyed", dust and visual pollution ("everywhere is dusty"), tourism/national image (embarrassment compared with Switzerland), waste still reaching rivers despite collection efforts</t>
+        </is>
+      </c>
+      <c r="E712" s="15" t="inlineStr">
+        <is>
+          <t>Panchkhal river impacts, daily smell, destroyed ecosystem, dusty landscape, national-image harm, Bagmati pollution despite donor projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B713" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C713" s="15" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D713" s="15" t="inlineStr">
+        <is>
+          <t>local residents and downstream communities (daily smell, Panchkhal negative impacts); rivers and the broader environment/ecosystem; Nepal's national image ("people call Nepal a beautiful country, like Switzerland, but everywhere is dusty")</t>
+        </is>
+      </c>
+      <c r="E713" s="15" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: local residents (smell); rivers/Panchkhal and broader environment; Nepal's international reputation. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B714" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C714" s="15" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D714" s="15" t="inlineStr">
+        <is>
+          <t>households/residents who leave plastic outside despite distributed containers, throw waste in forests, and fail to cooperate with segregation; the central/federal government ("big gap" with local government, slow progress, no master plans, draft act not reaching wards); pervasive plastic use in food packaging and single-use items without affordable systemic alternatives</t>
+        </is>
+      </c>
+      <c r="E714" s="15" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: uncooperative households; slow/weak central government planning; pervasive plastic consumption. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B715" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C715" s="15" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D715" s="15" t="inlineStr">
+        <is>
+          <t>the ward chairman personally (model zero-waste household behaviour, picks up litter, organic diet); Dhulikhel Municipality (segregating plastic and composting organic waste, transfer-station/landfill plan passed, contracting waste collection); Bhutan cited as an awareness example; researchers to find plastic alternatives; 2–4 workers separating recyclables at the dumping/refining site; international donors on Bagmati (World Bank, ADB)</t>
+        </is>
+      </c>
+      <c r="E715" s="15" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: ward chairman as personal model; Dhulikhel Municipality (segregation, transfer station plan); Bhutan awareness example; researchers; site workers separating recyclables; World Bank/ADB on Bagmati. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B716" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C716" s="15" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D716" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E716" s="15" t="inlineStr">
+        <is>
+          <t>Comparisons with Bhutan, Germany, Switzerland and the US; World Bank and Asian Development Bank funding on Bagmati.</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B717" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C717" s="15" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D717" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E717" s="15" t="inlineStr">
+        <is>
+          <t>Municipality contracts private collectors; ward coordinates with municipality; discussed refining with a company (agreements later terminated); 2–4 workers separate recyclables on site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B718" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C718" s="15" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D718" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E718" s="15" t="inlineStr">
+        <is>
+          <t>"Big gap between the local and federal governments"; debate over whether central government or municipality should lead; ward reports to municipality as main authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B719" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C719" s="15" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D719" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E719" s="15" t="inlineStr">
+        <is>
+          <t>RAM DEVI: central doesn't act, falls on municipality; ward head: state must be responsible OR municipality given full power — responsibility contested across levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B720" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C720" s="15" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D720" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E720" s="15" t="inlineStr">
+        <is>
+          <t>Restricts plastic beyond certain size; draft Waste Management Act; Bagmati projects with international donors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B721" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C721" s="15" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D721" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E721" s="15" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B722" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C722" s="15" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D722" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E722" s="15" t="inlineStr">
+        <is>
+          <t>Municipality provides funds through contracts; Dhulikhel segregating plastic and composting; transfer-station plan passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B723" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C723" s="15" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D723" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E723" s="15" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B724" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C724" s="15" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D724" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E724" s="15" t="inlineStr">
+        <is>
+          <t>Contractors collect/refine/manage waste; private companies visit monthly; processing companies (agreements terminated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B725" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C725" s="15" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D725" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E725" s="15" t="inlineStr">
+        <is>
+          <t>NA - not mentioned as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B726" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C726" s="15" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D726" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E726" s="15" t="inlineStr">
+        <is>
+          <t>"Researchers will know how to solve the problem by finding alternatives."</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B727" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C727" s="15" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D727" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E727" s="15" t="inlineStr">
+        <is>
+          <t>Household containers and source separation expected; ward chairman models zero household waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B728" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C728" s="15" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D728" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E728" s="15" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B729" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C729" s="15" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D729" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E729" s="15" t="inlineStr">
+        <is>
+          <t>NA - private collectors coded under Res_private_sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B730" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C730" s="15" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D730" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E730" s="15" t="inlineStr">
+        <is>
+          <t>"They keep making plans and talking, but progress is very slow"; no master plans; gap with local government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B731" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C731" s="15" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D731" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E731" s="15" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B732" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C732" s="15" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D732" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E732" s="15" t="inlineStr">
+        <is>
+          <t>NA - municipality portrayed partly as problem-solver (Dharan/Dhulikhel model), not primary culprit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B733" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C733" s="15" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D733" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E733" s="15" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B734" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C734" s="15" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D734" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E734" s="15" t="inlineStr">
+        <is>
+          <t>NA - contractors not blamed; processing agreements terminated but not framed as villain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B735" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C735" s="15" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D735" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E735" s="15" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B736" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C736" s="15" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D736" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E736" s="15" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B737" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C737" s="15" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D737" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E737" s="15" t="inlineStr">
+        <is>
+          <t>People left plastic outside despite containers; throw waste in forests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B738" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C738" s="15" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D738" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E738" s="15" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B739" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C739" s="15" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D739" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E739" s="15" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B740" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C740" s="15" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D740" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E740" s="15" t="inlineStr">
+        <is>
+          <t>"The state has to be responsible — the central government must take charge"; also calls for municipality to be given full power.</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B741" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C741" s="15" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D741" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E741" s="15" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B742" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C742" s="15" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D742" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E742" s="15" t="inlineStr">
+        <is>
+          <t>Municipality should make laws, set penalties and enforce them; Dhulikhel model like Dharan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B743" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C743" s="15" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D743" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E743" s="15" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B744" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C744" s="15" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D744" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E744" s="15" t="inlineStr">
+        <is>
+          <t>Private companies should collect separately by waste type; contractor improvements suggested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B745" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C745" s="15" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D745" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E745" s="15" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B746" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C746" s="15" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D746" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E746" s="15" t="inlineStr">
+        <is>
+          <t>Researchers to develop plastic alternatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B747" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C747" s="15" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D747" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E747" s="15" t="inlineStr">
+        <is>
+          <t>Door-to-door awareness; household separation of biodegradable and non-biodegradable waste; Germany-style differentiated fees discussed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B748" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C748" s="15" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D748" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E748" s="15" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B749" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C749" s="15" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D749" s="15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E749" s="15" t="inlineStr">
+        <is>
+          <t>NA - not named separately from private sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B750" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C750" s="15" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D750" s="15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E750" s="15" t="inlineStr">
+        <is>
+          <t>Long-serving elected ward chairman describing grassroots supervision, door-to-door programmes, dumping-site management and municipal coordination — street-level/local implementer (3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B751" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C751" s="15" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D751" s="15" t="inlineStr">
+        <is>
+          <t>As elected ward chairman (32 years, five terms) he supervises dumping sites, ran door-to-door container programmes, coordinates directly with the municipality on contractor arrangements, and requests land from the Nepal government — but has no formal ward-level waste-management staff, no separate ward budget (municipality contracts fund collection), and processing-company agreements were terminated.</t>
+        </is>
+      </c>
+      <c r="E751" s="15" t="inlineStr">
+        <is>
+          <t>Supervises dumping areas, distributed household containers, coordinates with municipality on contractors, requested Nepal-government land ownership in Ward No. 3 — but no formal ward waste staff or independent budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B752" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C752" s="15" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D752" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E752" s="15" t="inlineStr">
+        <is>
+          <t>"Cannot monitor 24/7"; people throw waste in forests when unobserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B753" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C753" s="15" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D753" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E753" s="15" t="inlineStr">
+        <is>
+          <t>Land purchase for transfer station difficult ("local people didn't give it freely"); processing agreements terminated; municipality funds via contracts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B754" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C754" s="15" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D754" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E754" s="15" t="inlineStr">
+        <is>
+          <t>Researchers expected to find alternatives to fast-food packaging plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B755" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C755" s="15" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D755" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E755" s="15" t="inlineStr">
+        <is>
+          <t>Transfer station and landfill planned (1–2 years); land in Thakuri village; access roads prepared in Ward No. 3; open dumping ~20–30 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B756" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C756" s="15" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D756" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E756" s="15" t="inlineStr">
+        <is>
+          <t>No designated ward-level waste-management personnel; relies on municipal contracts and 2–4 site workers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B757" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C757" s="15" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D757" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E757" s="15" t="inlineStr">
+        <is>
+          <t>"Enforcement is key. Lawmakers must make strict laws"; penalties and differentiated fees (Germany Rs 200 vs 500 example) needed — "just teaching won't be enough."</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B758" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C758" s="15" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D758" s="15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E758" s="15" t="inlineStr">
+        <is>
+          <t>Extended producer responsibility not mentioned in transcript.</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B759" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C759" s="15" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D759" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E759" s="15" t="inlineStr">
+        <is>
+          <t>Door-to-door programmes; Environment Day source collection and swap system; Bhutan-style public announcements cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B760" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C760" s="15" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D760" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E760" s="15" t="inlineStr">
+        <is>
+          <t>Awareness campaigns; municipal meetings on waste frequently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B761" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C761" s="15" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D761" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E761" s="15" t="inlineStr">
+        <is>
+          <t>"The Nepal government restricts plastic use beyond a certain size."</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B762" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C762" s="15" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D762" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E762" s="15" t="inlineStr">
+        <is>
+          <t>Cloth bags, natural-material baskets, paper bags promoted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B763" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C763" s="15" t="inlineStr">
+        <is>
+          <t>Pol_clean_up</t>
+        </is>
+      </c>
+      <c r="D763" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E763" s="15" t="inlineStr">
+        <is>
+          <t>Sweepers collect plastic; highway cleaning; Environment Day activities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B764" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C764" s="15" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D764" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E764" s="15" t="inlineStr">
+        <is>
+          <t>Plastic/paper/glass separated at site; refining at Rs 10–15/kg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B765" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C765" s="15" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D765" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E765" s="15" t="inlineStr">
+        <is>
+          <t>Sunday plastic collection; monthly private-company visits; trucks whistle to signal collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B766" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C766" s="15" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D766" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E766" s="15" t="inlineStr">
+        <is>
+          <t>Container programme failed; agreements terminated; waste still reaches rivers; federal-local gap slows progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B767" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C767" s="15" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D767" s="15" t="inlineStr">
+        <is>
+          <t>Door-to-door household containers "wasn't enough" because people left plastic outside; processing-company agreements "were terminated"; despite Sunday plastic collection and refining (Rs 10–15/kg), "even if there's a collection problem here, it still ends up in the river"; "now there's a big gap between the local and federal governments — they keep making plans and talking, but progress is very slow."</t>
+        </is>
+      </c>
+      <c r="E767" s="15" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B768" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C768" s="15" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D768" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E768" s="15" t="inlineStr">
+        <is>
+          <t>Central government must take charge OR municipality given full enforcement power.</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B769" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C769" s="15" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D769" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E769" s="15" t="inlineStr">
+        <is>
+          <t>Clarify state vs municipal responsibility; elected ward representative accountable to voters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B770" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C770" s="15" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D770" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E770" s="15" t="inlineStr">
+        <is>
+          <t>Door-to-door, Environment Day, Bhutan/Germany examples, public announcements on separation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B771" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C771" s="15" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D771" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E771" s="15" t="inlineStr">
+        <is>
+          <t>Sunday plastic collection; biodegradable/non-biodegradable household bins; separate collection days proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B772" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C772" s="15" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D772" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E772" s="15" t="inlineStr">
+        <is>
+          <t>On-site separation and refining; expand like Dharan/Dhulikhel municipal model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B773" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C773" s="15" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D773" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E773" s="15" t="inlineStr">
+        <is>
+          <t>Awareness that separation reduces fees (Germany example).</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B774" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C774" s="15" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D774" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E774" s="15" t="inlineStr">
+        <is>
+          <t>Designated personnel and formal ward-level contacts needed (currently none).</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B775" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C775" s="15" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D775" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E775" s="15" t="inlineStr">
+        <is>
+          <t>Differentiated fees for separated vs unseparated waste; municipality contract funding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B776" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C776" s="15" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D776" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E776" s="15" t="inlineStr">
+        <is>
+          <t>Transfer station, landfill, access roads in Ward No. 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B777" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C777" s="15" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D777" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E777" s="15" t="inlineStr">
+        <is>
+          <t>Natural baskets, paper bags, cloth bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B778" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C778" s="15" t="inlineStr">
+        <is>
+          <t>Sol_clean_up</t>
+        </is>
+      </c>
+      <c r="D778" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E778" s="15" t="inlineStr">
+        <is>
+          <t>Source collection, highway and neighbourhood cleaning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B779" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C779" s="15" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D779" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E779" s="15" t="inlineStr">
+        <is>
+          <t>Strict laws, penalties, differentiated waste fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B780" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C780" s="15" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D780" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E780" s="15" t="inlineStr">
+        <is>
+          <t>24/7 monitoring impossible — need systemic enforcement not just awareness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="15" t="inlineStr">
+        <is>
+          <t>NPL_10</t>
+        </is>
+      </c>
+      <c r="B781" s="15" t="inlineStr">
+        <is>
+          <t>Dhulikhel Municipality - Ward Chairman (32 years, five terms), Dhulikhel (Ward No. 3 per transcript; master list: Ward no. 7)</t>
+        </is>
+      </c>
+      <c r="C781" s="15" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D781" s="15" t="inlineStr">
+        <is>
+          <t>Baskets made from natural materials; paper bags used for vegetables; cloth bags encouraged; biodegradable vs. non-biodegradable household separation promoted in recent 1–2 year efforts.</t>
+        </is>
+      </c>
+      <c r="E781" s="15" t="inlineStr">
+        <is>
+          <t>Natural-material baskets, paper bags for vegetables, cloth bags, pre-plastic carrying practices.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Code NPL_11 Safa Urja Utpadan private sector interview
Add Safa Urja Utpadan waste-management contractor (Ratnanagar,
Khaireni & Kalika municipalities, Chitwan) as NPL_11 from full notes
and transcript. Codes loss-making municipal contract, facility-level
segregation, school/tourism awareness programmes, GPS/barcode tracking,
PPP planning, and implied NPF framing.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -62,56 +62,62 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBCEA2"/>
-        <bgColor rgb="00EBCEA2"/>
+        <fgColor rgb="00EBCAA2"/>
+        <bgColor rgb="00EBCAA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCEBA2"/>
-        <bgColor rgb="00DCEBA2"/>
+        <fgColor rgb="00E4EBA2"/>
+        <bgColor rgb="00E4EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B1EBA2"/>
-        <bgColor rgb="00B1EBA2"/>
+        <fgColor rgb="00BCEBA2"/>
+        <bgColor rgb="00BCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBBF"/>
-        <bgColor rgb="00A2EBBF"/>
+        <fgColor rgb="00A2EBAF"/>
+        <bgColor rgb="00A2EBAF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBD7"/>
+        <bgColor rgb="00A2EBD7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2BFEB"/>
-        <bgColor rgb="00A2BFEB"/>
+        <fgColor rgb="00A2D7EB"/>
+        <bgColor rgb="00A2D7EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B1A2EB"/>
-        <bgColor rgb="00B1A2EB"/>
+        <fgColor rgb="00A2AFEB"/>
+        <bgColor rgb="00A2AFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCA2EB"/>
-        <bgColor rgb="00DCA2EB"/>
+        <fgColor rgb="00BCA2EB"/>
+        <bgColor rgb="00BCA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2CE"/>
-        <bgColor rgb="00EBA2CE"/>
+        <fgColor rgb="00E4A2EB"/>
+        <bgColor rgb="00E4A2EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2CA"/>
+        <bgColor rgb="00EBA2CA"/>
       </patternFill>
     </fill>
   </fills>
@@ -141,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -186,6 +192,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -553,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -572,7 +581,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_10, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_11, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -652,87 +661,94 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  10. NPL_10 - Dhulikhel Municipality Ward Chairman (32 years, five terms), Dhulikhel. Master list label: Ward no. 7; transcript focal ward: Ward No. 3 (Thakuri village transfer-station planning). Interviewers: Ram Devi (Kathmandu University), Deep and F. Coded from the verbatim transcript; structured theme notes at the top of the source file (Bio-Camp, Plast Foundation, EPR policy content) excluded as they do not appear in this transcript.</t>
+          <t xml:space="preserve">  10. NPL_10 - Dhulikhel Municipality Ward Chairman (32 years, five terms), Dhulikhel. Master list label: Ward no. 7; transcript focal ward: Ward No. 3. Coded from verbatim transcript (theme notes at top of source file excluded).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  11. NPL_11 - Safa Urja Utpadan, private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities). Interviewers: Ram Devi (Kathmandu University) and Deep. Coded from both interview guideline notes and verbatim transcript.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_10, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_11, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_10) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_11) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1919,7 +1935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ11"/>
+  <dimension ref="A1:CQ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7266,6 +7282,483 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>private_sector</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O12" s="16" t="inlineStr">
+        <is>
+          <t>environment and land (improper disposal, long-term plastic impacts), agriculture (monsoon chemicals from plastic reach crops; soil pH and fertility affected; repeated tilling brings plastic to surface), health (winter home burning of plastics — smoke and carbon emissions), landfill pressure (Ratnanagar ~21 tractor loads/day; only small unusable fraction sent after company processing)</t>
+        </is>
+      </c>
+      <c r="P12" s="16" t="inlineStr">
+        <is>
+          <t>farmers and agricultural land (soil pH/fertility loss from plastic chemicals in monsoon); the environment and land; public health (smoke/carbon from winter burning); future generations ("breathe clean air and consume safely produced food")</t>
+        </is>
+      </c>
+      <c r="Q12" s="16" t="inlineStr">
+        <is>
+          <t>the general public/households (low awareness, careless disposal, night dumping in bazaars, burning plastics at home in winter, resistance to fines and fee increases, mentality that waste management is the company's job); the state/government ("we have not seen improvements from the state"; system not formalized); hotels/bazaar businesses that dump waste at night and resist proper fees</t>
+        </is>
+      </c>
+      <c r="R12" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan (collection, segregation, processing, GPS/barcode tracking, awareness programmes, paying NPR 6.6M+ annually to municipalities); school students who influence parents; planned PPP model across Ratnanagar, Khaireni and Kalika municipalities; paper alternatives for feast plastics</t>
+        </is>
+      </c>
+      <c r="S12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA12" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BB12" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja designs its own collection and segregation system (hazardous/food/non-harmful/plastic/textile streams), sets differentiated household/business fee schedules (NPR 25–300/month by category), deploys GPS-enabled vehicles and a planned barcode payment-tracking system, conducts awareness programmes on its own schedule (schools every 3 months; Sauraha tourism zone every 5–6 months), and negotiates PPP/TOR development across three municipalities — substantial organisational discretion within a loss-making municipal contract.</t>
+        </is>
+      </c>
+      <c r="BC12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI12" s="16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BP12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW12" s="16" t="inlineStr">
+        <is>
+          <t>Fines up to NPR 11,000 exist on paper but "can only be applied in certain areas; they cannot be enforced everywhere"; fee-increase proposals "aren't passing"; rates unchanged for seven years (only 10%/year added); "we have not seen improvements from the state"; household segregation compliance inconsistent despite company sorting at facility.</t>
+        </is>
+      </c>
+      <c r="BX12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM12" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO12" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP12" s="16" t="inlineStr">
+        <is>
+          <t>Some traditional knowledge mentioned but "no policy exists to reduce plastic"; plan to replace plastic plates/cups/bowls at feasts with paper alternatives; jute sacks/bags for purchased-plastic disposal proposed.</t>
+        </is>
+      </c>
+      <c r="CQ12" s="16" t="inlineStr">
+        <is>
+          <t>Master list label: "11. Private Sector Contractor/ SafaUrja Utpadan", affiliation: Safa Urja Utpadan. Interviewee: Safa Urja representative (name not given in transcript). Location: Khaireni, Chitwan district — operates across Ratnanagar, Khaireni and Kalika municipalities (16 wards; Sauraha tourism zone). Company operating ~2 years at time of interview; 70–80 staff; German operations manager; UK/US stakeholders. Interviewers: Ram Devi (Kathmandu University) and Deep. Coded from both the interview guideline notes and the full verbatim transcript. Landfill sites: Ratnanagar (Udaypur community forest; also Ratnanagar community forest near Ladhari/Kayar Khola cited); Khaireni (riverside below bridge). Pays municipality NPR 6.6M annually (increasing 10%/year). PPP model in planning across three municipalities. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7277,7 +7770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E781"/>
+  <dimension ref="A1:E861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28374,6 +28867,2166 @@
         </is>
       </c>
     </row>
+    <row r="782">
+      <c r="A782" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B782" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C782" s="16" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D782" s="16" t="inlineStr">
+        <is>
+          <t>private_sector</t>
+        </is>
+      </c>
+      <c r="E782" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan is a private-sector waste-management contractor (collection, segregation, processing) operating under municipal contracts in Chitwan district.</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B783" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C783" s="16" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D783" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E783" s="16" t="inlineStr">
+        <is>
+          <t>"Awareness in the environment is lacking"; people discard plastics carelessly, burn at home in winter, dump at night in bazaars, and assume waste management is the company's responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B784" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C784" s="16" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D784" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E784" s="16" t="inlineStr">
+        <is>
+          <t>"We have not seen improvements from the state"; government has not formalized the system; federal ministry policies unknown to interviewee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B785" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C785" s="16" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D785" s="16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E785" s="16" t="inlineStr">
+        <is>
+          <t>"Since we work in this field, we are very concerned"; operating in Nepal carries financial, social, ethical and political risks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B786" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C786" s="16" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D786" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E786" s="16" t="inlineStr">
+        <is>
+          <t>People throw plastic everywhere; bazaar waste dumped at night; scavengers, jackals and dogs scatter waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B787" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C787" s="16" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D787" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E787" s="16" t="inlineStr">
+        <is>
+          <t>Promotes minimising usage, reusable plastics, purchasing wisely, and using less plastic in households and businesses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B788" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C788" s="16" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D788" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E788" s="16" t="inlineStr">
+        <is>
+          <t>Company segregates and processes at facility; only unusable fraction to landfill; condenses 1–2 quintals to 8–10 kg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B789" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C789" s="16" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D789" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E789" s="16" t="inlineStr">
+        <is>
+          <t>Monsoon (Jestha–Shravan–Bhadra, ~4 months) makes collection and landfill operations very difficult; terrain delays vehicles; Ratnanagar alone ~21 tractor loads/day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B790" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C790" s="16" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D790" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E790" s="16" t="inlineStr">
+        <is>
+          <t>Discussion of PP vs LP plastic types and micron-thickness rules (40-micron standard; thicker = higher cost = less usage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B791" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C791" s="16" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D791" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E791" s="16" t="inlineStr">
+        <is>
+          <t>Paper plates/cups planned for feasts; jute sacks/bags for purchased-plastic disposal; no alternative technologies cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B792" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C792" s="16" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D792" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E792" s="16" t="inlineStr">
+        <is>
+          <t>Household segregation tried but compliance inconsistent; company sorts mixed waste at facility (glass, food, plastic, clothes, hazardous colour-coding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B793" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C793" s="16" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D793" s="16" t="inlineStr">
+        <is>
+          <t>environment and land (improper disposal, long-term plastic impacts), agriculture (monsoon chemicals from plastic reach crops; soil pH and fertility affected; repeated tilling brings plastic to surface), health (winter home burning of plastics — smoke and carbon emissions), landfill pressure (Ratnanagar ~21 tractor loads/day; only small unusable fraction sent after company processing)</t>
+        </is>
+      </c>
+      <c r="E793" s="16" t="inlineStr">
+        <is>
+          <t>Soil pH/fertility, crop contamination in monsoon, burning health effects, environmental pollution from improper disposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B794" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C794" s="16" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D794" s="16" t="inlineStr">
+        <is>
+          <t>farmers and agricultural land (soil pH/fertility loss from plastic chemicals in monsoon); the environment and land; public health (smoke/carbon from winter burning); future generations ("breathe clean air and consume safely produced food")</t>
+        </is>
+      </c>
+      <c r="E794" s="16" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: farmers/agricultural land; environment; public health from burning; future generations. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B795" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C795" s="16" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D795" s="16" t="inlineStr">
+        <is>
+          <t>the general public/households (low awareness, careless disposal, night dumping in bazaars, burning plastics at home in winter, resistance to fines and fee increases, mentality that waste management is the company's job); the state/government ("we have not seen improvements from the state"; system not formalized); hotels/bazaar businesses that dump waste at night and resist proper fees</t>
+        </is>
+      </c>
+      <c r="E795" s="16" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: unaware/careless public; state inaction; businesses dumping at night. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B796" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C796" s="16" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D796" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan (collection, segregation, processing, GPS/barcode tracking, awareness programmes, paying NPR 6.6M+ annually to municipalities); school students who influence parents; planned PPP model across Ratnanagar, Khaireni and Kalika municipalities; paper alternatives for feast plastics</t>
+        </is>
+      </c>
+      <c r="E796" s="16" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: Safa Urja company, school students as change agents, planned PPP model. Company positions itself as primary problem-solver. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B797" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C797" s="16" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D797" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E797" s="16" t="inlineStr">
+        <is>
+          <t>German operations manager; UK/US stakeholders/owners; comparison with DOKO Recyclers Kathmandu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B798" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C798" s="16" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D798" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E798" s="16" t="inlineStr">
+        <is>
+          <t>Company–municipality–community communication essential; temples, schools, cooperatives (~150+ public spots) need coordinated management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B799" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C799" s="16" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D799" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E799" s="16" t="inlineStr">
+        <is>
+          <t>Calls for coordinated regulation across municipality, provincial and central government; PPP across three municipalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B800" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C800" s="16" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D800" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E800" s="16" t="inlineStr">
+        <is>
+          <t>Public assumes free collection at temples/schools; leadership vs household responsibility debated; company pays municipality but community resists fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B801" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C801" s="16" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D801" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E801" s="16" t="inlineStr">
+        <is>
+          <t>Long-term government management needed; coordinated top-down regulation sought.</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B802" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C802" s="16" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D802" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E802" s="16" t="inlineStr">
+        <is>
+          <t>NA - provincial government mentioned only as part of desired coordinated regulation, not as current responsible actor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B803" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C803" s="16" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D803" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E803" s="16" t="inlineStr">
+        <is>
+          <t>"Responsibility ideally lies with the leadership"; municipality receives NPR 6.6M+ annual payment from company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B804" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C804" s="16" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D804" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E804" s="16" t="inlineStr">
+        <is>
+          <t>NA - students targeted for awareness but not described as responsible mitigation actors (coded under Tar_students).</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B805" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C805" s="16" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D805" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E805" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja collects, segregates, processes and manages landfill operations under contract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B806" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C806" s="16" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D806" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E806" s="16" t="inlineStr">
+        <is>
+          <t>NA - temples/schools/cooperatives discussed but not as formal responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B807" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C807" s="16" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D807" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E807" s="16" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B808" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C808" s="16" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D808" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E808" s="16" t="inlineStr">
+        <is>
+          <t>Every household must understand the system for management to work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B809" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C809" s="16" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D809" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E809" s="16" t="inlineStr">
+        <is>
+          <t>Schools receive awareness programmes every 3 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B810" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C810" s="16" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D810" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E810" s="16" t="inlineStr">
+        <is>
+          <t>Hotels, hardware stores, hostels, businesses pay tiered monthly fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B811" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C811" s="16" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D811" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E811" s="16" t="inlineStr">
+        <is>
+          <t>"We have not seen improvements from the state"; system not formalized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B812" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C812" s="16" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D812" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E812" s="16" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B813" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C813" s="16" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D813" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E813" s="16" t="inlineStr">
+        <is>
+          <t>NA - municipalities receive payments and are partners in PPP, not primarily blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B814" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C814" s="16" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D814" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E814" s="16" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B815" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C815" s="16" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D815" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E815" s="16" t="inlineStr">
+        <is>
+          <t>NA - Safa Urja is the interviewee; other private actors not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B816" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C816" s="16" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D816" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E816" s="16" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B817" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C817" s="16" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D817" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E817" s="16" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B818" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C818" s="16" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D818" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E818" s="16" t="inlineStr">
+        <is>
+          <t>Careless disposal, burning plastics, night dumping, fee resistance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B819" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C819" s="16" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D819" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E819" s="16" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B820" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C820" s="16" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D820" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E820" s="16" t="inlineStr">
+        <is>
+          <t>Bazaar businesses dump at night; some assume free collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B821" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C821" s="16" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D821" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E821" s="16" t="inlineStr">
+        <is>
+          <t>Coordinated regulation from central level sought.</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B822" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C822" s="16" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D822" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E822" s="16" t="inlineStr">
+        <is>
+          <t>NA - provincial level only in desired regulation, not as primary target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B823" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C823" s="16" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D823" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E823" s="16" t="inlineStr">
+        <is>
+          <t>Municipality must take responsibility across all areas and submit support proposals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B824" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C824" s="16" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D824" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E824" s="16" t="inlineStr">
+        <is>
+          <t>School awareness every 3 months — children influence parents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B825" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C825" s="16" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D825" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E825" s="16" t="inlineStr">
+        <is>
+          <t>PPP model for three municipalities; private sector engagement in new waste-management system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B826" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C826" s="16" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D826" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E826" s="16" t="inlineStr">
+        <is>
+          <t>NA - not named as primary target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B827" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C827" s="16" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D827" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E827" s="16" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B828" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C828" s="16" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D828" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E828" s="16" t="inlineStr">
+        <is>
+          <t>Household segregation, jute-sack disposal, fee compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B829" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C829" s="16" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D829" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E829" s="16" t="inlineStr">
+        <is>
+          <t>School programmes every 3 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B830" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C830" s="16" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D830" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E830" s="16" t="inlineStr">
+        <is>
+          <t>Sauraha tourism-zone hotels and businesses targeted every 5–6 months; tiered business fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B831" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C831" s="16" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D831" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E831" s="16" t="inlineStr">
+        <is>
+          <t>Company representative describes contract operations, fee structures, technology deployment, PPP planning and municipal negotiations — managerial/organisational implementer (2), not a policy formulator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B832" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C832" s="16" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D832" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja designs its own collection and segregation system (hazardous/food/non-harmful/plastic/textile streams), sets differentiated household/business fee schedules (NPR 25–300/month by category), deploys GPS-enabled vehicles and a planned barcode payment-tracking system, conducts awareness programmes on its own schedule (schools every 3 months; Sauraha tourism zone every 5–6 months), and negotiates PPP/TOR development across three municipalities — substantial organisational discretion within a loss-making municipal contract.</t>
+        </is>
+      </c>
+      <c r="E832" s="16" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell — GPS, barcodes, segregation streams, awareness scheduling, PPP/TOR development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B833" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C833" s="16" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D833" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E833" s="16" t="inlineStr">
+        <is>
+          <t>GPS-enabled vehicles; barcode payment-tracking system planned within 3 months; staff attendance recorded from home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B834" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C834" s="16" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D834" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E834" s="16" t="inlineStr">
+        <is>
+          <t>Operating at a loss every year; rates unchanged 7 years; fee increases face uproar; NPR 300,000/month needed for public-spot collection alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B835" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C835" s="16" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D835" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E835" s="16" t="inlineStr">
+        <is>
+          <t>NA - no research programmes mentioned (Deep references CREASION pellet factory visit but not attributed to Safa Urja).</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B836" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C836" s="16" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D836" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E836" s="16" t="inlineStr">
+        <is>
+          <t>Need proper landfill sites in good locations; existing sites in community forests and riverside land; terrain limits monsoon access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B837" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C837" s="16" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D837" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E837" s="16" t="inlineStr">
+        <is>
+          <t>70–80 workers; monsoon terrain difficulties; 21 tractor loads/day in Ratnanagar alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B838" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C838" s="16" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D838" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E838" s="16" t="inlineStr">
+        <is>
+          <t>Fines partial; cannot enforce everywhere; late payment up to 7 months; no late-payment penalty currently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B839" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C839" s="16" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D839" s="16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E839" s="16" t="inlineStr">
+        <is>
+          <t>Extended producer responsibility not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B840" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C840" s="16" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D840" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E840" s="16" t="inlineStr">
+        <is>
+          <t>School programmes every 3 months; Sauraha tourism programmes every 5–6 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B841" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C841" s="16" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D841" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E841" s="16" t="inlineStr">
+        <is>
+          <t>Children educated to influence families at home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B842" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C842" s="16" t="inlineStr">
+        <is>
+          <t>Pol_tax</t>
+        </is>
+      </c>
+      <c r="D842" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E842" s="16" t="inlineStr">
+        <is>
+          <t>Tiered household/business monthly fees; company pays NPR 6.6M+ annually to municipality as tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B843" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C843" s="16" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D843" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E843" s="16" t="inlineStr">
+        <is>
+          <t>40-micron standard discussed; above 40 microns not allowed (thicker = higher cost).</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B844" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C844" s="16" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D844" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E844" s="16" t="inlineStr">
+        <is>
+          <t>Jute sacks/bags; paper plates/cups for feasts planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B845" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C845" s="16" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D845" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E845" s="16" t="inlineStr">
+        <is>
+          <t>Facility-level segregation into compostable/recyclable streams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B846" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C846" s="16" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D846" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E846" s="16" t="inlineStr">
+        <is>
+          <t>Contracted municipal collection across 16 wards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B847" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C847" s="16" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D847" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E847" s="16" t="inlineStr">
+        <is>
+          <t>Fines and fees weakly enforced; state improvements not seen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B848" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C848" s="16" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D848" s="16" t="inlineStr">
+        <is>
+          <t>Fines up to NPR 11,000 exist on paper but "can only be applied in certain areas; they cannot be enforced everywhere"; fee-increase proposals "aren't passing"; rates unchanged for seven years (only 10%/year added); "we have not seen improvements from the state"; household segregation compliance inconsistent despite company sorting at facility.</t>
+        </is>
+      </c>
+      <c r="E848" s="16" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B849" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C849" s="16" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D849" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E849" s="16" t="inlineStr">
+        <is>
+          <t>PPP model across three municipalities with consultant/TOR study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B850" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C850" s="16" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D850" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E850" s="16" t="inlineStr">
+        <is>
+          <t>Clear communication between company, municipality and community.</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B851" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C851" s="16" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D851" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E851" s="16" t="inlineStr">
+        <is>
+          <t>Regular school and tourism-zone programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B852" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C852" s="16" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D852" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E852" s="16" t="inlineStr">
+        <is>
+          <t>Household and facility-level colour-coded segregation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B853" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C853" s="16" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D853" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E853" s="16" t="inlineStr">
+        <is>
+          <t>Process segregated streams; minimise landfill volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B854" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C854" s="16" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D854" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E854" s="16" t="inlineStr">
+        <is>
+          <t>Students as family influencers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B855" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C855" s="16" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D855" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E855" s="16" t="inlineStr">
+        <is>
+          <t>Worker responsibility training; 70–80 staff operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B856" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C856" s="16" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D856" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E856" s="16" t="inlineStr">
+        <is>
+          <t>Fee increases; late-payment penalties from municipality; PPP to address loss-making contract.</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B857" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C857" s="16" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D857" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E857" s="16" t="inlineStr">
+        <is>
+          <t>Proper landfill sites; GPS/barcode technology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B858" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C858" s="16" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D858" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E858" s="16" t="inlineStr">
+        <is>
+          <t>Paper feast ware; jute disposal bags; LP instead of PP plastic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B859" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C859" s="16" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D859" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E859" s="16" t="inlineStr">
+        <is>
+          <t>Progressive fines (NPR 5,000–10,000); differentiated fees for segregated vs unsegregated waste (discussed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B860" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C860" s="16" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D860" s="16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E860" s="16" t="inlineStr">
+        <is>
+          <t>GPS vehicles, barcode payment tracking, staff attendance system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="16" t="inlineStr">
+        <is>
+          <t>NPL_11</t>
+        </is>
+      </c>
+      <c r="B861" s="16" t="inlineStr">
+        <is>
+          <t>Safa Urja Utpadan - Private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities)</t>
+        </is>
+      </c>
+      <c r="C861" s="16" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D861" s="16" t="inlineStr">
+        <is>
+          <t>Some traditional knowledge mentioned but "no policy exists to reduce plastic"; plan to replace plastic plates/cups/bowls at feasts with paper alternatives; jute sacks/bags for purchased-plastic disposal proposed.</t>
+        </is>
+      </c>
+      <c r="E861" s="16" t="inlineStr">
+        <is>
+          <t>Some traditional knowledge acknowledged but no supporting policy; paper feast alternatives and jute bags proposed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Code NPL_12 Ministry for Urban Planning / MoUD interview
Add second MoUD policy-formulation interview (PEGO transcript) as
NPL_12 from full notes and transcript. Codes source segregation,
draft Solid Waste Management Act, EPR/PPP, Banchare Danda landfill
failure, and implied NPF framing. Notes substantive overlap with
NPL_8 but coded independently from this source.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -62,62 +62,68 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBCAA2"/>
-        <bgColor rgb="00EBCAA2"/>
+        <fgColor rgb="00EBC6A2"/>
+        <bgColor rgb="00EBC6A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4EBA2"/>
-        <bgColor rgb="00E4EBA2"/>
+        <fgColor rgb="00EBEBA2"/>
+        <bgColor rgb="00EBEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BCEBA2"/>
-        <bgColor rgb="00BCEBA2"/>
+        <fgColor rgb="00C6EBA2"/>
+        <bgColor rgb="00C6EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBAF"/>
-        <bgColor rgb="00A2EBAF"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD7"/>
-        <bgColor rgb="00A2EBD7"/>
+        <fgColor rgb="00A2EBC6"/>
+        <bgColor rgb="00A2EBC6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D7EB"/>
-        <bgColor rgb="00A2D7EB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2AFEB"/>
-        <bgColor rgb="00A2AFEB"/>
+        <fgColor rgb="00A2C6EB"/>
+        <bgColor rgb="00A2C6EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BCA2EB"/>
-        <bgColor rgb="00BCA2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4A2EB"/>
-        <bgColor rgb="00E4A2EB"/>
+        <fgColor rgb="00C6A2EB"/>
+        <bgColor rgb="00C6A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2CA"/>
-        <bgColor rgb="00EBA2CA"/>
+        <fgColor rgb="00EBA2EB"/>
+        <bgColor rgb="00EBA2EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2C6"/>
+        <bgColor rgb="00EBA2C6"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -195,6 +201,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -562,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -581,7 +590,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_11, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_12, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -668,87 +677,94 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  11. NPL_11 - Safa Urja Utpadan, private waste-management contractor, Khaireni/Chitwan (Ratnanagar, Khaireni &amp; Kalika municipalities). Interviewers: Ram Devi (Kathmandu University) and Deep. Coded from both interview guideline notes and verbatim transcript.</t>
+          <t xml:space="preserve">  11. NPL_11 - Safa Urja Utpadan, private waste-management contractor, Khaireni/Chitwan. Coded from notes and transcript.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  12. NPL_12 - Ministry for Urban Planning / Ministry of Urban Development (MoUD), policy official(s) involved in solid waste act and regulation formulation. Interviewer: PEGO team. Coded from notes and transcript. Substantively overlaps NPL_8 (same ministry); coded independently. NPF fields implied.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_11, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_12, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_11) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_12) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1935,7 +1951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ12"/>
+  <dimension ref="A1:CQ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7759,6 +7775,483 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>nat_government</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O13" s="17" t="inlineStr">
+        <is>
+          <t>rivers and canals (flow obstructed), sewer/water-line blockages, tourism (haphazard disposal), health (low-quality black plastic for meat/yogurt; public unaware of hazards), agriculture (productivity impacted), landfill/dumping sites (Banchare Danda designed 20 years but filled in 3–4 years; leachate, bad smells, visual disturbance), livestock consuming plastic, microeconomic/household-level damage, inter-municipal protests</t>
+        </is>
+      </c>
+      <c r="P13" s="17" t="inlineStr">
+        <is>
+          <t>the general public/households (health risks from black plastic food packaging; microeconomic damage); communities near landfill/dumping sites (leachate, smell, protests); farmers/agriculture (productivity loss); tourism and urban environments (old cities and emerging towns); rivers, canals and livestock</t>
+        </is>
+      </c>
+      <c r="Q13" s="17" t="inlineStr">
+        <is>
+          <t>the general public (convenience attachment to plastic, no segregation culture, haphazard disposal); plastic producers/industries (polluter-pays principle exists but implementation weak; EPR not yet enacted); municipalities operating sanitary landfills as open dumping sites (Banchare Danda deterrent); inter-municipal waste dumping and NIMBY conflicts</t>
+        </is>
+      </c>
+      <c r="R13" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / central government (draft Solid Waste Management Act with EPR, PPP, burning ban, three-tier roles); provincial/central assistance for landfill land acquisition; private sector (domestic and international) under PPP with sample agreements; MoUD training centre and municipal data software; source-segregation and circular-economy approach; international donor coordination</t>
+        </is>
+      </c>
+      <c r="S13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AS13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA13" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BB13" s="17" t="inlineStr">
+        <is>
+          <t>MoUD has authority to formulate policies, acts and regulations; drafts the Solid Waste Management Act, post-enactment regulations/guidelines (including 5 km/10 km distance management), PPP sample agreements, community-level plastic guidelines, municipal monitoring software, and coordinates international donor partner approvals.</t>
+        </is>
+      </c>
+      <c r="BC13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI13" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BN13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW13" s="17" t="inlineStr">
+        <is>
+          <t>Bagmati Cleaning Campaign running ~10 years but plastic remains the majority problem; Kathmandu source segregation only partial ("most not in the desired form"); polluter-pays principle in use but "implementation is weak"; Banchare Danda landfill designed for 20 years nearly filled within 3–4 years; no specific national plastic policy despite general solid waste framework.</t>
+        </is>
+      </c>
+      <c r="BX13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CA13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CH13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CM13" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO13" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP13" s="17" t="inlineStr">
+        <is>
+          <t>At low population density, waste was mostly organic and nature could absorb it; traditional leaf plates instead of plastic; natural consumption-land cycle (broken by plastic intervention); emerging household practice of separate decomposable and non-decomposable bins among younger generation.</t>
+        </is>
+      </c>
+      <c r="CQ13" s="17" t="inlineStr">
+        <is>
+          <t>Master list label: "12. Ministry for Urban Planning", affiliation: Ministry of Urban Development (MoUD), Government of Nepal. Interviewee name not given; role described as involved in formulating policies, acts and regulations for solid waste management and urban planning. Interviewer: PEGO project team. Coded from both the interview guideline notes and the full verbatim transcript. Substantively overlaps NPL_8 (also MoUD, 23 June 2025 session with named officials) but this appears to be a separate/cleaned transcript of the ministry policy perspective; coded independently from this source. Local Government Operation Act 2017 cited (NPL_8 referenced Self-Governance Act 2016). NPF fields implied, not explicit. Separate plastic waste management policy planned after Solid Waste Management Act.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7770,7 +8263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E861"/>
+  <dimension ref="A1:E940"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -31027,6 +31520,2139 @@
         </is>
       </c>
     </row>
+    <row r="862">
+      <c r="A862" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B862" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C862" s="17" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D862" s="17" t="inlineStr">
+        <is>
+          <t>nat_government</t>
+        </is>
+      </c>
+      <c r="E862" s="17" t="inlineStr">
+        <is>
+          <t>Interview at the Ministry of Urban Development (MoUD) / Ministry for Urban Planning — national government ministry with authority to formulate solid-waste policy, acts and regulations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B863" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C863" s="17" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D863" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E863" s="17" t="inlineStr">
+        <is>
+          <t>People lack segregation habits; lives "closely attached to plastic" for convenience; don't consider future public-health implications; heterogeneous waste thrown together on streets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B864" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C864" s="17" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D864" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E864" s="17" t="inlineStr">
+        <is>
+          <t>Municipalities confused about onboarding private sector and donor partners; no specific plastic policy yet; only general solid waste framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B865" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C865" s="17" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D865" s="17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E865" s="17" t="inlineStr">
+        <is>
+          <t>"Plastic is the component that disturbs society the most"; "Nepal government is very serious about this plastic waste"; remarkable volume in waste composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B866" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C866" s="17" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D866" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E866" s="17" t="inlineStr">
+        <is>
+          <t>Plastic visible everywhere in urban areas; waste thrown haphazardly without control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B867" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C867" s="17" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D867" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E867" s="17" t="inlineStr">
+        <is>
+          <t>Public convenience attachment to plastic for carrying goods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B868" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C868" s="17" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D868" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E868" s="17" t="inlineStr">
+        <is>
+          <t>Circular economy promoted but requires source segregation first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B869" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C869" s="17" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D869" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E869" s="17" t="inlineStr">
+        <is>
+          <t>Banchare Danda operated as dumping site (20-year design filled in 3–4 years); waste picked up and dumped without processing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B870" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C870" s="17" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D870" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E870" s="17" t="inlineStr">
+        <is>
+          <t>Producers/industries discussed under proposed EPR and weak polluter-pays implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B871" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C871" s="17" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D871" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E871" s="17" t="inlineStr">
+        <is>
+          <t>Separate plastics policy planned; foreign technology and investment welcomed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B872" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C872" s="17" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D872" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E872" s="17" t="inlineStr">
+        <is>
+          <t>"The main challenge is the separation of waste, specifically source segregation"; most Kathmandu waste not in desired form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B873" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C873" s="17" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D873" s="17" t="inlineStr">
+        <is>
+          <t>rivers and canals (flow obstructed), sewer/water-line blockages, tourism (haphazard disposal), health (low-quality black plastic for meat/yogurt; public unaware of hazards), agriculture (productivity impacted), landfill/dumping sites (Banchare Danda designed 20 years but filled in 3–4 years; leachate, bad smells, visual disturbance), livestock consuming plastic, microeconomic/household-level damage, inter-municipal protests</t>
+        </is>
+      </c>
+      <c r="E873" s="17" t="inlineStr">
+        <is>
+          <t>Rivers/canals, sewers, tourism, health (black plastic), agriculture, landfills, livestock, household microeconomics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B874" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C874" s="17" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D874" s="17" t="inlineStr">
+        <is>
+          <t>the general public/households (health risks from black plastic food packaging; microeconomic damage); communities near landfill/dumping sites (leachate, smell, protests); farmers/agriculture (productivity loss); tourism and urban environments (old cities and emerging towns); rivers, canals and livestock</t>
+        </is>
+      </c>
+      <c r="E874" s="17" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: public/households; communities near dumps; farmers; tourism/urban environments; rivers and livestock. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B875" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C875" s="17" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D875" s="17" t="inlineStr">
+        <is>
+          <t>the general public (convenience attachment to plastic, no segregation culture, haphazard disposal); plastic producers/industries (polluter-pays principle exists but implementation weak; EPR not yet enacted); municipalities operating sanitary landfills as open dumping sites (Banchare Danda deterrent); inter-municipal waste dumping and NIMBY conflicts</t>
+        </is>
+      </c>
+      <c r="E875" s="17" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: convenience-driven public; weakly regulated producers; municipalities running dumps; inter-municipal conflicts. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B876" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C876" s="17" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D876" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / central government (draft Solid Waste Management Act with EPR, PPP, burning ban, three-tier roles); provincial/central assistance for landfill land acquisition; private sector (domestic and international) under PPP with sample agreements; MoUD training centre and municipal data software; source-segregation and circular-economy approach; international donor coordination</t>
+        </is>
+      </c>
+      <c r="E876" s="17" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: MoUD/central government (new act, EPR, PPP); provincial/central landfill support; private sector; training centre/software; circular economy. Ministry positions itself as primary problem-solver. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B877" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C877" s="17" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D877" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E877" s="17" t="inlineStr">
+        <is>
+          <t>Foreign direct investment and international donor partner coordination; SDG and human-rights frameworks integrated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B878" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C878" s="17" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D878" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E878" s="17" t="inlineStr">
+        <is>
+          <t>Multi-stakeholder consultation — universities, private sector, mayors, industries; PPP between municipalities and private sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B879" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C879" s="17" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D879" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E879" s="17" t="inlineStr">
+        <is>
+          <t>New act defines central, provincial and local roles; provincial/central help acquire landfill land.</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B880" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C880" s="17" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D880" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E880" s="17" t="inlineStr">
+        <is>
+          <t>Three-tier roles being clarified in new act; municipalities need orientation beyond online posting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B881" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C881" s="17" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D881" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E881" s="17" t="inlineStr">
+        <is>
+          <t>MoUD develops policies, acts, regulations; coordinates donors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B882" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C882" s="17" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D882" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E882" s="17" t="inlineStr">
+        <is>
+          <t>Assists local governments with landfill land acquisition under new act.</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B883" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C883" s="17" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D883" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E883" s="17" t="inlineStr">
+        <is>
+          <t>Constitutionally responsible under Local Government Operation Act 2017.</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B884" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C884" s="17" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D884" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E884" s="17" t="inlineStr">
+        <is>
+          <t>NA - students not mentioned as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B885" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C885" s="17" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D885" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E885" s="17" t="inlineStr">
+        <is>
+          <t>Domestic and international partners under PPP; foreign technology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B886" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C886" s="17" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D886" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E886" s="17" t="inlineStr">
+        <is>
+          <t>NA - NGOs not described as current responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B887" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C887" s="17" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D887" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E887" s="17" t="inlineStr">
+        <is>
+          <t>Universities consulted in act formulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B888" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C888" s="17" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D888" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E888" s="17" t="inlineStr">
+        <is>
+          <t>Source segregation at household level essential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B889" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C889" s="17" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D889" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E889" s="17" t="inlineStr">
+        <is>
+          <t>NA - universities consulted but not ongoing responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B890" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C890" s="17" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D890" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E890" s="17" t="inlineStr">
+        <is>
+          <t>Producers/industries under proposed EPR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B891" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C891" s="17" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D891" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E891" s="17" t="inlineStr">
+        <is>
+          <t>NA - interviewee IS the national government; past weaknesses discussed but ministry positions itself as reformer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B892" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C892" s="17" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D892" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E892" s="17" t="inlineStr">
+        <is>
+          <t>NA - provincial government seen as future helper, not culprit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B893" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C893" s="17" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D893" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E893" s="17" t="inlineStr">
+        <is>
+          <t>Landfills operated as dumping sites (Banchare Danda example).</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B894" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C894" s="17" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D894" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E894" s="17" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B895" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C895" s="17" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D895" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E895" s="17" t="inlineStr">
+        <is>
+          <t>NA - private sector targeted for partnership, not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B896" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C896" s="17" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D896" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E896" s="17" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B897" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C897" s="17" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D897" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E897" s="17" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B898" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C898" s="17" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D898" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E898" s="17" t="inlineStr">
+        <is>
+          <t>No segregation culture; convenience attachment; haphazard disposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B899" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C899" s="17" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D899" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E899" s="17" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B900" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C900" s="17" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D900" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E900" s="17" t="inlineStr">
+        <is>
+          <t>Polluter-pays "implementation is weak."</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B901" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C901" s="17" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D901" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E901" s="17" t="inlineStr">
+        <is>
+          <t>Coordination, policy framework, donor partnerships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B902" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C902" s="17" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D902" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E902" s="17" t="inlineStr">
+        <is>
+          <t>Assistance with land acquisition and coordination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B903" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C903" s="17" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D903" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E903" s="17" t="inlineStr">
+        <is>
+          <t>Implementation, landfill operation, PPP agreements, orientation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B904" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C904" s="17" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D904" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E904" s="17" t="inlineStr">
+        <is>
+          <t>NA - not named as primary target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B905" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C905" s="17" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D905" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E905" s="17" t="inlineStr">
+        <is>
+          <t>Investment and technology partnership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B906" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C906" s="17" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D906" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E906" s="17" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B907" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C907" s="17" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D907" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E907" s="17" t="inlineStr">
+        <is>
+          <t>NA - researchers consulted but not primary target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B908" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C908" s="17" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D908" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E908" s="17" t="inlineStr">
+        <is>
+          <t>Source segregation habits; reducing plastic attachment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B909" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C909" s="17" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D909" s="17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E909" s="17" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B910" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C910" s="17" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D910" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E910" s="17" t="inlineStr">
+        <is>
+          <t>EPR, fee payments, post-enactment industry cooperation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B911" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C911" s="17" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D911" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E911" s="17" t="inlineStr">
+        <is>
+          <t>Respondent speaks as national policy formulator drafting the Solid Waste Management Act, regulations, guidelines and PPP templates — role 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B912" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C912" s="17" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D912" s="17" t="inlineStr">
+        <is>
+          <t>MoUD has authority to formulate policies, acts and regulations; drafts the Solid Waste Management Act, post-enactment regulations/guidelines (including 5 km/10 km distance management), PPP sample agreements, community-level plastic guidelines, municipal monitoring software, and coordinates international donor partner approvals.</t>
+        </is>
+      </c>
+      <c r="E912" s="17" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B913" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C913" s="17" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D913" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E913" s="17" t="inlineStr">
+        <is>
+          <t>Insufficient monitoring and technology for segregation patterns; planned municipal software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B914" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C914" s="17" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D914" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E914" s="17" t="inlineStr">
+        <is>
+          <t>Land acquisition difficult under separate Land Acquisition Act; circular economy needs financial sustainability support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B915" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C915" s="17" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D915" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E915" s="17" t="inlineStr">
+        <is>
+          <t>Universities and researchers consulted; welcomes international expertise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B916" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C916" s="17" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D916" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E916" s="17" t="inlineStr">
+        <is>
+          <t>Transfer stations exist in Kathmandu; sanitary landfill operation failing; PPP infrastructure provisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B917" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C917" s="17" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D917" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E917" s="17" t="inlineStr">
+        <is>
+          <t>Municipal elected leaders need technical orientation via training centre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B918" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C918" s="17" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D918" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E918" s="17" t="inlineStr">
+        <is>
+          <t>40-micron ban exists; burning prohibition with penalties in draft act; polluter-pays weak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B919" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C919" s="17" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D919" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E919" s="17" t="inlineStr">
+        <is>
+          <t>EPR proposed in draft act but not yet enacted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B920" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C920" s="17" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D920" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E920" s="17" t="inlineStr">
+        <is>
+          <t>Bagmati Cleaning Campaign (~10 years); provincial/district consultations planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B921" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C921" s="17" t="inlineStr">
+        <is>
+          <t>Pol_capacity</t>
+        </is>
+      </c>
+      <c r="D921" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E921" s="17" t="inlineStr">
+        <is>
+          <t>Training centre for local-government orientation packages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B922" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C922" s="17" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D922" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E922" s="17" t="inlineStr">
+        <is>
+          <t>Government banned plastic thinner than 40 microns; burning solid waste strictly prohibited in draft act.</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B923" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C923" s="17" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D923" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E923" s="17" t="inlineStr">
+        <is>
+          <t>Segregation and circular economy provisions; separate plastics policy planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B924" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C924" s="17" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D924" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E924" s="17" t="inlineStr">
+        <is>
+          <t>Act covers collection, transportation and disposal; transfer stations in Kathmandu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B925" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C925" s="17" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D925" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E925" s="17" t="inlineStr">
+        <is>
+          <t>Campaign, segregation, polluter-pays and landfill management all weak in practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B926" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C926" s="17" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D926" s="17" t="inlineStr">
+        <is>
+          <t>Bagmati Cleaning Campaign running ~10 years but plastic remains the majority problem; Kathmandu source segregation only partial ("most not in the desired form"); polluter-pays principle in use but "implementation is weak"; Banchare Danda landfill designed for 20 years nearly filled within 3–4 years; no specific national plastic policy despite general solid waste framework.</t>
+        </is>
+      </c>
+      <c r="E926" s="17" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B927" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C927" s="17" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D927" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E927" s="17" t="inlineStr">
+        <is>
+          <t>Three-tier role clarification in new act; central donor coordination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B928" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C928" s="17" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D928" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E928" s="17" t="inlineStr">
+        <is>
+          <t>EPR for producers; clear three-tier responsibilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B929" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C929" s="17" t="inlineStr">
+        <is>
+          <t>Sol_epr</t>
+        </is>
+      </c>
+      <c r="D929" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E929" s="17" t="inlineStr">
+        <is>
+          <t>Producers responsible for disposal or pay fee to local body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B930" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C930" s="17" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D930" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E930" s="17" t="inlineStr">
+        <is>
+          <t>Provincial/district consultations; not just website posting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B931" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C931" s="17" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D931" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E931" s="17" t="inlineStr">
+        <is>
+          <t>Primary solution enabling circular economy and waste reduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B932" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C932" s="17" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D932" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E932" s="17" t="inlineStr">
+        <is>
+          <t>Circular economy after segregation; separate plastics framework later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B933" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C933" s="17" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D933" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E933" s="17" t="inlineStr">
+        <is>
+          <t>Training centre orientation for municipalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B934" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C934" s="17" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D934" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E934" s="17" t="inlineStr">
+        <is>
+          <t>Guidelines and regulations post-enactment; municipal software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B935" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C935" s="17" t="inlineStr">
+        <is>
+          <t>Sol_RD</t>
+        </is>
+      </c>
+      <c r="D935" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E935" s="17" t="inlineStr">
+        <is>
+          <t>Foreign technology investment welcomed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B936" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C936" s="17" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D936" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E936" s="17" t="inlineStr">
+        <is>
+          <t>EPR fees; circular economy financial sustainability; donor coordination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B937" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C937" s="17" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D937" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E937" s="17" t="inlineStr">
+        <is>
+          <t>Sanitary landfill operation; transfer stations; PPP models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B938" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C938" s="17" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D938" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E938" s="17" t="inlineStr">
+        <is>
+          <t>Burning ban with penalties; EPR enforcement after enactment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B939" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C939" s="17" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D939" s="17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E939" s="17" t="inlineStr">
+        <is>
+          <t>Municipal software tracking population, production, segregation, disposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="17" t="inlineStr">
+        <is>
+          <t>NPL_12</t>
+        </is>
+      </c>
+      <c r="B940" s="17" t="inlineStr">
+        <is>
+          <t>Ministry of Urban Development / Ministry for Urban Planning - MoUD policy official(s), Kathmandu (PEGO interview)</t>
+        </is>
+      </c>
+      <c r="C940" s="17" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D940" s="17" t="inlineStr">
+        <is>
+          <t>At low population density, waste was mostly organic and nature could absorb it; traditional leaf plates instead of plastic; natural consumption-land cycle (broken by plastic intervention); emerging household practice of separate decomposable and non-decomposable bins among younger generation.</t>
+        </is>
+      </c>
+      <c r="E940" s="17" t="inlineStr">
+        <is>
+          <t>Leaf plates; organic waste cycle at low population density; separate household bins emerging.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Code NPL_13 Creasion recycling CSO interview
Add Creasion (Center for Research and Sustainable Development in Nepal)
as NPL_13 from guideline notes and field notes. Codes end-of-life plastic
concerns, microplastics from colored PET, scrap tax impacts, informal
picker exploitation, EU/CAP projects, and implied NPF framing.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -62,68 +62,74 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC6A2"/>
-        <bgColor rgb="00EBC6A2"/>
+        <fgColor rgb="00EBC4A2"/>
+        <bgColor rgb="00EBC4A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBEBA2"/>
-        <bgColor rgb="00EBEBA2"/>
+        <fgColor rgb="00EBE5A2"/>
+        <bgColor rgb="00EBE5A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EBA2"/>
-        <bgColor rgb="00C6EBA2"/>
+        <fgColor rgb="00CFEBA2"/>
+        <bgColor rgb="00CFEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA2"/>
-        <bgColor rgb="00A2EBA2"/>
+        <fgColor rgb="00ADEBA2"/>
+        <bgColor rgb="00ADEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBC6"/>
-        <bgColor rgb="00A2EBC6"/>
+        <fgColor rgb="00A2EBB8"/>
+        <bgColor rgb="00A2EBB8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBDA"/>
+        <bgColor rgb="00A2EBDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2C6EB"/>
-        <bgColor rgb="00A2C6EB"/>
+        <fgColor rgb="00A2DAEB"/>
+        <bgColor rgb="00A2DAEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A2EB"/>
-        <bgColor rgb="00A2A2EB"/>
+        <fgColor rgb="00A2B8EB"/>
+        <bgColor rgb="00A2B8EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6A2EB"/>
-        <bgColor rgb="00C6A2EB"/>
+        <fgColor rgb="00ADA2EB"/>
+        <bgColor rgb="00ADA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2EB"/>
-        <bgColor rgb="00EBA2EB"/>
+        <fgColor rgb="00CFA2EB"/>
+        <bgColor rgb="00CFA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C6"/>
-        <bgColor rgb="00EBA2C6"/>
+        <fgColor rgb="00EBA2E5"/>
+        <bgColor rgb="00EBA2E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2C4"/>
+        <bgColor rgb="00EBA2C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -204,6 +210,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -590,7 +599,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_12, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_13, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -684,87 +693,94 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  12. NPL_12 - Ministry for Urban Planning / Ministry of Urban Development (MoUD), policy official(s) involved in solid waste act and regulation formulation. Interviewer: PEGO team. Coded from notes and transcript. Substantively overlaps NPL_8 (same ministry); coded independently. NPF fields implied.</t>
+          <t xml:space="preserve">  12. NPL_12 - Ministry for Urban Planning / MoUD. Coded from notes and transcript.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  13. NPL_13 - Creasion, recycling and waste-management CSO (Center for Research and Sustainable Development in Nepal). Interview date: 23 June 2025 (~5:15pm). Coded from guideline notes and field notes (no full verbatim transcript). NPF fields implied.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_12, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_13, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_12) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_13) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1951,7 +1967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ13"/>
+  <dimension ref="A1:CQ14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8252,6 +8268,483 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>civil_society</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O14" s="18" t="inlineStr">
+        <is>
+          <t>end-of-life plastic fate; micro- and nano-plastics (colored PET bottles cannot be effectively reused — only transparent PET can; colored PET emits significant microplastics when processed); health hazards from recycled plastics in food-contact applications; carcinogenic emissions from poor recycling sector practices (processing at 100–200°C); exploitation of informal waste pickers (especially women) at landfills/dumpsites</t>
+        </is>
+      </c>
+      <c r="P14" s="18" t="inlineStr">
+        <is>
+          <t>informal waste pickers, particularly women selling PET from landfills/dumpsites for NPR 10 (vs NPR 25/kg formal rate) and facing intimidation/violence from intermediary "mafias"; the public exposed to unsafe recycled food-contact plastics and carcinogenic emissions from substandard recyclers; the environment from end-of-life plastics and microplastic release</t>
+        </is>
+      </c>
+      <c r="Q14" s="18" t="inlineStr">
+        <is>
+          <t>intermediary "mafias" who threaten and assault waste pickers who do not sell to them; substandard recyclers with "pathetic" social and environmental standards (100–200°C processing, carcinogenic emissions); the scrap tax on PET at municipal level (raising raw-material and granule costs); virgin-plastic preference among Nepali consumers and businesses; bureaucratic barriers (Department of Industry registration, 60% export condition after year three, repeated LG approvals on relocation); national government for not consulting recyclers on solid waste policy (improving only gradually)</t>
+        </is>
+      </c>
+      <c r="R14" s="18" t="inlineStr">
+        <is>
+          <t>Creasion (recycling, downsizing, product conversion, safety-tested granules, High-Effluent Treatment Plant recycling ~10,000 L water with no drainage outflow); EU-funded plastic-recovery and entrepreneurship project; CAP project (World Bank/UNOPS/SACEP) with sophisticated recycling technology; municipal collaboration to identify and formalize informal collectors; Plus Nepal and informal NRR associations; CSO trainings for sector coordination</t>
+        </is>
+      </c>
+      <c r="S14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AL14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AW14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA14" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BB14" s="18" t="inlineStr">
+        <is>
+          <t>Creasion designs its own recycling and product-conversion processes, develops granule quality/safety standards and government-standard testing before market release, runs EU and CAP projects, collaborates with municipalities to identify informal collectors, and builds entrepreneur capacity — but faces constrained discretion on bureaucratic setup (Dept of Industry, LG approvals) and export/tax policy conditions.</t>
+        </is>
+      </c>
+      <c r="BC14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI14" s="18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BL14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BP14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW14" s="18" t="inlineStr">
+        <is>
+          <t>Scrap tax on PET at municipal level raised raw-material and granule costs, making recycled products less competitive than virgin plastic; social/environmental standards across the broader recycling sector described as "pathetic" with weak enforcement; Creasion "not consulted" on solid waste management policy development (gradually being included); national plastic-generation estimates (60,000 t/year; 27% PET per World Bank) questioned as methodology unclear.</t>
+        </is>
+      </c>
+      <c r="BX14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CM14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO14" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP14" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CQ14" s="18" t="inlineStr">
+        <is>
+          <t>Master list label: "13. Creasion", affiliation: Center for Research and Sustainable Development in Nepal (Creasion). Interviewee name not given. Organization: recycling and waste-management CSO supporting informal waste workers and entrepreneurs. Interview date: 23 June 2025 (~5:15pm). Coded from interview guideline notes and bullet-point field notes (no full verbatim transcript supplied). ~70 t/month PET capacity cited. Two known recycling centers in Nepal mentioned. Associations: Plus Nepal (formal); Nepal Recycler and Reuse/NRR (informal/unregistered). CAP project throughput figures in source (1 t/h input vs 10 t/h granules) appear inconsistent — retained as stated. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8263,7 +8756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E940"/>
+  <dimension ref="A1:E1009"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33653,6 +34146,1869 @@
         </is>
       </c>
     </row>
+    <row r="941">
+      <c r="A941" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B941" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C941" s="18" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D941" s="18" t="inlineStr">
+        <is>
+          <t>civil_society</t>
+        </is>
+      </c>
+      <c r="E941" s="18" t="inlineStr">
+        <is>
+          <t>Creasion is a civil-society/recycling organization (Center for Research and Sustainable Development in Nepal) operating plastic recycling facilities and supporting informal waste workers and entrepreneurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B942" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C942" s="18" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D942" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E942" s="18" t="inlineStr">
+        <is>
+          <t>Most Nepali consumers/businesses prefer virgin over recycled plastic; unclear market demand for recycled granules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B943" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C943" s="18" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D943" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E943" s="18" t="inlineStr">
+        <is>
+          <t>Creasion not consulted on solid waste management policy (gradually being included); unclear national measurement methodology (60,000 t/year; 27% PET).</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B944" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C944" s="18" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D944" s="18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E944" s="18" t="inlineStr">
+        <is>
+          <t>Organization works directly on plastic end-of-life, food-packaging safety, and microplastics — high operational concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B945" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C945" s="18" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D945" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E945" s="18" t="inlineStr">
+        <is>
+          <t>Only two recycling centers identified; colored PET not effectively recyclable; sector standards "pathetic"; virgin plastic displaces recycled granules for food contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B946" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C946" s="18" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D946" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E946" s="18" t="inlineStr">
+        <is>
+          <t>End-of-life plastic fate; informal pickers exploited; bureaucratic barriers to establishing/moving recycling industry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B947" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C947" s="18" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D947" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E947" s="18" t="inlineStr">
+        <is>
+          <t>Virgin plastic preferred; 60% export condition after year three constrains recycler business models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B948" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C948" s="18" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D948" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E948" s="18" t="inlineStr">
+        <is>
+          <t>Need standardization of recycled granule quality and food-contact safety; recycled products could be cheaper without scrap tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B949" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C949" s="18" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D949" s="18" t="inlineStr">
+        <is>
+          <t>end-of-life plastic fate; micro- and nano-plastics (colored PET bottles cannot be effectively reused — only transparent PET can; colored PET emits significant microplastics when processed); health hazards from recycled plastics in food-contact applications; carcinogenic emissions from poor recycling sector practices (processing at 100–200°C); exploitation of informal waste pickers (especially women) at landfills/dumpsites</t>
+        </is>
+      </c>
+      <c r="E949" s="18" t="inlineStr">
+        <is>
+          <t>Micro/nano plastics from colored PET; food-contact safety risks; carcinogenic emissions from poor recyclers; informal picker exploitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B950" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C950" s="18" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D950" s="18" t="inlineStr">
+        <is>
+          <t>informal waste pickers, particularly women selling PET from landfills/dumpsites for NPR 10 (vs NPR 25/kg formal rate) and facing intimidation/violence from intermediary "mafias"; the public exposed to unsafe recycled food-contact plastics and carcinogenic emissions from substandard recyclers; the environment from end-of-life plastics and microplastic release</t>
+        </is>
+      </c>
+      <c r="E950" s="18" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: informal waste pickers (especially women); public exposed to unsafe recycled food plastics and emissions; environment from end-of-life plastics. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B951" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C951" s="18" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D951" s="18" t="inlineStr">
+        <is>
+          <t>intermediary "mafias" who threaten and assault waste pickers who do not sell to them; substandard recyclers with "pathetic" social and environmental standards (100–200°C processing, carcinogenic emissions); the scrap tax on PET at municipal level (raising raw-material and granule costs); virgin-plastic preference among Nepali consumers and businesses; bureaucratic barriers (Department of Industry registration, 60% export condition after year three, repeated LG approvals on relocation); national government for not consulting recyclers on solid waste policy (improving only gradually)</t>
+        </is>
+      </c>
+      <c r="E951" s="18" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: intermediary mafias; substandard recyclers; scrap tax; virgin-plastic market preference; bureaucratic/export policy barriers; government consultation gaps. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B952" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C952" s="18" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D952" s="18" t="inlineStr">
+        <is>
+          <t>Creasion (recycling, downsizing, product conversion, safety-tested granules, High-Effluent Treatment Plant recycling ~10,000 L water with no drainage outflow); EU-funded plastic-recovery and entrepreneurship project; CAP project (World Bank/UNOPS/SACEP) with sophisticated recycling technology; municipal collaboration to identify and formalize informal collectors; Plus Nepal and informal NRR associations; CSO trainings for sector coordination</t>
+        </is>
+      </c>
+      <c r="E952" s="18" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: Creasion, EU project, CAP/World Bank project, municipal formalization of informal collectors, Plus Nepal/NRR associations. Organization positions itself as primary problem-solver. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B953" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C953" s="18" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D953" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E953" s="18" t="inlineStr">
+        <is>
+          <t>EU-funded project; CAP project (World Bank, UNOPS, SACEP); 60% export condition from government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B954" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C954" s="18" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D954" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E954" s="18" t="inlineStr">
+        <is>
+          <t>Collaboration with municipalities, informal/formal associations (Plus Nepal, NRR), CSO trainings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B955" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C955" s="18" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D955" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E955" s="18" t="inlineStr">
+        <is>
+          <t>Department of Industry and local government approvals required for setup/relocation; municipal scrap tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B956" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C956" s="18" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D956" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E956" s="18" t="inlineStr">
+        <is>
+          <t>Who buys recycled granules unclear with only two centers; policy consultation gap for private recyclers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B957" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C957" s="18" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D957" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E957" s="18" t="inlineStr">
+        <is>
+          <t>Department of Industry (registration, utilities, export condition).</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B958" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C958" s="18" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D958" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E958" s="18" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B959" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C959" s="18" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D959" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E959" s="18" t="inlineStr">
+        <is>
+          <t>LG approvals for industry setup; municipal scrap tax collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B960" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C960" s="18" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D960" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E960" s="18" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B961" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C961" s="18" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D961" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E961" s="18" t="inlineStr">
+        <is>
+          <t>Recycling entrepreneurs and formal/informal recycler associations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B962" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C962" s="18" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D962" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E962" s="18" t="inlineStr">
+        <is>
+          <t>Creasion and CSO sector coordinating trainings and advocacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B963" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C963" s="18" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D963" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E963" s="18" t="inlineStr">
+        <is>
+          <t>NA - research on methodology questioned but no science actors named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B964" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C964" s="18" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D964" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E964" s="18" t="inlineStr">
+        <is>
+          <t>Consumer preference for virgin plastic affects market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B965" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C965" s="18" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D965" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E965" s="18" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B966" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C966" s="18" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D966" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E966" s="18" t="inlineStr">
+        <is>
+          <t>Buyers of recycled vs virgin granules; food vs non-food applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B967" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C967" s="18" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D967" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E967" s="18" t="inlineStr">
+        <is>
+          <t>Export conditionality; not consulting recyclers on policy; unclear data methodology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B968" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C968" s="18" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D968" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E968" s="18" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B969" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C969" s="18" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D969" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E969" s="18" t="inlineStr">
+        <is>
+          <t>See Cul_loc_government = yes (municipal scrap tax).</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B970" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C970" s="18" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D970" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E970" s="18" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B971" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C971" s="18" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D971" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E971" s="18" t="inlineStr">
+        <is>
+          <t>Substandard recyclers with carcinogenic emissions; intermediary mafias exploiting pickers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B972" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C972" s="18" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D972" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E972" s="18" t="inlineStr">
+        <is>
+          <t>NA - CSOs portrayed as heroes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B973" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C973" s="18" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D973" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E973" s="18" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B974" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C974" s="18" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D974" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E974" s="18" t="inlineStr">
+        <is>
+          <t>Virgin plastic preference limits recycled market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B975" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C975" s="18" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D975" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E975" s="18" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B976" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C976" s="18" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D976" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E976" s="18" t="inlineStr">
+        <is>
+          <t>NA - virgin preference coded under Cul_households/market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B977" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C977" s="18" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D977" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E977" s="18" t="inlineStr">
+        <is>
+          <t>NA - national level discussed as policy reform need but not primary target group in notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B978" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C978" s="18" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D978" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E978" s="18" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B979" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C979" s="18" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D979" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E979" s="18" t="inlineStr">
+        <is>
+          <t>Municipal collaboration to formalize informal collectors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B980" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C980" s="18" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D980" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E980" s="18" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B981" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C981" s="18" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D981" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E981" s="18" t="inlineStr">
+        <is>
+          <t>Recycling entrepreneurs need capacity-building and fair policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B982" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C982" s="18" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D982" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E982" s="18" t="inlineStr">
+        <is>
+          <t>CSO trainings; Plus Nepal and NRR as coordination channels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B983" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C983" s="18" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D983" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E983" s="18" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B984" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C984" s="18" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D984" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E984" s="18" t="inlineStr">
+        <is>
+          <t>Consumer awareness on recycled vs virgin plastic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B985" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C985" s="18" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D985" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E985" s="18" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B986" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C986" s="18" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D986" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E986" s="18" t="inlineStr">
+        <is>
+          <t>Industry standards and food-contact safety compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B987" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C987" s="18" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D987" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E987" s="18" t="inlineStr">
+        <is>
+          <t>Creasion operates recycling facilities, EU/CAP projects, entrepreneur capacity-building and municipal partnerships — managerial/organisational implementer (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B988" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C988" s="18" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D988" s="18" t="inlineStr">
+        <is>
+          <t>Creasion designs its own recycling and product-conversion processes, develops granule quality/safety standards and government-standard testing before market release, runs EU and CAP projects, collaborates with municipalities to identify informal collectors, and builds entrepreneur capacity — but faces constrained discretion on bureaucratic setup (Dept of Industry, LG approvals) and export/tax policy conditions.</t>
+        </is>
+      </c>
+      <c r="E988" s="18" t="inlineStr">
+        <is>
+          <t>Own processing standards, safety testing, water-recycling ATP, project design — but constrained by Dept of Industry/LG bureaucracy and tax/export rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B989" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C989" s="18" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D989" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E989" s="18" t="inlineStr">
+        <is>
+          <t>Weak sector standards enforcement; unclear national waste quantification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B990" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C990" s="18" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D990" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E990" s="18" t="inlineStr">
+        <is>
+          <t>Scrap tax raises costs; operating at competitive disadvantage vs virgin plastic; export condition after year 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B991" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C991" s="18" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D991" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E991" s="18" t="inlineStr">
+        <is>
+          <t>Questions World Bank PET percentage methodology; developing own granule standardization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B992" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C992" s="18" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D992" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E992" s="18" t="inlineStr">
+        <is>
+          <t>Bureaucratic hurdles for land, water, electricity on setup/relocation; ATP and CAP technology as infrastructure solutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B993" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C993" s="18" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D993" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E993" s="18" t="inlineStr">
+        <is>
+          <t>Building entrepreneur and informal-collector capacity via EU/CAP projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B994" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C994" s="18" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D994" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E994" s="18" t="inlineStr">
+        <is>
+          <t>Sector social/environmental standards weakly enforced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B995" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C995" s="18" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D995" s="18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E995" s="18" t="inlineStr">
+        <is>
+          <t>EPR not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B996" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C996" s="18" t="inlineStr">
+        <is>
+          <t>Pol_tax</t>
+        </is>
+      </c>
+      <c r="D996" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E996" s="18" t="inlineStr">
+        <is>
+          <t>Scrap tax on PET bottles paid at municipal level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B997" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C997" s="18" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D997" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E997" s="18" t="inlineStr">
+        <is>
+          <t>Creasion's recycling, downsizing and product-conversion operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B998" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C998" s="18" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D998" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E998" s="18" t="inlineStr">
+        <is>
+          <t>Tax undermines recycled competitiveness; weak standards; consultation gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B999" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C999" s="18" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D999" s="18" t="inlineStr">
+        <is>
+          <t>Scrap tax on PET at municipal level raised raw-material and granule costs, making recycled products less competitive than virgin plastic; social/environmental standards across the broader recycling sector described as "pathetic" with weak enforcement; Creasion "not consulted" on solid waste management policy development (gradually being included); national plastic-generation estimates (60,000 t/year; 27% PET per World Bank) questioned as methodology unclear.</t>
+        </is>
+      </c>
+      <c r="E999" s="18" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1000" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1000" s="18" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1000" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1000" s="18" t="inlineStr">
+        <is>
+          <t>Sector coordination via formal/informal associations and CSO trainings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1001" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1001" s="18" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1001" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1001" s="18" t="inlineStr">
+        <is>
+          <t>Entrepreneur and informal-worker support programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1002" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1002" s="18" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1002" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1002" s="18" t="inlineStr">
+        <is>
+          <t>High-quality granule production with safety testing; CAP technology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1003" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1003" s="18" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1003" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1003" s="18" t="inlineStr">
+        <is>
+          <t>CSO trainings for formal and informal associations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1004" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1004" s="18" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1004" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1004" s="18" t="inlineStr">
+        <is>
+          <t>EU project entrepreneurship support; CAP entrepreneur capacity-building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1005" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1005" s="18" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1005" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1005" s="18" t="inlineStr">
+        <is>
+          <t>Reconsider scrap tax and export conditionality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1006" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1006" s="18" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1006" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1006" s="18" t="inlineStr">
+        <is>
+          <t>Streamline Dept of Industry/LG approval processes; ATP water recycling model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1007" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1007" s="18" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1007" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1007" s="18" t="inlineStr">
+        <is>
+          <t>Standardize and enforce social/environmental standards across recyclers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1008" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1008" s="18" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1008" s="18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1008" s="18" t="inlineStr">
+        <is>
+          <t>Clearer national plastic-waste measurement methodology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="18" t="inlineStr">
+        <is>
+          <t>NPL_13</t>
+        </is>
+      </c>
+      <c r="B1009" s="18" t="inlineStr">
+        <is>
+          <t>Creasion - Recycling and waste-management CSO, Chitwan area (23 June 2025, ~5:15pm)</t>
+        </is>
+      </c>
+      <c r="C1009" s="18" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1009" s="18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1009" s="18" t="inlineStr">
+        <is>
+          <t>NA - not discussed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Code NPL_14 Hotel Silent Park Rajesh Aryal interview
Add Hotel Silent Park (Rajesh Aryal), Chitwan tourism/hotel sector as
NPL_14 from verbatim transcript. Codes animal ingestion, burning,
irregular Eco-Green/municipal collection, nature-guide cleanliness
model, and aluminum-foil concern. Exclude bundled policy-theme notes
not in this transcript.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -62,74 +62,80 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC4A2"/>
-        <bgColor rgb="00EBC4A2"/>
+        <fgColor rgb="00EBC1A2"/>
+        <bgColor rgb="00EBC1A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE5A2"/>
-        <bgColor rgb="00EBE5A2"/>
+        <fgColor rgb="00EBE0A2"/>
+        <bgColor rgb="00EBE0A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFEBA2"/>
-        <bgColor rgb="00CFEBA2"/>
+        <fgColor rgb="00D6EBA2"/>
+        <bgColor rgb="00D6EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADEBA2"/>
-        <bgColor rgb="00ADEBA2"/>
+        <fgColor rgb="00B7EBA2"/>
+        <bgColor rgb="00B7EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBB8"/>
-        <bgColor rgb="00A2EBB8"/>
+        <fgColor rgb="00A2EBAC"/>
+        <bgColor rgb="00A2EBAC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBDA"/>
-        <bgColor rgb="00A2EBDA"/>
+        <fgColor rgb="00A2EBCC"/>
+        <bgColor rgb="00A2EBCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2DAEB"/>
-        <bgColor rgb="00A2DAEB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2B8EB"/>
-        <bgColor rgb="00A2B8EB"/>
+        <fgColor rgb="00A2CCEB"/>
+        <bgColor rgb="00A2CCEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADA2EB"/>
-        <bgColor rgb="00ADA2EB"/>
+        <fgColor rgb="00A2ACEB"/>
+        <bgColor rgb="00A2ACEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFA2EB"/>
-        <bgColor rgb="00CFA2EB"/>
+        <fgColor rgb="00B7A2EB"/>
+        <bgColor rgb="00B7A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E5"/>
-        <bgColor rgb="00EBA2E5"/>
+        <fgColor rgb="00D6A2EB"/>
+        <bgColor rgb="00D6A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C4"/>
-        <bgColor rgb="00EBA2C4"/>
+        <fgColor rgb="00EBA2E0"/>
+        <bgColor rgb="00EBA2E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2C1"/>
+        <bgColor rgb="00EBA2C1"/>
       </patternFill>
     </fill>
   </fills>
@@ -159,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -213,6 +219,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -580,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -599,7 +608,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_13, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_14, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -700,87 +709,94 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  13. NPL_13 - Creasion, recycling and waste-management CSO (Center for Research and Sustainable Development in Nepal). Interview date: 23 June 2025 (~5:15pm). Coded from guideline notes and field notes (no full verbatim transcript). NPF fields implied.</t>
+          <t xml:space="preserve">  13. NPL_13 - Creasion, recycling CSO. Coded from notes and field notes.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  14. NPL_14 - Hotel Silent Park, Rajesh Aryal, Chitwan (26 June 2025). Coded from transcript; policy-theme notes at top of source file excluded (different interview). NPF fields implied.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_13, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_14, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_13) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_14) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1967,7 +1983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ14"/>
+  <dimension ref="A1:CQ15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8745,6 +8761,483 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>private_companies</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O15" s="19" t="inlineStr">
+        <is>
+          <t>wildlife and domestic animals (ingest salty plastic snack wrappers while eating food), air pollution (burning plastics), visual pollution and overflowing bins (wind and dogs/animals scatter uncollected waste), aluminum foil food packaging (greater disposal problem than plastic because recyclers do not collect it), tourism/safari area cleanliness</t>
+        </is>
+      </c>
+      <c r="P15" s="19" t="inlineStr">
+        <is>
+          <t>wildlife and domestic animals (ingesting plastic, especially salty snack wrappers); the local environment and air quality (burning plastics); the tourist/safari area and community when bins overflow and waste is scattered by wind and animals</t>
+        </is>
+      </c>
+      <c r="Q15" s="19" t="inlineStr">
+        <is>
+          <t>the general public/hotels (laziness, low awareness, convenience — plastic bags given free at shops; irregular use of cloth bags); shops/organizations that give plastic bags at no cost; municipal collection system (irregular Eco-Green bottle pickup every 15–20 days; municipal trucks not on time — bins overflow); hotel sector (thousands of hotels in Chitwan with discussion but no continuous waste-management action); aluminum foil packaging widely used for food wrapping without recycling route</t>
+        </is>
+      </c>
+      <c r="R15" s="19" t="inlineStr">
+        <is>
+          <t>nature guides (trained not to litter, collect wrappers during safari walks); park rangers and hotel associations (awareness/training); Eco-Green (recycles plastic bottles); informal collectors buying bottles at NPR 10–15/kg; safari dustbin system (compulsory bucket in vehicles); ward-level awareness and designated street cleaners (proposed); elephant-dung cleaning teams as a model (twice daily)</t>
+        </is>
+      </c>
+      <c r="S15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AW15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA15" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB15" s="19" t="inlineStr">
+        <is>
+          <t>As a hotel operator Rajesh Aryal stores plastic bottles for Eco-Green recycling, separates other plastics for municipal trucks, empties bottles before disposal, and participates in hotel-association discussions — but has no authority over municipal collection schedules, ward enforcement, or thousands of other hotels' waste practices in Chitwan.</t>
+        </is>
+      </c>
+      <c r="BC15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI15" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BS15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW15" s="19" t="inlineStr">
+        <is>
+          <t>Eco-Green collects bottles every 15–20 days but "it's irregular" and "this time it has been long since it has collected"; municipal dustbins provided but "if collection doesn't happen on time, wind spreads the waste"; awareness and cleanup programs exist "occasionally" but "there's no continuous action" — Environment Day "only one day, doesn't continue beyond that"; "no notices" from municipality on plastic removal.</t>
+        </is>
+      </c>
+      <c r="BX15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BY15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CN15" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO15" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP15" s="19" t="inlineStr">
+        <is>
+          <t>Cloth/fiber bags instead of plastic shopping bags; clay or cement pots instead of plastic flower pots.</t>
+        </is>
+      </c>
+      <c r="CQ15" s="19" t="inlineStr">
+        <is>
+          <t>Master list label: "14. Hotel Silent Park/ Rajesh Aryal", affiliation: Hotel Silent Park. Interviewee: Rajesh Aryal. Location: Chitwan (Sauraha/safari tourism area). Interview date: 26 June 2025. Interviewers: Ram Devi and Deep. Coded from the verbatim transcript and field notes attributable to this respondent. DATA-QUALITY NOTE: the structured theme notes at the top of the source document (PLEASE/Bio-Camp pilot, EPR nationwide, Plast Foundation, Solid Waste Management Association, comprehensive policy challenges, etc.) do not appear in the Rajesh Aryal transcript and were excluded as likely belonging to a different interview bundled in the same file. One bullet note states the respondent is "not so much concerned about plastics; more Aluminium foil" — coded as medium concern reflecting this nuance. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8756,7 +9249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1009"/>
+  <dimension ref="A1:E1079"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34925,7 +35418,7 @@
       </c>
       <c r="E969" s="18" t="inlineStr">
         <is>
-          <t>See Cul_loc_government = yes (municipal scrap tax).</t>
+          <t>Municipal scrap tax raising recycler costs.</t>
         </is>
       </c>
     </row>
@@ -36006,6 +36499,1896 @@
       <c r="E1009" s="18" t="inlineStr">
         <is>
           <t>NA - not discussed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1010" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1010" s="19" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1010" s="19" t="inlineStr">
+        <is>
+          <t>private_companies</t>
+        </is>
+      </c>
+      <c r="E1010" s="19" t="inlineStr">
+        <is>
+          <t>Rajesh Aryal is associated with Hotel Silent Park in Chitwan — coded as private_companies (hotel/tourism sector).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1011" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1011" s="19" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1011" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1011" s="19" t="inlineStr">
+        <is>
+          <t>"Ignorance and lack of awareness"; people lazy; plastic bags given free at shops; cloth bags not used consistently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1012" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1012" s="19" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1012" s="19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E1012" s="19" t="inlineStr">
+        <is>
+          <t>Acknowledges plastic pollution everywhere, burning, animal ingestion and need for management, but one field note states greater concern about aluminum foil than plastic — coded medium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1013" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1013" s="19" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1013" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1013" s="19" t="inlineStr">
+        <is>
+          <t>Bins overflow when collection delayed; wind spreads waste; dogs/animals scatter it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1014" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1014" s="19" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1014" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1014" s="19" t="inlineStr">
+        <is>
+          <t>"Plastic is easy and fast"; shoppers use free plastic bags instead of cloth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1015" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1015" s="19" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1015" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1015" s="19" t="inlineStr">
+        <is>
+          <t>Eco-Green bottle collection irregular; aluminum foil not taken by recyclers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1016" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1016" s="19" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1016" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1016" s="19" t="inlineStr">
+        <is>
+          <t>Collection system problematic — not on time; no continuous hotel/ward management programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1017" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1017" s="19" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1017" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1017" s="19" t="inlineStr">
+        <is>
+          <t>Cloth/fiber bags and clay/cement pots cited as alternatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1018" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1018" s="19" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1018" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1018" s="19" t="inlineStr">
+        <is>
+          <t>Bottles stored separately for Eco-Green; wrappers via municipal trucks; bottles emptied before disposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1019" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1019" s="19" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1019" s="19" t="inlineStr">
+        <is>
+          <t>wildlife and domestic animals (ingest salty plastic snack wrappers while eating food), air pollution (burning plastics), visual pollution and overflowing bins (wind and dogs/animals scatter uncollected waste), aluminum foil food packaging (greater disposal problem than plastic because recyclers do not collect it), tourism/safari area cleanliness</t>
+        </is>
+      </c>
+      <c r="E1019" s="19" t="inlineStr">
+        <is>
+          <t>Animal ingestion, burning air pollution, bin overflow, aluminum foil disposal gap, tourism area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1020" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1020" s="19" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1020" s="19" t="inlineStr">
+        <is>
+          <t>wildlife and domestic animals (ingesting plastic, especially salty snack wrappers); the local environment and air quality (burning plastics); the tourist/safari area and community when bins overflow and waste is scattered by wind and animals</t>
+        </is>
+      </c>
+      <c r="E1020" s="19" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: wildlife/domestic animals; environment/air; tourist area/community when waste spreads. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1021" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1021" s="19" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1021" s="19" t="inlineStr">
+        <is>
+          <t>the general public/hotels (laziness, low awareness, convenience — plastic bags given free at shops; irregular use of cloth bags); shops/organizations that give plastic bags at no cost; municipal collection system (irregular Eco-Green bottle pickup every 15–20 days; municipal trucks not on time — bins overflow); hotel sector (thousands of hotels in Chitwan with discussion but no continuous waste-management action); aluminum foil packaging widely used for food wrapping without recycling route</t>
+        </is>
+      </c>
+      <c r="E1021" s="19" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: lazy/unaware public; free plastic-bag distribution; irregular municipal/Eco-Green collection; hotels without continuous management. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1022" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1022" s="19" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1022" s="19" t="inlineStr">
+        <is>
+          <t>nature guides (trained not to litter, collect wrappers during safari walks); park rangers and hotel associations (awareness/training); Eco-Green (recycles plastic bottles); informal collectors buying bottles at NPR 10–15/kg; safari dustbin system (compulsory bucket in vehicles); ward-level awareness and designated street cleaners (proposed); elephant-dung cleaning teams as a model (twice daily)</t>
+        </is>
+      </c>
+      <c r="E1022" s="19" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: nature guides, park rangers, hotel associations, Eco-Green, informal bottle collectors, safari dustbin system, proposed ward cleaners. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1023" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1023" s="19" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D1023" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1023" s="19" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1024" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1024" s="19" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D1024" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1024" s="19" t="inlineStr">
+        <is>
+          <t>Hotel associations, NGOs, park rangers and nature guides coordinate awareness; Eco-Green and municipality split collection roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1025" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1025" s="19" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D1025" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1025" s="19" t="inlineStr">
+        <is>
+          <t>Municipal trucks vs private Eco-Green vs informal collectors; ward enforcement proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1026" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1026" s="19" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1026" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1026" s="19" t="inlineStr">
+        <is>
+          <t>NA - not explicitly discussed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1027" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1027" s="19" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1027" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1027" s="19" t="inlineStr">
+        <is>
+          <t>NA - not named as responsible actor in this interview.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1028" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1028" s="19" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1028" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1028" s="19" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1029" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1029" s="19" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1029" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1029" s="19" t="inlineStr">
+        <is>
+          <t>Municipal trucks collect bags/wrappers; dustbins provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1030" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1030" s="19" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1030" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1030" s="19" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1031" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1031" s="19" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1031" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1031" s="19" t="inlineStr">
+        <is>
+          <t>Eco-Green recycles bottles; informal collectors buy PET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1032" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1032" s="19" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1032" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1032" s="19" t="inlineStr">
+        <is>
+          <t>NGOs, park rangers, hotel associations train nature guides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1033" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1033" s="19" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1033" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1033" s="19" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1034" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1034" s="19" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1034" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1034" s="19" t="inlineStr">
+        <is>
+          <t>Store and separate waste at home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1035" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1035" s="19" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1035" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1035" s="19" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1036" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1036" s="19" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1036" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1036" s="19" t="inlineStr">
+        <is>
+          <t>Thousands of Chitwan hotels generate waste; hotel association discussions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1037" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1037" s="19" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1037" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1037" s="19" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1038" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1038" s="19" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1038" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1038" s="19" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1039" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1039" s="19" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1039" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1039" s="19" t="inlineStr">
+        <is>
+          <t>No municipal notices; irregular collection; streets not cleaned regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1040" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1040" s="19" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1040" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1040" s="19" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1041" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1041" s="19" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1041" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1041" s="19" t="inlineStr">
+        <is>
+          <t>NA - Eco-Green/informal collectors portrayed positively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1042" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1042" s="19" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1042" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1042" s="19" t="inlineStr">
+        <is>
+          <t>NA - NGOs/guides portrayed as heroes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1043" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1043" s="19" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1043" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1043" s="19" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1044" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1044" s="19" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1044" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1044" s="19" t="inlineStr">
+        <is>
+          <t>Laziness, ignorance, convenience, free plastic bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1045" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1045" s="19" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1045" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1045" s="19" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1046" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1046" s="19" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1046" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1046" s="19" t="inlineStr">
+        <is>
+          <t>Hotels discuss but lack continuous waste-management action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1047" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1047" s="19" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1047" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1047" s="19" t="inlineStr">
+        <is>
+          <t>NA - not named as target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1048" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1048" s="19" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1048" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1048" s="19" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1049" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1049" s="19" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1049" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1049" s="19" t="inlineStr">
+        <is>
+          <t>Ward should launch awareness campaigns, enforce rules, provide dustbins, designate street cleaners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1050" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1050" s="19" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1050" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1050" s="19" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1051" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1051" s="19" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1051" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1051" s="19" t="inlineStr">
+        <is>
+          <t>NA - informal collectors positive; hotel committee proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1052" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1052" s="19" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1052" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1052" s="19" t="inlineStr">
+        <is>
+          <t>Nature guides and hotel associations for sustained training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1053" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1053" s="19" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1053" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1053" s="19" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1054" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1054" s="19" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1054" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1054" s="19" t="inlineStr">
+        <is>
+          <t>Use cloth bags; reduce plastic attachment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1055" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1055" s="19" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1055" s="19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1055" s="19" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1056" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1056" s="19" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1056" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1056" s="19" t="inlineStr">
+        <is>
+          <t>Hotel business community could form cleanliness committee (rickshaw collection ~NPR 50,000/month proposed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1057" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1057" s="19" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1057" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1057" s="19" t="inlineStr">
+        <is>
+          <t>Hotel operator describing personal and sector waste practices as a target group of policies (role 4), not a policy formulator or primary implementer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1058" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1058" s="19" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1058" s="19" t="inlineStr">
+        <is>
+          <t>As a hotel operator Rajesh Aryal stores plastic bottles for Eco-Green recycling, separates other plastics for municipal trucks, empties bottles before disposal, and participates in hotel-association discussions — but has no authority over municipal collection schedules, ward enforcement, or thousands of other hotels' waste practices in Chitwan.</t>
+        </is>
+      </c>
+      <c r="E1058" s="19" t="inlineStr">
+        <is>
+          <t>Stores bottles for Eco-Green, separates waste for municipal collection, empties bottles — limited to own hotel/household practices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1059" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1059" s="19" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1059" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1059" s="19" t="inlineStr">
+        <is>
+          <t>No municipal notices or rules observed; irregular programme monitoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1060" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1060" s="19" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D1060" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1060" s="19" t="inlineStr">
+        <is>
+          <t>Hotel committee rickshaw collection (~NPR 50,000/month) proposed; bottle monetary value (NPR 10–15/kg) drives informal collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1061" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1061" s="19" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1061" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1061" s="19" t="inlineStr">
+        <is>
+          <t>Dustbins provided but overflow; safari vehicle buckets compulsory; need designated street cleaners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1062" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1062" s="19" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1062" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1062" s="19" t="inlineStr">
+        <is>
+          <t>No designated street cleaners (unlike elephant-dung teams); awareness programmes lack continuity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1063" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1063" s="19" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1063" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1063" s="19" t="inlineStr">
+        <is>
+          <t>No municipal enforcement notices; ward strict rules proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1064" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1064" s="19" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D1064" s="19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1064" s="19" t="inlineStr">
+        <is>
+          <t>EPR not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1065" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1065" s="19" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1065" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1065" s="19" t="inlineStr">
+        <is>
+          <t>Occasional programmes by NGOs, hotel associations, park rangers — not continuous.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1066" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1066" s="19" t="inlineStr">
+        <is>
+          <t>Pol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1066" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1066" s="19" t="inlineStr">
+        <is>
+          <t>Environment Day one-day events; safari dustbin rule; elephant-dung teams twice daily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1067" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1067" s="19" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1067" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1067" s="19" t="inlineStr">
+        <is>
+          <t>Eco-Green bottle collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1068" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1068" s="19" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1068" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1068" s="19" t="inlineStr">
+        <is>
+          <t>Municipal trucks for wrappers/bags; irregular schedules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1069" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1069" s="19" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1069" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1069" s="19" t="inlineStr">
+        <is>
+          <t>Irregular collection and awareness; no continuous action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1070" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1070" s="19" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1070" s="19" t="inlineStr">
+        <is>
+          <t>Eco-Green collects bottles every 15–20 days but "it's irregular" and "this time it has been long since it has collected"; municipal dustbins provided but "if collection doesn't happen on time, wind spreads the waste"; awareness and cleanup programs exist "occasionally" but "there's no continuous action" — Environment Day "only one day, doesn't continue beyond that"; "no notices" from municipality on plastic removal.</t>
+        </is>
+      </c>
+      <c r="E1070" s="19" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1071" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1071" s="19" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1071" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1071" s="19" t="inlineStr">
+        <is>
+          <t>Ward awareness campaigns to reduce negligence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1072" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1072" s="19" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1072" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1072" s="19" t="inlineStr">
+        <is>
+          <t>Sustained nature-guide and hotel-association training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1073" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1073" s="19" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1073" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1073" s="19" t="inlineStr">
+        <is>
+          <t>Train population through hotel association/NGO programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1074" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1074" s="19" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1074" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1074" s="19" t="inlineStr">
+        <is>
+          <t>Hotel committee fund for rickshaw waste collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1075" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1075" s="19" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1075" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1075" s="19" t="inlineStr">
+        <is>
+          <t>Ward dustbins; safari vehicle buckets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1076" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1076" s="19" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1076" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1076" s="19" t="inlineStr">
+        <is>
+          <t>Cloth/fiber bags; clay/cement pots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1077" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1077" s="19" t="inlineStr">
+        <is>
+          <t>Sol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1077" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1077" s="19" t="inlineStr">
+        <is>
+          <t>Designated street cleaners; daily collection like elephant-dung teams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1078" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1078" s="19" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1078" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1078" s="19" t="inlineStr">
+        <is>
+          <t>Ward strict rule enforcement proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1079" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1079" s="19" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1079" s="19" t="inlineStr">
+        <is>
+          <t>Cloth/fiber bags instead of plastic shopping bags; clay or cement pots instead of plastic flower pots.</t>
+        </is>
+      </c>
+      <c r="E1079" s="19" t="inlineStr">
+        <is>
+          <t>Cloth bags; clay/cement pots instead of plastic.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recode NPL_14 including full policy-themed guideline notes
Integrate Themes A-D policy content (EPR, PLEASE/Bio-Camp, informal
sector, Environmental Protection Act, microplastics, three-tier
governance) with Rajesh Aryal transcript rather than excluding
guideline notes as a separate interview.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -716,7 +716,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  14. NPL_14 - Hotel Silent Park, Rajesh Aryal, Chitwan (26 June 2025). Coded from transcript; policy-theme notes at top of source file excluded (different interview). NPF fields implied.</t>
+          <t xml:space="preserve">  14. NPL_14 - Hotel Silent Park, Rajesh Aryal, Chitwan (26 June 2025). Coded from full interview package (guideline policy themes and verbatim transcript). NPF fields implied.</t>
         </is>
       </c>
     </row>
@@ -8784,12 +8784,12 @@
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G15" s="19" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="L15" s="19" t="inlineStr">
@@ -8834,27 +8834,27 @@
       </c>
       <c r="O15" s="19" t="inlineStr">
         <is>
-          <t>wildlife and domestic animals (ingest salty plastic snack wrappers while eating food), air pollution (burning plastics), visual pollution and overflowing bins (wind and dogs/animals scatter uncollected waste), aluminum foil food packaging (greater disposal problem than plastic because recyclers do not collect it), tourism/safari area cleanliness</t>
+          <t>wildlife and domestic animals (ingest salty plastic snack wrappers); air pollution (burning plastics; poor communities use plastic as fire starters); microplastics contaminating soil, water, air, rivers, irrigation water and organic fertilisers (reducing soil moisture, potentially affecting crop yields); health (low-quality packaging may leach chemicals; unsafe bottled water/labelling practices); visual pollution and clogged drains/rivers; aluminum foil food packaging (greater disposal problem than plastic because recyclers do not collect it); tourism/safari area when bins overflow</t>
         </is>
       </c>
       <c r="P15" s="19" t="inlineStr">
         <is>
-          <t>wildlife and domestic animals (ingesting plastic, especially salty snack wrappers); the local environment and air quality (burning plastics); the tourist/safari area and community when bins overflow and waste is scattered by wind and animals</t>
+          <t>wildlife and domestic animals; poor communities exposed to burning and fire-starter practices; farmers/agriculture (microplastics in soil reducing moisture and crop yields); the general public (chemical leaching, unsafe bottled water); the tourist/safari area and local community when collection fails and waste spreads</t>
         </is>
       </c>
       <c r="Q15" s="19" t="inlineStr">
         <is>
-          <t>the general public/hotels (laziness, low awareness, convenience — plastic bags given free at shops; irregular use of cloth bags); shops/organizations that give plastic bags at no cost; municipal collection system (irregular Eco-Green bottle pickup every 15–20 days; municipal trucks not on time — bins overflow); hotel sector (thousands of hotels in Chitwan with discussion but no continuous waste-management action); aluminum foil packaging widely used for food wrapping without recycling route</t>
+          <t>the general public/hotels (low awareness, laziness, convenience, free plastic bags, perception that waste management is solely government's responsibility); national government (no comprehensive plastics policy — only general Environmental Protection Act; weak enforcement of &lt;40-micron ban; political instability delaying implementation); unclear federal/provincial/local authority division; municipal collection system (irregular Eco-Green and municipal trucks; bins overflow); hotel sector (thousands of Chitwan hotels with no continuous waste-management action); aluminum foil widely used without recycling route; heavy informal-sector reliance without formal integration</t>
         </is>
       </c>
       <c r="R15" s="19" t="inlineStr">
         <is>
-          <t>nature guides (trained not to litter, collect wrappers during safari walks); park rangers and hotel associations (awareness/training); Eco-Green (recycles plastic bottles); informal collectors buying bottles at NPR 10–15/kg; safari dustbin system (compulsory bucket in vehicles); ward-level awareness and designated street cleaners (proposed); elephant-dung cleaning teams as a model (twice daily)</t>
+          <t>nature guides and park rangers (trained not to litter, collect wrappers on safari); hotel associations and NGOs (awareness training); Eco-Green and informal collectors (NPR 10–15/kg for bottles; informal sector collects ~99% of valuable plastics from hotels); PLEASE and Bio-Camp pilot projects (segregation, recycling/upcycling); Solid Waste Management Association and Plast Foundation Nepal; safari dustbin system; proposed EPR nationwide and ward-level designated street cleaners; elephant-dung cleaning teams as operational model (twice daily)</t>
         </is>
       </c>
       <c r="S15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="T15" s="19" t="inlineStr">
@@ -8869,17 +8869,17 @@
       </c>
       <c r="V15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="X15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="Y15" s="19" t="inlineStr">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="AG15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AH15" s="19" t="inlineStr">
@@ -8974,7 +8974,7 @@
       </c>
       <c r="AQ15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AR15" s="19" t="inlineStr">
@@ -8994,7 +8994,7 @@
       </c>
       <c r="AU15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AV15" s="19" t="inlineStr">
@@ -9029,7 +9029,7 @@
       </c>
       <c r="BB15" s="19" t="inlineStr">
         <is>
-          <t>As a hotel operator Rajesh Aryal stores plastic bottles for Eco-Green recycling, separates other plastics for municipal trucks, empties bottles before disposal, and participates in hotel-association discussions — but has no authority over municipal collection schedules, ward enforcement, or thousands of other hotels' waste practices in Chitwan.</t>
+          <t>As a hotel operator Rajesh Aryal stores plastic bottles for Eco-Green recycling, separates other plastics for municipal trucks, empties bottles before disposal, and participates in hotel-association discussions — but has no authority over municipal collection schedules, national policy formulation, or thousands of other hotels' waste practices in Chitwan.</t>
         </is>
       </c>
       <c r="BC15" s="19" t="inlineStr">
@@ -9044,7 +9044,7 @@
       </c>
       <c r="BE15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BF15" s="19" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="BL15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BM15" s="19" t="inlineStr">
@@ -9099,12 +9099,12 @@
       </c>
       <c r="BP15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BQ15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BR15" s="19" t="inlineStr">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="BS15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BT15" s="19" t="inlineStr">
@@ -9134,22 +9134,22 @@
       </c>
       <c r="BW15" s="19" t="inlineStr">
         <is>
-          <t>Eco-Green collects bottles every 15–20 days but "it's irregular" and "this time it has been long since it has collected"; municipal dustbins provided but "if collection doesn't happen on time, wind spreads the waste"; awareness and cleanup programs exist "occasionally" but "there's no continuous action" — Environment Day "only one day, doesn't continue beyond that"; "no notices" from municipality on plastic removal.</t>
+          <t>Environmental Protection Act exists but no specific plastics policy; &lt;40-micron ban weakly enforced; federal government assessing new plastics act but guidelines unclear; Eco-Green bottle collection every 15–20 days but irregular; municipal collection not on time (bins overflow); awareness/cleanup programmes occasional — Environment Day "only one day"; PLEASE/Bio-Camp pilots show promise but not yet scaled; effectiveness limited by low enforcement, irregular collection and inconsistent public awareness.</t>
         </is>
       </c>
       <c r="BX15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BY15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="BZ15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="CA15" s="19" t="inlineStr">
@@ -9159,17 +9159,17 @@
       </c>
       <c r="CB15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="CC15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="CD15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="CE15" s="19" t="inlineStr">
@@ -9184,7 +9184,7 @@
       </c>
       <c r="CG15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="CH15" s="19" t="inlineStr">
@@ -9224,17 +9224,17 @@
       </c>
       <c r="CO15" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="CP15" s="19" t="inlineStr">
         <is>
-          <t>Cloth/fiber bags instead of plastic shopping bags; clay or cement pots instead of plastic flower pots.</t>
+          <t>Natural plates from banana leaves and pat leaves during feasts; cotton or towel bags for shopping; cloth/fiber bags and clay/cement pots instead of plastic; reuse of plastics before recycling.</t>
         </is>
       </c>
       <c r="CQ15" s="19" t="inlineStr">
         <is>
-          <t>Master list label: "14. Hotel Silent Park/ Rajesh Aryal", affiliation: Hotel Silent Park. Interviewee: Rajesh Aryal. Location: Chitwan (Sauraha/safari tourism area). Interview date: 26 June 2025. Interviewers: Ram Devi and Deep. Coded from the verbatim transcript and field notes attributable to this respondent. DATA-QUALITY NOTE: the structured theme notes at the top of the source document (PLEASE/Bio-Camp pilot, EPR nationwide, Plast Foundation, Solid Waste Management Association, comprehensive policy challenges, etc.) do not appear in the Rajesh Aryal transcript and were excluded as likely belonging to a different interview bundled in the same file. One bullet note states the respondent is "not so much concerned about plastics; more Aluminium foil" — coded as medium concern reflecting this nuance. NPF fields implied, not explicit.</t>
+          <t>Master list label: "14. Hotel Silent Park/ Rajesh Aryal", affiliation: Hotel Silent Park. Interviewee: Rajesh Aryal. Location: Chitwan (Sauraha/safari tourism area). Interview date: 26 June 2025. Interviewers: Ram Devi and Deep. Coded from the full interview package: structured guideline notes (Themes A–D, including national policy challenges, PLEASE/Bio-Camp pilots, EPR, informal sector, Plast Foundation Nepal, Solid Waste Management Association) AND the verbatim Rajesh Aryal transcript. One field bullet notes greater concern about aluminum foil than plastic at the hotel level; overall interview concern coded high given visible/invisible pollution and microplastic impacts in guideline notes. NPF fields implied, not explicit.</t>
         </is>
       </c>
     </row>
@@ -9249,7 +9249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1079"/>
+  <dimension ref="A1:E1094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36525,7 +36525,7 @@
       </c>
       <c r="E1010" s="19" t="inlineStr">
         <is>
-          <t>Rajesh Aryal is associated with Hotel Silent Park in Chitwan — coded as private_companies (hotel/tourism sector).</t>
+          <t>Rajesh Aryal, Hotel Silent Park, Chitwan tourism/hotel sector — coded as private_companies.</t>
         </is>
       </c>
     </row>
@@ -36552,7 +36552,7 @@
       </c>
       <c r="E1011" s="19" t="inlineStr">
         <is>
-          <t>"Ignorance and lack of awareness"; people lazy; plastic bags given free at shops; cloth bags not used consistently.</t>
+          <t>Low awareness of eco-friendly alternatives; ignorance and laziness; people do not reuse/recycle properly due to convenience; plastic bags given free at shops.</t>
         </is>
       </c>
     </row>
@@ -36569,17 +36569,17 @@
       </c>
       <c r="C1012" s="19" t="inlineStr">
         <is>
-          <t>Problem_concerndness</t>
+          <t>Problem_awareness_pol</t>
         </is>
       </c>
       <c r="D1012" s="19" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1012" s="19" t="inlineStr">
         <is>
-          <t>Acknowledges plastic pollution everywhere, burning, animal ingestion and need for management, but one field note states greater concern about aluminum foil than plastic — coded medium.</t>
+          <t>No comprehensive plastics policy (only Environmental Protection Act); federal assessing new act but guidelines unclear; unclear division of authority across three tiers.</t>
         </is>
       </c>
     </row>
@@ -36596,17 +36596,17 @@
       </c>
       <c r="C1013" s="19" t="inlineStr">
         <is>
-          <t>Problem_littering</t>
+          <t>Problem_concerndness</t>
         </is>
       </c>
       <c r="D1013" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E1013" s="19" t="inlineStr">
         <is>
-          <t>Bins overflow when collection delayed; wind spreads waste; dogs/animals scatter it.</t>
+          <t>Guideline notes: very concerned about visible litter and invisible microplastic contamination; transcript also flags aluminum foil as a particular hotel-level disposal concern.</t>
         </is>
       </c>
     </row>
@@ -36623,7 +36623,7 @@
       </c>
       <c r="C1014" s="19" t="inlineStr">
         <is>
-          <t>Problem_consumption</t>
+          <t>Problem_littering</t>
         </is>
       </c>
       <c r="D1014" s="19" t="inlineStr">
@@ -36633,7 +36633,7 @@
       </c>
       <c r="E1014" s="19" t="inlineStr">
         <is>
-          <t>"Plastic is easy and fast"; shoppers use free plastic bags instead of cloth.</t>
+          <t>Plastic everywhere urban and rural; bins overflow; wind and animals scatter waste; drains and rivers clogged.</t>
         </is>
       </c>
     </row>
@@ -36650,7 +36650,7 @@
       </c>
       <c r="C1015" s="19" t="inlineStr">
         <is>
-          <t>Problem_recycling</t>
+          <t>Problem_consumption</t>
         </is>
       </c>
       <c r="D1015" s="19" t="inlineStr">
@@ -36660,7 +36660,7 @@
       </c>
       <c r="E1015" s="19" t="inlineStr">
         <is>
-          <t>Eco-Green bottle collection irregular; aluminum foil not taken by recyclers.</t>
+          <t>Plastic easy and fast; free bags at shops; widespread packaging.</t>
         </is>
       </c>
     </row>
@@ -36677,7 +36677,7 @@
       </c>
       <c r="C1016" s="19" t="inlineStr">
         <is>
-          <t>Problem_waste_mgmt</t>
+          <t>Problem_recycling</t>
         </is>
       </c>
       <c r="D1016" s="19" t="inlineStr">
@@ -36687,7 +36687,7 @@
       </c>
       <c r="E1016" s="19" t="inlineStr">
         <is>
-          <t>Collection system problematic — not on time; no continuous hotel/ward management programmes.</t>
+          <t>Eco-Green irregular; aluminum foil not collected by recyclers; informal sector collects 99% of valuable hotel plastics.</t>
         </is>
       </c>
     </row>
@@ -36704,7 +36704,7 @@
       </c>
       <c r="C1017" s="19" t="inlineStr">
         <is>
-          <t>Problem_alternatives</t>
+          <t>Problem_waste_mgmt</t>
         </is>
       </c>
       <c r="D1017" s="19" t="inlineStr">
@@ -36714,7 +36714,7 @@
       </c>
       <c r="E1017" s="19" t="inlineStr">
         <is>
-          <t>Cloth/fiber bags and clay/cement pots cited as alternatives.</t>
+          <t>Irregular municipal/Eco-Green collection; heavy informal-sector reliance without formal integration; political instability delays implementation.</t>
         </is>
       </c>
     </row>
@@ -36731,7 +36731,7 @@
       </c>
       <c r="C1018" s="19" t="inlineStr">
         <is>
-          <t>Problem_waste_segregation</t>
+          <t>Problem_production</t>
         </is>
       </c>
       <c r="D1018" s="19" t="inlineStr">
@@ -36741,7 +36741,7 @@
       </c>
       <c r="E1018" s="19" t="inlineStr">
         <is>
-          <t>Bottles stored separately for Eco-Green; wrappers via municipal trucks; bottles emptied before disposal.</t>
+          <t>Upstream production and packaging implied in policy discussion; virgin plastic preference in food-contact applications.</t>
         </is>
       </c>
     </row>
@@ -36758,17 +36758,17 @@
       </c>
       <c r="C1019" s="19" t="inlineStr">
         <is>
-          <t>Impacts</t>
+          <t>Problem_alternatives</t>
         </is>
       </c>
       <c r="D1019" s="19" t="inlineStr">
         <is>
-          <t>wildlife and domestic animals (ingest salty plastic snack wrappers while eating food), air pollution (burning plastics), visual pollution and overflowing bins (wind and dogs/animals scatter uncollected waste), aluminum foil food packaging (greater disposal problem than plastic because recyclers do not collect it), tourism/safari area cleanliness</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1019" s="19" t="inlineStr">
         <is>
-          <t>Animal ingestion, burning air pollution, bin overflow, aluminum foil disposal gap, tourism area.</t>
+          <t>Cloth bags, clay/cement pots, leaf plates promoted but awareness low.</t>
         </is>
       </c>
     </row>
@@ -36785,17 +36785,17 @@
       </c>
       <c r="C1020" s="19" t="inlineStr">
         <is>
-          <t>NPF_victims</t>
+          <t>Problem_waste_segregation</t>
         </is>
       </c>
       <c r="D1020" s="19" t="inlineStr">
         <is>
-          <t>wildlife and domestic animals (ingesting plastic, especially salty snack wrappers); the local environment and air quality (burning plastics); the tourist/safari area and community when bins overflow and waste is scattered by wind and animals</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1020" s="19" t="inlineStr">
         <is>
-          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: wildlife/domestic animals; environment/air; tourist area/community when waste spreads. No FLAG needed.</t>
+          <t>Bottles stored for Eco-Green; wrappers via municipal trucks; PLEASE/Bio-Camp demonstrate segregation pilots.</t>
         </is>
       </c>
     </row>
@@ -36812,17 +36812,17 @@
       </c>
       <c r="C1021" s="19" t="inlineStr">
         <is>
-          <t>NPF_villains</t>
+          <t>Impacts</t>
         </is>
       </c>
       <c r="D1021" s="19" t="inlineStr">
         <is>
-          <t>the general public/hotels (laziness, low awareness, convenience — plastic bags given free at shops; irregular use of cloth bags); shops/organizations that give plastic bags at no cost; municipal collection system (irregular Eco-Green bottle pickup every 15–20 days; municipal trucks not on time — bins overflow); hotel sector (thousands of hotels in Chitwan with discussion but no continuous waste-management action); aluminum foil packaging widely used for food wrapping without recycling route</t>
+          <t>wildlife and domestic animals (ingest salty plastic snack wrappers); air pollution (burning plastics; poor communities use plastic as fire starters); microplastics contaminating soil, water, air, rivers, irrigation water and organic fertilisers (reducing soil moisture, potentially affecting crop yields); health (low-quality packaging may leach chemicals; unsafe bottled water/labelling practices); visual pollution and clogged drains/rivers; aluminum foil food packaging (greater disposal problem than plastic because recyclers do not collect it); tourism/safari area when bins overflow</t>
         </is>
       </c>
       <c r="E1021" s="19" t="inlineStr">
         <is>
-          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: lazy/unaware public; free plastic-bag distribution; irregular municipal/Eco-Green collection; hotels without continuous management. No FLAG needed.</t>
+          <t>Animals, burning, microplastics (soil/water/air/crops), health/leaching, drains, aluminum foil, tourism area.</t>
         </is>
       </c>
     </row>
@@ -36839,17 +36839,17 @@
       </c>
       <c r="C1022" s="19" t="inlineStr">
         <is>
-          <t>NPF_hero</t>
+          <t>NPF_victims</t>
         </is>
       </c>
       <c r="D1022" s="19" t="inlineStr">
         <is>
-          <t>nature guides (trained not to litter, collect wrappers during safari walks); park rangers and hotel associations (awareness/training); Eco-Green (recycles plastic bottles); informal collectors buying bottles at NPR 10–15/kg; safari dustbin system (compulsory bucket in vehicles); ward-level awareness and designated street cleaners (proposed); elephant-dung cleaning teams as a model (twice daily)</t>
+          <t>wildlife and domestic animals; poor communities exposed to burning and fire-starter practices; farmers/agriculture (microplastics in soil reducing moisture and crop yields); the general public (chemical leaching, unsafe bottled water); the tourist/safari area and local community when collection fails and waste spreads</t>
         </is>
       </c>
       <c r="E1022" s="19" t="inlineStr">
         <is>
-          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: nature guides, park rangers, hotel associations, Eco-Green, informal bottle collectors, safari dustbin system, proposed ward cleaners. No FLAG needed.</t>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: animals; poor communities; farmers; public health; tourist/community areas. No FLAG needed.</t>
         </is>
       </c>
     </row>
@@ -36866,17 +36866,17 @@
       </c>
       <c r="C1023" s="19" t="inlineStr">
         <is>
-          <t>Relevance_international_pol</t>
+          <t>NPF_villains</t>
         </is>
       </c>
       <c r="D1023" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>the general public/hotels (low awareness, laziness, convenience, free plastic bags, perception that waste management is solely government's responsibility); national government (no comprehensive plastics policy — only general Environmental Protection Act; weak enforcement of &lt;40-micron ban; political instability delaying implementation); unclear federal/provincial/local authority division; municipal collection system (irregular Eco-Green and municipal trucks; bins overflow); hotel sector (thousands of Chitwan hotels with no continuous waste-management action); aluminum foil widely used without recycling route; heavy informal-sector reliance without formal integration</t>
         </is>
       </c>
       <c r="E1023" s="19" t="inlineStr">
         <is>
-          <t>NA - not mentioned.</t>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: unaware public; weak national policy/enforcement; unclear governance; irregular collection; hotels; aluminum foil use; informal sector exploitation without integration. No FLAG needed.</t>
         </is>
       </c>
     </row>
@@ -36893,17 +36893,17 @@
       </c>
       <c r="C1024" s="19" t="inlineStr">
         <is>
-          <t>Coordination_sectoral</t>
+          <t>NPF_hero</t>
         </is>
       </c>
       <c r="D1024" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>nature guides and park rangers (trained not to litter, collect wrappers on safari); hotel associations and NGOs (awareness training); Eco-Green and informal collectors (NPR 10–15/kg for bottles; informal sector collects ~99% of valuable plastics from hotels); PLEASE and Bio-Camp pilot projects (segregation, recycling/upcycling); Solid Waste Management Association and Plast Foundation Nepal; safari dustbin system; proposed EPR nationwide and ward-level designated street cleaners; elephant-dung cleaning teams as operational model (twice daily)</t>
         </is>
       </c>
       <c r="E1024" s="19" t="inlineStr">
         <is>
-          <t>Hotel associations, NGOs, park rangers and nature guides coordinate awareness; Eco-Green and municipality split collection roles.</t>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: nature guides/rangers; PLEASE/Bio-Camp; Solid Waste Management Association; Plast Foundation; Eco-Green; informal collectors; proposed EPR. No FLAG needed.</t>
         </is>
       </c>
     </row>
@@ -36920,7 +36920,7 @@
       </c>
       <c r="C1025" s="19" t="inlineStr">
         <is>
-          <t>Coordination_levels</t>
+          <t>Relevance_international_pol</t>
         </is>
       </c>
       <c r="D1025" s="19" t="inlineStr">
@@ -36930,7 +36930,7 @@
       </c>
       <c r="E1025" s="19" t="inlineStr">
         <is>
-          <t>Municipal trucks vs private Eco-Green vs informal collectors; ward enforcement proposed.</t>
+          <t>UN plastic negotiations influence national policy development.</t>
         </is>
       </c>
     </row>
@@ -36947,17 +36947,17 @@
       </c>
       <c r="C1026" s="19" t="inlineStr">
         <is>
-          <t>Unclear_responsibilities</t>
+          <t>Coordination_sectoral</t>
         </is>
       </c>
       <c r="D1026" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1026" s="19" t="inlineStr">
         <is>
-          <t>NA - not explicitly discussed.</t>
+          <t>Solid Waste Management Association coordinates private operators; hotel associations, NGOs, park rangers; manufacturers/collectors/recyclers cooperation sought.</t>
         </is>
       </c>
     </row>
@@ -36974,17 +36974,17 @@
       </c>
       <c r="C1027" s="19" t="inlineStr">
         <is>
-          <t>Res_nat_government</t>
+          <t>Coordination_levels</t>
         </is>
       </c>
       <c r="D1027" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1027" s="19" t="inlineStr">
         <is>
-          <t>NA - not named as responsible actor in this interview.</t>
+          <t>Unclear federal/provincial/local roles; municipal vs Eco-Green vs informal collectors.</t>
         </is>
       </c>
     </row>
@@ -37001,17 +37001,17 @@
       </c>
       <c r="C1028" s="19" t="inlineStr">
         <is>
-          <t>Res_prov_government</t>
+          <t>Unclear_responsibilities</t>
         </is>
       </c>
       <c r="D1028" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1028" s="19" t="inlineStr">
         <is>
-          <t>NA - not mentioned.</t>
+          <t>Division of authority between federal, provincial and local levels; public sees waste as only government's job.</t>
         </is>
       </c>
     </row>
@@ -37028,7 +37028,7 @@
       </c>
       <c r="C1029" s="19" t="inlineStr">
         <is>
-          <t>Res_loc_government</t>
+          <t>Res_nat_government</t>
         </is>
       </c>
       <c r="D1029" s="19" t="inlineStr">
@@ -37038,7 +37038,7 @@
       </c>
       <c r="E1029" s="19" t="inlineStr">
         <is>
-          <t>Municipal trucks collect bags/wrappers; dustbins provided.</t>
+          <t>Federal government sets broad frameworks and assessments; new plastics act in development.</t>
         </is>
       </c>
     </row>
@@ -37055,17 +37055,17 @@
       </c>
       <c r="C1030" s="19" t="inlineStr">
         <is>
-          <t>Res_students</t>
+          <t>Res_prov_government</t>
         </is>
       </c>
       <c r="D1030" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1030" s="19" t="inlineStr">
         <is>
-          <t>NA - not mentioned.</t>
+          <t>Provincial level part of three-tier responsibility framework.</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37082,7 @@
       </c>
       <c r="C1031" s="19" t="inlineStr">
         <is>
-          <t>Res_private_sector</t>
+          <t>Res_loc_government</t>
         </is>
       </c>
       <c r="D1031" s="19" t="inlineStr">
@@ -37092,7 +37092,7 @@
       </c>
       <c r="E1031" s="19" t="inlineStr">
         <is>
-          <t>Eco-Green recycles bottles; informal collectors buy PET.</t>
+          <t>Municipalities/metropolitan cities gradually taking responsibility; municipal trucks and dustbins.</t>
         </is>
       </c>
     </row>
@@ -37109,17 +37109,17 @@
       </c>
       <c r="C1032" s="19" t="inlineStr">
         <is>
-          <t>Res_civil_society</t>
+          <t>Res_students</t>
         </is>
       </c>
       <c r="D1032" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E1032" s="19" t="inlineStr">
         <is>
-          <t>NGOs, park rangers, hotel associations train nature guides.</t>
+          <t>NA - not mentioned.</t>
         </is>
       </c>
     </row>
@@ -37136,17 +37136,17 @@
       </c>
       <c r="C1033" s="19" t="inlineStr">
         <is>
-          <t>Res_science</t>
+          <t>Res_private_sector</t>
         </is>
       </c>
       <c r="D1033" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1033" s="19" t="inlineStr">
         <is>
-          <t>NA - not mentioned.</t>
+          <t>Semi-formal private companies; Eco-Green; informal pickers (~99% hotel plastics).</t>
         </is>
       </c>
     </row>
@@ -37163,7 +37163,7 @@
       </c>
       <c r="C1034" s="19" t="inlineStr">
         <is>
-          <t>Res_households</t>
+          <t>Res_civil_society</t>
         </is>
       </c>
       <c r="D1034" s="19" t="inlineStr">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="E1034" s="19" t="inlineStr">
         <is>
-          <t>Store and separate waste at home.</t>
+          <t>Plast Foundation Nepal; NGOs training nature guides.</t>
         </is>
       </c>
     </row>
@@ -37190,7 +37190,7 @@
       </c>
       <c r="C1035" s="19" t="inlineStr">
         <is>
-          <t>Res_edu_institutions</t>
+          <t>Res_science</t>
         </is>
       </c>
       <c r="D1035" s="19" t="inlineStr">
@@ -37200,7 +37200,7 @@
       </c>
       <c r="E1035" s="19" t="inlineStr">
         <is>
-          <t>NA - not mentioned.</t>
+          <t>NA - research called for but no science actors named as responsible.</t>
         </is>
       </c>
     </row>
@@ -37217,7 +37217,7 @@
       </c>
       <c r="C1036" s="19" t="inlineStr">
         <is>
-          <t>Res_private_companies</t>
+          <t>Res_households</t>
         </is>
       </c>
       <c r="D1036" s="19" t="inlineStr">
@@ -37227,7 +37227,7 @@
       </c>
       <c r="E1036" s="19" t="inlineStr">
         <is>
-          <t>Thousands of Chitwan hotels generate waste; hotel association discussions.</t>
+          <t>Source separation and proper disposal expected.</t>
         </is>
       </c>
     </row>
@@ -37244,7 +37244,7 @@
       </c>
       <c r="C1037" s="19" t="inlineStr">
         <is>
-          <t>Cul_nat_government</t>
+          <t>Res_edu_institutions</t>
         </is>
       </c>
       <c r="D1037" s="19" t="inlineStr">
@@ -37254,7 +37254,7 @@
       </c>
       <c r="E1037" s="19" t="inlineStr">
         <is>
-          <t>NA - not blamed.</t>
+          <t>NA - not mentioned.</t>
         </is>
       </c>
     </row>
@@ -37271,17 +37271,17 @@
       </c>
       <c r="C1038" s="19" t="inlineStr">
         <is>
-          <t>Cul_prov_government</t>
+          <t>Res_private_companies</t>
         </is>
       </c>
       <c r="D1038" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1038" s="19" t="inlineStr">
         <is>
-          <t>NA - not blamed.</t>
+          <t>Hotels (thousands in Chitwan); retailers/shops giving free bags.</t>
         </is>
       </c>
     </row>
@@ -37298,7 +37298,7 @@
       </c>
       <c r="C1039" s="19" t="inlineStr">
         <is>
-          <t>Cul_loc_government</t>
+          <t>Cul_nat_government</t>
         </is>
       </c>
       <c r="D1039" s="19" t="inlineStr">
@@ -37308,7 +37308,7 @@
       </c>
       <c r="E1039" s="19" t="inlineStr">
         <is>
-          <t>No municipal notices; irregular collection; streets not cleaned regularly.</t>
+          <t>No specific plastics policy; weak &lt;40-micron enforcement; political instability.</t>
         </is>
       </c>
     </row>
@@ -37325,7 +37325,7 @@
       </c>
       <c r="C1040" s="19" t="inlineStr">
         <is>
-          <t>Cul_students</t>
+          <t>Cul_prov_government</t>
         </is>
       </c>
       <c r="D1040" s="19" t="inlineStr">
@@ -37335,7 +37335,7 @@
       </c>
       <c r="E1040" s="19" t="inlineStr">
         <is>
-          <t>NA - not blamed.</t>
+          <t>NA - provincial level not blamed specifically.</t>
         </is>
       </c>
     </row>
@@ -37352,17 +37352,17 @@
       </c>
       <c r="C1041" s="19" t="inlineStr">
         <is>
-          <t>Cul_private_sector</t>
+          <t>Cul_loc_government</t>
         </is>
       </c>
       <c r="D1041" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1041" s="19" t="inlineStr">
         <is>
-          <t>NA - Eco-Green/informal collectors portrayed positively.</t>
+          <t>Irregular collection; no municipal notices; streets not cleaned regularly.</t>
         </is>
       </c>
     </row>
@@ -37379,7 +37379,7 @@
       </c>
       <c r="C1042" s="19" t="inlineStr">
         <is>
-          <t>Cul_civil_society</t>
+          <t>Cul_students</t>
         </is>
       </c>
       <c r="D1042" s="19" t="inlineStr">
@@ -37389,7 +37389,7 @@
       </c>
       <c r="E1042" s="19" t="inlineStr">
         <is>
-          <t>NA - NGOs/guides portrayed as heroes.</t>
+          <t>NA - not blamed.</t>
         </is>
       </c>
     </row>
@@ -37406,7 +37406,7 @@
       </c>
       <c r="C1043" s="19" t="inlineStr">
         <is>
-          <t>Cul_science</t>
+          <t>Cul_private_sector</t>
         </is>
       </c>
       <c r="D1043" s="19" t="inlineStr">
@@ -37416,7 +37416,7 @@
       </c>
       <c r="E1043" s="19" t="inlineStr">
         <is>
-          <t>NA - not blamed.</t>
+          <t>NA - informal/private collectors largely portrayed positively.</t>
         </is>
       </c>
     </row>
@@ -37433,17 +37433,17 @@
       </c>
       <c r="C1044" s="19" t="inlineStr">
         <is>
-          <t>Cul_households</t>
+          <t>Cul_civil_society</t>
         </is>
       </c>
       <c r="D1044" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E1044" s="19" t="inlineStr">
         <is>
-          <t>Laziness, ignorance, convenience, free plastic bags.</t>
+          <t>NA - NGOs/guides portrayed as heroes.</t>
         </is>
       </c>
     </row>
@@ -37460,7 +37460,7 @@
       </c>
       <c r="C1045" s="19" t="inlineStr">
         <is>
-          <t>Cul_edu_institutions</t>
+          <t>Cul_science</t>
         </is>
       </c>
       <c r="D1045" s="19" t="inlineStr">
@@ -37487,7 +37487,7 @@
       </c>
       <c r="C1046" s="19" t="inlineStr">
         <is>
-          <t>Cul_private_companies</t>
+          <t>Cul_households</t>
         </is>
       </c>
       <c r="D1046" s="19" t="inlineStr">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="E1046" s="19" t="inlineStr">
         <is>
-          <t>Hotels discuss but lack continuous waste-management action.</t>
+          <t>Low awareness, convenience, waste seen as government's job only.</t>
         </is>
       </c>
     </row>
@@ -37514,7 +37514,7 @@
       </c>
       <c r="C1047" s="19" t="inlineStr">
         <is>
-          <t>Tar_nat_government</t>
+          <t>Cul_edu_institutions</t>
         </is>
       </c>
       <c r="D1047" s="19" t="inlineStr">
@@ -37524,7 +37524,7 @@
       </c>
       <c r="E1047" s="19" t="inlineStr">
         <is>
-          <t>NA - not named as target group.</t>
+          <t>NA - not blamed.</t>
         </is>
       </c>
     </row>
@@ -37541,17 +37541,17 @@
       </c>
       <c r="C1048" s="19" t="inlineStr">
         <is>
-          <t>Tar_prov_government</t>
+          <t>Cul_private_companies</t>
         </is>
       </c>
       <c r="D1048" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1048" s="19" t="inlineStr">
         <is>
-          <t>NA - not named.</t>
+          <t>Hotels lack continuous waste-management action.</t>
         </is>
       </c>
     </row>
@@ -37568,7 +37568,7 @@
       </c>
       <c r="C1049" s="19" t="inlineStr">
         <is>
-          <t>Tar_loc_government</t>
+          <t>Tar_nat_government</t>
         </is>
       </c>
       <c r="D1049" s="19" t="inlineStr">
@@ -37578,7 +37578,7 @@
       </c>
       <c r="E1049" s="19" t="inlineStr">
         <is>
-          <t>Ward should launch awareness campaigns, enforce rules, provide dustbins, designate street cleaners.</t>
+          <t>Coordination, EPR implementation, regulate imported plastics, support research.</t>
         </is>
       </c>
     </row>
@@ -37595,7 +37595,7 @@
       </c>
       <c r="C1050" s="19" t="inlineStr">
         <is>
-          <t>Tar_students</t>
+          <t>Tar_prov_government</t>
         </is>
       </c>
       <c r="D1050" s="19" t="inlineStr">
@@ -37605,7 +37605,7 @@
       </c>
       <c r="E1050" s="19" t="inlineStr">
         <is>
-          <t>NA - not named.</t>
+          <t>NA - not named as primary target group.</t>
         </is>
       </c>
     </row>
@@ -37622,17 +37622,17 @@
       </c>
       <c r="C1051" s="19" t="inlineStr">
         <is>
-          <t>Tar_private_sector</t>
+          <t>Tar_loc_government</t>
         </is>
       </c>
       <c r="D1051" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1051" s="19" t="inlineStr">
         <is>
-          <t>NA - informal collectors positive; hotel committee proposed.</t>
+          <t>Inspections, local enforcement, designated street cleaners, dustbins.</t>
         </is>
       </c>
     </row>
@@ -37649,17 +37649,17 @@
       </c>
       <c r="C1052" s="19" t="inlineStr">
         <is>
-          <t>Tar_civil_society</t>
+          <t>Tar_students</t>
         </is>
       </c>
       <c r="D1052" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E1052" s="19" t="inlineStr">
         <is>
-          <t>Nature guides and hotel associations for sustained training.</t>
+          <t>NA - not named.</t>
         </is>
       </c>
     </row>
@@ -37676,17 +37676,17 @@
       </c>
       <c r="C1053" s="19" t="inlineStr">
         <is>
-          <t>Tar_science</t>
+          <t>Tar_private_sector</t>
         </is>
       </c>
       <c r="D1053" s="19" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1053" s="19" t="inlineStr">
         <is>
-          <t>NA - not named.</t>
+          <t>Semi-formal collectors, recyclers, hotel committees.</t>
         </is>
       </c>
     </row>
@@ -37703,7 +37703,7 @@
       </c>
       <c r="C1054" s="19" t="inlineStr">
         <is>
-          <t>Tar_households</t>
+          <t>Tar_civil_society</t>
         </is>
       </c>
       <c r="D1054" s="19" t="inlineStr">
@@ -37713,7 +37713,7 @@
       </c>
       <c r="E1054" s="19" t="inlineStr">
         <is>
-          <t>Use cloth bags; reduce plastic attachment.</t>
+          <t>Nature guides, park rangers, NGO training programmes.</t>
         </is>
       </c>
     </row>
@@ -37730,7 +37730,7 @@
       </c>
       <c r="C1055" s="19" t="inlineStr">
         <is>
-          <t>Tar_edu_institutions</t>
+          <t>Tar_science</t>
         </is>
       </c>
       <c r="D1055" s="19" t="inlineStr">
@@ -37740,7 +37740,7 @@
       </c>
       <c r="E1055" s="19" t="inlineStr">
         <is>
-          <t>NA - not named.</t>
+          <t>NA - research support via federal govt, not science actors as targets.</t>
         </is>
       </c>
     </row>
@@ -37757,7 +37757,7 @@
       </c>
       <c r="C1056" s="19" t="inlineStr">
         <is>
-          <t>Tar_private_companies</t>
+          <t>Tar_households</t>
         </is>
       </c>
       <c r="D1056" s="19" t="inlineStr">
@@ -37767,7 +37767,7 @@
       </c>
       <c r="E1056" s="19" t="inlineStr">
         <is>
-          <t>Hotel business community could form cleanliness committee (rickshaw collection ~NPR 50,000/month proposed).</t>
+          <t>Awareness, 3R/4R, proper disposal.</t>
         </is>
       </c>
     </row>
@@ -37784,17 +37784,17 @@
       </c>
       <c r="C1057" s="19" t="inlineStr">
         <is>
-          <t>Actor_role</t>
+          <t>Tar_edu_institutions</t>
         </is>
       </c>
       <c r="D1057" s="19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E1057" s="19" t="inlineStr">
         <is>
-          <t>Hotel operator describing personal and sector waste practices as a target group of policies (role 4), not a policy formulator or primary implementer.</t>
+          <t>NA - not named.</t>
         </is>
       </c>
     </row>
@@ -37811,17 +37811,17 @@
       </c>
       <c r="C1058" s="19" t="inlineStr">
         <is>
-          <t>Discretion</t>
+          <t>Tar_private_companies</t>
         </is>
       </c>
       <c r="D1058" s="19" t="inlineStr">
         <is>
-          <t>As a hotel operator Rajesh Aryal stores plastic bottles for Eco-Green recycling, separates other plastics for municipal trucks, empties bottles before disposal, and participates in hotel-association discussions — but has no authority over municipal collection schedules, ward enforcement, or thousands of other hotels' waste practices in Chitwan.</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1058" s="19" t="inlineStr">
         <is>
-          <t>Stores bottles for Eco-Green, separates waste for municipal collection, empties bottles — limited to own hotel/household practices.</t>
+          <t>Hotels, small businesses, retailers.</t>
         </is>
       </c>
     </row>
@@ -37838,17 +37838,17 @@
       </c>
       <c r="C1059" s="19" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Actor_role</t>
         </is>
       </c>
       <c r="D1059" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E1059" s="19" t="inlineStr">
         <is>
-          <t>No municipal notices or rules observed; irregular programme monitoring.</t>
+          <t>Hotel operator as target group (role 4) — describes ground-level hotel/tourism practices while interview also covers national policy themes.</t>
         </is>
       </c>
     </row>
@@ -37865,17 +37865,17 @@
       </c>
       <c r="C1060" s="19" t="inlineStr">
         <is>
-          <t>Financial_resources</t>
+          <t>Discretion</t>
         </is>
       </c>
       <c r="D1060" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>As a hotel operator Rajesh Aryal stores plastic bottles for Eco-Green recycling, separates other plastics for municipal trucks, empties bottles before disposal, and participates in hotel-association discussions — but has no authority over municipal collection schedules, national policy formulation, or thousands of other hotels' waste practices in Chitwan.</t>
         </is>
       </c>
       <c r="E1060" s="19" t="inlineStr">
         <is>
-          <t>Hotel committee rickshaw collection (~NPR 50,000/month) proposed; bottle monetary value (NPR 10–15/kg) drives informal collection.</t>
+          <t>Limited to own hotel waste-handling practices; no policy or municipal authority.</t>
         </is>
       </c>
     </row>
@@ -37892,7 +37892,7 @@
       </c>
       <c r="C1061" s="19" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="D1061" s="19" t="inlineStr">
@@ -37902,7 +37902,7 @@
       </c>
       <c r="E1061" s="19" t="inlineStr">
         <is>
-          <t>Dustbins provided but overflow; safari vehicle buckets compulsory; need designated street cleaners.</t>
+          <t>Weak enforcement; limited testing-lab capacity nationally; no municipal notices locally.</t>
         </is>
       </c>
     </row>
@@ -37919,7 +37919,7 @@
       </c>
       <c r="C1062" s="19" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Financial_resources</t>
         </is>
       </c>
       <c r="D1062" s="19" t="inlineStr">
@@ -37929,7 +37929,7 @@
       </c>
       <c r="E1062" s="19" t="inlineStr">
         <is>
-          <t>No designated street cleaners (unlike elephant-dung teams); awareness programmes lack continuity.</t>
+          <t>Local governments face resource gaps; hotel committee rickshaw collection (~NPR 50,000/month) proposed; financial support for private collection initiatives.</t>
         </is>
       </c>
     </row>
@@ -37946,7 +37946,7 @@
       </c>
       <c r="C1063" s="19" t="inlineStr">
         <is>
-          <t>Enforcement</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D1063" s="19" t="inlineStr">
@@ -37956,7 +37956,7 @@
       </c>
       <c r="E1063" s="19" t="inlineStr">
         <is>
-          <t>No municipal enforcement notices; ward strict rules proposed.</t>
+          <t>Research needed on microplastics, burning impacts, agriculture and water contamination.</t>
         </is>
       </c>
     </row>
@@ -37973,17 +37973,17 @@
       </c>
       <c r="C1064" s="19" t="inlineStr">
         <is>
-          <t>Pol_epr</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D1064" s="19" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1064" s="19" t="inlineStr">
         <is>
-          <t>EPR not mentioned.</t>
+          <t>Need dustbins, shredders, transfer stations; safari buckets; ward cleaners.</t>
         </is>
       </c>
     </row>
@@ -38000,7 +38000,7 @@
       </c>
       <c r="C1065" s="19" t="inlineStr">
         <is>
-          <t>Pol_awareness</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="D1065" s="19" t="inlineStr">
@@ -38010,7 +38010,7 @@
       </c>
       <c r="E1065" s="19" t="inlineStr">
         <is>
-          <t>Occasional programmes by NGOs, hotel associations, park rangers — not continuous.</t>
+          <t>Limited technical capacity (testing labs); no designated street cleaners; training needed for collectors and nature guides.</t>
         </is>
       </c>
     </row>
@@ -38027,7 +38027,7 @@
       </c>
       <c r="C1066" s="19" t="inlineStr">
         <is>
-          <t>Pol_clean_up</t>
+          <t>Enforcement</t>
         </is>
       </c>
       <c r="D1066" s="19" t="inlineStr">
@@ -38037,7 +38037,7 @@
       </c>
       <c r="E1066" s="19" t="inlineStr">
         <is>
-          <t>Environment Day one-day events; safari dustbin rule; elephant-dung teams twice daily.</t>
+          <t>Weak ban enforcement; ward strict rules proposed.</t>
         </is>
       </c>
     </row>
@@ -38054,17 +38054,17 @@
       </c>
       <c r="C1067" s="19" t="inlineStr">
         <is>
-          <t>Pol_recycling</t>
+          <t>Pol_epr</t>
         </is>
       </c>
       <c r="D1067" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E1067" s="19" t="inlineStr">
         <is>
-          <t>Eco-Green bottle collection.</t>
+          <t>EPR proposed as future solution but not currently in place.</t>
         </is>
       </c>
     </row>
@@ -38081,7 +38081,7 @@
       </c>
       <c r="C1068" s="19" t="inlineStr">
         <is>
-          <t>Pol_waste_collection</t>
+          <t>Pol_awareness</t>
         </is>
       </c>
       <c r="D1068" s="19" t="inlineStr">
@@ -38091,7 +38091,7 @@
       </c>
       <c r="E1068" s="19" t="inlineStr">
         <is>
-          <t>Municipal trucks for wrappers/bags; irregular schedules.</t>
+          <t>Irregular campaigns; Environment Day one day only; nature-guide training.</t>
         </is>
       </c>
     </row>
@@ -38108,7 +38108,7 @@
       </c>
       <c r="C1069" s="19" t="inlineStr">
         <is>
-          <t>Pol_effectiveness</t>
+          <t>Pol_education</t>
         </is>
       </c>
       <c r="D1069" s="19" t="inlineStr">
@@ -38118,7 +38118,7 @@
       </c>
       <c r="E1069" s="19" t="inlineStr">
         <is>
-          <t>Irregular collection and awareness; no continuous action.</t>
+          <t>Training for waste collectors and nature guides.</t>
         </is>
       </c>
     </row>
@@ -38135,17 +38135,17 @@
       </c>
       <c r="C1070" s="19" t="inlineStr">
         <is>
-          <t>Pol_effectiveness_example</t>
+          <t>Pol_ban</t>
         </is>
       </c>
       <c r="D1070" s="19" t="inlineStr">
         <is>
-          <t>Eco-Green collects bottles every 15–20 days but "it's irregular" and "this time it has been long since it has collected"; municipal dustbins provided but "if collection doesn't happen on time, wind spreads the waste"; awareness and cleanup programs exist "occasionally" but "there's no continuous action" — Environment Day "only one day, doesn't continue beyond that"; "no notices" from municipality on plastic removal.</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E1070" s="19" t="inlineStr">
         <is>
-          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+          <t>&lt;40-micron plastics ban weakly enforced.</t>
         </is>
       </c>
     </row>
@@ -38162,7 +38162,7 @@
       </c>
       <c r="C1071" s="19" t="inlineStr">
         <is>
-          <t>Sol_awareness</t>
+          <t>Pol_subsitutes</t>
         </is>
       </c>
       <c r="D1071" s="19" t="inlineStr">
@@ -38172,7 +38172,7 @@
       </c>
       <c r="E1071" s="19" t="inlineStr">
         <is>
-          <t>Ward awareness campaigns to reduce negligence.</t>
+          <t>Cloth bags, clay/cement pots, leaf plates.</t>
         </is>
       </c>
     </row>
@@ -38189,7 +38189,7 @@
       </c>
       <c r="C1072" s="19" t="inlineStr">
         <is>
-          <t>Sol_education</t>
+          <t>Pol_clean_up</t>
         </is>
       </c>
       <c r="D1072" s="19" t="inlineStr">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="E1072" s="19" t="inlineStr">
         <is>
-          <t>Sustained nature-guide and hotel-association training.</t>
+          <t>Environment Day; safari dustbin rule; elephant-dung teams.</t>
         </is>
       </c>
     </row>
@@ -38216,7 +38216,7 @@
       </c>
       <c r="C1073" s="19" t="inlineStr">
         <is>
-          <t>Sol_capacity</t>
+          <t>Pol_upcycling</t>
         </is>
       </c>
       <c r="D1073" s="19" t="inlineStr">
@@ -38226,7 +38226,7 @@
       </c>
       <c r="E1073" s="19" t="inlineStr">
         <is>
-          <t>Train population through hotel association/NGO programmes.</t>
+          <t>Bio-Camp pilots (flowerpots, plastic boards).</t>
         </is>
       </c>
     </row>
@@ -38243,7 +38243,7 @@
       </c>
       <c r="C1074" s="19" t="inlineStr">
         <is>
-          <t>Sol_finance</t>
+          <t>Pol_recycling</t>
         </is>
       </c>
       <c r="D1074" s="19" t="inlineStr">
@@ -38253,7 +38253,7 @@
       </c>
       <c r="E1074" s="19" t="inlineStr">
         <is>
-          <t>Hotel committee fund for rickshaw waste collection.</t>
+          <t>Eco-Green bottles; PLEASE/Bio-Camp segregation/recycling.</t>
         </is>
       </c>
     </row>
@@ -38270,7 +38270,7 @@
       </c>
       <c r="C1075" s="19" t="inlineStr">
         <is>
-          <t>Sol_infrastructure</t>
+          <t>Pol_waste_collection</t>
         </is>
       </c>
       <c r="D1075" s="19" t="inlineStr">
@@ -38280,7 +38280,7 @@
       </c>
       <c r="E1075" s="19" t="inlineStr">
         <is>
-          <t>Ward dustbins; safari vehicle buckets.</t>
+          <t>Municipal trucks; informal sector; irregular schedules.</t>
         </is>
       </c>
     </row>
@@ -38297,7 +38297,7 @@
       </c>
       <c r="C1076" s="19" t="inlineStr">
         <is>
-          <t>Sol_subsitutes</t>
+          <t>Pol_effectiveness</t>
         </is>
       </c>
       <c r="D1076" s="19" t="inlineStr">
@@ -38307,7 +38307,7 @@
       </c>
       <c r="E1076" s="19" t="inlineStr">
         <is>
-          <t>Cloth/fiber bags; clay/cement pots.</t>
+          <t>Limited due to weak enforcement, irregular collection, policy gaps.</t>
         </is>
       </c>
     </row>
@@ -38324,17 +38324,17 @@
       </c>
       <c r="C1077" s="19" t="inlineStr">
         <is>
-          <t>Sol_clean_up</t>
+          <t>Pol_effectiveness_example</t>
         </is>
       </c>
       <c r="D1077" s="19" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Environmental Protection Act exists but no specific plastics policy; &lt;40-micron ban weakly enforced; federal government assessing new plastics act but guidelines unclear; Eco-Green bottle collection every 15–20 days but irregular; municipal collection not on time (bins overflow); awareness/cleanup programmes occasional — Environment Day "only one day"; PLEASE/Bio-Camp pilots show promise but not yet scaled; effectiveness limited by low enforcement, irregular collection and inconsistent public awareness.</t>
         </is>
       </c>
       <c r="E1077" s="19" t="inlineStr">
         <is>
-          <t>Designated street cleaners; daily collection like elephant-dung teams.</t>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
         </is>
       </c>
     </row>
@@ -38351,7 +38351,7 @@
       </c>
       <c r="C1078" s="19" t="inlineStr">
         <is>
-          <t>Sol_enforcement</t>
+          <t>Sol_lead_agency</t>
         </is>
       </c>
       <c r="D1078" s="19" t="inlineStr">
@@ -38361,7 +38361,7 @@
       </c>
       <c r="E1078" s="19" t="inlineStr">
         <is>
-          <t>Ward strict rule enforcement proposed.</t>
+          <t>Clear three-tier responsibilities; Solid Waste Management Association coordination.</t>
         </is>
       </c>
     </row>
@@ -38378,17 +38378,422 @@
       </c>
       <c r="C1079" s="19" t="inlineStr">
         <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1079" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1079" s="19" t="inlineStr">
+        <is>
+          <t>Clarify federal/provincial/local roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1080" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1080" s="19" t="inlineStr">
+        <is>
+          <t>Sol_epr</t>
+        </is>
+      </c>
+      <c r="D1080" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1080" s="19" t="inlineStr">
+        <is>
+          <t>Implement EPR nationwide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1081" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1081" s="19" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1081" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1081" s="19" t="inlineStr">
+        <is>
+          <t>Sustained public-awareness campaigns; ward programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1082" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1082" s="19" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1082" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1082" s="19" t="inlineStr">
+        <is>
+          <t>Household and hotel source segregation; scale PLEASE/Bio-Camp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1083" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1083" s="19" t="inlineStr">
+        <is>
+          <t>Sol_upcycling</t>
+        </is>
+      </c>
+      <c r="D1083" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1083" s="19" t="inlineStr">
+        <is>
+          <t>Scale Bio-Camp upcycling models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1084" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1084" s="19" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1084" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1084" s="19" t="inlineStr">
+        <is>
+          <t>Strengthen formal recycling; integrate informal sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1085" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1085" s="19" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1085" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1085" s="19" t="inlineStr">
+        <is>
+          <t>3R/4R, lifecycle assessment, eco-friendly alternatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1086" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1086" s="19" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1086" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1086" s="19" t="inlineStr">
+        <is>
+          <t>Labs, trained workforce, segregation skills, nature-guide training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1087" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1087" s="19" t="inlineStr">
+        <is>
+          <t>Sol_RD</t>
+        </is>
+      </c>
+      <c r="D1087" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1087" s="19" t="inlineStr">
+        <is>
+          <t>Research on microplastics, burning, agriculture, water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1088" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1088" s="19" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1088" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1088" s="19" t="inlineStr">
+        <is>
+          <t>Support private collection initiatives; hotel committee funding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1089" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1089" s="19" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1089" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1089" s="19" t="inlineStr">
+        <is>
+          <t>Dustbins, shredders, transfer stations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1090" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1090" s="19" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1090" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1090" s="19" t="inlineStr">
+        <is>
+          <t>Leaf plates, cotton/towel bags, clay pots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1091" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1091" s="19" t="inlineStr">
+        <is>
+          <t>Sol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1091" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1091" s="19" t="inlineStr">
+        <is>
+          <t>Designated street cleaners; daily collection model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1092" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1092" s="19" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1092" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1092" s="19" t="inlineStr">
+        <is>
+          <t>Local inspections; enforce bans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1093" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1093" s="19" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1093" s="19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1093" s="19" t="inlineStr">
+        <is>
+          <t>Stronger enforcement and data systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="19" t="inlineStr">
+        <is>
+          <t>NPL_14</t>
+        </is>
+      </c>
+      <c r="B1094" s="19" t="inlineStr">
+        <is>
+          <t>Hotel Silent Park - Rajesh Aryal, Chitwan/Sauraha tourism area (26 June 2025)</t>
+        </is>
+      </c>
+      <c r="C1094" s="19" t="inlineStr">
+        <is>
           <t>Traditions to build on (free-hand)</t>
         </is>
       </c>
-      <c r="D1079" s="19" t="inlineStr">
-        <is>
-          <t>Cloth/fiber bags instead of plastic shopping bags; clay or cement pots instead of plastic flower pots.</t>
-        </is>
-      </c>
-      <c r="E1079" s="19" t="inlineStr">
-        <is>
-          <t>Cloth bags; clay/cement pots instead of plastic.</t>
+      <c r="D1094" s="19" t="inlineStr">
+        <is>
+          <t>Natural plates from banana leaves and pat leaves during feasts; cotton or towel bags for shopping; cloth/fiber bags and clay/cement pots instead of plastic; reuse of plastics before recycling.</t>
+        </is>
+      </c>
+      <c r="E1094" s="19" t="inlineStr">
+        <is>
+          <t>Banana/pat leaf plates; cotton/towel bags; clay pots; reuse before recycle.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NPL_15 coding for KTM Environment Inspector Suna Maya Margen
Code interview no. 2 (23 June 2025) from guideline/field notes: public
education, composting programmes, Doko Recyclers Cluster 7 MoU, land/MRF
barriers, Mayors Forum provisions, UNDP partnership, and Newari Lapti
traditions. Register as NPL_15 with full Coding_Explanations.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -62,80 +62,86 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC1A2"/>
-        <bgColor rgb="00EBC1A2"/>
+        <fgColor rgb="00EBBFA2"/>
+        <bgColor rgb="00EBBFA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE0A2"/>
-        <bgColor rgb="00EBE0A2"/>
+        <fgColor rgb="00EBDCA2"/>
+        <bgColor rgb="00EBDCA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6EBA2"/>
-        <bgColor rgb="00D6EBA2"/>
+        <fgColor rgb="00DCEBA2"/>
+        <bgColor rgb="00DCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B7EBA2"/>
-        <bgColor rgb="00B7EBA2"/>
+        <fgColor rgb="00BFEBA2"/>
+        <bgColor rgb="00BFEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBAC"/>
-        <bgColor rgb="00A2EBAC"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBCC"/>
-        <bgColor rgb="00A2EBCC"/>
+        <fgColor rgb="00A2EBBF"/>
+        <bgColor rgb="00A2EBBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBDC"/>
+        <bgColor rgb="00A2EBDC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2CCEB"/>
-        <bgColor rgb="00A2CCEB"/>
+        <fgColor rgb="00A2DCEB"/>
+        <bgColor rgb="00A2DCEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2ACEB"/>
-        <bgColor rgb="00A2ACEB"/>
+        <fgColor rgb="00A2BFEB"/>
+        <bgColor rgb="00A2BFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B7A2EB"/>
-        <bgColor rgb="00B7A2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6A2EB"/>
-        <bgColor rgb="00D6A2EB"/>
+        <fgColor rgb="00BFA2EB"/>
+        <bgColor rgb="00BFA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E0"/>
-        <bgColor rgb="00EBA2E0"/>
+        <fgColor rgb="00DCA2EB"/>
+        <bgColor rgb="00DCA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C1"/>
-        <bgColor rgb="00EBA2C1"/>
+        <fgColor rgb="00EBA2DC"/>
+        <bgColor rgb="00EBA2DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2BF"/>
+        <bgColor rgb="00EBA2BF"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -222,6 +228,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -589,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -608,7 +617,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_14, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_15, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -721,82 +730,89 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  15. NPL_15 - Kathmandu Metropolitan City, Ms. Suna Maya Margen (Environment Inspector, Public Education), Kathmandu (23 June 2025, internal interview no. 2). Coded from interview guideline/field notes only (no full verbatim transcript). Overlaps thematically with NPL_3 (same municipality) but distinct respondent.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_14, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_15, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Colour key: each interview (NPL_1 through NPL_14) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
-    </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1983,7 +1999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ15"/>
+  <dimension ref="A1:CQ16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9238,6 +9254,483 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="O16" s="20" t="inlineStr">
+        <is>
+          <t>visual pollution (described as the biggest problem visually since 1998, linked to tourists and lifestyle), drainage blockage and riverbank dumping, rising share of low-value multi-layer plastics (8% rising to 15%), microplastics impacts on health, environment and wildlife (raised as a public knowledge gap)</t>
+        </is>
+      </c>
+      <c r="P16" s="20" t="inlineStr">
+        <is>
+          <t>rivers and riverbanks (dumping, drainage blockage), drainage/sewer systems, the visual environment and tourism image of Kathmandu, neighbouring municipalities/communities opposing MRF siting, wildlife and the broader environment (microplastics), and valley residents affected by inadequate processing capacity despite sufficient waste volumes</t>
+        </is>
+      </c>
+      <c r="Q16" s="20" t="inlineStr">
+        <is>
+          <t>consumers and lifestyle/tourism-driven plastic use (visual pollution); multi-layer plastic producers/suppliers (low-value plastics with "no value" left behind); unregistered/informal private actors (KMC works only with registered private sector and explicitly does not work with the informal sector); residents who oppose MRF/waste facilities nearby ("people don't want wastes everywhere"); and uncertain import flows ("import of plastics??" raised as an open policy issue)</t>
+        </is>
+      </c>
+      <c r="R16" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (public education, composting programmes at household/community/school levels, landfill site management for 23 municipalities, riverbed debris excavation/transfer); registered private partners under MoUs (Doko Recyclers collecting Cluster 7); UNDP (MoU for plastics recovery and plastic study); department stores voluntarily providing cloth bags instead of polythene; Newari festival traditions using leaf plates (Lapti); and planned measures (action plan, producer subsidies, single-use plastics ban, subsidised alternatives)</t>
+        </is>
+      </c>
+      <c r="S16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Y16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AA16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AL16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AS16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA16" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BB16" s="20" t="inlineStr">
+        <is>
+          <t>As an Environment Inspector focused on public education, Ms. Margen implements composting and plastics-reduction programmes at household, community and school levels and works within KMC's framework of MoUs with registered private partners (e.g. Doko Recyclers in Cluster 7) — but has limited discretion over land procurement (federal land authority), engagement with the informal sector (explicitly excluded), national policy revision timelines, or siting MRF facilities opposed by neighbouring municipalities.</t>
+        </is>
+      </c>
+      <c r="BC16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI16" s="20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ16" s="20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BK16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BS16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW16" s="20" t="inlineStr">
+        <is>
+          <t>Ministry of Forest and Environment plastics policy "not implemented and currently under revision"; KMC relies on the Environment Act 2077 and Natural Resource Management Act 2007 rather than a plastics-specific local ordinance; single-use plastics ban is still at the planning stage; no assessment yet of the 40-micron notification; sufficient waste is collected but KMC cannot procure land for MRF/processing — effectiveness limited by land, technology and enforcement gaps.</t>
+        </is>
+      </c>
+      <c r="BX16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH16" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CJ16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CN16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO16" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP16" s="20" t="inlineStr">
+        <is>
+          <t>Newari community festival practices that try to minimise plastics by using leaf plates (Lapti) instead of disposable plastic — effective culturally but expensive, with cheaper plastic alternatives still dominating unless subsidised.</t>
+        </is>
+      </c>
+      <c r="CQ16" s="20" t="inlineStr">
+        <is>
+          <t>Master list label: "15. Kathmandu Metropolitan City/ Suna Maya Margen", affiliation: Kathmandu Metropolitan City - Environment Division / Public Education &amp; Inspection. Interviewee: Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education. Interview date: 23 June 2025; internal interview no. 2. Coded from interview guideline/field notes only (no full verbatim transcript supplied). Data-quality notes: the follow-up on concern level (Q1) and Q2 (visible effects) were left blank in the source; ministry-template follow-ups Q4a/Q4b and Q4 effectiveness follow-up were also blank. Overlap with NPL_3 (same municipality, Doko Recyclers Cluster 7, land/MRF challenges, Lapti tradition, UNDP MoU) but distinct respondent with emphasis on public education, composting and inspection rather than SWM office policy formulation. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9249,7 +9742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1094"/>
+  <dimension ref="A1:E1178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -38797,6 +39290,2274 @@
         </is>
       </c>
     </row>
+    <row r="1095">
+      <c r="A1095" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1095" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1095" s="20" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1095" s="20" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="E1095" s="20" t="inlineStr">
+        <is>
+          <t>Ms. Suna Maya Margen is an Environment Inspector in Kathmandu Metropolitan City's Environment Division (Public Education &amp; Inspection) — coded as loc_government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1096" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1096" s="20" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1096" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1096" s="20" t="inlineStr">
+        <is>
+          <t>Follow-up Q10 asks what people need to learn more about (assessment of the 40-micron notification; microplastics impacts) — implying public knowledge gaps despite KMC's public education work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1097" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1097" s="20" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D1097" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1097" s="20" t="inlineStr">
+        <is>
+          <t>Ministry of Forest and Environment plastics policy is "not implemented and currently under revision"; KMC has no direct plastics ordinance and instead relies on broader environment acts — indicating policy-framework gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1098" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1098" s="20" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1098" s="20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1098" s="20" t="inlineStr">
+        <is>
+          <t>Plastic described as "the biggest problem visually since 1998" with rising multi-layer share (8% to 15%), riverbank dumping and drainage blockage. The explicit follow-up on concern level was left blank in the source notes, but the overall framing reflects high institutional concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1099" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1099" s="20" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1099" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1099" s="20" t="inlineStr">
+        <is>
+          <t>"Dumped at river-banks"; drainage blockage; visual pollution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1100" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1100" s="20" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1100" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1100" s="20" t="inlineStr">
+        <is>
+          <t>Visual pollution attributed to "tourists" and "life-style" — ongoing consumption patterns driving visible waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1101" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1101" s="20" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1101" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1101" s="20" t="inlineStr">
+        <is>
+          <t>"8% and before now 15%" multi-layer plastics with "no value" — low-value plastics not economically recycled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1102" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1102" s="20" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1102" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1102" s="20" t="inlineStr">
+        <is>
+          <t>"Sufficient waste but unable to procure land"; lack of land/space within Kathmandu city; 23 municipalities in four districts dispose at KMC's landfill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1103" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1103" s="20" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1103" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1103" s="20" t="inlineStr">
+        <is>
+          <t>Multi-layer plastic share rising (8% to 15%); future solutions include "provide subsidies to producers" — implying upstream production/composition is part of the problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1104" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1104" s="20" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1104" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1104" s="20" t="inlineStr">
+        <is>
+          <t>"Lapti" leaf plates and other alternatives "are expensive"; "alternatives are expensive" relative to cheap plastic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1105" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1105" s="20" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1105" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1105" s="20" t="inlineStr">
+        <is>
+          <t>"Lack of land, we can segregate (no space within the Kathmandu city)" — segregation hampered by space constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1106" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1106" s="20" t="inlineStr">
+        <is>
+          <t>Problem_import</t>
+        </is>
+      </c>
+      <c r="D1106" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1106" s="20" t="inlineStr">
+        <is>
+          <t>"Import of plastics??" raised as an open policy question in future measures — suggesting imports may undermine domestic management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1107" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1107" s="20" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1107" s="20" t="inlineStr">
+        <is>
+          <t>visual pollution (described as the biggest problem visually since 1998, linked to tourists and lifestyle), drainage blockage and riverbank dumping, rising share of low-value multi-layer plastics (8% rising to 15%), microplastics impacts on health, environment and wildlife (raised as a public knowledge gap)</t>
+        </is>
+      </c>
+      <c r="E1107" s="20" t="inlineStr">
+        <is>
+          <t>See Coded_Data Impacts cell — visual pollution since 1998, drainage blockage, riverbank dumping, multi-layer plastic share, microplastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1108" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1108" s="20" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1108" s="20" t="inlineStr">
+        <is>
+          <t>rivers and riverbanks (dumping, drainage blockage), drainage/sewer systems, the visual environment and tourism image of Kathmandu, neighbouring municipalities/communities opposing MRF siting, wildlife and the broader environment (microplastics), and valley residents affected by inadequate processing capacity despite sufficient waste volumes</t>
+        </is>
+      </c>
+      <c r="E1108" s="20" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: rivers/drainage systems, tourism/visual environment, neighbouring communities near proposed MRF sites, wildlife and public health (microplastics). No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1109" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1109" s="20" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1109" s="20" t="inlineStr">
+        <is>
+          <t>consumers and lifestyle/tourism-driven plastic use (visual pollution); multi-layer plastic producers/suppliers (low-value plastics with "no value" left behind); unregistered/informal private actors (KMC works only with registered private sector and explicitly does not work with the informal sector); residents who oppose MRF/waste facilities nearby ("people don't want wastes everywhere"); and uncertain import flows ("import of plastics??" raised as an open policy issue)</t>
+        </is>
+      </c>
+      <c r="E1109" s="20" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: lifestyle/tourism consumers; multi-layer plastic producers; unregistered/informal sector (excluded from KMC partnerships); NIMBY opposition to waste facilities; possible plastic importers. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1110" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1110" s="20" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1110" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City (public education, composting programmes at household/community/school levels, landfill site management for 23 municipalities, riverbed debris excavation/transfer); registered private partners under MoUs (Doko Recyclers collecting Cluster 7); UNDP (MoU for plastics recovery and plastic study); department stores voluntarily providing cloth bags instead of polythene; Newari festival traditions using leaf plates (Lapti); and planned measures (action plan, producer subsidies, single-use plastics ban, subsidised alternatives)</t>
+        </is>
+      </c>
+      <c r="E1110" s="20" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: KMC (education, composting, landfill management, riverbed clean-up); Doko Recyclers; UNDP; stores using cloth bags; Newari Lapti traditions; planned subsidies and bans. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1111" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1111" s="20" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D1111" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1111" s="20" t="inlineStr">
+        <is>
+          <t>UNDP donor partnership (MoU) for plastics recovery and plastic study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1112" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1112" s="20" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D1112" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1112" s="20" t="inlineStr">
+        <is>
+          <t>KMC coordinates with registered private sector (MoUs), UNDP donor partner, and Mayors Forum (18 municipalities) on plastic and solid waste management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1113" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1113" s="20" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D1113" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1113" s="20" t="inlineStr">
+        <is>
+          <t>"Land authority is with federal and implementation is by LG, its difficult for LG, better coordination and collaboration with provincial and district [needed]"; central/provincial governments should help provide land within the metro city or valley.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1114" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1114" s="20" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1114" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1114" s="20" t="inlineStr">
+        <is>
+          <t>Federal government holds land authority while local government must implement; ministry plastics policy under revision and not implemented — unclear national-local division of roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1115" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1115" s="20" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1115" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1115" s="20" t="inlineStr">
+        <is>
+          <t>Ministry of Forest and Environment (national plastics policy under revision); federal land authority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1116" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1116" s="20" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1116" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1116" s="20" t="inlineStr">
+        <is>
+          <t>"Central and provincial government provide [land] within metro city or in the valley" — provincial role in land/support explicitly invoked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1117" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1117" s="20" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1117" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1117" s="20" t="inlineStr">
+        <is>
+          <t>"KTM city" responsible; manages landfill site used by 23 municipalities in four districts; implements environment acts and solid waste management at city level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1118" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1118" s="20" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1118" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1118" s="20" t="inlineStr">
+        <is>
+          <t>Composting programmes run at school level — students/schools are implementation partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1119" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1119" s="20" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1119" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1119" s="20" t="inlineStr">
+        <is>
+          <t>Registered private sector engaged via MoUs (e.g. Doko Recyclers collecting Cluster 7); solid waste management provisions for private sector engagement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1120" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1120" s="20" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1120" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1120" s="20" t="inlineStr">
+        <is>
+          <t>NA - Doko Recyclers coded under private sector; no NGOs/CSOs named as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1121" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1121" s="20" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1121" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1121" s="20" t="inlineStr">
+        <is>
+          <t>NA - research needs mentioned but no scientific institutions named as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1122" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1122" s="20" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1122" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1122" s="20" t="inlineStr">
+        <is>
+          <t>Composting promoted at household level as part of KMC public education work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1123" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1123" s="20" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1123" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1123" s="20" t="inlineStr">
+        <is>
+          <t>School-level composting programmes — schools as implementation sites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1124" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1124" s="20" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1124" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1124" s="20" t="inlineStr">
+        <is>
+          <t>Department stores that provide cloth bags and do not give out polythene bags — retail companies exercising responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1125" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1125" s="20" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1125" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1125" s="20" t="inlineStr">
+        <is>
+          <t>Land authority rests with federal government while local government must implement; national ministry policy "not implemented and currently under revision."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1126" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1126" s="20" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1126" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1126" s="20" t="inlineStr">
+        <is>
+          <t>NA - provincial government portrayed as needed helper, not primarily blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1127" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1127" s="20" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1127" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1127" s="20" t="inlineStr">
+        <is>
+          <t>NA - interviewee represents KMC; municipality portrayed as implementer facing external constraints rather than primary culprit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1128" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1128" s="20" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1128" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1128" s="20" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1129" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1129" s="20" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1129" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1129" s="20" t="inlineStr">
+        <is>
+          <t>Historical note that private-sector partners "were not legalized"; KMC now works only with registered private sector and not with the informal sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1130" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1130" s="20" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1130" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1130" s="20" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1131" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1131" s="20" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1131" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1131" s="20" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1132" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1132" s="20" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1132" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1132" s="20" t="inlineStr">
+        <is>
+          <t>"Public opposition – people don't want wastes everywhere"; neighbouring municipalities oppose MRF facilities nearby.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1133" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1133" s="20" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1133" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1133" s="20" t="inlineStr">
+        <is>
+          <t>NA - schools are programme sites, not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1134" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1134" s="20" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1134" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1134" s="20" t="inlineStr">
+        <is>
+          <t>NA - stores with cloth bags portrayed positively; importers only raised as open question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1135" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1135" s="20" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1135" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1135" s="20" t="inlineStr">
+        <is>
+          <t>Central government should provide land and revise/implement national plastics policy; subsidies to producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1136" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1136" s="20" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1136" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1136" s="20" t="inlineStr">
+        <is>
+          <t>Provincial government should help provide land and coordinate with local government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1137" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1137" s="20" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1137" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1137" s="20" t="inlineStr">
+        <is>
+          <t>Better rules and regulation "within our areas"; MRF siting and implementation accountability at municipal level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1138" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1138" s="20" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1138" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1138" s="20" t="inlineStr">
+        <is>
+          <t>School-level composting and education programmes target students.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1139" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1139" s="20" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1139" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1139" s="20" t="inlineStr">
+        <is>
+          <t>NA - registered private partners discussed as collaborators rather than primary policy targets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1140" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1140" s="20" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1140" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1140" s="20" t="inlineStr">
+        <is>
+          <t>NA - not named as target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1141" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1141" s="20" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1141" s="20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1141" s="20" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1142" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1142" s="20" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1142" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1142" s="20" t="inlineStr">
+        <is>
+          <t>Household composting programmes and public education on plastics imply households as a target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1143" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1143" s="20" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1143" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1143" s="20" t="inlineStr">
+        <is>
+          <t>Schools are explicit sites for composting and education programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1144" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1144" s="20" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1144" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1144" s="20" t="inlineStr">
+        <is>
+          <t>Q9: "stores in Nepal but u get cloth bags and don't get plastics (polythene)" — retailers/stores named as focus for future policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1145" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1145" s="20" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1145" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E1145" s="20" t="inlineStr">
+        <is>
+          <t>Environment Inspector conducting public education, composting programmes and ground-level implementation — street-level implementer (role 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1146" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1146" s="20" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1146" s="20" t="inlineStr">
+        <is>
+          <t>As an Environment Inspector focused on public education, Ms. Margen implements composting and plastics-reduction programmes at household, community and school levels and works within KMC's framework of MoUs with registered private partners (e.g. Doko Recyclers in Cluster 7) — but has limited discretion over land procurement (federal land authority), engagement with the informal sector (explicitly excluded), national policy revision timelines, or siting MRF facilities opposed by neighbouring municipalities.</t>
+        </is>
+      </c>
+      <c r="E1146" s="20" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1147" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1147" s="20" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1147" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1147" s="20" t="inlineStr">
+        <is>
+          <t>"Assessment of the 40m notification" needed — explicit monitoring/evaluation gap for existing ban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1148" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1148" s="20" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D1148" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1148" s="20" t="inlineStr">
+        <is>
+          <t>Calls for subsidies to producers and to companies producing alternatives; donor support via UNDP MoU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1149" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1149" s="20" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D1149" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1149" s="20" t="inlineStr">
+        <is>
+          <t>UNDP MoU includes "plastic study"; microplastics impacts need more public knowledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1150" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1150" s="20" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1150" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1150" s="20" t="inlineStr">
+        <is>
+          <t>"Technology, recycling factory" lacking; need MRF and land from central/provincial government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1151" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1151" s="20" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1151" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1151" s="20" t="inlineStr">
+        <is>
+          <t>Technology and recycling-factory capacity gaps explicitly named among main challenges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1152" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1152" s="20" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1152" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1152" s="20" t="inlineStr">
+        <is>
+          <t>"Rules &amp; regulation within our areas" and need to assess 40-micron notification — implying enforcement/monitoring gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1153" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1153" s="20" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D1153" s="20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1153" s="20" t="inlineStr">
+        <is>
+          <t>Producer subsidies discussed but no extended producer responsibility framework mentioned — coded no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1154" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1154" s="20" t="inlineStr">
+        <is>
+          <t>Pol_import</t>
+        </is>
+      </c>
+      <c r="D1154" s="20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1154" s="20" t="inlineStr">
+        <is>
+          <t>Import of plastics raised only as an open question ("import of plastics??") with no effective import-control mechanism described.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1155" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1155" s="20" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1155" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1155" s="20" t="inlineStr">
+        <is>
+          <t>Interviewee's public-education role; KMC runs awareness-oriented programmes on plastics reduction and composting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1156" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1156" s="20" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D1156" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1156" s="20" t="inlineStr">
+        <is>
+          <t>Public education is the interviewee's field of work; composting education at household, community and school levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1157" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1157" s="20" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1157" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1157" s="20" t="inlineStr">
+        <is>
+          <t>"Single-use plastics ban — planning" — ban under development, not yet fully operational.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1158" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1158" s="20" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1158" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1158" s="20" t="inlineStr">
+        <is>
+          <t>Stores provide cloth bags instead of polythene; planned government subsidies for companies producing alternatives; Lapti leaf plates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1159" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1159" s="20" t="inlineStr">
+        <is>
+          <t>Pol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1159" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1159" s="20" t="inlineStr">
+        <is>
+          <t>"We did collaborated with wastes at debris near river beds (excavate and transfer)" — active clean-up of riverbed debris.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1160" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1160" s="20" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1160" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1160" s="20" t="inlineStr">
+        <is>
+          <t>Doko Recyclers MoU collecting from Cluster 7; Mayors Forum provisions for plastic management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1161" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1161" s="20" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1161" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1161" s="20" t="inlineStr">
+        <is>
+          <t>Cluster-based collection via registered private partners; landfill site management for 23 municipalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1162" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1162" s="20" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1162" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1162" s="20" t="inlineStr">
+        <is>
+          <t>National policy not implemented; ban only planning stage; no 40-m assessment; land/technology gaps limit effectiveness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1163" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1163" s="20" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1163" s="20" t="inlineStr">
+        <is>
+          <t>Ministry of Forest and Environment plastics policy "not implemented and currently under revision"; KMC relies on the Environment Act 2077 and Natural Resource Management Act 2007 rather than a plastics-specific local ordinance; single-use plastics ban is still at the planning stage; no assessment yet of the 40-micron notification; sufficient waste is collected but KMC cannot procure land for MRF/processing — effectiveness limited by land, technology and enforcement gaps.</t>
+        </is>
+      </c>
+      <c r="E1163" s="20" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1164" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1164" s="20" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1164" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1164" s="20" t="inlineStr">
+        <is>
+          <t>Better coordination between federal (land authority), provincial, district and local government; action plan referenced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1165" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1165" s="20" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1165" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1165" s="20" t="inlineStr">
+        <is>
+          <t>Clarify federal land authority vs local implementation; Mayors Forum and ministry revision to assign roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1166" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1166" s="20" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1166" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1166" s="20" t="inlineStr">
+        <is>
+          <t>Continued public education on microplastics and 40-micron notification assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1167" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1167" s="20" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1167" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1167" s="20" t="inlineStr">
+        <is>
+          <t>Segregation desired but blocked by lack of land/space — future solution requires land and MRF infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1168" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1168" s="20" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1168" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1168" s="20" t="inlineStr">
+        <is>
+          <t>Recycling factory/technology and MRF needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1169" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1169" s="20" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1169" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1169" s="20" t="inlineStr">
+        <is>
+          <t>Public education on microplastics, health/environment/wildlife impacts and composting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1170" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1170" s="20" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1170" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1170" s="20" t="inlineStr">
+        <is>
+          <t>Technology and recycling-factory capacity building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1171" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1171" s="20" t="inlineStr">
+        <is>
+          <t>Sol_ban</t>
+        </is>
+      </c>
+      <c r="D1171" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1171" s="20" t="inlineStr">
+        <is>
+          <t>Single-use plastics ban in planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1172" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1172" s="20" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1172" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1172" s="20" t="inlineStr">
+        <is>
+          <t>Subsidies to producers; government subsidies for alternative-product companies; UNDP donor support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1173" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1173" s="20" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1173" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1173" s="20" t="inlineStr">
+        <is>
+          <t>MRF and land provision by central/provincial government within metro city or valley.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1174" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1174" s="20" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1174" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1174" s="20" t="inlineStr">
+        <is>
+          <t>Subsidise companies producing alternatives; promote Lapti and cloth bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1175" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1175" s="20" t="inlineStr">
+        <is>
+          <t>Sol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1175" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1175" s="20" t="inlineStr">
+        <is>
+          <t>Riverbed debris excavation and transfer (ongoing collaborative work).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1176" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1176" s="20" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1176" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1176" s="20" t="inlineStr">
+        <is>
+          <t>"Rules &amp; regulation within our areas"; assess and enforce 40-micron notification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1177" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1177" s="20" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1177" s="20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1177" s="20" t="inlineStr">
+        <is>
+          <t>Assessment of 40-micron notification; plastic study with UNDP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="20" t="inlineStr">
+        <is>
+          <t>NPL_15</t>
+        </is>
+      </c>
+      <c r="B1178" s="20" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City - Ms. Suna Maya Margen (30 years), Environment Inspector, Public Education &amp; Inspection, Kathmandu (23 June 2025, internal interview no. 2)</t>
+        </is>
+      </c>
+      <c r="C1178" s="20" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1178" s="20" t="inlineStr">
+        <is>
+          <t>Newari community festival practices that try to minimise plastics by using leaf plates (Lapti) instead of disposable plastic — effective culturally but expensive, with cheaper plastic alternatives still dominating unless subsidised.</t>
+        </is>
+      </c>
+      <c r="E1178" s="20" t="inlineStr">
+        <is>
+          <t>Newari festival leaf plates (Lapti) — culturally rooted plastic reduction but cost barrier.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_16 coding for Kathmandu Ward No. 6 solid waste respondent
Code ward-level interview from 22 June 2025 field notes: 40-micron ban
ineffectiveness, no source segregation, paper-bag hospital advocacy,
private waste contractor, Ward 8 landfill, and proposed household pilot
committees. Document possible Dhulikhel-context overlap in Notes.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -62,86 +62,92 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBBFA2"/>
-        <bgColor rgb="00EBBFA2"/>
+        <fgColor rgb="00EBBDA2"/>
+        <bgColor rgb="00EBBDA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBDCA2"/>
-        <bgColor rgb="00EBDCA2"/>
+        <fgColor rgb="00EBD9A2"/>
+        <bgColor rgb="00EBD9A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCEBA2"/>
-        <bgColor rgb="00DCEBA2"/>
+        <fgColor rgb="00E2EBA2"/>
+        <bgColor rgb="00E2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BFEBA2"/>
-        <bgColor rgb="00BFEBA2"/>
+        <fgColor rgb="00C6EBA2"/>
+        <bgColor rgb="00C6EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA2"/>
-        <bgColor rgb="00A2EBA2"/>
+        <fgColor rgb="00ABEBA2"/>
+        <bgColor rgb="00ABEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBBF"/>
-        <bgColor rgb="00A2EBBF"/>
+        <fgColor rgb="00A2EBB4"/>
+        <bgColor rgb="00A2EBB4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBDC"/>
-        <bgColor rgb="00A2EBDC"/>
+        <fgColor rgb="00A2EBD0"/>
+        <bgColor rgb="00A2EBD0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2DCEB"/>
-        <bgColor rgb="00A2DCEB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2BFEB"/>
-        <bgColor rgb="00A2BFEB"/>
+        <fgColor rgb="00A2D0EB"/>
+        <bgColor rgb="00A2D0EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A2EB"/>
-        <bgColor rgb="00A2A2EB"/>
+        <fgColor rgb="00A2B4EB"/>
+        <bgColor rgb="00A2B4EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BFA2EB"/>
-        <bgColor rgb="00BFA2EB"/>
+        <fgColor rgb="00ABA2EB"/>
+        <bgColor rgb="00ABA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCA2EB"/>
-        <bgColor rgb="00DCA2EB"/>
+        <fgColor rgb="00C6A2EB"/>
+        <bgColor rgb="00C6A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2DC"/>
-        <bgColor rgb="00EBA2DC"/>
+        <fgColor rgb="00E2A2EB"/>
+        <bgColor rgb="00E2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2BF"/>
-        <bgColor rgb="00EBA2BF"/>
+        <fgColor rgb="00EBA2D9"/>
+        <bgColor rgb="00EBA2D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2BD"/>
+        <bgColor rgb="00EBA2BD"/>
       </patternFill>
     </fill>
   </fills>
@@ -171,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -231,6 +237,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -598,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -617,7 +626,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_15, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_16, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -737,82 +746,89 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  16. NPL_16 - Kathmandu Metropolitan City Ward No. 6, ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1). Coded from guideline/field notes only. Source notes flag possible context overlap with Dhulikhel ward interviews (12 wards, Ward 8 landfill, Panchkal).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_15, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_16, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_14) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_16) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
-    </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -1999,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ16"/>
+  <dimension ref="A1:CQ17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9731,6 +9747,483 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O17" s="21" t="inlineStr">
+        <is>
+          <t>plastics spread across water bodies and rivers; agricultural land (plastic in fields reducing soil fertility); downstream areas affected when collected waste is dumped and rain washes it downhill; health and environmental impacts (raised as areas where public knowledge is currently limited); Panchkal open sewerage noted in the locality</t>
+        </is>
+      </c>
+      <c r="P17" s="21" t="inlineStr">
+        <is>
+          <t>rivers and water bodies; farmers and agricultural land (soil fertility loss); downstream settlements below the dumping area when it rains; the general public (limited knowledge of health/environment impacts); and the local environment around Panchkal open sewerage</t>
+        </is>
+      </c>
+      <c r="Q17" s="21" t="inlineStr">
+        <is>
+          <t>the general public/households (plastic chosen because it is "affordable and easily available"; alternatives not used because they are not "available and accessible"); national government (40-micron ban notification issued ~3–4 years ago but "did not work"; "no regulatory mechanism in place"; many policies on paper with weak implementation); and capacity gaps among local actors ("people are not able to do management")</t>
+        </is>
+      </c>
+      <c r="R17" s="21" t="inlineStr">
+        <is>
+          <t>the ward office as the front-line coordinator ("it's our responsibility to manage at ward level"); community/hospital advocacy (1,000 paper bags distributed with community to hospitals); a private waste-management company currently collecting waste (proposed to be given clearer responsibility); a single NGO that once worked on recycling (now absent); past household-level "punching plastics &amp; hocking" collection (~10 years ago); and proposed pilot household committees (100–200 households) for segregation, recycling and networking</t>
+        </is>
+      </c>
+      <c r="S17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AW17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA17" s="21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BB17" s="21" t="inlineStr">
+        <is>
+          <t>The ward carries out advocacy and awareness campaigns, distributed 1,000 paper bags with the community to hospitals, and can propose pilot household committees (100–200 households) for segregation and recycling — but has "no adhikar (authority/responsibility) to formulate rules and guidelines to manage plastics", no ward-level budget (a private company manages waste), and cannot enforce the micron ban or control where/how collected waste is dumped (all ward waste goes to the Ward No. 8 landfill site).</t>
+        </is>
+      </c>
+      <c r="BC17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI17" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW17" s="21" t="inlineStr">
+        <is>
+          <t>"Advocacy carried out on it but not sustainable, and not working too well" (paper-bag initiative); "Nothing in particular we have done" about plastics in water bodies; 40-micron ban made ~3–4 years ago "but did not working"; "Many policies are in place, but implementation is lacking properly"; Q4 effectiveness follow-up not answered in source notes.</t>
+        </is>
+      </c>
+      <c r="BX17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CJ17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM17" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO17" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP17" s="21" t="inlineStr">
+        <is>
+          <t>"Old times we did not have plastics. We need to revive the old ways without plastics" — paper thungas, leaves and other natural materials for carrying and packaging instead of plastic.</t>
+        </is>
+      </c>
+      <c r="CQ17" s="21" t="inlineStr">
+        <is>
+          <t>Master list label: "16. Kathmandu Ward no.6", affiliation: Kathmandu Metropolitan City - Ward No. 6 (ward-level solid waste management). Interviewee name and specific role/title not given in source notes. Interview date: 22 June 2025 (Sunday), 11:30am–12:30pm; internal Kathmandu interview no. 1. Coded from interview guideline/field notes only (no full verbatim transcript supplied). Data-quality notes: source header identifies Kathmandu Ward No. 6, but contextual details (all 12 wards' waste going to a landfill in Ward No. 8; Panchkal open sewerage; hospital paper-bag campaign) closely parallel Dhulikhel ward interviews (NPL_9/NPL_10) — retained as labelled but flagged here. Q4 effectiveness follow-up and Theme C level-difference follow-up were blank. Hospital collaboration and paper-bag initiative described as not sustainable/working well. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9742,7 +10235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1178"/>
+  <dimension ref="A1:E1256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -41558,6 +42051,2112 @@
         </is>
       </c>
     </row>
+    <row r="1179">
+      <c r="A1179" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1179" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1179" s="21" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1179" s="21" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="E1179" s="21" t="inlineStr">
+        <is>
+          <t>Ward-level solid waste management respondent at Kathmandu Metropolitan City Ward No. 6 — coded as loc_government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1180" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1180" s="21" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1180" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1180" s="21" t="inlineStr">
+        <is>
+          <t>"People are not comfortable use other options as its not available and accessible"; "Impacts and effects of plastic on environmental n health is needed. Less knowledge about this."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1181" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1181" s="21" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D1181" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1181" s="21" t="inlineStr">
+        <is>
+          <t>"Problem at Source – budgetary and alternative sources. And no regulatory mechanism in place"; "Many policies are in place, but implementation is lacking properly."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1182" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1182" s="21" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1182" s="21" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1182" s="21" t="inlineStr">
+        <is>
+          <t>"It is a problem everywhere"; "Plastics all over water bodies and rivers. Nothing in particular we have done"; hospital/paper-bag initiative "not sustainable, and not working too well."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1183" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1183" s="21" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1183" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1183" s="21" t="inlineStr">
+        <is>
+          <t>"Plastics all over water bodies and rivers"; waste dumped in one place and washed downstream when it rains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1184" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1184" s="21" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1184" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1184" s="21" t="inlineStr">
+        <is>
+          <t>"Plastic is affordable and easily available"; "Everything literally comes in plastics."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1185" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1185" s="21" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1185" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1185" s="21" t="inlineStr">
+        <is>
+          <t>"Other recycling options need to be explored"; "Only once did an NGO work on this, and now there is none"; past household "punching plastics &amp; hocking and collecting from hh level" (~10 years ago).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1186" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1186" s="21" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1186" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1186" s="21" t="inlineStr">
+        <is>
+          <t>Waste gathered and collected twice a week then dumped in one place; hospital collaboration "did not work"; no ward dumping site; private company currently manages waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1187" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1187" s="21" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1187" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1187" s="21" t="inlineStr">
+        <is>
+          <t>"Need to alternative, lots of talk but nothing really happening to find other alternatives"; people not comfortable without accessible substitutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1188" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1188" s="21" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1188" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1188" s="21" t="inlineStr">
+        <is>
+          <t>"No segregation at source, but there is segregation at the dumping site."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1189" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1189" s="21" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1189" s="21" t="inlineStr">
+        <is>
+          <t>plastics spread across water bodies and rivers; agricultural land (plastic in fields reducing soil fertility); downstream areas affected when collected waste is dumped and rain washes it downhill; health and environmental impacts (raised as areas where public knowledge is currently limited); Panchkal open sewerage noted in the locality</t>
+        </is>
+      </c>
+      <c r="E1189" s="21" t="inlineStr">
+        <is>
+          <t>Water bodies/rivers; agricultural land and soil fertility; downstream areas; health/environment knowledge gap; Panchkal open sewerage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1190" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1190" s="21" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1190" s="21" t="inlineStr">
+        <is>
+          <t>rivers and water bodies; farmers and agricultural land (soil fertility loss); downstream settlements below the dumping area when it rains; the general public (limited knowledge of health/environment impacts); and the local environment around Panchkal open sewerage</t>
+        </is>
+      </c>
+      <c r="E1190" s="21" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: rivers/water bodies; farmers/agricultural land; downstream settlements; public health/environment. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1191" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1191" s="21" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1191" s="21" t="inlineStr">
+        <is>
+          <t>the general public/households (plastic chosen because it is "affordable and easily available"; alternatives not used because they are not "available and accessible"); national government (40-micron ban notification issued ~3–4 years ago but "did not work"; "no regulatory mechanism in place"; many policies on paper with weak implementation); and capacity gaps among local actors ("people are not able to do management")</t>
+        </is>
+      </c>
+      <c r="E1191" s="21" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: affordability-driven public; weak national regulation/enforcement; implementation gaps. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1192" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1192" s="21" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1192" s="21" t="inlineStr">
+        <is>
+          <t>the ward office as the front-line coordinator ("it's our responsibility to manage at ward level"); community/hospital advocacy (1,000 paper bags distributed with community to hospitals); a private waste-management company currently collecting waste (proposed to be given clearer responsibility); a single NGO that once worked on recycling (now absent); past household-level "punching plastics &amp; hocking" collection (~10 years ago); and proposed pilot household committees (100–200 households) for segregation, recycling and networking</t>
+        </is>
+      </c>
+      <c r="E1192" s="21" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: ward office; community/hospital paper-bag initiative; private waste company; past/proposed NGO and household-committee pilots; traditional materials. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1193" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1193" s="21" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D1193" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1193" s="21" t="inlineStr">
+        <is>
+          <t>Attempted hospital collaboration on waste management; community paper-bag distribution; one NGO previously worked on recycling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1194" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1194" s="21" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D1194" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1194" s="21" t="inlineStr">
+        <is>
+          <t>"We have no adhikar (authority/responsibility) – to formulate rules and guidelines to manage plastics"; ward has no budget while a private company manages waste at municipal level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1195" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1195" s="21" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1195" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1195" s="21" t="inlineStr">
+        <is>
+          <t>"It's everyone's responsibility" alongside ward having no rule-making authority and policies existing on paper with weak implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1196" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1196" s="21" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1196" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1196" s="21" t="inlineStr">
+        <is>
+          <t>40-micron plastics ban initiated with notification issued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1197" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1197" s="21" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1197" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1197" s="21" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1198" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1198" s="21" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1198" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1198" s="21" t="inlineStr">
+        <is>
+          <t>"It's our responsibility to manage at ward level"; municipality/ward system gathers and dumps waste; private company contracted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1199" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1199" s="21" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1199" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1199" s="21" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1200" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1200" s="21" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1200" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1200" s="21" t="inlineStr">
+        <is>
+          <t>Private company currently managing ward waste; proposed to be given clearer responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1201" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1201" s="21" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1201" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1201" s="21" t="inlineStr">
+        <is>
+          <t>One NGO once worked on recycling (now absent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1202" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1202" s="21" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1202" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1202" s="21" t="inlineStr">
+        <is>
+          <t>NA - research need mentioned but no scientific actors named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1203" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1203" s="21" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1203" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1203" s="21" t="inlineStr">
+        <is>
+          <t>"At the household level, we need to work from there to manage plastics"; proposed 100–200 household pilot committees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1204" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1204" s="21" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1204" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1204" s="21" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1205" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1205" s="21" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1205" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1205" s="21" t="inlineStr">
+        <is>
+          <t>Hospital has a waste-management unit with agreement on dumpsite/open-space deposit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1206" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1206" s="21" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1206" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1206" s="21" t="inlineStr">
+        <is>
+          <t>40-micron ban made ~3–4 years ago "but did not working"; "no regulatory mechanism in place"; implementation lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1207" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1207" s="21" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1207" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1207" s="21" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1208" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1208" s="21" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1208" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1208" s="21" t="inlineStr">
+        <is>
+          <t>Ward has no budget for waste management despite operational responsibility at ward level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1209" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1209" s="21" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1209" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1209" s="21" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1210" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1210" s="21" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1210" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1210" s="21" t="inlineStr">
+        <is>
+          <t>NA - private waste company portrayed as solution, not culprit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1211" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1211" s="21" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1211" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1211" s="21" t="inlineStr">
+        <is>
+          <t>NA - NGO absence noted but not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1212" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1212" s="21" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1212" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1212" s="21" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1213" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1213" s="21" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1213" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1213" s="21" t="inlineStr">
+        <is>
+          <t>Public chooses plastic because alternatives are unavailable/inaccessible and plastic is cheap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1214" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1214" s="21" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1214" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1214" s="21" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1215" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1215" s="21" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1215" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1215" s="21" t="inlineStr">
+        <is>
+          <t>NA - hospitals discussed as partners, not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1216" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1216" s="21" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1216" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1216" s="21" t="inlineStr">
+        <is>
+          <t>Regulating plastics under 40 microns with enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1217" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1217" s="21" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1217" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1217" s="21" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1218" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1218" s="21" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1218" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1218" s="21" t="inlineStr">
+        <is>
+          <t>Ward/municipal implementation; give private waste company clearer responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1219" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1219" s="21" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1219" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1219" s="21" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1220" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1220" s="21" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1220" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1220" s="21" t="inlineStr">
+        <is>
+          <t>Private waste-management company should be given responsibility "so they can better manage."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1221" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1221" s="21" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1221" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1221" s="21" t="inlineStr">
+        <is>
+          <t>NGO recycling work referenced — only one NGO worked before, needs enforcement/support to scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1222" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1222" s="21" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1222" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1222" s="21" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1223" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1223" s="21" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1223" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1223" s="21" t="inlineStr">
+        <is>
+          <t>Household-level management; pilot committees of 100–200 households.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1224" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1224" s="21" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1224" s="21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1224" s="21" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1225" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1225" s="21" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1225" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1225" s="21" t="inlineStr">
+        <is>
+          <t>Hospitals targeted in paper-bag advocacy; drinking-water bottles named for replacement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1226" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1226" s="21" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1226" s="21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E1226" s="21" t="inlineStr">
+        <is>
+          <t>Ward-level respondent describing grassroots advocacy, hospital/community paper-bag distribution and proposed household pilot committees — street-level implementer (role 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1227" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1227" s="21" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1227" s="21" t="inlineStr">
+        <is>
+          <t>The ward carries out advocacy and awareness campaigns, distributed 1,000 paper bags with the community to hospitals, and can propose pilot household committees (100–200 households) for segregation and recycling — but has "no adhikar (authority/responsibility) to formulate rules and guidelines to manage plastics", no ward-level budget (a private company manages waste), and cannot enforce the micron ban or control where/how collected waste is dumped (all ward waste goes to the Ward No. 8 landfill site).</t>
+        </is>
+      </c>
+      <c r="E1227" s="21" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1228" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1228" s="21" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1228" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1228" s="21" t="inlineStr">
+        <is>
+          <t>Ban effectiveness questioned; implementation gaps; no assessment of impacts communicated to public.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1229" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1229" s="21" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D1229" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1229" s="21" t="inlineStr">
+        <is>
+          <t>"Problem at Source – budgetary"; "At the ward level – there is no budget"; paper-bag initiative not sustainable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1230" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1230" s="21" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D1230" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1230" s="21" t="inlineStr">
+        <is>
+          <t>"Impacts and effects of plastic on environmental n health is needed. Less knowledge about this."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1231" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1231" s="21" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1231" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1231" s="21" t="inlineStr">
+        <is>
+          <t>No ward dumping site; hospital lacks dumping site; open-space deposit and burning suggested but difficult due to volume; all ward waste goes to Ward No. 8 landfill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1232" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1232" s="21" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1232" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1232" s="21" t="inlineStr">
+        <is>
+          <t>"Capacity – people are not able to do management."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1233" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1233" s="21" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1233" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1233" s="21" t="inlineStr">
+        <is>
+          <t>40-micron ban "did not working"; NGO recycling "needs enforcement"; implementation lacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1234" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1234" s="21" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D1234" s="21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1234" s="21" t="inlineStr">
+        <is>
+          <t>Extended producer responsibility not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1235" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1235" s="21" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1235" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1235" s="21" t="inlineStr">
+        <is>
+          <t>"Advocacy/awareness is carried out at every level"; ward paper-bag distribution to hospitals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1236" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1236" s="21" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D1236" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1236" s="21" t="inlineStr">
+        <is>
+          <t>"Campaigns are carried out."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1237" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1237" s="21" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1237" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1237" s="21" t="inlineStr">
+        <is>
+          <t>40-micron plastics ban initiated; notification issued ~3–4 years ago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1238" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1238" s="21" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1238" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1238" s="21" t="inlineStr">
+        <is>
+          <t>1,000 paper bags distributed with community to hospitals; paper thungas, leaves and natural materials promoted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1239" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1239" s="21" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1239" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1239" s="21" t="inlineStr">
+        <is>
+          <t>Segregation at dumping site; past NGO recycling work; household punching/hooking collection ~10 years ago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1240" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1240" s="21" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1240" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1240" s="21" t="inlineStr">
+        <is>
+          <t>Waste gathered and collected twice a week, then dumped in one place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1241" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1241" s="21" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1241" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1241" s="21" t="inlineStr">
+        <is>
+          <t>Awareness/paper-bag initiative not sustainable; ban ineffective; many policies on paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1242" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1242" s="21" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1242" s="21" t="inlineStr">
+        <is>
+          <t>"Advocacy carried out on it but not sustainable, and not working too well" (paper-bag initiative); "Nothing in particular we have done" about plastics in water bodies; 40-micron ban made ~3–4 years ago "but did not working"; "Many policies are in place, but implementation is lacking properly"; Q4 effectiveness follow-up not answered in source notes.</t>
+        </is>
+      </c>
+      <c r="E1242" s="21" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1243" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1243" s="21" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1243" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1243" s="21" t="inlineStr">
+        <is>
+          <t>Pilot household committees (100–200 households) to coordinate segregation, recycling, processing and networking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1244" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1244" s="21" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1244" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1244" s="21" t="inlineStr">
+        <is>
+          <t>Give private waste company clearer responsibility; clarify ward vs municipal roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1245" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1245" s="21" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1245" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1245" s="21" t="inlineStr">
+        <is>
+          <t>"Awareness is necessary."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1246" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1246" s="21" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1246" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1246" s="21" t="inlineStr">
+        <is>
+          <t>Source segregation via household committees; segregation currently only at dumping site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1247" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1247" s="21" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1247" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1247" s="21" t="inlineStr">
+        <is>
+          <t>Explore recycling options beyond a single NGO; revive household collection models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1248" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1248" s="21" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1248" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1248" s="21" t="inlineStr">
+        <is>
+          <t>Public education on health/environment impacts of plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1249" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1249" s="21" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1249" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1249" s="21" t="inlineStr">
+        <is>
+          <t>Build management capacity at ward and household levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1250" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1250" s="21" t="inlineStr">
+        <is>
+          <t>Sol_ban</t>
+        </is>
+      </c>
+      <c r="D1250" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1250" s="21" t="inlineStr">
+        <is>
+          <t>Make 40-micron regulation work with enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1251" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1251" s="21" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1251" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1251" s="21" t="inlineStr">
+        <is>
+          <t>Address budgetary constraints at source and ward level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1252" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1252" s="21" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1252" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1252" s="21" t="inlineStr">
+        <is>
+          <t>Proper dumping/processing sites; replace open-space deposit/burning practices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1253" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1253" s="21" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1253" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1253" s="21" t="inlineStr">
+        <is>
+          <t>Provide sustainable alternatives; revive paper thungas, leaves and natural materials; start by replacing drinking-water bottles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1254" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1254" s="21" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1254" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1254" s="21" t="inlineStr">
+        <is>
+          <t>Enforcement needed for ban and NGO recycling models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1255" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1255" s="21" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1255" s="21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1255" s="21" t="inlineStr">
+        <is>
+          <t>Assess policy implementation and communicate plastic impacts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="21" t="inlineStr">
+        <is>
+          <t>NPL_16</t>
+        </is>
+      </c>
+      <c r="B1256" s="21" t="inlineStr">
+        <is>
+          <t>Kathmandu Metropolitan City Ward No. 6 - ward-level solid waste management respondent (name/role not given), Kathmandu (22 June 2025, 11:30am–12:30pm; internal interview no. 1)</t>
+        </is>
+      </c>
+      <c r="C1256" s="21" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1256" s="21" t="inlineStr">
+        <is>
+          <t>"Old times we did not have plastics. We need to revive the old ways without plastics" — paper thungas, leaves and other natural materials for carrying and packaging instead of plastic.</t>
+        </is>
+      </c>
+      <c r="E1256" s="21" t="inlineStr">
+        <is>
+          <t>Pre-plastic practices; paper thungas, leaves and natural materials.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_18 coding for dry waste practitioner/consultant interview
Code unnamed dry waste management practitioner active since 2017
(Kathmandu & Pokhara): UNDP training/consulting, multilayer plastics,
Bhaktapur campaigns, UK university policy research, EPR advocacy, and
cherry-picking/value-chain gaps. Matches Q3a content excluded from NPL_3.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -62,98 +62,104 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBBCA2"/>
-        <bgColor rgb="00EBBCA2"/>
+        <fgColor rgb="00EBBAA2"/>
+        <bgColor rgb="00EBBAA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD5A2"/>
-        <bgColor rgb="00EBD5A2"/>
+        <fgColor rgb="00EBD3A2"/>
+        <bgColor rgb="00EBD3A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7EBA2"/>
-        <bgColor rgb="00E7EBA2"/>
+        <fgColor rgb="00EBEBA2"/>
+        <bgColor rgb="00EBEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CDEBA2"/>
-        <bgColor rgb="00CDEBA2"/>
+        <fgColor rgb="00D3EBA2"/>
+        <bgColor rgb="00D3EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B3EBA2"/>
-        <bgColor rgb="00B3EBA2"/>
+        <fgColor rgb="00BAEBA2"/>
+        <bgColor rgb="00BAEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBAB"/>
-        <bgColor rgb="00A2EBAB"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBC4"/>
-        <bgColor rgb="00A2EBC4"/>
+        <fgColor rgb="00A2EBBA"/>
+        <bgColor rgb="00A2EBBA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBDE"/>
-        <bgColor rgb="00A2EBDE"/>
+        <fgColor rgb="00A2EBD3"/>
+        <bgColor rgb="00A2EBD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2DEEB"/>
-        <bgColor rgb="00A2DEEB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2C4EB"/>
-        <bgColor rgb="00A2C4EB"/>
+        <fgColor rgb="00A2D3EB"/>
+        <bgColor rgb="00A2D3EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2ABEB"/>
-        <bgColor rgb="00A2ABEB"/>
+        <fgColor rgb="00A2BAEB"/>
+        <bgColor rgb="00A2BAEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B3A2EB"/>
-        <bgColor rgb="00B3A2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CDA2EB"/>
-        <bgColor rgb="00CDA2EB"/>
+        <fgColor rgb="00BAA2EB"/>
+        <bgColor rgb="00BAA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7A2EB"/>
-        <bgColor rgb="00E7A2EB"/>
+        <fgColor rgb="00D3A2EB"/>
+        <bgColor rgb="00D3A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D5"/>
-        <bgColor rgb="00EBA2D5"/>
+        <fgColor rgb="00EBA2EB"/>
+        <bgColor rgb="00EBA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2BC"/>
-        <bgColor rgb="00EBA2BC"/>
+        <fgColor rgb="00EBA2D3"/>
+        <bgColor rgb="00EBA2D3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2BA"/>
+        <bgColor rgb="00EBA2BA"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -249,6 +255,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -616,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -635,7 +644,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_17, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_18, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -769,82 +778,89 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  18. NPL_18 - Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017). Coded from guideline/field notes. Content matches Q3a bullets previously excluded from NPL_3; thematically overlaps NPL_5.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_17, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_18, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_17) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_18) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2031,7 +2047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ18"/>
+  <dimension ref="A1:CQ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10717,6 +10733,483 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>private_sector</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O19" s="23" t="inlineStr">
+        <is>
+          <t>low-value and multi-layer plastics discarded at riverbanks and dump sites when they lack market value; broader environmental pollution from unmanaged plastic fractions left outside the profitable recycling stream</t>
+        </is>
+      </c>
+      <c r="P19" s="23" t="inlineStr">
+        <is>
+          <t>rivers and riverbank/dump-site environments where plastics with little or no market value are discarded; communities and ecosystems affected by unmanaged low-value plastic fractions; the public affected by inadequate end-of-life management rather than plastic use alone</t>
+        </is>
+      </c>
+      <c r="Q19" s="23" t="inlineStr">
+        <is>
+          <t>plastic producers without extended producer responsibility; informal/formal scrap collectors engaging in "cherry-picking" (only high-value plastics collected, low-value fractions left behind); the national government (unclear lead department, no dedicated plastic mandate, no coordinating/implementing body, fragmented policies); key decision-makers and the public who do not take plastic pollution seriously enough; and poorly coordinated stakeholders (government, private sector, communities, donors) working in isolation</t>
+        </is>
+      </c>
+      <c r="R19" s="23" t="inlineStr">
+        <is>
+          <t>the interviewee's own dry-waste management practice (sorting plastics into grades for downstream recyclers since 2017); UNDP-funded training and consulting (Pokhara, ~400 participants, multilayer-plastic focus); Bhaktapur awareness campaigns; UK-university policy research on household product end-of-life management; municipalities as key local implementers; waste managers needing formal support; and proposed EPR, sector incentives, and processing facilities for low-value plastics</t>
+        </is>
+      </c>
+      <c r="S19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AJ19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AL19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA19" s="23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BB19" s="23" t="inlineStr">
+        <is>
+          <t>The interviewee operates dry-waste sorting and grade-based handoff to downstream recyclers, designs UNDP-funded training programmes (including multilayer-plastic projects in Pokhara), runs Bhaktapur awareness campaigns, consults for UNDP on waste management, and conducts UK-university policy research — but has limited influence over national policy architecture, which department should lead, or sector-wide incentives/infrastructure.</t>
+        </is>
+      </c>
+      <c r="BC19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI19" s="23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BO19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BT19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW19" s="23" t="inlineStr">
+        <is>
+          <t>"Largely ineffective": planned single-use plastics ban above 40 microns discussed nationally but "not been fully implemented/enforced"; "very few national-level policies in place"; municipalities develop their own policies resulting in a "fragmented and uneven policy landscape" without shared framework or resources.</t>
+        </is>
+      </c>
+      <c r="BX19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CA19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CD19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CH19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CM19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO19" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP19" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CQ19" s="23" t="inlineStr">
+        <is>
+          <t>Master list label: "18. Dry waste management practitioner/ consultant (unnamed)", affiliation: dry waste management practitioner; consultant and researcher (Kathmandu &amp; Pokhara). Interviewee name not given. Active in dry waste management since 2017 (~8 years). Interview date not stated in source notes. Coded from structured guideline/field notes only (Theme A Q1/Q2 on plastic problem/concern and visible effects were blank; Q4a/Q4b ministry template questions blank; Theme C level-difference follow-up blank). DATA-QUALITY NOTE: this content matches the Q3a bullet list previously excluded from NPL_3 (KTM Municipal Office) as belonging to a different respondent; thematically overlaps NPL_5 (Doco Recyclers) on EPR, cherry-picking and multilayer plastics but coded here as a separate unnamed practitioner/consultant interview per the research team. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10728,7 +11221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1337"/>
+  <dimension ref="A1:E1418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -46837,6 +47330,2193 @@
         </is>
       </c>
     </row>
+    <row r="1338">
+      <c r="A1338" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1338" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1338" s="23" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1338" s="23" t="inlineStr">
+        <is>
+          <t>private_sector</t>
+        </is>
+      </c>
+      <c r="E1338" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner, consultant and researcher operating in Kathmandu and Pokhara since 2017 — coded as private_sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1339" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1339" s="23" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1339" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1339" s="23" t="inlineStr">
+        <is>
+          <t>"Plastic pollution is not taken seriously enough by key decision-makers and the public"; follow-up calls to reduce public ignorance through education.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1340" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1340" s="23" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D1340" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1340" s="23" t="inlineStr">
+        <is>
+          <t>"Lack of coherent policy"; fragmented municipal policies without national framework; unclear which department should lead; no dedicated plastic-specific mandate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1341" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1341" s="23" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1341" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1341" s="23" t="inlineStr">
+        <is>
+          <t>NA - Theme A Q1 (is plastic a problem?) and concern follow-up were left blank in the source notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1342" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1342" s="23" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1342" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1342" s="23" t="inlineStr">
+        <is>
+          <t>Plastics with little or no market value "end up discarded at riverbanks and dump sites."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1343" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1343" s="23" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1343" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1343" s="23" t="inlineStr">
+        <is>
+          <t>Q9 targets consumers/households to reduce plastic consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1344" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1344" s="23" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1344" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1344" s="23" t="inlineStr">
+        <is>
+          <t>No established value chain; cherry-picking leaves low-value plastics unaddressed; inadequate processing/recycling infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1345" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1345" s="23" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1345" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1345" s="23" t="inlineStr">
+        <is>
+          <t>Inadequate infrastructure for collection, processing and recycling at scale; missing implementing/coordinating body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1346" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1346" s="23" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1346" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1346" s="23" t="inlineStr">
+        <is>
+          <t>Producers face no EPR obligation for end-of-life plastics they put on the market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1347" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1347" s="23" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1347" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1347" s="23" t="inlineStr">
+        <is>
+          <t>Core practice is sorting collected plastics into different grades — implies segregation is needed but value-chain gaps limit effective downstream use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1348" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1348" s="23" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1348" s="23" t="inlineStr">
+        <is>
+          <t>low-value and multi-layer plastics discarded at riverbanks and dump sites when they lack market value; broader environmental pollution from unmanaged plastic fractions left outside the profitable recycling stream</t>
+        </is>
+      </c>
+      <c r="E1348" s="23" t="inlineStr">
+        <is>
+          <t>Riverbanks and dump sites receiving discarded low-value/multi-layer plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1349" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1349" s="23" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1349" s="23" t="inlineStr">
+        <is>
+          <t>rivers and riverbank/dump-site environments where plastics with little or no market value are discarded; communities and ecosystems affected by unmanaged low-value plastic fractions; the public affected by inadequate end-of-life management rather than plastic use alone</t>
+        </is>
+      </c>
+      <c r="E1349" s="23" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: riverbank/dump-site environments; communities/ecosystems; public affected by poor end-of-life management. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1350" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1350" s="23" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1350" s="23" t="inlineStr">
+        <is>
+          <t>plastic producers without extended producer responsibility; informal/formal scrap collectors engaging in "cherry-picking" (only high-value plastics collected, low-value fractions left behind); the national government (unclear lead department, no dedicated plastic mandate, no coordinating/implementing body, fragmented policies); key decision-makers and the public who do not take plastic pollution seriously enough; and poorly coordinated stakeholders (government, private sector, communities, donors) working in isolation</t>
+        </is>
+      </c>
+      <c r="E1350" s="23" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: producers without EPR; cherry-picking collectors; weak/fragmented national governance; unserious public/decision-makers; poor stakeholder coordination. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1351" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1351" s="23" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1351" s="23" t="inlineStr">
+        <is>
+          <t>the interviewee's own dry-waste management practice (sorting plastics into grades for downstream recyclers since 2017); UNDP-funded training and consulting (Pokhara, ~400 participants, multilayer-plastic focus); Bhaktapur awareness campaigns; UK-university policy research on household product end-of-life management; municipalities as key local implementers; waste managers needing formal support; and proposed EPR, sector incentives, and processing facilities for low-value plastics</t>
+        </is>
+      </c>
+      <c r="E1351" s="23" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: practitioner/operator; UNDP; municipalities; waste managers; researchers; proposed EPR and sector incentives. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1352" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1352" s="23" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D1352" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1352" s="23" t="inlineStr">
+        <is>
+          <t>Policy research with a UK university; technology transfer from countries that have solved these problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1353" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1353" s="23" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D1353" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1353" s="23" t="inlineStr">
+        <is>
+          <t>"Poor coordination among stakeholders — government, private sector, communities, and donors are not working in alignment."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1354" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1354" s="23" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D1354" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1354" s="23" t="inlineStr">
+        <is>
+          <t>Unclear national lead department; municipalities acting in isolation; Department of Environment without clear coordination with local communities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1355" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1355" s="23" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1355" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1355" s="23" t="inlineStr">
+        <is>
+          <t>"Uncertain which Department should look after"; plastic governance subsumed under Municipal Solid Waste Management Act with no dedicated mandate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1356" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1356" s="23" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1356" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1356" s="23" t="inlineStr">
+        <is>
+          <t>Government of Nepal — but unclear lead department.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1357" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1357" s="23" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1357" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1357" s="23" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1358" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1358" s="23" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1358" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1358" s="23" t="inlineStr">
+        <is>
+          <t>Municipalities are "key actors" bearing practical burden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1359" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1359" s="23" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1359" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1359" s="23" t="inlineStr">
+        <is>
+          <t>NA - students targeted via curriculum but not named as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1360" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1360" s="23" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1360" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1360" s="23" t="inlineStr">
+        <is>
+          <t>Private sector participates; informal scrap collectors recover valuable plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1361" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1361" s="23" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1361" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1361" s="23" t="inlineStr">
+        <is>
+          <t>Community groups worked with on multilayer plastic management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1362" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1362" s="23" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1362" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1362" s="23" t="inlineStr">
+        <is>
+          <t>UK-university collaboration on end-of-life policy research.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1363" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1363" s="23" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1363" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1363" s="23" t="inlineStr">
+        <is>
+          <t>Consumers/households responsible for reducing consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1364" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1364" s="23" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1364" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1364" s="23" t="inlineStr">
+        <is>
+          <t>Schools proposed for waste-management curriculum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1365" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1365" s="23" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1365" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1365" s="23" t="inlineStr">
+        <is>
+          <t>Producers should bear EPR responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1366" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1366" s="23" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1366" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1366" s="23" t="inlineStr">
+        <is>
+          <t>No dedicated governing/implementing body; no EPR; fragmented national policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1367" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1367" s="23" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1367" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1367" s="23" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1368" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1368" s="23" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1368" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1368" s="23" t="inlineStr">
+        <is>
+          <t>Fragmented municipal policies without shared national framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1369" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1369" s="23" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1369" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1369" s="23" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1370" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1370" s="23" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1370" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1370" s="23" t="inlineStr">
+        <is>
+          <t>"Cherry-picking" — only high-value plastics collected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1371" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1371" s="23" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1371" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1371" s="23" t="inlineStr">
+        <is>
+          <t>NA - community groups portrayed as partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1372" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1372" s="23" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1372" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1372" s="23" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1373" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1373" s="23" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1373" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1373" s="23" t="inlineStr">
+        <is>
+          <t>Public/consumers not taking issue seriously enough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1374" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1374" s="23" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1374" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1374" s="23" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1375" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1375" s="23" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1375" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1375" s="23" t="inlineStr">
+        <is>
+          <t>NA - producers targeted via EPR, not primarily blamed as companies separate from production responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1376" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1376" s="23" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1376" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1376" s="23" t="inlineStr">
+        <is>
+          <t>Coherent national framework and coordination needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1377" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1377" s="23" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1377" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1377" s="23" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1378" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1378" s="23" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1378" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1378" s="23" t="inlineStr">
+        <is>
+          <t>Municipalities should be primary implementing/monitoring body and made accountable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1379" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1379" s="23" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1379" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1379" s="23" t="inlineStr">
+        <is>
+          <t>"As young as you can catch them"; embed waste management in education system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1380" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1380" s="23" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1380" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1380" s="23" t="inlineStr">
+        <is>
+          <t>Waste managers need formal support and recognition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1381" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1381" s="23" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1381" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1381" s="23" t="inlineStr">
+        <is>
+          <t>NA - not named as primary target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1382" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1382" s="23" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1382" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1382" s="23" t="inlineStr">
+        <is>
+          <t>NA - researchers partners, not primary target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1383" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1383" s="23" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1383" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1383" s="23" t="inlineStr">
+        <is>
+          <t>Reduce plastic consumption at household/individual level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1384" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1384" s="23" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1384" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1384" s="23" t="inlineStr">
+        <is>
+          <t>Formal school curriculum for waste management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1385" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1385" s="23" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1385" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1385" s="23" t="inlineStr">
+        <is>
+          <t>Producers through EPR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1386" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1386" s="23" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1386" s="23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1386" s="23" t="inlineStr">
+        <is>
+          <t>Practitioner/consultant operating sorting systems, UNDP training, awareness campaigns and policy research — managerial/organisational implementer (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1387" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1387" s="23" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1387" s="23" t="inlineStr">
+        <is>
+          <t>The interviewee operates dry-waste sorting and grade-based handoff to downstream recyclers, designs UNDP-funded training programmes (including multilayer-plastic projects in Pokhara), runs Bhaktapur awareness campaigns, consults for UNDP on waste management, and conducts UK-university policy research — but has limited influence over national policy architecture, which department should lead, or sector-wide incentives/infrastructure.</t>
+        </is>
+      </c>
+      <c r="E1387" s="23" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1388" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1388" s="23" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1388" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1388" s="23" t="inlineStr">
+        <is>
+          <t>SUP ban not fully enforced/monitored; no national monitoring framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1389" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1389" s="23" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D1389" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1389" s="23" t="inlineStr">
+        <is>
+          <t>Private sector hesitant to invest; sector lacks incentives and long-term viability confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1390" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1390" s="23" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D1390" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1390" s="23" t="inlineStr">
+        <is>
+          <t>UK-university end-of-life policy research; UNDP consulting; multilayer-plastic project focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1391" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1391" s="23" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1391" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1391" s="23" t="inlineStr">
+        <is>
+          <t>Inadequate collection, processing and recycling infrastructure at scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1392" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1392" s="23" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1392" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1392" s="23" t="inlineStr">
+        <is>
+          <t>Sector needs incentives, technology transfer and human-capacity building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1393" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1393" s="23" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1393" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1393" s="23" t="inlineStr">
+        <is>
+          <t>Planned &gt;40-micron SUP ban not fully implemented/enforced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1394" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1394" s="23" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D1394" s="23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1394" s="23" t="inlineStr">
+        <is>
+          <t>EPR "has not been introduced in Nepal."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1395" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1395" s="23" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1395" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1395" s="23" t="inlineStr">
+        <is>
+          <t>Bhaktapur awareness campaigns on plastic reduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1396" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1396" s="23" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D1396" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1396" s="23" t="inlineStr">
+        <is>
+          <t>UNDP skill development training (~400 participants, Pokhara); school curriculum proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1397" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1397" s="23" t="inlineStr">
+        <is>
+          <t>Pol_RD</t>
+        </is>
+      </c>
+      <c r="D1397" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1397" s="23" t="inlineStr">
+        <is>
+          <t>Policy research with UK university on household product end-of-life management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1398" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1398" s="23" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1398" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1398" s="23" t="inlineStr">
+        <is>
+          <t>Planned ban on single-use plastics above 40 microns discussed nationally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1399" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1399" s="23" t="inlineStr">
+        <is>
+          <t>Pol_upcycling</t>
+        </is>
+      </c>
+      <c r="D1399" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1399" s="23" t="inlineStr">
+        <is>
+          <t>UNDP training covered upcycling and paper upcycling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1400" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1400" s="23" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1400" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1400" s="23" t="inlineStr">
+        <is>
+          <t>Interviewee sorts plastics into grades and passes to downstream recyclers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1401" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1401" s="23" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1401" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1401" s="23" t="inlineStr">
+        <is>
+          <t>Collection chains discussed as needing financing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1402" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1402" s="23" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1402" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1402" s="23" t="inlineStr">
+        <is>
+          <t>Largely ineffective — ban not enforced; fragmented municipal policies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1403" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1403" s="23" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1403" s="23" t="inlineStr">
+        <is>
+          <t>"Largely ineffective": planned single-use plastics ban above 40 microns discussed nationally but "not been fully implemented/enforced"; "very few national-level policies in place"; municipalities develop their own policies resulting in a "fragmented and uneven policy landscape" without shared framework or resources.</t>
+        </is>
+      </c>
+      <c r="E1403" s="23" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1404" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1404" s="23" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1404" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1404" s="23" t="inlineStr">
+        <is>
+          <t>Dedicated guiding governing/implementing body needed (Ministry of Environment as natural candidate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1405" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1405" s="23" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1405" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1405" s="23" t="inlineStr">
+        <is>
+          <t>Clarify national lead; make municipalities accountable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1406" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1406" s="23" t="inlineStr">
+        <is>
+          <t>Sol_epr</t>
+        </is>
+      </c>
+      <c r="D1406" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1406" s="23" t="inlineStr">
+        <is>
+          <t>"Single most important first step" — producers accountable for end-of-life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1407" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1407" s="23" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1407" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1407" s="23" t="inlineStr">
+        <is>
+          <t>Bhaktapur campaigns; reduce public ignorance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1408" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1408" s="23" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1408" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1408" s="23" t="inlineStr">
+        <is>
+          <t>Sorting into grades as part of value-chain solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1409" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1409" s="23" t="inlineStr">
+        <is>
+          <t>Sol_upcycling</t>
+        </is>
+      </c>
+      <c r="D1409" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1409" s="23" t="inlineStr">
+        <is>
+          <t>Upcycling covered in UNDP training programmes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1410" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1410" s="23" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1410" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1410" s="23" t="inlineStr">
+        <is>
+          <t>Invest in processing/treatment/recycling facilities, especially for low-value plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1411" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1411" s="23" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1411" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1411" s="23" t="inlineStr">
+        <is>
+          <t>Waste management in formal school curriculum from early age.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1412" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1412" s="23" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1412" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1412" s="23" t="inlineStr">
+        <is>
+          <t>Technology transfer — "do not reinvent the wheel."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1413" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1413" s="23" t="inlineStr">
+        <is>
+          <t>Sol_RD</t>
+        </is>
+      </c>
+      <c r="D1413" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1413" s="23" t="inlineStr">
+        <is>
+          <t>Continued policy and end-of-life research.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1414" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1414" s="23" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1414" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1414" s="23" t="inlineStr">
+        <is>
+          <t>Funding for collection chains and recycling facilities; sector incentives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1415" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1415" s="23" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1415" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1415" s="23" t="inlineStr">
+        <is>
+          <t>Processing facilities for low-value plastics; collection-chain infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1416" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1416" s="23" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1416" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1416" s="23" t="inlineStr">
+        <is>
+          <t>Implement and monitor SUP ban; practical guidelines needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1417" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1417" s="23" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1417" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1417" s="23" t="inlineStr">
+        <is>
+          <t>Municipalities as implementing/monitoring partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" s="23" t="inlineStr">
+        <is>
+          <t>NPL_18</t>
+        </is>
+      </c>
+      <c r="B1418" s="23" t="inlineStr">
+        <is>
+          <t>Dry waste management practitioner / consultant &amp; researcher (unnamed), Kathmandu &amp; Pokhara (active since 2017; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1418" s="23" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1418" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1418" s="23" t="inlineStr">
+        <is>
+          <t>NA - not discussed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_19 coding for TAAN Trekking Association president
Code verbatim interview on tourism-sector plastic governance: trail litter,
domestic tourism, guide/porter training, ACAP partnerships, Mustang/Manaslu
deposit policy, Pokhara lake cleanup, and traditional Gurung Bhangra/dal bhat
alternatives.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -62,104 +62,110 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBBAA2"/>
-        <bgColor rgb="00EBBAA2"/>
+        <fgColor rgb="00EBB9A2"/>
+        <bgColor rgb="00EBB9A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD3A2"/>
-        <bgColor rgb="00EBD3A2"/>
+        <fgColor rgb="00EBD0A2"/>
+        <bgColor rgb="00EBD0A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBEBA2"/>
-        <bgColor rgb="00EBEBA2"/>
+        <fgColor rgb="00EBE7A2"/>
+        <bgColor rgb="00EBE7A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3EBA2"/>
-        <bgColor rgb="00D3EBA2"/>
+        <fgColor rgb="00D8EBA2"/>
+        <bgColor rgb="00D8EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BAEBA2"/>
-        <bgColor rgb="00BAEBA2"/>
+        <fgColor rgb="00C1EBA2"/>
+        <bgColor rgb="00C1EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA2"/>
-        <bgColor rgb="00A2EBA2"/>
+        <fgColor rgb="00AAEBA2"/>
+        <bgColor rgb="00AAEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBBA"/>
-        <bgColor rgb="00A2EBBA"/>
+        <fgColor rgb="00A2EBB1"/>
+        <bgColor rgb="00A2EBB1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD3"/>
-        <bgColor rgb="00A2EBD3"/>
+        <fgColor rgb="00A2EBC8"/>
+        <bgColor rgb="00A2EBC8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBDF"/>
+        <bgColor rgb="00A2EBDF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D3EB"/>
-        <bgColor rgb="00A2D3EB"/>
+        <fgColor rgb="00A2DFEB"/>
+        <bgColor rgb="00A2DFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2BAEB"/>
-        <bgColor rgb="00A2BAEB"/>
+        <fgColor rgb="00A2C8EB"/>
+        <bgColor rgb="00A2C8EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A2EB"/>
-        <bgColor rgb="00A2A2EB"/>
+        <fgColor rgb="00A2B1EB"/>
+        <bgColor rgb="00A2B1EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BAA2EB"/>
-        <bgColor rgb="00BAA2EB"/>
+        <fgColor rgb="00AAA2EB"/>
+        <bgColor rgb="00AAA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3A2EB"/>
-        <bgColor rgb="00D3A2EB"/>
+        <fgColor rgb="00C1A2EB"/>
+        <bgColor rgb="00C1A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2EB"/>
-        <bgColor rgb="00EBA2EB"/>
+        <fgColor rgb="00D8A2EB"/>
+        <bgColor rgb="00D8A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D3"/>
-        <bgColor rgb="00EBA2D3"/>
+        <fgColor rgb="00EBA2E7"/>
+        <bgColor rgb="00EBA2E7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2BA"/>
-        <bgColor rgb="00EBA2BA"/>
+        <fgColor rgb="00EBA2D0"/>
+        <bgColor rgb="00EBA2D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B9"/>
+        <bgColor rgb="00EBA2B9"/>
       </patternFill>
     </fill>
   </fills>
@@ -189,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -258,6 +264,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -644,7 +653,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_18, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_19, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -785,82 +794,89 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  19. NPL_19 - TAAN (Trekking Agencies' Association of Nepal), president (unnamed), Pokhara; also Ethical Trekking founder. Coded from full verbatim transcript. Tourism/trekking sector focus.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_18, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_19, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_18) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_19) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
-    </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2047,7 +2063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ19"/>
+  <dimension ref="A1:CQ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11210,6 +11226,483 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>civil_society</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O20" s="24" t="inlineStr">
+        <is>
+          <t>environment and ecological systems (plastic harms "all living and non-living beings"; trails and mountains above 3,000 m littered), wildlife (animals eat plastic), health (side effects from plastic and from burning it), tourism and national image ("bad impression of the image of the whole country"; trash undermines visitors coming to see natural resources and mountains), Pokhara Lakeside garbage management failures, and air pollution from open burning of plastic waste</t>
+        </is>
+      </c>
+      <c r="P20" s="24" t="inlineStr">
+        <is>
+          <t>wildlife and mountain ecosystems; Nepal's tourism reputation and natural-resource image; communities and porters/guides (off-season unemployment; trails as workplace); the public affected by health impacts of plastic and burning; and Pokhara Lakeside residents/visitors facing inadequate garbage disposal options</t>
+        </is>
+      </c>
+      <c r="Q20" s="24" t="inlineStr">
+        <is>
+          <t>domestic tourists who "throw plastics out of the bus"; plastic producers/factories (especially plastic-bag factories the interviewee says should be closed); junk-food/noodle/beer-bottle consumption on treks; the national government (policies exist but are not implemented, current act is old, no fines for plastic bags, lack of monitoring and willingness to enforce); people who burn plastic waste; and new road access making checkpoint/deposit enforcement harder in restricted areas (Upper Mustang, Manaslu)</t>
+        </is>
+      </c>
+      <c r="R20" s="24" t="inlineStr">
+        <is>
+          <t>TAAN and tourism entrepreneurs (minimize plastic use, train guides/porters, collect trash above 3,000 m); Ethical Trekking (eco-friendly trekking model); ACAP and local governments as partners; guides and porters in proposed paid "clean campaigns"; mother groups and youth clubs (weekly cleanups); schools banning junk food/noodles; Nepal Army and NTNC; Pokhara municipality recycling-factory plans; Tourism Minister lake-cleaning campaign; and traditional alternatives (Gurung Bhangra bags, leaf plates, dal bhat, metal bottles)</t>
+        </is>
+      </c>
+      <c r="S20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AC20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AD20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AQ20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AX20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA20" s="24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BB20" s="24" t="inlineStr">
+        <is>
+          <t>As TAAN president (and Ethical Trekking operator), the interviewee runs guide/porter training programmes (~150 students), discourages trekker plastic-bottle use, coordinates with ACAP and local governments on trail cleanups, and launched association-wide campaigns (e.g. Pokhara lake cleaning with the Tourism Minister) — but cannot enforce national plastic policy, close plastic factories, fund off-season clean campaigns without external support, or control domestic-tourism littering nationwide.</t>
+        </is>
+      </c>
+      <c r="BC20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI20" s="24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BP20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BS20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW20" s="24" t="inlineStr">
+        <is>
+          <t>"We have policies, but they are not implemented properly"; Upper Mustang/Manaslu garbage-listing and deposit system exists but "implementation is not easy" (especially with new roads); black plastics banned but plastic factories remain; "lack of monitoring and a lack of willingness to implement policies"; "currently, there are no fines in Nepal for using plastic bags, only monthly fees for trash collection"; "if the law were strictly implemented, it could be cured."</t>
+        </is>
+      </c>
+      <c r="BX20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI20" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CN20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO20" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP20" s="24" t="inlineStr">
+        <is>
+          <t>Gurung Bhangra woven bags for carrying goods; leaf plates and mud cups; copper plates at home; promoting dal bhat (local vegetables/lentils, no plastic packaging) over noodles/spaghetti in plastic; metal bottles and treated/filtered water instead of plastic bottles.</t>
+        </is>
+      </c>
+      <c r="CQ20" s="24" t="inlineStr">
+        <is>
+          <t>Master list label: "19. TAAN Trekking Association", affiliation: Trekking Agencies' Association of Nepal (TAAN), Pokhara. Interviewee name not given; respondent is TAAN president (first elected without contest; former treasurer/vice president) and founder/operator of Ethical Trekking. Also founded a self-sustaining NGO/orphanage (closed 2019) — background narrative included in transcript but plastic-governance coding focuses on TAAN/tourism role. Interviewers: PEGO team. Interview date not stated. Coded from full verbatim transcript. ~180 trekking companies in Pokhara; TAAN established 42 years ago. Partners mentioned: ACAP, NTNC, Nepal Army, Tourism Minister. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11221,7 +11714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1418"/>
+  <dimension ref="A1:E1500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -49517,6 +50010,2220 @@
         </is>
       </c>
     </row>
+    <row r="1419">
+      <c r="A1419" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1419" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1419" s="24" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1419" s="24" t="inlineStr">
+        <is>
+          <t>civil_society</t>
+        </is>
+      </c>
+      <c r="E1419" s="24" t="inlineStr">
+        <is>
+          <t>Respondent is president of TAAN (Trekking Agencies' Association of Nepal), an industry association representing trekking agencies — coded as civil_society.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1420" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1420" s="24" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1420" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1420" s="24" t="inlineStr">
+        <is>
+          <t>Domestic tourists "throw plastics out of the bus"; people "don't have a culture of carrying shopping bags yet"; nationwide school campaigns needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1421" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1421" s="24" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D1421" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1421" s="24" t="inlineStr">
+        <is>
+          <t>"We have policies, but they are not implemented properly"; current act "quite old"; lack of monitoring and willingness to implement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1422" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1422" s="24" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1422" s="24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1422" s="24" t="inlineStr">
+        <is>
+          <t>"As the president of TAAN, it really pains me to see trash and plastic everywhere"; TAAN and trekking companies "very aware" of plastic issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1423" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1423" s="24" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1423" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1423" s="24" t="inlineStr">
+        <is>
+          <t>Trash and plastic "everywhere" on trails and nationally; Pokhara Lakeside garbage problems; difficulty bringing all trail waste back down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1424" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1424" s="24" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1424" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1424" s="24" t="inlineStr">
+        <is>
+          <t>Junk food, noodles, beer bottles and plastic bottles described as "a massive problem" on treks; domestic tourism consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1425" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1425" s="24" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1425" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1425" s="24" t="inlineStr">
+        <is>
+          <t>TAAN works to promote recycling; Pokhara municipality planning recycling factories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1426" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1426" s="24" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1426" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1426" s="24" t="inlineStr">
+        <is>
+          <t>Pokhara Lakeside — "nowhere to throw" garbage sometimes; villages bury or burn waste; trails above 3,000 m hard to manage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1427" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1427" s="24" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1427" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1427" s="24" t="inlineStr">
+        <is>
+          <t>"Close the factories that make plastic bags"; government should "totally ban plastic factories."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1428" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1428" s="24" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1428" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1428" s="24" t="inlineStr">
+        <is>
+          <t>Discourage plastic bottles; filters/tablets for local water; metal bottles; traditional woven bags and leaf plates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1429" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1429" s="24" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1429" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1429" s="24" t="inlineStr">
+        <is>
+          <t>Need deposit/separation places with sheds so trash "doesn't fly away."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1430" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1430" s="24" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1430" s="24" t="inlineStr">
+        <is>
+          <t>environment and ecological systems (plastic harms "all living and non-living beings"; trails and mountains above 3,000 m littered), wildlife (animals eat plastic), health (side effects from plastic and from burning it), tourism and national image ("bad impression of the image of the whole country"; trash undermines visitors coming to see natural resources and mountains), Pokhara Lakeside garbage management failures, and air pollution from open burning of plastic waste</t>
+        </is>
+      </c>
+      <c r="E1430" s="24" t="inlineStr">
+        <is>
+          <t>Environment, wildlife, health, burning, tourism/national image, Pokhara Lakeside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1431" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1431" s="24" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1431" s="24" t="inlineStr">
+        <is>
+          <t>wildlife and mountain ecosystems; Nepal's tourism reputation and natural-resource image; communities and porters/guides (off-season unemployment; trails as workplace); the public affected by health impacts of plastic and burning; and Pokhara Lakeside residents/visitors facing inadequate garbage disposal options</t>
+        </is>
+      </c>
+      <c r="E1431" s="24" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: wildlife; mountain ecosystems; tourism/national image; porters/guides; public health. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1432" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1432" s="24" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1432" s="24" t="inlineStr">
+        <is>
+          <t>domestic tourists who "throw plastics out of the bus"; plastic producers/factories (especially plastic-bag factories the interviewee says should be closed); junk-food/noodle/beer-bottle consumption on treks; the national government (policies exist but are not implemented, current act is old, no fines for plastic bags, lack of monitoring and willingness to enforce); people who burn plastic waste; and new road access making checkpoint/deposit enforcement harder in restricted areas (Upper Mustang, Manaslu)</t>
+        </is>
+      </c>
+      <c r="E1432" s="24" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: domestic litterers; plastic factories; weak government enforcement; junk-food consumption; road access undermining checkpoints. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1433" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1433" s="24" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1433" s="24" t="inlineStr">
+        <is>
+          <t>TAAN and tourism entrepreneurs (minimize plastic use, train guides/porters, collect trash above 3,000 m); Ethical Trekking (eco-friendly trekking model); ACAP and local governments as partners; guides and porters in proposed paid "clean campaigns"; mother groups and youth clubs (weekly cleanups); schools banning junk food/noodles; Nepal Army and NTNC; Pokhara municipality recycling-factory plans; Tourism Minister lake-cleaning campaign; and traditional alternatives (Gurung Bhangra bags, leaf plates, dal bhat, metal bottles)</t>
+        </is>
+      </c>
+      <c r="E1433" s="24" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: TAAN, Ethical Trekking, tourism sector, ACAP, local government, guides/porters, schools, traditional alternatives. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1434" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1434" s="24" t="inlineStr">
+        <is>
+          <t>Relevance_international_pol</t>
+        </is>
+      </c>
+      <c r="D1434" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1434" s="24" t="inlineStr">
+        <is>
+          <t>International trekking promotion (Europe); research needed to affect government policy; tourism-dependent economy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1435" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1435" s="24" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D1435" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1435" s="24" t="inlineStr">
+        <is>
+          <t>TAAN works with stakeholders, local governments, ACAP, Nepal Army, NTNC, Tourism Minister, mother groups and youth clubs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1436" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1436" s="24" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D1436" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1436" s="24" t="inlineStr">
+        <is>
+          <t>National policies vs local implementation gaps; checkpoint deposit systems in restricted areas vs municipal collection in Pokhara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1437" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1437" s="24" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1437" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1437" s="24" t="inlineStr">
+        <is>
+          <t>Government should be strict but lacks monitoring/willingness; "encourage the government to do its job now."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1438" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1438" s="24" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1438" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1438" s="24" t="inlineStr">
+        <is>
+          <t>Policies, bans, fines, factory regulation, strict implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1439" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1439" s="24" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1439" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1439" s="24" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1440" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1440" s="24" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1440" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1440" s="24" t="inlineStr">
+        <is>
+          <t>Local governments trying "their best"; reward minimisers; recycling factory plans in Pokhara; black-plastic prohibitions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1441" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1441" s="24" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1441" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1441" s="24" t="inlineStr">
+        <is>
+          <t>NA - students targeted via schools but not named as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1442" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1442" s="24" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1442" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1442" s="24" t="inlineStr">
+        <is>
+          <t>Trekking agencies, guides and porters responsible for trail trash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1443" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1443" s="24" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1443" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1443" s="24" t="inlineStr">
+        <is>
+          <t>TAAN, mother groups, youth clubs running cleanups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1444" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1444" s="24" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1444" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1444" s="24" t="inlineStr">
+        <is>
+          <t>Research needed "to affect government policy."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1445" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1445" s="24" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1445" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1445" s="24" t="inlineStr">
+        <is>
+          <t>Public should carry own bags and reduce plastic consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1446" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1446" s="24" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1446" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1446" s="24" t="inlineStr">
+        <is>
+          <t>Schools banning junk food; nationwide school campaigns proposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1447" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1447" s="24" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1447" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1447" s="24" t="inlineStr">
+        <is>
+          <t>Plastic-bag factories; trekking/tourism companies under TAAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1448" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1448" s="24" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1448" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1448" s="24" t="inlineStr">
+        <is>
+          <t>Policies not implemented; old act; no bag fines; weak monitoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1449" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1449" s="24" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1449" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1449" s="24" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1450" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1450" s="24" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1450" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1450" s="24" t="inlineStr">
+        <is>
+          <t>NA - local government portrayed as trying and planning recycling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1451" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1451" s="24" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1451" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1451" s="24" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1452" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1452" s="24" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1452" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1452" s="24" t="inlineStr">
+        <is>
+          <t>NA - trekking sector portrayed as relatively conscious; TAAN leads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1453" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1453" s="24" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1453" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1453" s="24" t="inlineStr">
+        <is>
+          <t>NA - CSOs portrayed as heroes (cleanups).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1454" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1454" s="24" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1454" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1454" s="24" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1455" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1455" s="24" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1455" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1455" s="24" t="inlineStr">
+        <is>
+          <t>Domestic tourism littering; no shopping-bag culture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1456" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1456" s="24" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1456" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1456" s="24" t="inlineStr">
+        <is>
+          <t>NA - schools portrayed positively (junk-food bans).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1457" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1457" s="24" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1457" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1457" s="24" t="inlineStr">
+        <is>
+          <t>Plastic-bag factories should be closed; junk-food packaging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1458" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1458" s="24" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1458" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1458" s="24" t="inlineStr">
+        <is>
+          <t>Strict implementation, updated legislation, factory bans, fines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1459" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1459" s="24" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1459" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1459" s="24" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1460" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1460" s="24" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1460" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1460" s="24" t="inlineStr">
+        <is>
+          <t>Rewards for minimisers; garbage management (Pokhara); recycling infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1461" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1461" s="24" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1461" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1461" s="24" t="inlineStr">
+        <is>
+          <t>Nationwide school campaigns; schools already banning junk food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1462" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1462" s="24" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1462" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1462" s="24" t="inlineStr">
+        <is>
+          <t>Guides/porters training and paid off-season clean campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1463" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1463" s="24" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1463" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1463" s="24" t="inlineStr">
+        <is>
+          <t>NA - CSOs already active; not primary target framing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1464" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1464" s="24" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1464" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1464" s="24" t="inlineStr">
+        <is>
+          <t>Research to inform government policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1465" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1465" s="24" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1465" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1465" s="24" t="inlineStr">
+        <is>
+          <t>Reduce plastic consumption; adopt reusable bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1466" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1466" s="24" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1466" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1466" s="24" t="inlineStr">
+        <is>
+          <t>School campaigns and junk-food bans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1467" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1467" s="24" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1467" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1467" s="24" t="inlineStr">
+        <is>
+          <t>Trekking agencies and plastic producers/factories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1468" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1468" s="24" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1468" s="24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1468" s="24" t="inlineStr">
+        <is>
+          <t>TAAN president organising training (~150 guide/porter students), campaigns, stakeholder coordination and policy advocacy — managerial/organisational implementer (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1469" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1469" s="24" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1469" s="24" t="inlineStr">
+        <is>
+          <t>As TAAN president (and Ethical Trekking operator), the interviewee runs guide/porter training programmes (~150 students), discourages trekker plastic-bottle use, coordinates with ACAP and local governments on trail cleanups, and launched association-wide campaigns (e.g. Pokhara lake cleaning with the Tourism Minister) — but cannot enforce national plastic policy, close plastic factories, fund off-season clean campaigns without external support, or control domestic-tourism littering nationwide.</t>
+        </is>
+      </c>
+      <c r="E1469" s="24" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1470" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1470" s="24" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1470" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1470" s="24" t="inlineStr">
+        <is>
+          <t>Lack of monitoring cited; checkpoint deposit system hard to enforce with roads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1471" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1471" s="24" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D1471" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1471" s="24" t="inlineStr">
+        <is>
+          <t>Off-season porters need paid clean-campaign funding; economic support for remote mountain areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1472" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1472" s="24" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D1472" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1472" s="24" t="inlineStr">
+        <is>
+          <t>"We need research like yours to affect government policy."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1473" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1473" s="24" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1473" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1473" s="24" t="inlineStr">
+        <is>
+          <t>Deposit/separation sheds; Pokhara twice-weekly collection vs village bury/burn; planned recycling factory land.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1474" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1474" s="24" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1474" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1474" s="24" t="inlineStr">
+        <is>
+          <t>Train guides/porters but need jobs in off-season to prevent migration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1475" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1475" s="24" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1475" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1475" s="24" t="inlineStr">
+        <is>
+          <t>Deposit/checkpoint policy in Mustang/Manaslu; proposed fines and strict law implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1476" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1476" s="24" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D1476" s="24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1476" s="24" t="inlineStr">
+        <is>
+          <t>Extended producer responsibility not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1477" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1477" s="24" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1477" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1477" s="24" t="inlineStr">
+        <is>
+          <t>Lake-cleaning campaign with Tourism Minister; TAAN promotion campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1478" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1478" s="24" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D1478" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1478" s="24" t="inlineStr">
+        <is>
+          <t>Guide/porter training for ~150 students on trash responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1479" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1479" s="24" t="inlineStr">
+        <is>
+          <t>Pol_tax</t>
+        </is>
+      </c>
+      <c r="D1479" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1479" s="24" t="inlineStr">
+        <is>
+          <t>Monthly trash-collection fees in Pokhara (no fines for plastic bags).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1480" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1480" s="24" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1480" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1480" s="24" t="inlineStr">
+        <is>
+          <t>Black plastics prohibited/banned; proposes total plastic-factory ban; some schools ban junk food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1481" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1481" s="24" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1481" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1481" s="24" t="inlineStr">
+        <is>
+          <t>Water filters/tablets, metal bottles, traditional bags and leaf plates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1482" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1482" s="24" t="inlineStr">
+        <is>
+          <t>Pol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1482" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1482" s="24" t="inlineStr">
+        <is>
+          <t>Lake cleanup; weekly mother-group/youth-club cleanups; collect trash above 3,000 m; proposed paid clean campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1483" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1483" s="24" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1483" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1483" s="24" t="inlineStr">
+        <is>
+          <t>TAAN promotes recycling; Pokhara municipality recycling-factory plans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1484" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1484" s="24" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1484" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1484" s="24" t="inlineStr">
+        <is>
+          <t>Pokhara trucks twice weekly; Mustang/Manaslu garbage listing and deposit at checkpoints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1485" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1485" s="24" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1485" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1485" s="24" t="inlineStr">
+        <is>
+          <t>Policies exist but poorly implemented/monitored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1486" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1486" s="24" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1486" s="24" t="inlineStr">
+        <is>
+          <t>"We have policies, but they are not implemented properly"; Upper Mustang/Manaslu garbage-listing and deposit system exists but "implementation is not easy" (especially with new roads); black plastics banned but plastic factories remain; "lack of monitoring and a lack of willingness to implement policies"; "currently, there are no fines in Nepal for using plastic bags, only monthly fees for trash collection"; "if the law were strictly implemented, it could be cured."</t>
+        </is>
+      </c>
+      <c r="E1486" s="24" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1487" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1487" s="24" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1487" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1487" s="24" t="inlineStr">
+        <is>
+          <t>Strict government implementation; TAAN/stakeholder coordination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1488" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1488" s="24" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1488" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1488" s="24" t="inlineStr">
+        <is>
+          <t>Government strictness; municipalities accountable for garbage management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1489" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1489" s="24" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1489" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1489" s="24" t="inlineStr">
+        <is>
+          <t>More campaigns nationwide, especially schools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1490" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1490" s="24" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1490" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1490" s="24" t="inlineStr">
+        <is>
+          <t>Deposit places with sheds for separated trash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1491" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1491" s="24" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1491" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1491" s="24" t="inlineStr">
+        <is>
+          <t>Pokhara recycling factories; promote recycling via TAAN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1492" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1492" s="24" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1492" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1492" s="24" t="inlineStr">
+        <is>
+          <t>School campaigns; guide/porter training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1493" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1493" s="24" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1493" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1493" s="24" t="inlineStr">
+        <is>
+          <t>Train and employ porters/guides in off-season clean campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1494" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1494" s="24" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1494" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1494" s="24" t="inlineStr">
+        <is>
+          <t>Economic support/funding for remote-area clean campaigns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1495" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1495" s="24" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1495" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1495" s="24" t="inlineStr">
+        <is>
+          <t>Segregation deposit sheds; municipal recycling facilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1496" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1496" s="24" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1496" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1496" s="24" t="inlineStr">
+        <is>
+          <t>Metal bottles, filters, Gurung Bhangra, leaf plates, dal bhat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1497" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1497" s="24" t="inlineStr">
+        <is>
+          <t>Sol_clean_up</t>
+        </is>
+      </c>
+      <c r="D1497" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1497" s="24" t="inlineStr">
+        <is>
+          <t>Paid off-season trail clean campaigns; lake and weekly community cleanups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1498" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1498" s="24" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1498" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1498" s="24" t="inlineStr">
+        <is>
+          <t>Strict law implementation; fines; checkpoint deposit system enforced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1499" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1499" s="24" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1499" s="24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1499" s="24" t="inlineStr">
+        <is>
+          <t>Better monitoring and willingness to implement existing policies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" s="24" t="inlineStr">
+        <is>
+          <t>NPL_19</t>
+        </is>
+      </c>
+      <c r="B1500" s="24" t="inlineStr">
+        <is>
+          <t>TAAN (Trekking Agencies' Association of Nepal) - President (unnamed), Pokhara; also founder of Ethical Trekking (interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1500" s="24" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1500" s="24" t="inlineStr">
+        <is>
+          <t>Gurung Bhangra woven bags for carrying goods; leaf plates and mud cups; copper plates at home; promoting dal bhat (local vegetables/lentils, no plastic packaging) over noodles/spaghetti in plastic; metal bottles and treated/filtered water instead of plastic bottles.</t>
+        </is>
+      </c>
+      <c r="E1500" s="24" t="inlineStr">
+        <is>
+          <t>Gurung Bhangra, leaf plates, mud/copper vessels, dal bhat over packaged noodles.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_20 coding for municipality Environment Officer (Chitwan area)
Code integrated guideline notes and verbatim transcript for the small
Chitwan-area municipal Environment Officer interview (Safa Urja contractor,
visual pollution, cloth-bag campaigns, inter-municipal PPP landfill planning).
Updates workbook to NPL_1 through NPL_20.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -62,110 +62,116 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB9A2"/>
-        <bgColor rgb="00EBB9A2"/>
+        <fgColor rgb="00EBB8A2"/>
+        <bgColor rgb="00EBB8A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD0A2"/>
-        <bgColor rgb="00EBD0A2"/>
+        <fgColor rgb="00EBCEA2"/>
+        <bgColor rgb="00EBCEA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE7A2"/>
-        <bgColor rgb="00EBE7A2"/>
+        <fgColor rgb="00EBE4A2"/>
+        <bgColor rgb="00EBE4A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D8EBA2"/>
-        <bgColor rgb="00D8EBA2"/>
+        <fgColor rgb="00DCEBA2"/>
+        <bgColor rgb="00DCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C1EBA2"/>
-        <bgColor rgb="00C1EBA2"/>
+        <fgColor rgb="00C6EBA2"/>
+        <bgColor rgb="00C6EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00AAEBA2"/>
-        <bgColor rgb="00AAEBA2"/>
+        <fgColor rgb="00B1EBA2"/>
+        <bgColor rgb="00B1EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBB1"/>
-        <bgColor rgb="00A2EBB1"/>
+        <fgColor rgb="00A2EBA9"/>
+        <bgColor rgb="00A2EBA9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBC8"/>
-        <bgColor rgb="00A2EBC8"/>
+        <fgColor rgb="00A2EBBF"/>
+        <bgColor rgb="00A2EBBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBDF"/>
-        <bgColor rgb="00A2EBDF"/>
+        <fgColor rgb="00A2EBD5"/>
+        <bgColor rgb="00A2EBD5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2DFEB"/>
-        <bgColor rgb="00A2DFEB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2C8EB"/>
-        <bgColor rgb="00A2C8EB"/>
+        <fgColor rgb="00A2D5EB"/>
+        <bgColor rgb="00A2D5EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2B1EB"/>
-        <bgColor rgb="00A2B1EB"/>
+        <fgColor rgb="00A2BFEB"/>
+        <bgColor rgb="00A2BFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00AAA2EB"/>
-        <bgColor rgb="00AAA2EB"/>
+        <fgColor rgb="00A2A9EB"/>
+        <bgColor rgb="00A2A9EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C1A2EB"/>
-        <bgColor rgb="00C1A2EB"/>
+        <fgColor rgb="00B1A2EB"/>
+        <bgColor rgb="00B1A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D8A2EB"/>
-        <bgColor rgb="00D8A2EB"/>
+        <fgColor rgb="00C6A2EB"/>
+        <bgColor rgb="00C6A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E7"/>
-        <bgColor rgb="00EBA2E7"/>
+        <fgColor rgb="00DCA2EB"/>
+        <bgColor rgb="00DCA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D0"/>
-        <bgColor rgb="00EBA2D0"/>
+        <fgColor rgb="00EBA2E4"/>
+        <bgColor rgb="00EBA2E4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B9"/>
-        <bgColor rgb="00EBA2B9"/>
+        <fgColor rgb="00EBA2CE"/>
+        <bgColor rgb="00EBA2CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B8"/>
+        <bgColor rgb="00EBA2B8"/>
       </patternFill>
     </fill>
   </fills>
@@ -195,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -267,6 +273,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -634,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -653,7 +662,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_19, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_20, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -801,82 +810,89 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  20. NPL_20 - Municipality Environment Officer (unnamed), small Chitwan-area municipality. Coded from integrated guideline notes and verbatim transcript (Marlene Kammerer/Ram Devi/Deep). Safa Urja contractor; overlap with NPL_11.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_19, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_20, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_19) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_20) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-    </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2063,7 +2079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ20"/>
+  <dimension ref="A1:CQ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11703,6 +11719,483 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" s="25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O21" s="25" t="inlineStr">
+        <is>
+          <t>visual/aesthetic pollution (scattered noodle/chips/gutka packets — "the most obvious effect"; reduces aesthetics for residents and tourism), environment (non-biodegradable plastics persist in soil/farmlands; sub-40-micron and black plastics visible in farmlands), and air/climate (burning plastics releases gases contributing to global warming — limited locally; only 1–2 burning complaints this year)</t>
+        </is>
+      </c>
+      <c r="P21" s="25" t="inlineStr">
+        <is>
+          <t>residents and local communities who want a clean environment; tourism/aesthetic appeal of the municipality; farmlands/soil where small plastic packets persist; and the broader environment affected by non-biodegradable litter</t>
+        </is>
+      </c>
+      <c r="Q21" s="25" t="inlineStr">
+        <is>
+          <t>the public/households (inconsistent use of dustbins; littering despite bins; moderate but incomplete awareness); weak and flexible national/local laws with infrequent enforcement; plastic producers of banned sub-40-micron and black plastics (ban incomplete); and infrastructure/land gaps that leave municipalities dependent on private contractors dumping residual waste at riverbanks</t>
+        </is>
+      </c>
+      <c r="R21" s="25" t="inlineStr">
+        <is>
+          <t>the municipality (cloth-bag distribution, reduce/reuse/recycle campaigns, dustbins, penalties under Natural Resource Protection Act, Environment &amp; Disaster budget); Safa Urja Utpadan (contracted collection, partial segregation, recycling facilities and own land); proposed inter-municipal integrated landfill/PPP (Ratnanagar, Kalika, Khaireni, Rapti); and promoted alternatives (cloth/fiber bags, 3R/4R principles, shredders/green roads)</t>
+        </is>
+      </c>
+      <c r="S21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AB21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AV21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA21" s="25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BB21" s="25" t="inlineStr">
+        <is>
+          <t>As a municipal Environment Officer, the interviewee oversees waste/plastic management operations, distributes cloth bags, runs awareness campaigns, allocates budget under Environment &amp; Disaster, and contracts Safa Urja for collection — but is not involved in drafting the national Solid Waste Management bill, cannot acquire municipal landfill land, and relies on the private contractor for most collection, segregation and recycling.</t>
+        </is>
+      </c>
+      <c r="BC21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BE21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BF21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI21" s="25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="BJ21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BR21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW21" s="25" t="inlineStr">
+        <is>
+          <t>40-micron and black-plastic production bans exist but "enforcement is incomplete" and bans are "only partially effective"; dustbins placed "at every corner" but littering continues; penalties under Natural Resource Protection Act exist but laws are "weak and flexible" with infrequent enforcement; Solid Waste Management bill recently sent to Council of Ministers but officer not involved in drafting — overall guidance exists but "enforcement and awareness remain weak."</t>
+        </is>
+      </c>
+      <c r="BX21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BZ21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CG21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CK21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO21" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CP21" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CQ21" s="25" t="inlineStr">
+        <is>
+          <t>Master list label: "20. Municipality Environment Officer (Chitwan area)", affiliation: local government — Environment Officer (small municipality). Interviewee name not given. Municipality described as small (one hospital, one cinema hall, few restaurants). Location/context: Chitwan area — Safa Urja Utpadan contracted for collection; neighbouring municipalities Ratnanagar, Kalika, Khaireni and Rapti discussed for integrated landfill/PPP. Interviewers: Marlene Kammerer (University of Bern), Ram Devi, Deep. Interview date not stated. Coded from integrated structured guideline notes and full verbatim transcript (with interpreter Deep). Overlap with NPL_11 (Safa Urja Utpadan — same contractor, same area) but distinct municipal-government perspective. Q4a/Q4b ministry follow-ups blank. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11714,7 +12207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1500"/>
+  <dimension ref="A1:E1578"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -52224,6 +52717,2112 @@
         </is>
       </c>
     </row>
+    <row r="1501">
+      <c r="A1501" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1501" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1501" s="25" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1501" s="25" t="inlineStr">
+        <is>
+          <t>loc_government</t>
+        </is>
+      </c>
+      <c r="E1501" s="25" t="inlineStr">
+        <is>
+          <t>Municipal Environment Officer in a small Chitwan-area municipality — coded as loc_government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1502" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1502" s="25" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1502" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1502" s="25" t="inlineStr">
+        <is>
+          <t>"Public unawareness of proper disposal methods"; dustbins provided but littering continues; "whether their awareness level has not reached that point."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1503" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1503" s="25" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pol</t>
+        </is>
+      </c>
+      <c r="D1503" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1503" s="25" t="inlineStr">
+        <is>
+          <t>"Weak enforcement; laws are broad and flexible"; "guidance exists but enforcement and awareness remain weak"; officer not involved in drafting national SWM bill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1504" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1504" s="25" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1504" s="25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1504" s="25" t="inlineStr">
+        <is>
+          <t>"Officer is very concerned"; "Concerned very much"; municipality launching campaigns and distributing cloth bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1505" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1505" s="25" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1505" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1505" s="25" t="inlineStr">
+        <is>
+          <t>Visual pollution from scattered noodle/chips/gutka packets; dustbins at corners but people still litter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1506" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1506" s="25" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1506" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1506" s="25" t="inlineStr">
+        <is>
+          <t>Small single-use packets (noodles, chips, Kurkure) with no reuse value persist in environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1507" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1507" s="25" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1507" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1507" s="25" t="inlineStr">
+        <is>
+          <t>Private contractor recycles most waste but technology gaps (shredders, advanced processing) remain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1508" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1508" s="25" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1508" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1508" s="25" t="inlineStr">
+        <is>
+          <t>No municipal engineered landfill; municipality relies on private sector; residual waste dumped at riverbank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1509" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1509" s="25" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1509" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1509" s="25" t="inlineStr">
+        <is>
+          <t>Production of plastics below 40 microns and black plastics banned but "enforcement is incomplete."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1510" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1510" s="25" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1510" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1510" s="25" t="inlineStr">
+        <is>
+          <t>"Lack of proper alternatives for banned plastics"; promotes cloth bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1511" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1511" s="25" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1511" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1511" s="25" t="inlineStr">
+        <is>
+          <t>Safa Urja performs partial segregation with own machine; municipality does not segregate directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1512" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1512" s="25" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1512" s="25" t="inlineStr">
+        <is>
+          <t>visual/aesthetic pollution (scattered noodle/chips/gutka packets — "the most obvious effect"; reduces aesthetics for residents and tourism), environment (non-biodegradable plastics persist in soil/farmlands; sub-40-micron and black plastics visible in farmlands), and air/climate (burning plastics releases gases contributing to global warming — limited locally; only 1–2 burning complaints this year)</t>
+        </is>
+      </c>
+      <c r="E1512" s="25" t="inlineStr">
+        <is>
+          <t>Visual/aesthetic pollution; farmlands; environment; limited burning/global warming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1513" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1513" s="25" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1513" s="25" t="inlineStr">
+        <is>
+          <t>residents and local communities who want a clean environment; tourism/aesthetic appeal of the municipality; farmlands/soil where small plastic packets persist; and the broader environment affected by non-biodegradable litter</t>
+        </is>
+      </c>
+      <c r="E1513" s="25" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: residents; tourists; farmlands/environment. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1514" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1514" s="25" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1514" s="25" t="inlineStr">
+        <is>
+          <t>the public/households (inconsistent use of dustbins; littering despite bins; moderate but incomplete awareness); weak and flexible national/local laws with infrequent enforcement; plastic producers of banned sub-40-micron and black plastics (ban incomplete); and infrastructure/land gaps that leave municipalities dependent on private contractors dumping residual waste at riverbanks</t>
+        </is>
+      </c>
+      <c r="E1514" s="25" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: public littering; weak enforcement; banned plastic production; land/infrastructure gaps. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1515" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1515" s="25" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1515" s="25" t="inlineStr">
+        <is>
+          <t>the municipality (cloth-bag distribution, reduce/reuse/recycle campaigns, dustbins, penalties under Natural Resource Protection Act, Environment &amp; Disaster budget); Safa Urja Utpadan (contracted collection, partial segregation, recycling facilities and own land); proposed inter-municipal integrated landfill/PPP (Ratnanagar, Kalika, Khaireni, Rapti); and promoted alternatives (cloth/fiber bags, 3R/4R principles, shredders/green roads)</t>
+        </is>
+      </c>
+      <c r="E1515" s="25" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: municipality; Safa Urja; cloth-bag/campaign measures; planned inter-municipal PPP landfill. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1516" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1516" s="25" t="inlineStr">
+        <is>
+          <t>Coordination_sectoral</t>
+        </is>
+      </c>
+      <c r="D1516" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1516" s="25" t="inlineStr">
+        <is>
+          <t>Municipality contracts Safa Urja; NGOs/private sector mentioned as shared responsibility; hospitals/businesses targeted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1517" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1517" s="25" t="inlineStr">
+        <is>
+          <t>Coordination_levels</t>
+        </is>
+      </c>
+      <c r="D1517" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1517" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up: challenges differ — local operational/resource gaps vs federal policy clarity/coordination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1518" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1518" s="25" t="inlineStr">
+        <is>
+          <t>Unclear_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1518" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1518" s="25" t="inlineStr">
+        <is>
+          <t>Responsibility shared among municipality, government and private sector/NGOs; national bill drafting not involving this officer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1519" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1519" s="25" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1519" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1519" s="25" t="inlineStr">
+        <is>
+          <t>40-micron/black-plastic bans; Solid Waste Management bill; Natural Resource Protection Act penalties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1520" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1520" s="25" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1520" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1520" s="25" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1521" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1521" s="25" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1521" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1521" s="25" t="inlineStr">
+        <is>
+          <t>Municipality oversees operations, dustbins, budget, campaigns, enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1522" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1522" s="25" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1522" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1522" s="25" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1523" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1523" s="25" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1523" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1523" s="25" t="inlineStr">
+        <is>
+          <t>Safa Urja contracted for collection, partial segregation, recycling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1524" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1524" s="25" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1524" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1524" s="25" t="inlineStr">
+        <is>
+          <t>NA - NGOs mentioned generally but not as formal responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1525" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1525" s="25" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1525" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1525" s="25" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1526" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1526" s="25" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1526" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1526" s="25" t="inlineStr">
+        <is>
+          <t>Households must use dustbins and cloth bags; compliance varies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1527" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1527" s="25" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1527" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1527" s="25" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1528" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1528" s="25" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1528" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1528" s="25" t="inlineStr">
+        <is>
+          <t>Safa Urja and small businesses/restaurants/hospital.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1529" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1529" s="25" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1529" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1529" s="25" t="inlineStr">
+        <is>
+          <t>Weak/flexible laws; incomplete ban enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1530" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1530" s="25" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1530" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1530" s="25" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1531" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1531" s="25" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1531" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1531" s="25" t="inlineStr">
+        <is>
+          <t>NA - municipality portrayed as active implementer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1532" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1532" s="25" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1532" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1532" s="25" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1533" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1533" s="25" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1533" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1533" s="25" t="inlineStr">
+        <is>
+          <t>NA - Safa Urja portrayed as central solution partner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1534" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1534" s="25" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1534" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1534" s="25" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1535" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1535" s="25" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1535" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1535" s="25" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1536" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1536" s="25" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1536" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1536" s="25" t="inlineStr">
+        <is>
+          <t>Inconsistent dustbin use; littering; moderate awareness gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1537" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1537" s="25" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1537" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1537" s="25" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1538" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1538" s="25" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1538" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1538" s="25" t="inlineStr">
+        <is>
+          <t>NA - businesses targeted for policy, not primarily blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1539" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1539" s="25" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1539" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1539" s="25" t="inlineStr">
+        <is>
+          <t>Stronger laws and national policy clarity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1540" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1540" s="25" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1540" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1540" s="25" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1541" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1541" s="25" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1541" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1541" s="25" t="inlineStr">
+        <is>
+          <t>Municipal investment in infrastructure; integrated landfill planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1542" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1542" s="25" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1542" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1542" s="25" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1543" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1543" s="25" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1543" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1543" s="25" t="inlineStr">
+        <is>
+          <t>Safa Urja coordination; private sector central to collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1544" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1544" s="25" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1544" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1544" s="25" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1545" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1545" s="25" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1545" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1545" s="25" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1546" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1546" s="25" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1546" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1546" s="25" t="inlineStr">
+        <is>
+          <t>Primary target alongside small businesses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1547" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1547" s="25" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1547" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1547" s="25" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1548" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1548" s="25" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1548" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1548" s="25" t="inlineStr">
+        <is>
+          <t>Restaurants, cinema hall, hospital; autoclave disposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1549" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1549" s="25" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1549" s="25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E1549" s="25" t="inlineStr">
+        <is>
+          <t>Environment Officer managing municipal campaigns, contractor oversight and local implementation — managerial/organisational implementer (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1550" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1550" s="25" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1550" s="25" t="inlineStr">
+        <is>
+          <t>As a municipal Environment Officer, the interviewee oversees waste/plastic management operations, distributes cloth bags, runs awareness campaigns, allocates budget under Environment &amp; Disaster, and contracts Safa Urja for collection — but is not involved in drafting the national Solid Waste Management bill, cannot acquire municipal landfill land, and relies on the private contractor for most collection, segregation and recycling.</t>
+        </is>
+      </c>
+      <c r="E1550" s="25" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1551" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1551" s="25" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1551" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1551" s="25" t="inlineStr">
+        <is>
+          <t>Penalties for open dumping/burning; only 1–2 burning complaints this year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1552" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1552" s="25" t="inlineStr">
+        <is>
+          <t>Financial_resources</t>
+        </is>
+      </c>
+      <c r="D1552" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1552" s="25" t="inlineStr">
+        <is>
+          <t>Municipality budget under Environment &amp; Disaster; minimal direct investment; private sector pays municipality; land acquisition problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1553" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1553" s="25" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D1553" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1553" s="25" t="inlineStr">
+        <is>
+          <t>NA - not mentioned as active research actor (interview is part of research project).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1554" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1554" s="25" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1554" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1554" s="25" t="inlineStr">
+        <is>
+          <t>No municipal landfill; lack of shredders/transfer stations; private sector has land and MRF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1555" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1555" s="25" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1555" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1555" s="25" t="inlineStr">
+        <is>
+          <t>Municipality can formulate local policy but implementation depends on public compliance; technology gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1556" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1556" s="25" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1556" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1556" s="25" t="inlineStr">
+        <is>
+          <t>Penalties exist but infrequent; bans partially effective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1557" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1557" s="25" t="inlineStr">
+        <is>
+          <t>Pol_epr</t>
+        </is>
+      </c>
+      <c r="D1557" s="25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E1557" s="25" t="inlineStr">
+        <is>
+          <t>Extended producer responsibility not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1558" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1558" s="25" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1558" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1558" s="25" t="inlineStr">
+        <is>
+          <t>Municipality campaigns on reduction, reuse, recycling; cloth-bag distribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1559" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1559" s="25" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D1559" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1559" s="25" t="inlineStr">
+        <is>
+          <t>Public awareness campaigns alongside laws.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1560" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1560" s="25" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1560" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1560" s="25" t="inlineStr">
+        <is>
+          <t>Ban on production below 40 microns and black plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1561" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1561" s="25" t="inlineStr">
+        <is>
+          <t>Pol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1561" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1561" s="25" t="inlineStr">
+        <is>
+          <t>Cloth/fiber bags promoted and distributed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1562" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1562" s="25" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1562" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1562" s="25" t="inlineStr">
+        <is>
+          <t>Safa Urja recycling facilities; reuse of shredded plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1563" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1563" s="25" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1563" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1563" s="25" t="inlineStr">
+        <is>
+          <t>Municipality contracts Safa Urja for household collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1564" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1564" s="25" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1564" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1564" s="25" t="inlineStr">
+        <is>
+          <t>Bans and bins only partially effective; weak enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1565" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1565" s="25" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1565" s="25" t="inlineStr">
+        <is>
+          <t>40-micron and black-plastic production bans exist but "enforcement is incomplete" and bans are "only partially effective"; dustbins placed "at every corner" but littering continues; penalties under Natural Resource Protection Act exist but laws are "weak and flexible" with infrequent enforcement; Solid Waste Management bill recently sent to Council of Ministers but officer not involved in drafting — overall guidance exists but "enforcement and awareness remain weak."</t>
+        </is>
+      </c>
+      <c r="E1565" s="25" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1566" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1566" s="25" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1566" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1566" s="25" t="inlineStr">
+        <is>
+          <t>Inter-municipal integrated waste management/PPP landfill across neighbouring municipalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1567" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1567" s="25" t="inlineStr">
+        <is>
+          <t>Sol_responsibilities</t>
+        </is>
+      </c>
+      <c r="D1567" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1567" s="25" t="inlineStr">
+        <is>
+          <t>Clarify roles between municipality and private contractor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1568" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1568" s="25" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1568" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1568" s="25" t="inlineStr">
+        <is>
+          <t>Promote awareness alongside laws; 3R/4R principles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1569" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1569" s="25" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1569" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1569" s="25" t="inlineStr">
+        <is>
+          <t>Improve segregation via private-sector facilities and public compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1570" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1570" s="25" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1570" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1570" s="25" t="inlineStr">
+        <is>
+          <t>Shredders, recycling facilities, green roads, reuse of plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1571" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1571" s="25" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1571" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1571" s="25" t="inlineStr">
+        <is>
+          <t>Awareness campaigns for citizen compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1572" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1572" s="25" t="inlineStr">
+        <is>
+          <t>Sol_capacity</t>
+        </is>
+      </c>
+      <c r="D1572" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1572" s="25" t="inlineStr">
+        <is>
+          <t>Technology transfer and shredder infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1573" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1573" s="25" t="inlineStr">
+        <is>
+          <t>Sol_finance</t>
+        </is>
+      </c>
+      <c r="D1573" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1573" s="25" t="inlineStr">
+        <is>
+          <t>Initial investment high but reduces costs over time; municipal budget limits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1574" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1574" s="25" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1574" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1574" s="25" t="inlineStr">
+        <is>
+          <t>Landfills, transfer stations, shredders, common landfill across municipalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1575" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1575" s="25" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1575" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1575" s="25" t="inlineStr">
+        <is>
+          <t>Cloth bags; minimize plastic at source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1576" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1576" s="25" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1576" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1576" s="25" t="inlineStr">
+        <is>
+          <t>Stronger laws and stricter penalties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1577" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1577" s="25" t="inlineStr">
+        <is>
+          <t>Sol_monitoring</t>
+        </is>
+      </c>
+      <c r="D1577" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1577" s="25" t="inlineStr">
+        <is>
+          <t>Better enforcement of existing penalties and bans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" s="25" t="inlineStr">
+        <is>
+          <t>NPL_20</t>
+        </is>
+      </c>
+      <c r="B1578" s="25" t="inlineStr">
+        <is>
+          <t>Municipality Environment Officer (unnamed), small Chitwan-area municipality (Safa Urja contractor; Ratnanagar/Kalika/Khaireni/Rapti context; interview date not stated)</t>
+        </is>
+      </c>
+      <c r="C1578" s="25" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1578" s="25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1578" s="25" t="inlineStr">
+        <is>
+          <t>NA - not discussed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_21 coding for ordinary person/citizen interview (Feb 2026)
Code structured guideline notes for unnamed ordinary-person interview
(concern about plastic convenience vs environment, mixed municipal
collection, weak ban enforcement, separate-collection infrastructure
needed). Updates workbook to NPL_1 through NPL_21.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -62,116 +62,122 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB8A2"/>
-        <bgColor rgb="00EBB8A2"/>
+        <fgColor rgb="00EBB7A2"/>
+        <bgColor rgb="00EBB7A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBCEA2"/>
-        <bgColor rgb="00EBCEA2"/>
+        <fgColor rgb="00EBCCA2"/>
+        <bgColor rgb="00EBCCA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE4A2"/>
-        <bgColor rgb="00EBE4A2"/>
+        <fgColor rgb="00EBE0A2"/>
+        <bgColor rgb="00EBE0A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCEBA2"/>
-        <bgColor rgb="00DCEBA2"/>
+        <fgColor rgb="00E0EBA2"/>
+        <bgColor rgb="00E0EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EBA2"/>
-        <bgColor rgb="00C6EBA2"/>
+        <fgColor rgb="00CCEBA2"/>
+        <bgColor rgb="00CCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B1EBA2"/>
-        <bgColor rgb="00B1EBA2"/>
+        <fgColor rgb="00B7EBA2"/>
+        <bgColor rgb="00B7EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA9"/>
-        <bgColor rgb="00A2EBA9"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBBF"/>
-        <bgColor rgb="00A2EBBF"/>
+        <fgColor rgb="00A2EBB7"/>
+        <bgColor rgb="00A2EBB7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD5"/>
-        <bgColor rgb="00A2EBD5"/>
+        <fgColor rgb="00A2EBCC"/>
+        <bgColor rgb="00A2EBCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBE0"/>
+        <bgColor rgb="00A2EBE0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D5EB"/>
-        <bgColor rgb="00A2D5EB"/>
+        <fgColor rgb="00A2E0EB"/>
+        <bgColor rgb="00A2E0EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2BFEB"/>
-        <bgColor rgb="00A2BFEB"/>
+        <fgColor rgb="00A2CCEB"/>
+        <bgColor rgb="00A2CCEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A9EB"/>
-        <bgColor rgb="00A2A9EB"/>
+        <fgColor rgb="00A2B7EB"/>
+        <bgColor rgb="00A2B7EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B1A2EB"/>
-        <bgColor rgb="00B1A2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6A2EB"/>
-        <bgColor rgb="00C6A2EB"/>
+        <fgColor rgb="00B7A2EB"/>
+        <bgColor rgb="00B7A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCA2EB"/>
-        <bgColor rgb="00DCA2EB"/>
+        <fgColor rgb="00CCA2EB"/>
+        <bgColor rgb="00CCA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E4"/>
-        <bgColor rgb="00EBA2E4"/>
+        <fgColor rgb="00E0A2EB"/>
+        <bgColor rgb="00E0A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2CE"/>
-        <bgColor rgb="00EBA2CE"/>
+        <fgColor rgb="00EBA2E0"/>
+        <bgColor rgb="00EBA2E0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B8"/>
-        <bgColor rgb="00EBA2B8"/>
+        <fgColor rgb="00EBA2CC"/>
+        <bgColor rgb="00EBA2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B7"/>
+        <bgColor rgb="00EBA2B7"/>
       </patternFill>
     </fill>
   </fills>
@@ -201,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -276,6 +282,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -643,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -662,7 +671,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_20, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_21, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -817,82 +826,89 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  21. NPL_21 - Ordinary person / citizen (unnamed), Nepal (17 February 2026). Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured guideline/field notes only. Q3, Q6, Q9 and Q10 not fully asked.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_20, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_21, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_20) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_21) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2079,7 +2095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ21"/>
+  <dimension ref="A1:CQ22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12196,6 +12212,483 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>households</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O22" s="26" t="inlineStr">
+        <is>
+          <t>health (burning plastics is "very bad for the health" — main health impact cited; plastic itself not harmful unless burned), visual/aesthetic pollution, blocked pipes/drainage, and contaminated agricultural plots; environment (plastics are non-biodegradable)</t>
+        </is>
+      </c>
+      <c r="P22" s="26" t="inlineStr">
+        <is>
+          <t>people exposed to burning plastics (health); agricultural plots contaminated by plastic waste; drainage/pipe infrastructure blocked by litter; and residents affected by visual/aesthetic pollution</t>
+        </is>
+      </c>
+      <c r="Q22" s="26" t="inlineStr">
+        <is>
+          <t>households/the public ("people know the rules but do not follow them"; no information on single-use vs other plastic types; read a little about plastic then forget; continue using plastic because it is "very convenient"); and government (spreads information but "do not enforce" and "there is not monitoring"; past plastic ban "did not work")</t>
+        </is>
+      </c>
+      <c r="R22" s="26" t="inlineStr">
+        <is>
+          <t>local government imposing regulation (ward, mayor and ministry); separate waste-collection vehicles for different waste streams to enable segregation; and traditional alternatives (paper bags and baskets — though plastic is more convenient)</t>
+        </is>
+      </c>
+      <c r="S22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AY22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA22" s="26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB22" s="26" t="inlineStr">
+        <is>
+          <t>As an ordinary resident the interviewee is concerned about plastic pollution but continues to use plastic because it is convenient; puts out mixed wet and dry waste for the municipality's daily collection vehicle with no household segregation — and has no authority to change enforcement, monitoring or the collection system (separate vehicles would need to be provided by local government).</t>
+        </is>
+      </c>
+      <c r="BC22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BH22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BL22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW22" s="26" t="inlineStr">
+        <is>
+          <t>Ban of black plastic bags exists and "there was a ban of plastics some years ago, but it did not work"; daily municipal collection vehicle takes mixed waste to landfill but "there are not further policies"; wet and dry waste mixed at household level with no segregation.</t>
+        </is>
+      </c>
+      <c r="BX22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CB22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CC22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CF22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN22" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO22" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP22" s="26" t="inlineStr">
+        <is>
+          <t>Traditionally paper bags and baskets were used to carry goods, but plastic is "much more convenient."</t>
+        </is>
+      </c>
+      <c r="CQ22" s="26" t="inlineStr">
+        <is>
+          <t>Master list label: "21. Ordinary person (unnamed)", affiliation: ordinary person/citizen. Interviewee name not given. Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Q3 (main challenges) not asked separately — integrated in Q2 notes. Q6 and Q6 follow-up not asked (enforcement/monitoring gap noted in passing). Q9 (target groups) not asked. Q10 not asked (infrastructure for separate collection mentioned under solutions). NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12207,7 +12700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1578"/>
+  <dimension ref="A1:E1636"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54823,6 +55316,1572 @@
         </is>
       </c>
     </row>
+    <row r="1579">
+      <c r="A1579" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1579" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1579" s="26" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1579" s="26" t="inlineStr">
+        <is>
+          <t>households</t>
+        </is>
+      </c>
+      <c r="E1579" s="26" t="inlineStr">
+        <is>
+          <t>Interviewee described as "ordinary person" — coded as households.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1580" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1580" s="26" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1580" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1580" s="26" t="inlineStr">
+        <is>
+          <t>"They have no information about single use and other types of the plastic"; "People read a little about the plastic and then forget about it."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1581" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1581" s="26" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1581" s="26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1581" s="26" t="inlineStr">
+        <is>
+          <t>"Yes, concerned about plastic pollution" — but also notes plastic is "very convenient to use."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1582" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1582" s="26" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1582" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1582" s="26" t="inlineStr">
+        <is>
+          <t>Visual pollution/aesthetic effects cited as an impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1583" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1583" s="26" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1583" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1583" s="26" t="inlineStr">
+        <is>
+          <t>Plastic is "very convenient to use" despite environmental concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1584" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1584" s="26" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1584" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1584" s="26" t="inlineStr">
+        <is>
+          <t>Daily collection to landfill but no household segregation; wet and dry waste mixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1585" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1585" s="26" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1585" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1585" s="26" t="inlineStr">
+        <is>
+          <t>Traditionally paper bags and baskets were used but plastic is more convenient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1586" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1586" s="26" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1586" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1586" s="26" t="inlineStr">
+        <is>
+          <t>"Not segregated at household level, i.e. also wet and dry waste are mixed together."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1587" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1587" s="26" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1587" s="26" t="inlineStr">
+        <is>
+          <t>health (burning plastics is "very bad for the health" — main health impact cited; plastic itself not harmful unless burned), visual/aesthetic pollution, blocked pipes/drainage, and contaminated agricultural plots; environment (plastics are non-biodegradable)</t>
+        </is>
+      </c>
+      <c r="E1587" s="26" t="inlineStr">
+        <is>
+          <t>Health (burning), visual pollution, blocked drainage, contaminated agricultural plots, non-biodegradability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1588" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1588" s="26" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1588" s="26" t="inlineStr">
+        <is>
+          <t>people exposed to burning plastics (health); agricultural plots contaminated by plastic waste; drainage/pipe infrastructure blocked by litter; and residents affected by visual/aesthetic pollution</t>
+        </is>
+      </c>
+      <c r="E1588" s="26" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: health from burning; agricultural plots; drainage; residents from visual pollution. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1589" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1589" s="26" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1589" s="26" t="inlineStr">
+        <is>
+          <t>households/the public ("people know the rules but do not follow them"; no information on single-use vs other plastic types; read a little about plastic then forget; continue using plastic because it is "very convenient"); and government (spreads information but "do not enforce" and "there is not monitoring"; past plastic ban "did not work")</t>
+        </is>
+      </c>
+      <c r="E1589" s="26" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: public/households (non-compliance, convenience); government (weak enforcement/monitoring). No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1590" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1590" s="26" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1590" s="26" t="inlineStr">
+        <is>
+          <t>local government imposing regulation (ward, mayor and ministry); separate waste-collection vehicles for different waste streams to enable segregation; and traditional alternatives (paper bags and baskets — though plastic is more convenient)</t>
+        </is>
+      </c>
+      <c r="E1590" s="26" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: local government regulation; separate collection vehicles; traditional paper bags/baskets. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1591" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1591" s="26" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1591" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1591" s="26" t="inlineStr">
+        <is>
+          <t>Ministry mentioned alongside ward and mayor as needing to impose regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1592" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1592" s="26" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1592" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1592" s="26" t="inlineStr">
+        <is>
+          <t>NA - provincial government not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1593" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1593" s="26" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1593" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1593" s="26" t="inlineStr">
+        <is>
+          <t>"Local government" responsible for managing plastics/waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1594" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1594" s="26" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1594" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1594" s="26" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1595" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1595" s="26" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1595" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1595" s="26" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1596" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1596" s="26" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1596" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1596" s="26" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1597" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1597" s="26" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1597" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1597" s="26" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1598" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1598" s="26" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1598" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1598" s="26" t="inlineStr">
+        <is>
+          <t>Households produce mixed waste and do not segregate at source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1599" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1599" s="26" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1599" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1599" s="26" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1600" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1600" s="26" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1600" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1600" s="26" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1601" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1601" s="26" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1601" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1601" s="26" t="inlineStr">
+        <is>
+          <t>"Govt. spreads the information, but they do not enforce, there is not monitoring"; past ban did not work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1602" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1602" s="26" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1602" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1602" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1603" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1603" s="26" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1603" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1603" s="26" t="inlineStr">
+        <is>
+          <t>NA - local government portrayed as responsible actor to strengthen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1604" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1604" s="26" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1604" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1604" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1605" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1605" s="26" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1605" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1605" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1606" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1606" s="26" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1606" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1606" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1607" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1607" s="26" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1607" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1607" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1608" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1608" s="26" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1608" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1608" s="26" t="inlineStr">
+        <is>
+          <t>"People know the rules but do not follow them"; limited information and forgetfulness; convenience-driven plastic use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1609" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1609" s="26" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1609" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1609" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1610" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1610" s="26" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1610" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1610" s="26" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1611" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1611" s="26" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1611" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1611" s="26" t="inlineStr">
+        <is>
+          <t>Ministry named as part of actors who should impose regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1612" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1612" s="26" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1612" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1612" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1613" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1613" s="26" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1613" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1613" s="26" t="inlineStr">
+        <is>
+          <t>"Local government has to impose the regulation, i.e. the ward, mayor and the ministry."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1614" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1614" s="26" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1614" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1614" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1615" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1615" s="26" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1615" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1615" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1616" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1616" s="26" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1616" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1616" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1617" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1617" s="26" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1617" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1617" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1618" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1618" s="26" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1618" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1618" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named as policy target (local government emphasised).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1619" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1619" s="26" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1619" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1619" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1620" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1620" s="26" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1620" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1620" s="26" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1621" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1621" s="26" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1621" s="26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1621" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary citizen as target group / affected resident (role 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1622" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1622" s="26" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1622" s="26" t="inlineStr">
+        <is>
+          <t>As an ordinary resident the interviewee is concerned about plastic pollution but continues to use plastic because it is convenient; puts out mixed wet and dry waste for the municipality's daily collection vehicle with no household segregation — and has no authority to change enforcement, monitoring or the collection system (separate vehicles would need to be provided by local government).</t>
+        </is>
+      </c>
+      <c r="E1622" s="26" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1623" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1623" s="26" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1623" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1623" s="26" t="inlineStr">
+        <is>
+          <t>No monitoring of waste/plastic rules cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1624" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1624" s="26" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1624" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1624" s="26" t="inlineStr">
+        <is>
+          <t>Separate vehicles for different waste types needed to enable segregation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1625" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1625" s="26" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1625" s="26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1625" s="26" t="inlineStr">
+        <is>
+          <t>NA - not discussed as an implementation barrier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1626" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1626" s="26" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1626" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1626" s="26" t="inlineStr">
+        <is>
+          <t>Government spreads information but does not enforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1627" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1627" s="26" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1627" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1627" s="26" t="inlineStr">
+        <is>
+          <t>Ban of black plastic bags; earlier plastics ban "some years ago" that did not work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1628" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1628" s="26" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1628" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1628" s="26" t="inlineStr">
+        <is>
+          <t>Municipality-organised daily collection vehicle picks up waste and drops at landfill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1629" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1629" s="26" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1629" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1629" s="26" t="inlineStr">
+        <is>
+          <t>Past ban ineffective; only basic collection in place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1630" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1630" s="26" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1630" s="26" t="inlineStr">
+        <is>
+          <t>Ban of black plastic bags exists and "there was a ban of plastics some years ago, but it did not work"; daily municipal collection vehicle takes mixed waste to landfill but "there are not further policies"; wet and dry waste mixed at household level with no segregation.</t>
+        </is>
+      </c>
+      <c r="E1630" s="26" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1631" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1631" s="26" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1631" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1631" s="26" t="inlineStr">
+        <is>
+          <t>Local government (ward, mayor, ministry) should impose regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1632" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1632" s="26" t="inlineStr">
+        <is>
+          <t>Sol_segregation</t>
+        </is>
+      </c>
+      <c r="D1632" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1632" s="26" t="inlineStr">
+        <is>
+          <t>Different vehicles for different wastes would make segregation easier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1633" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1633" s="26" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1633" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1633" s="26" t="inlineStr">
+        <is>
+          <t>Better waste collection infrastructure with separate streams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1634" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1634" s="26" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1634" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1634" s="26" t="inlineStr">
+        <is>
+          <t>Traditional paper bags and baskets as alternatives to plastic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1635" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1635" s="26" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1635" s="26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1635" s="26" t="inlineStr">
+        <is>
+          <t>Regulation needs to be imposed by local government.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" s="26" t="inlineStr">
+        <is>
+          <t>NPL_21</t>
+        </is>
+      </c>
+      <c r="B1636" s="26" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1636" s="26" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1636" s="26" t="inlineStr">
+        <is>
+          <t>Traditionally paper bags and baskets were used to carry goods, but plastic is "much more convenient."</t>
+        </is>
+      </c>
+      <c r="E1636" s="26" t="inlineStr">
+        <is>
+          <t>Paper bags and baskets traditionally used.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_22 coding for second ordinary-person interview (Feb 2026)
Code structured guideline notes for second unnamed ordinary-person
respondent (low personal concern, burning/livestock impacts, abolished
segregation, weak campaign effectiveness). Distinct from NPL_21 on same
date. Updates workbook to NPL_1 through NPL_22.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="24">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -62,122 +62,128 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB7A2"/>
-        <bgColor rgb="00EBB7A2"/>
+        <fgColor rgb="00EBB6A2"/>
+        <bgColor rgb="00EBB6A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBCCA2"/>
-        <bgColor rgb="00EBCCA2"/>
+        <fgColor rgb="00EBCAA2"/>
+        <bgColor rgb="00EBCAA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE0A2"/>
-        <bgColor rgb="00EBE0A2"/>
+        <fgColor rgb="00EBDEA2"/>
+        <bgColor rgb="00EBDEA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0EBA2"/>
-        <bgColor rgb="00E0EBA2"/>
+        <fgColor rgb="00E4EBA2"/>
+        <bgColor rgb="00E4EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCEBA2"/>
-        <bgColor rgb="00CCEBA2"/>
+        <fgColor rgb="00D0EBA2"/>
+        <bgColor rgb="00D0EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B7EBA2"/>
-        <bgColor rgb="00B7EBA2"/>
+        <fgColor rgb="00BCEBA2"/>
+        <bgColor rgb="00BCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA2"/>
-        <bgColor rgb="00A2EBA2"/>
+        <fgColor rgb="00A9EBA2"/>
+        <bgColor rgb="00A9EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBB7"/>
-        <bgColor rgb="00A2EBB7"/>
+        <fgColor rgb="00A2EBAF"/>
+        <bgColor rgb="00A2EBAF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBCC"/>
-        <bgColor rgb="00A2EBCC"/>
+        <fgColor rgb="00A2EBC3"/>
+        <bgColor rgb="00A2EBC3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBE0"/>
-        <bgColor rgb="00A2EBE0"/>
+        <fgColor rgb="00A2EBD7"/>
+        <bgColor rgb="00A2EBD7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2E0EB"/>
-        <bgColor rgb="00A2E0EB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2CCEB"/>
-        <bgColor rgb="00A2CCEB"/>
+        <fgColor rgb="00A2D7EB"/>
+        <bgColor rgb="00A2D7EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2B7EB"/>
-        <bgColor rgb="00A2B7EB"/>
+        <fgColor rgb="00A2C3EB"/>
+        <bgColor rgb="00A2C3EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A2EB"/>
-        <bgColor rgb="00A2A2EB"/>
+        <fgColor rgb="00A2AFEB"/>
+        <bgColor rgb="00A2AFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B7A2EB"/>
-        <bgColor rgb="00B7A2EB"/>
+        <fgColor rgb="00A9A2EB"/>
+        <bgColor rgb="00A9A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCA2EB"/>
-        <bgColor rgb="00CCA2EB"/>
+        <fgColor rgb="00BCA2EB"/>
+        <bgColor rgb="00BCA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0A2EB"/>
-        <bgColor rgb="00E0A2EB"/>
+        <fgColor rgb="00D0A2EB"/>
+        <bgColor rgb="00D0A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E0"/>
-        <bgColor rgb="00EBA2E0"/>
+        <fgColor rgb="00E4A2EB"/>
+        <bgColor rgb="00E4A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2CC"/>
-        <bgColor rgb="00EBA2CC"/>
+        <fgColor rgb="00EBA2DE"/>
+        <bgColor rgb="00EBA2DE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B7"/>
-        <bgColor rgb="00EBA2B7"/>
+        <fgColor rgb="00EBA2CA"/>
+        <bgColor rgb="00EBA2CA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B6"/>
+        <bgColor rgb="00EBA2B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -207,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -285,6 +291,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -652,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -671,7 +680,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_21, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_22, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -833,82 +842,89 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  22. NPL_22 - Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026). Same interview team and date as NPL_21 but distinct respondent (lower personal concern; burning/livestock impacts; segregation abolished). Coded from guideline/field notes only.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_21, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_22, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_21) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_22) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2095,7 +2111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ22"/>
+  <dimension ref="A1:CQ23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12689,6 +12705,483 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>households</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O23" s="27" t="inlineStr">
+        <is>
+          <t>livestock (animals eat plastics), health (burning plastics — smell and coughing; air pollution from burning), contaminated agricultural plots, and blocked pipes/drainage</t>
+        </is>
+      </c>
+      <c r="P23" s="27" t="inlineStr">
+        <is>
+          <t>livestock that ingest plastic waste; people affected by burning plastics (smell, coughing, air pollution); agricultural plots contaminated by plastic; and drainage/pipe infrastructure blocked by litter</t>
+        </is>
+      </c>
+      <c r="Q23" s="27" t="inlineStr">
+        <is>
+          <t>households/residents (plastic is "very convenient" — buy and throw to dustbin; "do not want to engage with the waste themselves"; do not make compost); government ("does not enforce" and "there is no monitoring"; information about impacts "not taught to people"); and plastic producers ("stop production" suggested as solution)</t>
+        </is>
+      </c>
+      <c r="R23" s="27" t="inlineStr">
+        <is>
+          <t>local government enforcing regulation; stopping plastic production; strict regulations for carrying plastic bags; awareness-raising about impacts; and traditional/modern alternatives (paper bags, bamboo leaves/baskets, cloth bags — used more often but not yet frequently)</t>
+        </is>
+      </c>
+      <c r="S23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AR23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AY23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA23" s="27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB23" s="27" t="inlineStr">
+        <is>
+          <t>As an ordinary resident the interviewee is "not very concerned about pollution" but recognises burning as a problem; uses plastic for convenience and throws it in the dustbin; does not segregate waste or make compost at home (segregation was abolished; residents "don't want to engage with the waste themselves") — and has no authority over municipal enforcement, production bans or monitoring.</t>
+        </is>
+      </c>
+      <c r="BC23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BH23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BU23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW23" s="27" t="inlineStr">
+        <is>
+          <t>Campaign not to use plastics "did not work well"; daily municipal waste pick-up in place but "segregation was abolished"; municipality makes compost but residents do not use it (no agricultural plots nearby) and "do not make compost themselves"; overall "measures are not very effective so far."</t>
+        </is>
+      </c>
+      <c r="BX23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CF23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CJ23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CL23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN23" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO23" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP23" s="27" t="inlineStr">
+        <is>
+          <t>Traditionally paper bags and bamboo leaves/baskets were used to carry goods, but plastic is "much more convenient"; cloth bags exist today and are used more often but "not yet used frequently."</t>
+        </is>
+      </c>
+      <c r="CQ23" s="27" t="inlineStr">
+        <is>
+          <t>Master list label: "22. Ordinary person (unnamed, 2nd respondent)", affiliation: ordinary person/citizen. Interviewee name not given. Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Second ordinary-person interview on the same date as NPL_21 — distinct respondent with lower personal concern and emphasis on burning/livestock impacts. Q3 not asked separately. Q6 and Q6 follow-up not asked (enforcement/monitoring and awareness gaps noted in passing). Q9 and Q10 not asked. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12700,7 +13193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1636"/>
+  <dimension ref="A1:E1695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -56882,6 +57375,1599 @@
         </is>
       </c>
     </row>
+    <row r="1637">
+      <c r="A1637" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1637" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1637" s="27" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1637" s="27" t="inlineStr">
+        <is>
+          <t>households</t>
+        </is>
+      </c>
+      <c r="E1637" s="27" t="inlineStr">
+        <is>
+          <t>Interviewee described as "ordinary person" — coded as households.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1638" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1638" s="27" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1638" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1638" s="27" t="inlineStr">
+        <is>
+          <t>"Information about the impacts is not taught to people -&gt; need to increase awareness."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1639" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1639" s="27" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1639" s="27" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E1639" s="27" t="inlineStr">
+        <is>
+          <t>"Not very concerned about pollution" — though burning is recognised as a problem (smell, coughing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1640" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1640" s="27" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1640" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1640" s="27" t="inlineStr">
+        <is>
+          <t>Livestock eat plastics; blocked drainage pipes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1641" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1641" s="27" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1641" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1641" s="27" t="inlineStr">
+        <is>
+          <t>Plastic is "very convenient" — buy and throw to dustbin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1642" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1642" s="27" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1642" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1642" s="27" t="inlineStr">
+        <is>
+          <t>Municipality makes compost but residents do not use it; residents do not make compost themselves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1643" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1643" s="27" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1643" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1643" s="27" t="inlineStr">
+        <is>
+          <t>Segregation abolished; residents do not engage with waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1644" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1644" s="27" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1644" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1644" s="27" t="inlineStr">
+        <is>
+          <t>"Stop production" suggested as future measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1645" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1645" s="27" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1645" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1645" s="27" t="inlineStr">
+        <is>
+          <t>"Segregation was abolished."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1646" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1646" s="27" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1646" s="27" t="inlineStr">
+        <is>
+          <t>livestock (animals eat plastics), health (burning plastics — smell and coughing; air pollution from burning), contaminated agricultural plots, and blocked pipes/drainage</t>
+        </is>
+      </c>
+      <c r="E1646" s="27" t="inlineStr">
+        <is>
+          <t>Livestock, burning/air pollution/health, agricultural plots, blocked drainage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1647" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1647" s="27" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1647" s="27" t="inlineStr">
+        <is>
+          <t>livestock that ingest plastic waste; people affected by burning plastics (smell, coughing, air pollution); agricultural plots contaminated by plastic; and drainage/pipe infrastructure blocked by litter</t>
+        </is>
+      </c>
+      <c r="E1647" s="27" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: livestock; health from burning; agricultural plots; drainage. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1648" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1648" s="27" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1648" s="27" t="inlineStr">
+        <is>
+          <t>households/residents (plastic is "very convenient" — buy and throw to dustbin; "do not want to engage with the waste themselves"; do not make compost); government ("does not enforce" and "there is no monitoring"; information about impacts "not taught to people"); and plastic producers ("stop production" suggested as solution)</t>
+        </is>
+      </c>
+      <c r="E1648" s="27" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: households (convenience, non-engagement); government (no enforcement/monitoring, lack of education); producers (stop production). No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1649" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1649" s="27" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1649" s="27" t="inlineStr">
+        <is>
+          <t>local government enforcing regulation; stopping plastic production; strict regulations for carrying plastic bags; awareness-raising about impacts; and traditional/modern alternatives (paper bags, bamboo leaves/baskets, cloth bags — used more often but not yet frequently)</t>
+        </is>
+      </c>
+      <c r="E1649" s="27" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: local government enforcement; production stop; strict bag rules; awareness; traditional/modern bag alternatives. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1650" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1650" s="27" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1650" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1650" s="27" t="inlineStr">
+        <is>
+          <t>NA - national government not named as formal responsible actor (only blamed for enforcement gap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1651" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1651" s="27" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1651" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1651" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1652" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1652" s="27" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1652" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1652" s="27" t="inlineStr">
+        <is>
+          <t>"Local government" responsible for managing plastics/waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1653" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1653" s="27" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1653" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1653" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1654" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1654" s="27" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1654" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1654" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1655" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1655" s="27" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1655" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1655" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1656" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1656" s="27" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1656" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1656" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1657" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1657" s="27" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1657" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1657" s="27" t="inlineStr">
+        <is>
+          <t>Residents produce waste, use dustbins, but do not segregate or compost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1658" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1658" s="27" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1658" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1658" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1659" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1659" s="27" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1659" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1659" s="27" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1660" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1660" s="27" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1660" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1660" s="27" t="inlineStr">
+        <is>
+          <t>"Govt. does not enforce, there is no monitoring"; impacts not taught to people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1661" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1661" s="27" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1661" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1661" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1662" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1662" s="27" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1662" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1662" s="27" t="inlineStr">
+        <is>
+          <t>NA - local government portrayed as actor to strengthen enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1663" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1663" s="27" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1663" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1663" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1664" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1664" s="27" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1664" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1664" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1665" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1665" s="27" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1665" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1665" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1666" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1666" s="27" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1666" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1666" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1667" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1667" s="27" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1667" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1667" s="27" t="inlineStr">
+        <is>
+          <t>Convenience-driven plastic use; "don't want to engage with the waste themselves"; do not make compost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1668" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1668" s="27" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1668" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1668" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1669" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1669" s="27" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1669" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1669" s="27" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1670" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1670" s="27" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1670" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1670" s="27" t="inlineStr">
+        <is>
+          <t>"Stop production" implies national-level production regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1671" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1671" s="27" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1671" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1671" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1672" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1672" s="27" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1672" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1672" s="27" t="inlineStr">
+        <is>
+          <t>"Local government has to enforce the regulation."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1673" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1673" s="27" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1673" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1673" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1674" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1674" s="27" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1674" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1674" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1675" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1675" s="27" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1675" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1675" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1676" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1676" s="27" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1676" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1676" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1677" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1677" s="27" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1677" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1677" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named as policy target (local government emphasised).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1678" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1678" s="27" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1678" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1678" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1679" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1679" s="27" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1679" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1679" s="27" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1680" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1680" s="27" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1680" s="27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1680" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary citizen as target group / affected resident (role 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1681" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1681" s="27" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1681" s="27" t="inlineStr">
+        <is>
+          <t>As an ordinary resident the interviewee is "not very concerned about pollution" but recognises burning as a problem; uses plastic for convenience and throws it in the dustbin; does not segregate waste or make compost at home (segregation was abolished; residents "don't want to engage with the waste themselves") — and has no authority over municipal enforcement, production bans or monitoring.</t>
+        </is>
+      </c>
+      <c r="E1681" s="27" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1682" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1682" s="27" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1682" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1682" s="27" t="inlineStr">
+        <is>
+          <t>"There is no monitoring."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1683" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1683" s="27" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1683" s="27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1683" s="27" t="inlineStr">
+        <is>
+          <t>NA - not discussed as an implementation barrier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1684" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1684" s="27" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1684" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1684" s="27" t="inlineStr">
+        <is>
+          <t>Government does not enforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1685" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1685" s="27" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1685" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1685" s="27" t="inlineStr">
+        <is>
+          <t>Campaign not to use plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1686" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1686" s="27" t="inlineStr">
+        <is>
+          <t>Pol_recycling</t>
+        </is>
+      </c>
+      <c r="D1686" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1686" s="27" t="inlineStr">
+        <is>
+          <t>Municipality makes compost (unused by residents).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1687" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1687" s="27" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1687" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1687" s="27" t="inlineStr">
+        <is>
+          <t>Daily waste pick-up from municipality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1688" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1688" s="27" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1688" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1688" s="27" t="inlineStr">
+        <is>
+          <t>Campaign did not work; segregation abolished; compost unused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1689" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1689" s="27" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1689" s="27" t="inlineStr">
+        <is>
+          <t>Campaign not to use plastics "did not work well"; daily municipal waste pick-up in place but "segregation was abolished"; municipality makes compost but residents do not use it (no agricultural plots nearby) and "do not make compost themselves"; overall "measures are not very effective so far."</t>
+        </is>
+      </c>
+      <c r="E1689" s="27" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1690" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1690" s="27" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1690" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1690" s="27" t="inlineStr">
+        <is>
+          <t>Local government must enforce regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1691" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1691" s="27" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1691" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1691" s="27" t="inlineStr">
+        <is>
+          <t>Increase awareness about impacts (not currently taught).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1692" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1692" s="27" t="inlineStr">
+        <is>
+          <t>Sol_ban</t>
+        </is>
+      </c>
+      <c r="D1692" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1692" s="27" t="inlineStr">
+        <is>
+          <t>"Stop production" and strict regulations for carrying plastic bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1693" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1693" s="27" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1693" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1693" s="27" t="inlineStr">
+        <is>
+          <t>Paper bags, bamboo leaves/baskets, cloth bags (increasing but not frequent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1694" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1694" s="27" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1694" s="27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1694" s="27" t="inlineStr">
+        <is>
+          <t>Local government enforcement of regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="27" t="inlineStr">
+        <is>
+          <t>NPL_22</t>
+        </is>
+      </c>
+      <c r="B1695" s="27" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 2nd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21)</t>
+        </is>
+      </c>
+      <c r="C1695" s="27" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1695" s="27" t="inlineStr">
+        <is>
+          <t>Traditionally paper bags and bamboo leaves/baskets were used to carry goods, but plastic is "much more convenient"; cloth bags exist today and are used more often but "not yet used frequently."</t>
+        </is>
+      </c>
+      <c r="E1695" s="27" t="inlineStr">
+        <is>
+          <t>Paper bags and bamboo leaves/baskets; cloth bags today.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_23 coding for shop owner interview (Feb 2026)
Code structured guideline notes for unnamed shop-owner respondent
(low concern, black-bag ban, white/blue bags at 3 NPR, customer demand
for bags). Updates workbook to NPL_1 through NPL_23.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -62,128 +62,134 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB6A2"/>
-        <bgColor rgb="00EBB6A2"/>
+        <fgColor rgb="00EBB5A2"/>
+        <bgColor rgb="00EBB5A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBCAA2"/>
-        <bgColor rgb="00EBCAA2"/>
+        <fgColor rgb="00EBC8A2"/>
+        <bgColor rgb="00EBC8A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBDEA2"/>
-        <bgColor rgb="00EBDEA2"/>
+        <fgColor rgb="00EBDBA2"/>
+        <bgColor rgb="00EBDBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4EBA2"/>
-        <bgColor rgb="00E4EBA2"/>
+        <fgColor rgb="00E8EBA2"/>
+        <bgColor rgb="00E8EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D0EBA2"/>
-        <bgColor rgb="00D0EBA2"/>
+        <fgColor rgb="00D5EBA2"/>
+        <bgColor rgb="00D5EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BCEBA2"/>
-        <bgColor rgb="00BCEBA2"/>
+        <fgColor rgb="00C2EBA2"/>
+        <bgColor rgb="00C2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A9EBA2"/>
-        <bgColor rgb="00A9EBA2"/>
+        <fgColor rgb="00AFEBA2"/>
+        <bgColor rgb="00AFEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBAF"/>
-        <bgColor rgb="00A2EBAF"/>
+        <fgColor rgb="00A2EBA8"/>
+        <bgColor rgb="00A2EBA8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBC3"/>
-        <bgColor rgb="00A2EBC3"/>
+        <fgColor rgb="00A2EBBB"/>
+        <bgColor rgb="00A2EBBB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD7"/>
-        <bgColor rgb="00A2EBD7"/>
+        <fgColor rgb="00A2EBCE"/>
+        <bgColor rgb="00A2EBCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBE1"/>
+        <bgColor rgb="00A2EBE1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D7EB"/>
-        <bgColor rgb="00A2D7EB"/>
+        <fgColor rgb="00A2E1EB"/>
+        <bgColor rgb="00A2E1EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2C3EB"/>
-        <bgColor rgb="00A2C3EB"/>
+        <fgColor rgb="00A2CEEB"/>
+        <bgColor rgb="00A2CEEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2AFEB"/>
-        <bgColor rgb="00A2AFEB"/>
+        <fgColor rgb="00A2BBEB"/>
+        <bgColor rgb="00A2BBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A9A2EB"/>
-        <bgColor rgb="00A9A2EB"/>
+        <fgColor rgb="00A2A8EB"/>
+        <bgColor rgb="00A2A8EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BCA2EB"/>
-        <bgColor rgb="00BCA2EB"/>
+        <fgColor rgb="00AFA2EB"/>
+        <bgColor rgb="00AFA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D0A2EB"/>
-        <bgColor rgb="00D0A2EB"/>
+        <fgColor rgb="00C2A2EB"/>
+        <bgColor rgb="00C2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E4A2EB"/>
-        <bgColor rgb="00E4A2EB"/>
+        <fgColor rgb="00D5A2EB"/>
+        <bgColor rgb="00D5A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2DE"/>
-        <bgColor rgb="00EBA2DE"/>
+        <fgColor rgb="00E8A2EB"/>
+        <bgColor rgb="00E8A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2CA"/>
-        <bgColor rgb="00EBA2CA"/>
+        <fgColor rgb="00EBA2DB"/>
+        <bgColor rgb="00EBA2DB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B6"/>
-        <bgColor rgb="00EBA2B6"/>
+        <fgColor rgb="00EBA2C8"/>
+        <bgColor rgb="00EBA2C8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B5"/>
+        <bgColor rgb="00EBA2B5"/>
       </patternFill>
     </fill>
   </fills>
@@ -213,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -294,6 +300,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -661,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -680,7 +689,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_22, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_23, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -849,82 +858,89 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  23. NPL_23 - Shop owner (unnamed), Nepal (17 February 2026). Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from guideline/field notes only. Black-bag ban; white/blue bags (3 NPR); customers request bags for home waste. Q6, Q8 and Q10 not asked.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_22, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_23, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
-    </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_22) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_23) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
-    </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2111,7 +2127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ23"/>
+  <dimension ref="A1:CQ24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13182,6 +13198,483 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>private_companies</t>
+        </is>
+      </c>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O24" s="28" t="inlineStr">
+        <is>
+          <t>environment (negative environmental impact acknowledged — "the respondent sees the problem but has no idea how to proceed with it"; described as a "problem which is not a problem" from the shopkeeper's practical perspective)</t>
+        </is>
+      </c>
+      <c r="P24" s="28" t="inlineStr">
+        <is>
+          <t>the environment (negative impact acknowledged but not elaborated in detail); implicitly the wider community affected by plastic pollution</t>
+        </is>
+      </c>
+      <c r="Q24" s="28" t="inlineStr">
+        <is>
+          <t>pervasive plastic packaging and supply chains ("everything comes in plastic" and it is "not manageable to get things without it"); customers/households who "come and ask for plastic bags in a shop to manage their waste at home"; and changed food culture (shift away from traditional packaging toward more plastic bags)</t>
+        </is>
+      </c>
+      <c r="R24" s="28" t="inlineStr">
+        <is>
+          <t>everyone sharing responsibility ("everyone should be responsible"); regulated bag policy (ban on black bags; white and blue bags only); and traditional alternatives (paper bags — women used to make bags themselves)</t>
+        </is>
+      </c>
+      <c r="S24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AG24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AT24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BA24" s="28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB24" s="28" t="inlineStr">
+        <is>
+          <t>As a shop owner the interviewee is not very concerned about plastic pollution and sees it as practically unavoidable because "everything comes in plastic"; customers routinely ask for plastic bags to manage household waste; the shop complies with the black-bag ban by supplying only white and blue bags (3 NPR per blue bag) — but has no authority over production, national policy or customers' waste practices.</t>
+        </is>
+      </c>
+      <c r="BC24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BH24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BI24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BL24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BP24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BQ24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW24" s="28" t="inlineStr">
+        <is>
+          <t>Ban of black plastic bags in place; people are allowed to use only white and blue bags (3 NPR for one blue bag). Follow-up: "People don't use dangerous black bags" — partially effective for the specific black-bag ban.</t>
+        </is>
+      </c>
+      <c r="BX24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BY24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CB24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CF24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CL24" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CO24" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP24" s="28" t="inlineStr">
+        <is>
+          <t>Previously people used paper bags to carry each item; women made bags themselves. Food culture changed, therefore there are more plastic bags now.</t>
+        </is>
+      </c>
+      <c r="CQ24" s="28" t="inlineStr">
+        <is>
+          <t>Master list label: "23. Shop owner (unnamed)", affiliation: shop-owner/retailer. Interviewee name not given. Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Q6 and Q6 follow-up not asked. Q8 (future measures) not asked. Q10 not asked. Same interview date as NPL_21/NPL_22 but distinct retail-sector respondent. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13193,7 +13686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1695"/>
+  <dimension ref="A1:E1743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58968,6 +59461,1302 @@
         </is>
       </c>
     </row>
+    <row r="1696">
+      <c r="A1696" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1696" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1696" s="28" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1696" s="28" t="inlineStr">
+        <is>
+          <t>private_companies</t>
+        </is>
+      </c>
+      <c r="E1696" s="28" t="inlineStr">
+        <is>
+          <t>Interviewee described as "shop-owner" — coded as private_companies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1697" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1697" s="28" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1697" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1697" s="28" t="inlineStr">
+        <is>
+          <t>Customers "come and ask for plastic bags in a shop to manage their waste at home" — implying household demand drives shop plastic-bag supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1698" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1698" s="28" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1698" s="28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="E1698" s="28" t="inlineStr">
+        <is>
+          <t>"Respondent is not very concerned"; describes it as a "problem which is not a problem" from a practical shopkeeper perspective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1699" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1699" s="28" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1699" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1699" s="28" t="inlineStr">
+        <is>
+          <t>"Everything comes in plastic" and it is "not manageable to get things without it."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1700" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1700" s="28" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1700" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1700" s="28" t="inlineStr">
+        <is>
+          <t>No practical alternatives for shopkeeper to source goods without plastic packaging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1701" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1701" s="28" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1701" s="28" t="inlineStr">
+        <is>
+          <t>environment (negative environmental impact acknowledged — "the respondent sees the problem but has no idea how to proceed with it"; described as a "problem which is not a problem" from the shopkeeper's practical perspective)</t>
+        </is>
+      </c>
+      <c r="E1701" s="28" t="inlineStr">
+        <is>
+          <t>Negative environmental impact acknowledged but respondent "has no idea how to proceed."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1702" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1702" s="28" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1702" s="28" t="inlineStr">
+        <is>
+          <t>the environment (negative impact acknowledged but not elaborated in detail); implicitly the wider community affected by plastic pollution</t>
+        </is>
+      </c>
+      <c r="E1702" s="28" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: the environment. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1703" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1703" s="28" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1703" s="28" t="inlineStr">
+        <is>
+          <t>pervasive plastic packaging and supply chains ("everything comes in plastic" and it is "not manageable to get things without it"); customers/households who "come and ask for plastic bags in a shop to manage their waste at home"; and changed food culture (shift away from traditional packaging toward more plastic bags)</t>
+        </is>
+      </c>
+      <c r="E1703" s="28" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: plastic supply/packaging system; customers asking for bags; changed food culture. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1704" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1704" s="28" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1704" s="28" t="inlineStr">
+        <is>
+          <t>everyone sharing responsibility ("everyone should be responsible"); regulated bag policy (ban on black bags; white and blue bags only); and traditional alternatives (paper bags — women used to make bags themselves)</t>
+        </is>
+      </c>
+      <c r="E1704" s="28" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: shared responsibility (everyone); regulated white/blue bag policy; traditional paper bags. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1705" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1705" s="28" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1705" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1705" s="28" t="inlineStr">
+        <is>
+          <t>NA - national government not named separately as responsible actor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1706" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1706" s="28" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1706" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1706" s="28" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1707" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1707" s="28" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1707" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1707" s="28" t="inlineStr">
+        <is>
+          <t>Municipal/national bag policy (black ban, white/blue only) shapes shop practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1708" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1708" s="28" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1708" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1708" s="28" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1709" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1709" s="28" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1709" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1709" s="28" t="inlineStr">
+        <is>
+          <t>NA - not mentioned separately from shop/private_companies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1710" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1710" s="28" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1710" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1710" s="28" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1711" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1711" s="28" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1711" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1711" s="28" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1712" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1712" s="28" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1712" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1712" s="28" t="inlineStr">
+        <is>
+          <t>"Everyone should be responsible"; customers request plastic bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1713" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1713" s="28" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1713" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1713" s="28" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1714" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1714" s="28" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1714" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1714" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner supplies bags and sells packaged goods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1715" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1715" s="28" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1715" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1715" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1716" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1716" s="28" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1716" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1716" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1717" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1717" s="28" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1717" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1717" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1718" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1718" s="28" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1718" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1718" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1719" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1719" s="28" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1719" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1719" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1720" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1720" s="28" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1720" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1720" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1721" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1721" s="28" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1721" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1721" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1722" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1722" s="28" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1722" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1722" s="28" t="inlineStr">
+        <is>
+          <t>Customers ask shop for plastic bags to manage home waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1723" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1723" s="28" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1723" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1723" s="28" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1724" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1724" s="28" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1724" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1724" s="28" t="inlineStr">
+        <is>
+          <t>NA - shop owner not blamed; portrayed as constrained by supply and customer demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1725" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1725" s="28" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1725" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1725" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1726" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1726" s="28" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1726" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1726" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1727" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1727" s="28" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1727" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1727" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named as specific target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1728" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1728" s="28" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1728" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1728" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1729" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1729" s="28" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1729" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1729" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1730" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1730" s="28" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1730" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1730" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1731" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1731" s="28" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1731" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1731" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1732" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1732" s="28" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1732" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1732" s="28" t="inlineStr">
+        <is>
+          <t>"Everyone should be responsible."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1733" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1733" s="28" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1733" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1733" s="28" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1734" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1734" s="28" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1734" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1734" s="28" t="inlineStr">
+        <is>
+          <t>Retailers/shops implied as part of "everyone."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1735" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1735" s="28" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1735" s="28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1735" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner as target group / retail actor (role 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1736" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1736" s="28" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1736" s="28" t="inlineStr">
+        <is>
+          <t>As a shop owner the interviewee is not very concerned about plastic pollution and sees it as practically unavoidable because "everything comes in plastic"; customers routinely ask for plastic bags to manage household waste; the shop complies with the black-bag ban by supplying only white and blue bags (3 NPR per blue bag) — but has no authority over production, national policy or customers' waste practices.</t>
+        </is>
+      </c>
+      <c r="E1736" s="28" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1737" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1737" s="28" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1737" s="28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1737" s="28" t="inlineStr">
+        <is>
+          <t>NA - Q6 not asked; implementation barriers not discussed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1738" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1738" s="28" t="inlineStr">
+        <is>
+          <t>Pol_tax</t>
+        </is>
+      </c>
+      <c r="D1738" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1738" s="28" t="inlineStr">
+        <is>
+          <t>3 NPR charge for one blue bag (price measure on permitted bags).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1739" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1739" s="28" t="inlineStr">
+        <is>
+          <t>Pol_ban</t>
+        </is>
+      </c>
+      <c r="D1739" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1739" s="28" t="inlineStr">
+        <is>
+          <t>Ban of black plastic bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1740" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1740" s="28" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1740" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1740" s="28" t="inlineStr">
+        <is>
+          <t>Black-bag ban partially effective — people don't use "dangerous black bags."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1741" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1741" s="28" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1741" s="28" t="inlineStr">
+        <is>
+          <t>Ban of black plastic bags in place; people are allowed to use only white and blue bags (3 NPR for one blue bag). Follow-up: "People don't use dangerous black bags" — partially effective for the specific black-bag ban.</t>
+        </is>
+      </c>
+      <c r="E1741" s="28" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1742" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1742" s="28" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1742" s="28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1742" s="28" t="inlineStr">
+        <is>
+          <t>Traditional paper bags; women used to make bags themselves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="28" t="inlineStr">
+        <is>
+          <t>NPL_23</t>
+        </is>
+      </c>
+      <c r="B1743" s="28" t="inlineStr">
+        <is>
+          <t>Shop owner (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1743" s="28" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1743" s="28" t="inlineStr">
+        <is>
+          <t>Previously people used paper bags to carry each item; women made bags themselves. Food culture changed, therefore there are more plastic bags now.</t>
+        </is>
+      </c>
+      <c r="E1743" s="28" t="inlineStr">
+        <is>
+          <t>Paper bags; women making bags; food culture change noted as driver of more plastic.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_24 coding for graduated young man interview (Feb 2026)
Code structured guideline notes for unnamed mechanical-engineering
graduate (moderate concern, awareness gaps, schools/young people as
policy focus). Updates workbook to NPL_1 through NPL_24.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="26">
+  <fills count="27">
     <fill>
       <patternFill/>
     </fill>
@@ -62,134 +62,140 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB5A2"/>
-        <bgColor rgb="00EBB5A2"/>
+        <fgColor rgb="00EBB4A2"/>
+        <bgColor rgb="00EBB4A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC8A2"/>
-        <bgColor rgb="00EBC8A2"/>
+        <fgColor rgb="00EBC6A2"/>
+        <bgColor rgb="00EBC6A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBDBA2"/>
-        <bgColor rgb="00EBDBA2"/>
+        <fgColor rgb="00EBD9A2"/>
+        <bgColor rgb="00EBD9A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8EBA2"/>
-        <bgColor rgb="00E8EBA2"/>
+        <fgColor rgb="00EBEBA2"/>
+        <bgColor rgb="00EBEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5EBA2"/>
-        <bgColor rgb="00D5EBA2"/>
+        <fgColor rgb="00D9EBA2"/>
+        <bgColor rgb="00D9EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C2EBA2"/>
-        <bgColor rgb="00C2EBA2"/>
+        <fgColor rgb="00C6EBA2"/>
+        <bgColor rgb="00C6EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00AFEBA2"/>
-        <bgColor rgb="00AFEBA2"/>
+        <fgColor rgb="00B4EBA2"/>
+        <bgColor rgb="00B4EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA8"/>
-        <bgColor rgb="00A2EBA8"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBBB"/>
-        <bgColor rgb="00A2EBBB"/>
+        <fgColor rgb="00A2EBB4"/>
+        <bgColor rgb="00A2EBB4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBCE"/>
-        <bgColor rgb="00A2EBCE"/>
+        <fgColor rgb="00A2EBC6"/>
+        <bgColor rgb="00A2EBC6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBE1"/>
-        <bgColor rgb="00A2EBE1"/>
+        <fgColor rgb="00A2EBD9"/>
+        <bgColor rgb="00A2EBD9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2E1EB"/>
-        <bgColor rgb="00A2E1EB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2CEEB"/>
-        <bgColor rgb="00A2CEEB"/>
+        <fgColor rgb="00A2D9EB"/>
+        <bgColor rgb="00A2D9EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2BBEB"/>
-        <bgColor rgb="00A2BBEB"/>
+        <fgColor rgb="00A2C6EB"/>
+        <bgColor rgb="00A2C6EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A8EB"/>
-        <bgColor rgb="00A2A8EB"/>
+        <fgColor rgb="00A2B4EB"/>
+        <bgColor rgb="00A2B4EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00AFA2EB"/>
-        <bgColor rgb="00AFA2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C2A2EB"/>
-        <bgColor rgb="00C2A2EB"/>
+        <fgColor rgb="00B4A2EB"/>
+        <bgColor rgb="00B4A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5A2EB"/>
-        <bgColor rgb="00D5A2EB"/>
+        <fgColor rgb="00C6A2EB"/>
+        <bgColor rgb="00C6A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8A2EB"/>
-        <bgColor rgb="00E8A2EB"/>
+        <fgColor rgb="00D9A2EB"/>
+        <bgColor rgb="00D9A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2DB"/>
-        <bgColor rgb="00EBA2DB"/>
+        <fgColor rgb="00EBA2EB"/>
+        <bgColor rgb="00EBA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C8"/>
-        <bgColor rgb="00EBA2C8"/>
+        <fgColor rgb="00EBA2D9"/>
+        <bgColor rgb="00EBA2D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B5"/>
-        <bgColor rgb="00EBA2B5"/>
+        <fgColor rgb="00EBA2C6"/>
+        <bgColor rgb="00EBA2C6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B4"/>
+        <bgColor rgb="00EBA2B4"/>
       </patternFill>
     </fill>
   </fills>
@@ -219,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -303,6 +309,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -670,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -689,7 +698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_23, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_24, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -865,82 +874,89 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  24. NPL_24 - Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026). Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from guideline/field notes only. Awareness/education focus; young people and schools as policy targets. Q5, Q6, Q8 traditions and Q10 not asked.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_23, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_24, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_23) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_24) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
-    </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2127,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ24"/>
+  <dimension ref="A1:CQ25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13675,6 +13691,483 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>science</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O25" s="29" t="inlineStr">
+        <is>
+          <t>health ("plastic is toxic, it affects health") and environment ("bad for the environment"; waste "everywhere on the streets")</t>
+        </is>
+      </c>
+      <c r="P25" s="29" t="inlineStr">
+        <is>
+          <t>public health (toxic plastics affecting health); the environment; and residents affected by street litter/waste accumulation</t>
+        </is>
+      </c>
+      <c r="Q25" s="29" t="inlineStr">
+        <is>
+          <t>society-wide lack of awareness ("no awareness in society"; elderly people "have no knowledge about plastics pollution"); continued plastic use despite municipal anti-plastic messaging ("everyone continues to use it"); and inadequate school education (respondent "was not taught about it at school")</t>
+        </is>
+      </c>
+      <c r="R25" s="29" t="inlineStr">
+        <is>
+          <t>young people sharing information with elderly; schools and education campaigns; municipal anti-plastic initiatives; and raising public awareness ("people need to be aware")</t>
+        </is>
+      </c>
+      <c r="S25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AA25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AT25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AU25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA25" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB25" s="29" t="inlineStr">
+        <is>
+          <t>As a recently graduated young man in mechanical engineering the interviewee is moderately concerned about street litter and plastic's health/environmental impacts but has no formal role in waste governance — can advocate awareness among elderly and peers but was not taught about plastic pollution at school and cannot implement municipal policies.</t>
+        </is>
+      </c>
+      <c r="BC25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BH25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BI25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BM25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW25" s="29" t="inlineStr">
+        <is>
+          <t>Municipalities' idea was not to use plastics, but "everyone continues to use it" — awareness/education measures ineffective so far; respondent was not taught about plastic pollution at school.</t>
+        </is>
+      </c>
+      <c r="BX25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BY25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE25" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CL25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CM25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CO25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP25" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CQ25" s="29" t="inlineStr">
+        <is>
+          <t>Master list label: "24. Graduated young man (unnamed)", affiliation: graduated young man; area of expertise: mechanical engineering sphere. Interviewee name not given. Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Q5 (responsibility), Q6/Q6 follow-up, Q8 traditions follow-up and Q10 not asked. Same interview date as NPL_21–NPL_23 but distinct young-educated-respondent perspective. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13686,7 +14179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1743"/>
+  <dimension ref="A1:E1792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -60757,6 +61250,1329 @@
         </is>
       </c>
     </row>
+    <row r="1744">
+      <c r="A1744" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1744" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1744" s="29" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1744" s="29" t="inlineStr">
+        <is>
+          <t>science</t>
+        </is>
+      </c>
+      <c r="E1744" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man in mechanical engineering sphere — coded as science.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1745" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1745" s="29" t="inlineStr">
+        <is>
+          <t>Problem_awareness_pop</t>
+        </is>
+      </c>
+      <c r="D1745" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1745" s="29" t="inlineStr">
+        <is>
+          <t>"No awareness in society"; elderly people "have no knowledge about plastics pollution."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1746" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1746" s="29" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1746" s="29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E1746" s="29" t="inlineStr">
+        <is>
+          <t>"A little bit concerned" because waste is "everywhere on the streets."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1747" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1747" s="29" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1747" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1747" s="29" t="inlineStr">
+        <is>
+          <t>Waste "everywhere on the streets."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1748" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1748" s="29" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1748" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1748" s="29" t="inlineStr">
+        <is>
+          <t>"Everyone continues to use" plastic despite municipal messaging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1749" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1749" s="29" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1749" s="29" t="inlineStr">
+        <is>
+          <t>health ("plastic is toxic, it affects health") and environment ("bad for the environment"; waste "everywhere on the streets")</t>
+        </is>
+      </c>
+      <c r="E1749" s="29" t="inlineStr">
+        <is>
+          <t>Health (toxic plastics) and environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1750" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1750" s="29" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1750" s="29" t="inlineStr">
+        <is>
+          <t>public health (toxic plastics affecting health); the environment; and residents affected by street litter/waste accumulation</t>
+        </is>
+      </c>
+      <c r="E1750" s="29" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: health; environment; residents affected by street litter. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1751" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1751" s="29" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1751" s="29" t="inlineStr">
+        <is>
+          <t>society-wide lack of awareness ("no awareness in society"; elderly people "have no knowledge about plastics pollution"); continued plastic use despite municipal anti-plastic messaging ("everyone continues to use it"); and inadequate school education (respondent "was not taught about it at school")</t>
+        </is>
+      </c>
+      <c r="E1751" s="29" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: societal lack of awareness; elderly knowledge gap; continued use; inadequate school education. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1752" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1752" s="29" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1752" s="29" t="inlineStr">
+        <is>
+          <t>young people sharing information with elderly; schools and education campaigns; municipal anti-plastic initiatives; and raising public awareness ("people need to be aware")</t>
+        </is>
+      </c>
+      <c r="E1752" s="29" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: young people; schools; awareness campaigns; intergenerational knowledge sharing. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1753" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1753" s="29" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1753" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1753" s="29" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1754" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1754" s="29" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1754" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1754" s="29" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1755" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1755" s="29" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1755" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1755" s="29" t="inlineStr">
+        <is>
+          <t>Municipalities promoted idea not to use plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1756" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1756" s="29" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1756" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1756" s="29" t="inlineStr">
+        <is>
+          <t>Young people should share information with elderly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1757" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1757" s="29" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1757" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1757" s="29" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1758" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1758" s="29" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1758" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1758" s="29" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1759" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1759" s="29" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1759" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1759" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named as formal responsible actor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1760" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1760" s="29" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1760" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1760" s="29" t="inlineStr">
+        <is>
+          <t>Elderly households lack knowledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1761" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1761" s="29" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1761" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1761" s="29" t="inlineStr">
+        <is>
+          <t>Schools should teach plastic pollution (respondent was not taught).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1762" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1762" s="29" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1762" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1762" s="29" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1763" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1763" s="29" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1763" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1763" s="29" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1764" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1764" s="29" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1764" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1764" s="29" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1765" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1765" s="29" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1765" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1765" s="29" t="inlineStr">
+        <is>
+          <t>NA - municipality portrayed as trying but ineffective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1766" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1766" s="29" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1766" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1766" s="29" t="inlineStr">
+        <is>
+          <t>NA - young people portrayed as solution, not cause.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1767" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1767" s="29" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1767" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1767" s="29" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1768" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1768" s="29" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1768" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1768" s="29" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1769" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1769" s="29" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1769" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1769" s="29" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1770" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1770" s="29" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1770" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1770" s="29" t="inlineStr">
+        <is>
+          <t>Elderly people lack knowledge about plastic pollution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1771" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1771" s="29" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1771" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1771" s="29" t="inlineStr">
+        <is>
+          <t>NA - schools portrayed as needing strengthening, not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1772" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1772" s="29" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1772" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1772" s="29" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1773" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1773" s="29" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1773" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1773" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1774" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1774" s="29" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1774" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1774" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1775" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1775" s="29" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1775" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1775" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named as specific target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1776" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1776" s="29" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1776" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1776" s="29" t="inlineStr">
+        <is>
+          <t>"Young people" should be focus of future policies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1777" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1777" s="29" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1777" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1777" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1778" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1778" s="29" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1778" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1778" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1779" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1779" s="29" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1779" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1779" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1780" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1780" s="29" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1780" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1780" s="29" t="inlineStr">
+        <is>
+          <t>Elderly people targeted via young people's information-sharing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1781" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1781" s="29" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1781" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1781" s="29" t="inlineStr">
+        <is>
+          <t>"Schools" named as policy focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1782" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1782" s="29" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1782" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1782" s="29" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1783" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1783" s="29" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1783" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1783" s="29" t="inlineStr">
+        <is>
+          <t>Young graduate as target group / awareness advocate (role 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1784" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1784" s="29" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1784" s="29" t="inlineStr">
+        <is>
+          <t>As a recently graduated young man in mechanical engineering the interviewee is moderately concerned about street litter and plastic's health/environmental impacts but has no formal role in waste governance — can advocate awareness among elderly and peers but was not taught about plastic pollution at school and cannot implement municipal policies.</t>
+        </is>
+      </c>
+      <c r="E1784" s="29" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1785" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1785" s="29" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1785" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1785" s="29" t="inlineStr">
+        <is>
+          <t>NA - Q6 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1786" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1786" s="29" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1786" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1786" s="29" t="inlineStr">
+        <is>
+          <t>Municipalities' idea was not to use plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1787" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1787" s="29" t="inlineStr">
+        <is>
+          <t>Pol_education</t>
+        </is>
+      </c>
+      <c r="D1787" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1787" s="29" t="inlineStr">
+        <is>
+          <t>School education on plastic pollution absent for this respondent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1788" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1788" s="29" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1788" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1788" s="29" t="inlineStr">
+        <is>
+          <t>Everyone continues to use plastic — municipal message ineffective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1789" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1789" s="29" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1789" s="29" t="inlineStr">
+        <is>
+          <t>Municipalities' idea was not to use plastics, but "everyone continues to use it" — awareness/education measures ineffective so far; respondent was not taught about plastic pollution at school.</t>
+        </is>
+      </c>
+      <c r="E1789" s="29" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1790" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1790" s="29" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1790" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1790" s="29" t="inlineStr">
+        <is>
+          <t>"People need to be aware."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1791" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1791" s="29" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1791" s="29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1791" s="29" t="inlineStr">
+        <is>
+          <t>Young people should share information with elderly; schools as focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="29" t="inlineStr">
+        <is>
+          <t>NPL_24</t>
+        </is>
+      </c>
+      <c r="B1792" s="29" t="inlineStr">
+        <is>
+          <t>Graduated young man (unnamed), mechanical engineering sphere, Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1792" s="29" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1792" s="29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1792" s="29" t="inlineStr">
+        <is>
+          <t>NA - Q8 traditions follow-up not asked.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_25 coding for third ordinary-person interview (Feb 2026)
Code structured guideline notes for unnamed ordinary-person respondent
(high concern, health/diseases, diapers/packaging, temple taboo and god
monuments). Distinct from NPL_21/NPL_22. Updates workbook to NPL_25.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="28">
     <fill>
       <patternFill/>
     </fill>
@@ -62,140 +62,146 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB4A2"/>
-        <bgColor rgb="00EBB4A2"/>
+        <fgColor rgb="00EBB3A2"/>
+        <bgColor rgb="00EBB3A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC6A2"/>
-        <bgColor rgb="00EBC6A2"/>
+        <fgColor rgb="00EBC5A2"/>
+        <bgColor rgb="00EBC5A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD9A2"/>
-        <bgColor rgb="00EBD9A2"/>
+        <fgColor rgb="00EBD6A2"/>
+        <bgColor rgb="00EBD6A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBEBA2"/>
-        <bgColor rgb="00EBEBA2"/>
+        <fgColor rgb="00EBE8A2"/>
+        <bgColor rgb="00EBE8A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EBA2"/>
-        <bgColor rgb="00D9EBA2"/>
+        <fgColor rgb="00DCEBA2"/>
+        <bgColor rgb="00DCEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EBA2"/>
-        <bgColor rgb="00C6EBA2"/>
+        <fgColor rgb="00CBEBA2"/>
+        <bgColor rgb="00CBEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4EBA2"/>
-        <bgColor rgb="00B4EBA2"/>
+        <fgColor rgb="00B9EBA2"/>
+        <bgColor rgb="00B9EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA2"/>
-        <bgColor rgb="00A2EBA2"/>
+        <fgColor rgb="00A8EBA2"/>
+        <bgColor rgb="00A8EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBB4"/>
-        <bgColor rgb="00A2EBB4"/>
+        <fgColor rgb="00A2EBAE"/>
+        <bgColor rgb="00A2EBAE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBC6"/>
-        <bgColor rgb="00A2EBC6"/>
+        <fgColor rgb="00A2EBBF"/>
+        <bgColor rgb="00A2EBBF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD9"/>
-        <bgColor rgb="00A2EBD9"/>
+        <fgColor rgb="00A2EBD1"/>
+        <bgColor rgb="00A2EBD1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBE2"/>
+        <bgColor rgb="00A2EBE2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D9EB"/>
-        <bgColor rgb="00A2D9EB"/>
+        <fgColor rgb="00A2E2EB"/>
+        <bgColor rgb="00A2E2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2C6EB"/>
-        <bgColor rgb="00A2C6EB"/>
+        <fgColor rgb="00A2D1EB"/>
+        <bgColor rgb="00A2D1EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2B4EB"/>
-        <bgColor rgb="00A2B4EB"/>
+        <fgColor rgb="00A2BFEB"/>
+        <bgColor rgb="00A2BFEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A2EB"/>
-        <bgColor rgb="00A2A2EB"/>
+        <fgColor rgb="00A2AEEB"/>
+        <bgColor rgb="00A2AEEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4A2EB"/>
-        <bgColor rgb="00B4A2EB"/>
+        <fgColor rgb="00A8A2EB"/>
+        <bgColor rgb="00A8A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6A2EB"/>
-        <bgColor rgb="00C6A2EB"/>
+        <fgColor rgb="00B9A2EB"/>
+        <bgColor rgb="00B9A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9A2EB"/>
-        <bgColor rgb="00D9A2EB"/>
+        <fgColor rgb="00CBA2EB"/>
+        <bgColor rgb="00CBA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2EB"/>
-        <bgColor rgb="00EBA2EB"/>
+        <fgColor rgb="00DCA2EB"/>
+        <bgColor rgb="00DCA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D9"/>
-        <bgColor rgb="00EBA2D9"/>
+        <fgColor rgb="00EBA2E8"/>
+        <bgColor rgb="00EBA2E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C6"/>
-        <bgColor rgb="00EBA2C6"/>
+        <fgColor rgb="00EBA2D6"/>
+        <bgColor rgb="00EBA2D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B4"/>
-        <bgColor rgb="00EBA2B4"/>
+        <fgColor rgb="00EBA2C5"/>
+        <bgColor rgb="00EBA2C5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B3"/>
+        <bgColor rgb="00EBA2B3"/>
       </patternFill>
     </fill>
   </fills>
@@ -225,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -312,6 +318,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -679,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -698,7 +707,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_24, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_25, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -881,82 +890,89 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  25. NPL_25 - Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026). Same interview team/date as NPL_21/NPL_22 but distinct (high concern, health/diseases, diapers/packaging, religious taboo at temples, god monuments). Q4 effectiveness, Q6 level follow-up, Q9 and Q10 not asked.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_24, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_25, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_24) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_25) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
-    </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2143,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ25"/>
+  <dimension ref="A1:CQ26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14168,6 +14184,483 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="C26" s="30" t="inlineStr">
+        <is>
+          <t>households</t>
+        </is>
+      </c>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F26" s="30" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O26" s="30" t="inlineStr">
+        <is>
+          <t>health ("impact on health"; "different diseases appear")</t>
+        </is>
+      </c>
+      <c r="P26" s="30" t="inlineStr">
+        <is>
+          <t>public health — people affected by diseases linked to plastic pollution</t>
+        </is>
+      </c>
+      <c r="Q26" s="30" t="inlineStr">
+        <is>
+          <t>government ("not much has been done yet by government"); households/residents ("people want to have a comfortable life" with "no wish to make efforts for segregation"); and rising plastic consumption (more packaging, plastic bottles, diapers for babies and elderly people) — plastics that unlike other waste "can[not] be decomposed"</t>
+        </is>
+      </c>
+      <c r="R26" s="30" t="inlineStr">
+        <is>
+          <t>local government and mayor (responsible for waste management; daily collection vehicle); religious/cultural norms prohibiting waste dumping near saint places/temples; and municipal use of god monuments at open dumping sites to deter littering</t>
+        </is>
+      </c>
+      <c r="S26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AO26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AY26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA26" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB26" s="30" t="inlineStr">
+        <is>
+          <t>As an ordinary resident the interviewee is very concerned about plastic's health impacts but relies on the municipality's daily collection vehicle and has "no wish to make efforts for segregation"; cannot influence government action beyond noting that "not much has been done yet" — comfort-oriented plastic use (packaging, bottles, diapers) continues.</t>
+        </is>
+      </c>
+      <c r="BC26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BG26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BH26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BL26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BV26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BW26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BX26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BY26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CF26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CJ26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CL26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CM26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN26" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO26" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP26" s="30" t="inlineStr">
+        <is>
+          <t>Religious/cultural taboo against throwing waste near saint places (temples) — municipalities strategically place god monuments at open dumping sites. However, "people don't want to return to traditions"; "plastics make life more comfortable."</t>
+        </is>
+      </c>
+      <c r="CQ26" s="30" t="inlineStr">
+        <is>
+          <t>Master list label: "25. Ordinary person (unnamed, 3rd respondent)", affiliation: ordinary person/citizen. Interviewee name not given. Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Third ordinary-person interview on the same date as NPL_21/NPL_22 — distinct respondent with high concern and health focus; unique religious/cultural anti-littering mechanism (temples, god monuments). Q4 effectiveness follow-up, Q6 level follow-up, Q9 and Q10 not asked. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14179,7 +14672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1792"/>
+  <dimension ref="A1:E1843"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -62573,6 +63066,1383 @@
         </is>
       </c>
     </row>
+    <row r="1793">
+      <c r="A1793" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1793" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1793" s="30" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1793" s="30" t="inlineStr">
+        <is>
+          <t>households</t>
+        </is>
+      </c>
+      <c r="E1793" s="30" t="inlineStr">
+        <is>
+          <t>Interviewee described as "ordinary person" — coded as households.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1794" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1794" s="30" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1794" s="30" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1794" s="30" t="inlineStr">
+        <is>
+          <t>"Very much concerned."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1795" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1795" s="30" t="inlineStr">
+        <is>
+          <t>Problem_consumption</t>
+        </is>
+      </c>
+      <c r="D1795" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1795" s="30" t="inlineStr">
+        <is>
+          <t>More plastics in packaging, plastic bottles; use of diapers by babies and elderly people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1796" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1796" s="30" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1796" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1796" s="30" t="inlineStr">
+        <is>
+          <t>Plastics cannot be decomposed unlike some other waste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1797" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1797" s="30" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1797" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1797" s="30" t="inlineStr">
+        <is>
+          <t>Government "not much has been done yet"; residents unwilling to segregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1798" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1798" s="30" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1798" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1798" s="30" t="inlineStr">
+        <is>
+          <t>"Plastics make life more comfortable"; people don't want to return to traditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1799" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1799" s="30" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1799" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1799" s="30" t="inlineStr">
+        <is>
+          <t>"No wish to make efforts for segregation."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1800" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1800" s="30" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1800" s="30" t="inlineStr">
+        <is>
+          <t>health ("impact on health"; "different diseases appear")</t>
+        </is>
+      </c>
+      <c r="E1800" s="30" t="inlineStr">
+        <is>
+          <t>Health — "different diseases appear."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1801" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1801" s="30" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1801" s="30" t="inlineStr">
+        <is>
+          <t>public health — people affected by diseases linked to plastic pollution</t>
+        </is>
+      </c>
+      <c r="E1801" s="30" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: public health/disease sufferers. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1802" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1802" s="30" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1802" s="30" t="inlineStr">
+        <is>
+          <t>government ("not much has been done yet by government"); households/residents ("people want to have a comfortable life" with "no wish to make efforts for segregation"); and rising plastic consumption (more packaging, plastic bottles, diapers for babies and elderly people) — plastics that unlike other waste "can[not] be decomposed"</t>
+        </is>
+      </c>
+      <c r="E1802" s="30" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: government inaction; household comfort-seeking; rising plastic consumption (packaging, bottles, diapers). No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1803" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1803" s="30" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1803" s="30" t="inlineStr">
+        <is>
+          <t>local government and mayor (responsible for waste management; daily collection vehicle); religious/cultural norms prohibiting waste dumping near saint places/temples; and municipal use of god monuments at open dumping sites to deter littering</t>
+        </is>
+      </c>
+      <c r="E1803" s="30" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: local government/mayor; daily collection; religious taboo at temples; god monuments at dump sites. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1804" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1804" s="30" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1804" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1804" s="30" t="inlineStr">
+        <is>
+          <t>Government cited as not having done much yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1805" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1805" s="30" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1805" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1805" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1806" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1806" s="30" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1806" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1806" s="30" t="inlineStr">
+        <is>
+          <t>"Local government; mayor" responsible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1807" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1807" s="30" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1807" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1807" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1808" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1808" s="30" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1808" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1808" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1809" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1809" s="30" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1809" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1809" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1810" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1810" s="30" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1810" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1810" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1811" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1811" s="30" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1811" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1811" s="30" t="inlineStr">
+        <is>
+          <t>Households produce waste including diapers; unwilling to segregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1812" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1812" s="30" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1812" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1812" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1813" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1813" s="30" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1813" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1813" s="30" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1814" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1814" s="30" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1814" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1814" s="30" t="inlineStr">
+        <is>
+          <t>"Not much has been done yet by government."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1815" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1815" s="30" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1815" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1815" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1816" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1816" s="30" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1816" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1816" s="30" t="inlineStr">
+        <is>
+          <t>NA - local government portrayed as responsible/collection actor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1817" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1817" s="30" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1817" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1817" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1818" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1818" s="30" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1818" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1818" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1819" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1819" s="30" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1819" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1819" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1820" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1820" s="30" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1820" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1820" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1821" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1821" s="30" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1821" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1821" s="30" t="inlineStr">
+        <is>
+          <t>Comfort-oriented behaviour; no wish to segregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1822" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1822" s="30" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1822" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1822" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1823" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1823" s="30" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1823" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1823" s="30" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1824" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1824" s="30" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1824" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1824" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named as specific target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1825" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1825" s="30" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1825" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1825" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1826" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1826" s="30" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1826" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1826" s="30" t="inlineStr">
+        <is>
+          <t>Local government/mayor named as responsible actor to strengthen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1827" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1827" s="30" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1827" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1827" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1828" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1828" s="30" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1828" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1828" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1829" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1829" s="30" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1829" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1829" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1830" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1830" s="30" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1830" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1830" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1831" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1831" s="30" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1831" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1831" s="30" t="inlineStr">
+        <is>
+          <t>NA - Q9 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1832" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1832" s="30" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1832" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1832" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1833" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1833" s="30" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1833" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1833" s="30" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1834" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1834" s="30" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1834" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1834" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary citizen as target group (role 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1835" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1835" s="30" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1835" s="30" t="inlineStr">
+        <is>
+          <t>As an ordinary resident the interviewee is very concerned about plastic's health impacts but relies on the municipality's daily collection vehicle and has "no wish to make efforts for segregation"; cannot influence government action beyond noting that "not much has been done yet" — comfort-oriented plastic use (packaging, bottles, diapers) continues.</t>
+        </is>
+      </c>
+      <c r="E1835" s="30" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1836" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1836" s="30" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1836" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1836" s="30" t="inlineStr">
+        <is>
+          <t>Government has not done much; residents unwilling to segregate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1837" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1837" s="30" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1837" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1837" s="30" t="inlineStr">
+        <is>
+          <t>Religious/cultural enforcement via saint places/temples and god monuments at open dumping sites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1838" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1838" s="30" t="inlineStr">
+        <is>
+          <t>Pol_waste_collection</t>
+        </is>
+      </c>
+      <c r="D1838" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1838" s="30" t="inlineStr">
+        <is>
+          <t>Daily municipal collection vehicle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1839" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1839" s="30" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1839" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1839" s="30" t="inlineStr">
+        <is>
+          <t>NA - Q4 effectiveness follow-up not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1840" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1840" s="30" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1840" s="30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1840" s="30" t="inlineStr">
+        <is>
+          <t>NA - Q4 effectiveness follow-up not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1841" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1841" s="30" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1841" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1841" s="30" t="inlineStr">
+        <is>
+          <t>Cultural/religious norms around saint places deter open dumping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1842" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1842" s="30" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1842" s="30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1842" s="30" t="inlineStr">
+        <is>
+          <t>Municipal god monuments at open spaces to reduce littering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" s="30" t="inlineStr">
+        <is>
+          <t>NPL_25</t>
+        </is>
+      </c>
+      <c r="B1843" s="30" t="inlineStr">
+        <is>
+          <t>Ordinary person / citizen (unnamed, 3rd respondent), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording; distinct from NPL_21/NPL_22)</t>
+        </is>
+      </c>
+      <c r="C1843" s="30" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1843" s="30" t="inlineStr">
+        <is>
+          <t>Religious/cultural taboo against throwing waste near saint places (temples) — municipalities strategically place god monuments at open dumping sites. However, "people don't want to return to traditions"; "plastics make life more comfortable."</t>
+        </is>
+      </c>
+      <c r="E1843" s="30" t="inlineStr">
+        <is>
+          <t>Temple/saint-place taboo against waste dumping; god monuments — but people don't want to return to older traditions.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_26 coding for cafe workers interview (Feb 2026)
Code structured guideline notes for unnamed cafe workers (concern about
burning smog, collection centres needed, ineffective anti-plastic
campaign, local government enforcement). Updates workbook to NPL_26.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="28">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -68,134 +68,140 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC5A2"/>
-        <bgColor rgb="00EBC5A2"/>
+        <fgColor rgb="00EBC4A2"/>
+        <bgColor rgb="00EBC4A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD6A2"/>
-        <bgColor rgb="00EBD6A2"/>
+        <fgColor rgb="00EBD4A2"/>
+        <bgColor rgb="00EBD4A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE8A2"/>
-        <bgColor rgb="00EBE8A2"/>
+        <fgColor rgb="00EBE5A2"/>
+        <bgColor rgb="00EBE5A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCEBA2"/>
-        <bgColor rgb="00DCEBA2"/>
+        <fgColor rgb="00E0EBA2"/>
+        <bgColor rgb="00E0EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CBEBA2"/>
-        <bgColor rgb="00CBEBA2"/>
+        <fgColor rgb="00CFEBA2"/>
+        <bgColor rgb="00CFEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B9EBA2"/>
-        <bgColor rgb="00B9EBA2"/>
+        <fgColor rgb="00BEEBA2"/>
+        <bgColor rgb="00BEEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A8EBA2"/>
-        <bgColor rgb="00A8EBA2"/>
+        <fgColor rgb="00ADEBA2"/>
+        <bgColor rgb="00ADEBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBAE"/>
-        <bgColor rgb="00A2EBAE"/>
+        <fgColor rgb="00A2EBA8"/>
+        <bgColor rgb="00A2EBA8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBBF"/>
-        <bgColor rgb="00A2EBBF"/>
+        <fgColor rgb="00A2EBB8"/>
+        <bgColor rgb="00A2EBB8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBD1"/>
-        <bgColor rgb="00A2EBD1"/>
+        <fgColor rgb="00A2EBC9"/>
+        <bgColor rgb="00A2EBC9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBE2"/>
-        <bgColor rgb="00A2EBE2"/>
+        <fgColor rgb="00A2EBDA"/>
+        <bgColor rgb="00A2EBDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2E2EB"/>
-        <bgColor rgb="00A2E2EB"/>
+        <fgColor rgb="00A2EBEB"/>
+        <bgColor rgb="00A2EBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2D1EB"/>
-        <bgColor rgb="00A2D1EB"/>
+        <fgColor rgb="00A2DAEB"/>
+        <bgColor rgb="00A2DAEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2BFEB"/>
-        <bgColor rgb="00A2BFEB"/>
+        <fgColor rgb="00A2C9EB"/>
+        <bgColor rgb="00A2C9EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2AEEB"/>
-        <bgColor rgb="00A2AEEB"/>
+        <fgColor rgb="00A2B8EB"/>
+        <bgColor rgb="00A2B8EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A8A2EB"/>
-        <bgColor rgb="00A8A2EB"/>
+        <fgColor rgb="00A2A8EB"/>
+        <bgColor rgb="00A2A8EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B9A2EB"/>
-        <bgColor rgb="00B9A2EB"/>
+        <fgColor rgb="00ADA2EB"/>
+        <bgColor rgb="00ADA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CBA2EB"/>
-        <bgColor rgb="00CBA2EB"/>
+        <fgColor rgb="00BEA2EB"/>
+        <bgColor rgb="00BEA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCA2EB"/>
-        <bgColor rgb="00DCA2EB"/>
+        <fgColor rgb="00CFA2EB"/>
+        <bgColor rgb="00CFA2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E8"/>
-        <bgColor rgb="00EBA2E8"/>
+        <fgColor rgb="00E0A2EB"/>
+        <bgColor rgb="00E0A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D6"/>
-        <bgColor rgb="00EBA2D6"/>
+        <fgColor rgb="00EBA2E5"/>
+        <bgColor rgb="00EBA2E5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C5"/>
-        <bgColor rgb="00EBA2C5"/>
+        <fgColor rgb="00EBA2D4"/>
+        <bgColor rgb="00EBA2D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2C4"/>
+        <bgColor rgb="00EBA2C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -231,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -321,6 +327,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -688,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -707,7 +716,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_25, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_26, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -897,82 +906,89 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  26. NPL_26 - Cafe workers (unnamed), Nepal (17 February 2026). Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from guideline/field notes only. Collection centres, anti-plastic campaign, dustbins, alternatives. Q6, Q8 traditions, Q9 and Q10 not asked.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_25, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_26, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
-    </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_25) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_26) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-    </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2159,7 +2175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ26"/>
+  <dimension ref="A1:CQ27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14661,6 +14677,483 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>private_companies</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F27" s="31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O27" s="31" t="inlineStr">
+        <is>
+          <t>visual/aesthetic pollution ("it doesn't look nice"), air pollution (smog after burning — "that's the only effect they know"), animals, water and agriculture ("plants cannot grow up")</t>
+        </is>
+      </c>
+      <c r="P27" s="31" t="inlineStr">
+        <is>
+          <t>animals, water bodies and agriculture (plants cannot grow); residents affected by visual pollution and smog from burning plastics</t>
+        </is>
+      </c>
+      <c r="Q27" s="31" t="inlineStr">
+        <is>
+          <t>government ("does not enforce" and "there is no monitoring"; national anti-plastic campaign "did not work well"); lack of plastics collection infrastructure; and continued plastic production/consumption</t>
+        </is>
+      </c>
+      <c r="R27" s="31" t="inlineStr">
+        <is>
+          <t>local government enforcing regulation; plastics collection centers; dustbins everywhere; alternative plastic products; and stopping plastic production</t>
+        </is>
+      </c>
+      <c r="S27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AE27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AF27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AH27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AY27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AZ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA27" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BB27" s="31" t="inlineStr">
+        <is>
+          <t>As cafe workers the interviewees are concerned about plastic pollution (mainly smog from burning and visual impacts) but have limited knowledge of broader effects; operate in the food-service sector with no authority over national campaigns, enforcement, collection-centre infrastructure or production bans — rely on local government action.</t>
+        </is>
+      </c>
+      <c r="BC27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BD27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BH27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BI27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BL27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BW27" s="31" t="inlineStr">
+        <is>
+          <t>Campaign not to use plastics "all over Nepal" but "it did not work well" — measures "not very effective so far"; government "does not enforce" and "there is no monitoring."</t>
+        </is>
+      </c>
+      <c r="BX27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BY27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CB27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CE27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CF27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CJ27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CL27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN27" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP27" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CQ27" s="31" t="inlineStr">
+        <is>
+          <t>Master list label: "26. Cafe workers (unnamed)", affiliation: cafe workers. General information lists interviewee name as "Cafe" (likely cafe name or placeholder; individual names not given). Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Q6 not asked (enforcement/monitoring gap noted in passing). Q8 traditions follow-up, Q9 and Q10 not asked. Same interview date as NPL_21–NPL_25. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14672,7 +15165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1843"/>
+  <dimension ref="A1:E1900"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -64443,6 +64936,1545 @@
         </is>
       </c>
     </row>
+    <row r="1844">
+      <c r="A1844" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1844" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1844" s="31" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1844" s="31" t="inlineStr">
+        <is>
+          <t>private_companies</t>
+        </is>
+      </c>
+      <c r="E1844" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers — coded as private_companies (food-service sector).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1845" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1845" s="31" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1845" s="31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E1845" s="31" t="inlineStr">
+        <is>
+          <t>"They are concerned" but smog from burning is "the only effect they know" — moderate concern with limited knowledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1846" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1846" s="31" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1846" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1846" s="31" t="inlineStr">
+        <is>
+          <t>"It doesn't look nice" — visual/aesthetic impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1847" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1847" s="31" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1847" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1847" s="31" t="inlineStr">
+        <is>
+          <t>Need to "create plastics collection centers."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1848" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1848" s="31" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1848" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1848" s="31" t="inlineStr">
+        <is>
+          <t>Collection-centre infrastructure gap identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1849" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1849" s="31" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1849" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1849" s="31" t="inlineStr">
+        <is>
+          <t>"Stop producing plastics" suggested as solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1850" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1850" s="31" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1850" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1850" s="31" t="inlineStr">
+        <is>
+          <t>"Alternative plastic products" suggested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1851" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1851" s="31" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1851" s="31" t="inlineStr">
+        <is>
+          <t>visual/aesthetic pollution ("it doesn't look nice"), air pollution (smog after burning — "that's the only effect they know"), animals, water and agriculture ("plants cannot grow up")</t>
+        </is>
+      </c>
+      <c r="E1851" s="31" t="inlineStr">
+        <is>
+          <t>Visual pollution, smog from burning, animals, water, agriculture (plants cannot grow).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1852" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1852" s="31" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1852" s="31" t="inlineStr">
+        <is>
+          <t>animals, water bodies and agriculture (plants cannot grow); residents affected by visual pollution and smog from burning plastics</t>
+        </is>
+      </c>
+      <c r="E1852" s="31" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: animals; water; agriculture; residents (visual/smog). No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1853" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1853" s="31" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1853" s="31" t="inlineStr">
+        <is>
+          <t>government ("does not enforce" and "there is no monitoring"; national anti-plastic campaign "did not work well"); lack of plastics collection infrastructure; and continued plastic production/consumption</t>
+        </is>
+      </c>
+      <c r="E1853" s="31" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: government (weak enforcement/monitoring, ineffective campaign); lack of collection infrastructure; continued production. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1854" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1854" s="31" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1854" s="31" t="inlineStr">
+        <is>
+          <t>local government enforcing regulation; plastics collection centers; dustbins everywhere; alternative plastic products; and stopping plastic production</t>
+        </is>
+      </c>
+      <c r="E1854" s="31" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: local government; collection centers; dustbins; alternatives; production stop. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1855" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1855" s="31" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1855" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1855" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named as formal responsible actor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1856" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1856" s="31" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1856" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1856" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1857" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1857" s="31" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1857" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1857" s="31" t="inlineStr">
+        <is>
+          <t>"Local government" responsible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1858" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1858" s="31" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1858" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1858" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1859" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1859" s="31" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1859" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1859" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1860" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1860" s="31" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1860" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1860" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1861" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1861" s="31" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1861" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1861" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1862" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1862" s="31" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1862" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1862" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1863" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1863" s="31" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1863" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1863" s="31" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1864" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1864" s="31" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1864" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1864" s="31" t="inlineStr">
+        <is>
+          <t>NA - cafe workers are respondents, not named as responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1865" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1865" s="31" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1865" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1865" s="31" t="inlineStr">
+        <is>
+          <t>"Govt. does not enforce, there is no monitoring"; campaign ineffective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1866" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1866" s="31" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1866" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1866" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1867" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1867" s="31" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1867" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1867" s="31" t="inlineStr">
+        <is>
+          <t>NA - local government portrayed as actor to strengthen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1868" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1868" s="31" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1868" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1868" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1869" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1869" s="31" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1869" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1869" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1870" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1870" s="31" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1870" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1870" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1871" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1871" s="31" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1871" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1871" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1872" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1872" s="31" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1872" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1872" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1873" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1873" s="31" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1873" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1873" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1874" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1874" s="31" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1874" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1874" s="31" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1875" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1875" s="31" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1875" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1875" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1876" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1876" s="31" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1876" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1876" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1877" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1877" s="31" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1877" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1877" s="31" t="inlineStr">
+        <is>
+          <t>"Local government has to enforce the regulation"; local government "in charge."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1878" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1878" s="31" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1878" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1878" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1879" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1879" s="31" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1879" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1879" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1880" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1880" s="31" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1880" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1880" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1881" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1881" s="31" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1881" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1881" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1882" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1882" s="31" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1882" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1882" s="31" t="inlineStr">
+        <is>
+          <t>NA - Q9 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1883" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1883" s="31" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1883" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1883" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1884" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1884" s="31" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1884" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1884" s="31" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1885" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1885" s="31" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1885" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E1885" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers as target group / food-service sector (role 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1886" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1886" s="31" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1886" s="31" t="inlineStr">
+        <is>
+          <t>As cafe workers the interviewees are concerned about plastic pollution (mainly smog from burning and visual impacts) but have limited knowledge of broader effects; operate in the food-service sector with no authority over national campaigns, enforcement, collection-centre infrastructure or production bans — rely on local government action.</t>
+        </is>
+      </c>
+      <c r="E1886" s="31" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1887" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1887" s="31" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D1887" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1887" s="31" t="inlineStr">
+        <is>
+          <t>"There is no monitoring."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1888" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1888" s="31" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1888" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1888" s="31" t="inlineStr">
+        <is>
+          <t>Need plastics collection centers; dustbins everywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1889" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1889" s="31" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1889" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1889" s="31" t="inlineStr">
+        <is>
+          <t>NA - Q6 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1890" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1890" s="31" t="inlineStr">
+        <is>
+          <t>Enforcement</t>
+        </is>
+      </c>
+      <c r="D1890" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1890" s="31" t="inlineStr">
+        <is>
+          <t>Government does not enforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1891" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1891" s="31" t="inlineStr">
+        <is>
+          <t>Pol_awareness</t>
+        </is>
+      </c>
+      <c r="D1891" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1891" s="31" t="inlineStr">
+        <is>
+          <t>Campaign not to use plastics all over Nepal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1892" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1892" s="31" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1892" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1892" s="31" t="inlineStr">
+        <is>
+          <t>Campaign "did not work well"; measures not very effective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1893" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1893" s="31" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1893" s="31" t="inlineStr">
+        <is>
+          <t>Campaign not to use plastics "all over Nepal" but "it did not work well" — measures "not very effective so far"; government "does not enforce" and "there is no monitoring."</t>
+        </is>
+      </c>
+      <c r="E1893" s="31" t="inlineStr">
+        <is>
+          <t>See Pol_effectiveness — quoted directly in Coded_Data cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1894" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1894" s="31" t="inlineStr">
+        <is>
+          <t>Sol_lead_agency</t>
+        </is>
+      </c>
+      <c r="D1894" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1894" s="31" t="inlineStr">
+        <is>
+          <t>Local government enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1895" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1895" s="31" t="inlineStr">
+        <is>
+          <t>Sol_recycling</t>
+        </is>
+      </c>
+      <c r="D1895" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1895" s="31" t="inlineStr">
+        <is>
+          <t>Plastics collection centers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1896" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1896" s="31" t="inlineStr">
+        <is>
+          <t>Sol_ban</t>
+        </is>
+      </c>
+      <c r="D1896" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1896" s="31" t="inlineStr">
+        <is>
+          <t>Stop producing plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1897" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1897" s="31" t="inlineStr">
+        <is>
+          <t>Sol_infrastructure</t>
+        </is>
+      </c>
+      <c r="D1897" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1897" s="31" t="inlineStr">
+        <is>
+          <t>Set up dustbins everywhere; plastics collection centers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1898" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1898" s="31" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1898" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1898" s="31" t="inlineStr">
+        <is>
+          <t>Alternative plastic products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1899" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1899" s="31" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1899" s="31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1899" s="31" t="inlineStr">
+        <is>
+          <t>Local government must enforce regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" s="31" t="inlineStr">
+        <is>
+          <t>NPL_26</t>
+        </is>
+      </c>
+      <c r="B1900" s="31" t="inlineStr">
+        <is>
+          <t>Cafe workers (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1900" s="31" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1900" s="31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1900" s="31" t="inlineStr">
+        <is>
+          <t>NA - Q8 traditions follow-up not asked.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add NPL_27 coding for school teacher interview (Feb 2026)
Code structured guideline notes for unnamed school teacher (high concern,
no waste collection, monthly plastic burning, school education for
children, cloth bags). Updates workbook to NPL_27.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
+++ b/nepal_plastic_coding/Nepal_Plastic_Governance_Coding.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="29">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -62,152 +62,158 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBB3A2"/>
-        <bgColor rgb="00EBB3A2"/>
+        <fgColor rgb="00EBB2A2"/>
+        <bgColor rgb="00EBB2A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBC4A2"/>
-        <bgColor rgb="00EBC4A2"/>
+        <fgColor rgb="00EBC2A2"/>
+        <bgColor rgb="00EBC2A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBD4A2"/>
-        <bgColor rgb="00EBD4A2"/>
+        <fgColor rgb="00EBD3A2"/>
+        <bgColor rgb="00EBD3A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBE5A2"/>
-        <bgColor rgb="00EBE5A2"/>
+        <fgColor rgb="00EBE3A2"/>
+        <bgColor rgb="00EBE3A2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0EBA2"/>
-        <bgColor rgb="00E0EBA2"/>
+        <fgColor rgb="00E3EBA2"/>
+        <bgColor rgb="00E3EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFEBA2"/>
-        <bgColor rgb="00CFEBA2"/>
+        <fgColor rgb="00D3EBA2"/>
+        <bgColor rgb="00D3EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BEEBA2"/>
-        <bgColor rgb="00BEEBA2"/>
+        <fgColor rgb="00C2EBA2"/>
+        <bgColor rgb="00C2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADEBA2"/>
-        <bgColor rgb="00ADEBA2"/>
+        <fgColor rgb="00B2EBA2"/>
+        <bgColor rgb="00B2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBA8"/>
-        <bgColor rgb="00A2EBA8"/>
+        <fgColor rgb="00A2EBA2"/>
+        <bgColor rgb="00A2EBA2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBB8"/>
-        <bgColor rgb="00A2EBB8"/>
+        <fgColor rgb="00A2EBB2"/>
+        <bgColor rgb="00A2EBB2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBC9"/>
-        <bgColor rgb="00A2EBC9"/>
+        <fgColor rgb="00A2EBC2"/>
+        <bgColor rgb="00A2EBC2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBDA"/>
-        <bgColor rgb="00A2EBDA"/>
+        <fgColor rgb="00A2EBD3"/>
+        <bgColor rgb="00A2EBD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2EBEB"/>
-        <bgColor rgb="00A2EBEB"/>
+        <fgColor rgb="00A2EBE3"/>
+        <bgColor rgb="00A2EBE3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2DAEB"/>
-        <bgColor rgb="00A2DAEB"/>
+        <fgColor rgb="00A2E3EB"/>
+        <bgColor rgb="00A2E3EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2C9EB"/>
-        <bgColor rgb="00A2C9EB"/>
+        <fgColor rgb="00A2D3EB"/>
+        <bgColor rgb="00A2D3EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2B8EB"/>
-        <bgColor rgb="00A2B8EB"/>
+        <fgColor rgb="00A2C2EB"/>
+        <bgColor rgb="00A2C2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A2A8EB"/>
-        <bgColor rgb="00A2A8EB"/>
+        <fgColor rgb="00A2B2EB"/>
+        <bgColor rgb="00A2B2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADA2EB"/>
-        <bgColor rgb="00ADA2EB"/>
+        <fgColor rgb="00A2A2EB"/>
+        <bgColor rgb="00A2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BEA2EB"/>
-        <bgColor rgb="00BEA2EB"/>
+        <fgColor rgb="00B2A2EB"/>
+        <bgColor rgb="00B2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFA2EB"/>
-        <bgColor rgb="00CFA2EB"/>
+        <fgColor rgb="00C2A2EB"/>
+        <bgColor rgb="00C2A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0A2EB"/>
-        <bgColor rgb="00E0A2EB"/>
+        <fgColor rgb="00D3A2EB"/>
+        <bgColor rgb="00D3A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2E5"/>
-        <bgColor rgb="00EBA2E5"/>
+        <fgColor rgb="00E3A2EB"/>
+        <bgColor rgb="00E3A2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2D4"/>
-        <bgColor rgb="00EBA2D4"/>
+        <fgColor rgb="00EBA2E3"/>
+        <bgColor rgb="00EBA2E3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2C4"/>
-        <bgColor rgb="00EBA2C4"/>
+        <fgColor rgb="00EBA2D3"/>
+        <bgColor rgb="00EBA2D3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBA2B3"/>
-        <bgColor rgb="00EBA2B3"/>
+        <fgColor rgb="00EBA2C2"/>
+        <bgColor rgb="00EBA2C2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBA2B2"/>
+        <bgColor rgb="00EBA2B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -237,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -330,6 +336,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -697,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -716,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_26, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
+          <t>This workbook applies the supplied codebook (see 'Codebook' sheet) to the Nepal interview list. 'Coded_Data' contains one row per fully coded interview (NPL_1 through NPL_27, in that order). Unfilled placeholder rows are not included. Column names and order follow exactly the variable list supplied by the research team.</t>
         </is>
       </c>
     </row>
@@ -913,82 +922,89 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  27. NPL_27 - School teacher (unnamed), Nepal (17 February 2026). Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. No waste collection; monthly plastic burning; school education for children. Q4, Q6, Q8 traditions, Q9 and Q10 not asked.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook:</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_26, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+          <t xml:space="preserve">  - Codebook: the variable dictionary, listed in the exact same order as the columns in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Coded_Data: wide-format matrix, one row per coded interview (NPL_1-NPL_27, in order), one column per codebook variable, including a free-hand 'Notes' column. Each interview's row is filled with a distinct colour so interviews are easy to tell apart at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Coding_Explanations: long-format table giving the quote/observation behind each coded value, one row per Interview x Variable. As requested, the following columns ALWAYS have an explanation row for every interview, even when the value is NA: NPF_victims, NPF_villains, NPF_hero, all Res_/Cul_/Tar_ actor-grid columns, Actor_role, Discretion, Capacity, Pol_effectiveness and Pol_effectiveness_example. For NPF fields, explanations explicitly note when victims/villains/hero are implied rather than named, or FLAG when none are mentioned directly or even implied. Other columns are documented only where a specific explanation was written. Rows are colour-matched to the same interview colour used in 'Coded_Data'.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-    </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Colour key: each interview (NPL_1 through NPL_26) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Colour key: each interview (NPL_1 through NPL_27) has a distinct colour spread evenly across the colour wheel so adjacent IDs are easy to tell apart.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Coding conventions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+          <t xml:space="preserve">  - 'yes' / 'no' / 'NA': NA means the topic was not addressed in that interview (no evidence either way); 'no' is only used where the interviewee explicitly said the item is not an issue / not in place (e.g. Pol_epr = no where EPR is proposed but not yet enacted).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Free-hand fields (Impacts, NPF_victims/villains/hero, Discretion, Pol_effectiveness_example, 'Traditions to build on') contain short descriptive text derived directly from the interview content, or 'NA' if not discussed/not yet coded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Actor_role: 1 = formulation/policy actor, 2 = managerial/organisational implementer, 3 = street-level implementer, 4 = target group (comma-separated if more than one applies), derived from what the interview describes the interviewee's organisation/role as actually doing - not simply from their actor type. Ganesh Shah (NPL_2) is coded as role 1 (formulation/policy actor), reflecting his role as a former Minister and policy/science-diplomacy advocate rather than a current day-to-day implementer; Discretion is therefore marked NA for that row, as the field only applies to roles 2/3.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Note on source material: an earlier version of this workbook coded NPL_7 from short bullet-point notes only. That row has now been fully recoded from the complete interview guideline notes and verbatim transcript supplied for this respondent.</t>
         </is>
@@ -2175,7 +2191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ27"/>
+  <dimension ref="A1:CQ28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15154,6 +15170,483 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>edu_institutions</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O28" s="32" t="inlineStr">
+        <is>
+          <t>health ("burning has much impact on human health" — monthly plastic burning because no collection and plastics are not compostable), and livestock ("life stock eats plastics")</t>
+        </is>
+      </c>
+      <c r="P28" s="32" t="inlineStr">
+        <is>
+          <t>human health (from monthly plastic burning); livestock that ingest plastic waste; and the teacher's household/community lacking waste collection</t>
+        </is>
+      </c>
+      <c r="Q28" s="32" t="inlineStr">
+        <is>
+          <t>absence of waste collection ("no waste collection at all"; "they do not have pick-up" forcing monthly burning of non-compostable plastics with large volume); continued plastic production (shutting down production seen as desirable but "impossible"); and insufficient education ("children need to be taught about it")</t>
+        </is>
+      </c>
+      <c r="R28" s="32" t="inlineStr">
+        <is>
+          <t>community members; local government enforcing regulation; higher authorities; cloth bags ("carry around cloth bags"); school-based education for children; volunteers sharing information; and plastic-free areas (seen as desirable but "impossible")</t>
+        </is>
+      </c>
+      <c r="S28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="T28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="X28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Z28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AE28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AF28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AG28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AH28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AI28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AJ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AK28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AL28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AM28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AN28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AO28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AP28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AQ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AR28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AS28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AT28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AU28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AV28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AW28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AX28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AY28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AZ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BA28" s="32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BB28" s="32" t="inlineStr">
+        <is>
+          <t>As a school teacher the interviewee is very concerned about plastic pollution and can teach children and mobilise community awareness, but personally must burn plastics monthly because there is no municipal pick-up and plastics cannot be composted (organic waste is composted for an agricultural plot) — cannot enforce regulation, shut production or establish plastic-free zones.</t>
+        </is>
+      </c>
+      <c r="BC28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BD28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BE28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BF28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="BG28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BH28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BI28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BJ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BK28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BL28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BM28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BN28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BO28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BP28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BQ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BR28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BS28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BT28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BU28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BW28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BX28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BY28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BZ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CA28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CB28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CC28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CD28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CE28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CF28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CG28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CH28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CI28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CJ28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CK28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CL28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CM28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CN28" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="CO28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CP28" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="CQ28" s="32" t="inlineStr">
+        <is>
+          <t>Master list label: "27. School teacher (unnamed)", affiliation: teacher at school. Interviewee name not given. Interview date: 17 February 2026. Interviewers: Ram Devi, Marlene Kammerer, Anastasiia. Consent given; no recording. Coded from structured interview guideline/field notes only (no verbatim transcript). Informal discussion noted: children need to be taught; volunteers may be needed to share information. Q3 integrated (no collection); Q4/Q4 follow-up and Q6/Q6 follow-up not asked. Q8 traditions, Q9 and Q10 not asked. Same interview date as NPL_21–NPL_26. NPF fields implied, not explicit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15165,7 +15658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1900"/>
+  <dimension ref="A1:E1954"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -66475,6 +66968,1464 @@
         </is>
       </c>
     </row>
+    <row r="1901">
+      <c r="A1901" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1901" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1901" s="32" t="inlineStr">
+        <is>
+          <t>Actortype</t>
+        </is>
+      </c>
+      <c r="D1901" s="32" t="inlineStr">
+        <is>
+          <t>edu_institutions</t>
+        </is>
+      </c>
+      <c r="E1901" s="32" t="inlineStr">
+        <is>
+          <t>Teacher at school — coded as edu_institutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1902" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1902" s="32" t="inlineStr">
+        <is>
+          <t>Problem_concerndness</t>
+        </is>
+      </c>
+      <c r="D1902" s="32" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E1902" s="32" t="inlineStr">
+        <is>
+          <t>"Very much concerned."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1903" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1903" s="32" t="inlineStr">
+        <is>
+          <t>Problem_littering</t>
+        </is>
+      </c>
+      <c r="D1903" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1903" s="32" t="inlineStr">
+        <is>
+          <t>Livestock eat plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1904" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1904" s="32" t="inlineStr">
+        <is>
+          <t>Problem_recycling</t>
+        </is>
+      </c>
+      <c r="D1904" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1904" s="32" t="inlineStr">
+        <is>
+          <t>Plastics not compostable; must be burned monthly (large volume).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1905" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1905" s="32" t="inlineStr">
+        <is>
+          <t>Problem_waste_mgmt</t>
+        </is>
+      </c>
+      <c r="D1905" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1905" s="32" t="inlineStr">
+        <is>
+          <t>"No waste collection at all"; no pick-up service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1906" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1906" s="32" t="inlineStr">
+        <is>
+          <t>Problem_production</t>
+        </is>
+      </c>
+      <c r="D1906" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1906" s="32" t="inlineStr">
+        <is>
+          <t>Shutting down production suggested but seen as "impossible."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1907" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1907" s="32" t="inlineStr">
+        <is>
+          <t>Problem_alternatives</t>
+        </is>
+      </c>
+      <c r="D1907" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1907" s="32" t="inlineStr">
+        <is>
+          <t>Cloth bags suggested; plastic-free area desired but "impossible."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1908" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1908" s="32" t="inlineStr">
+        <is>
+          <t>Problem_waste_segregation</t>
+        </is>
+      </c>
+      <c r="D1908" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1908" s="32" t="inlineStr">
+        <is>
+          <t>Organic waste composted for agricultural plot; plastics separated and burned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1909" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1909" s="32" t="inlineStr">
+        <is>
+          <t>Impacts</t>
+        </is>
+      </c>
+      <c r="D1909" s="32" t="inlineStr">
+        <is>
+          <t>health ("burning has much impact on human health" — monthly plastic burning because no collection and plastics are not compostable), and livestock ("life stock eats plastics")</t>
+        </is>
+      </c>
+      <c r="E1909" s="32" t="inlineStr">
+        <is>
+          <t>Health from burning; livestock ingesting plastics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1910" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1910" s="32" t="inlineStr">
+        <is>
+          <t>NPF_victims</t>
+        </is>
+      </c>
+      <c r="D1910" s="32" t="inlineStr">
+        <is>
+          <t>human health (from monthly plastic burning); livestock that ingest plastic waste; and the teacher's household/community lacking waste collection</t>
+        </is>
+      </c>
+      <c r="E1910" s="32" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: human health; livestock; community without collection. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1911" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1911" s="32" t="inlineStr">
+        <is>
+          <t>NPF_villains</t>
+        </is>
+      </c>
+      <c r="D1911" s="32" t="inlineStr">
+        <is>
+          <t>absence of waste collection ("no waste collection at all"; "they do not have pick-up" forcing monthly burning of non-compostable plastics with large volume); continued plastic production (shutting down production seen as desirable but "impossible"); and insufficient education ("children need to be taught about it")</t>
+        </is>
+      </c>
+      <c r="E1911" s="32" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: absence of collection infrastructure; continued production; inadequate school education. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1912" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1912" s="32" t="inlineStr">
+        <is>
+          <t>NPF_hero</t>
+        </is>
+      </c>
+      <c r="D1912" s="32" t="inlineStr">
+        <is>
+          <t>community members; local government enforcing regulation; higher authorities; cloth bags ("carry around cloth bags"); school-based education for children; volunteers sharing information; and plastic-free areas (seen as desirable but "impossible")</t>
+        </is>
+      </c>
+      <c r="E1912" s="32" t="inlineStr">
+        <is>
+          <t>NOT named in explicit NPF narrative language, but clearly IMPLIED: community members; local government; higher authorities; cloth bags; school education; volunteers. No FLAG needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1913" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1913" s="32" t="inlineStr">
+        <is>
+          <t>Res_nat_government</t>
+        </is>
+      </c>
+      <c r="D1913" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1913" s="32" t="inlineStr">
+        <is>
+          <t>"Higher authorities" responsible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1914" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1914" s="32" t="inlineStr">
+        <is>
+          <t>Res_prov_government</t>
+        </is>
+      </c>
+      <c r="D1914" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1914" s="32" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1915" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1915" s="32" t="inlineStr">
+        <is>
+          <t>Res_loc_government</t>
+        </is>
+      </c>
+      <c r="D1915" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1915" s="32" t="inlineStr">
+        <is>
+          <t>"Local government" responsible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1916" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1916" s="32" t="inlineStr">
+        <is>
+          <t>Res_students</t>
+        </is>
+      </c>
+      <c r="D1916" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1916" s="32" t="inlineStr">
+        <is>
+          <t>NA - children mentioned as learners, not formal responsible actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1917" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1917" s="32" t="inlineStr">
+        <is>
+          <t>Res_private_sector</t>
+        </is>
+      </c>
+      <c r="D1917" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1917" s="32" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1918" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1918" s="32" t="inlineStr">
+        <is>
+          <t>Res_civil_society</t>
+        </is>
+      </c>
+      <c r="D1918" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1918" s="32" t="inlineStr">
+        <is>
+          <t>NA - volunteers mentioned informally but not as formal actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1919" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1919" s="32" t="inlineStr">
+        <is>
+          <t>Res_science</t>
+        </is>
+      </c>
+      <c r="D1919" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1919" s="32" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1920" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1920" s="32" t="inlineStr">
+        <is>
+          <t>Res_households</t>
+        </is>
+      </c>
+      <c r="D1920" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1920" s="32" t="inlineStr">
+        <is>
+          <t>"Community members" cited in solutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1921" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1921" s="32" t="inlineStr">
+        <is>
+          <t>Res_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1921" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1921" s="32" t="inlineStr">
+        <is>
+          <t>Teacher role; informal note that children need to be taught.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1922" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1922" s="32" t="inlineStr">
+        <is>
+          <t>Res_private_companies</t>
+        </is>
+      </c>
+      <c r="D1922" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1922" s="32" t="inlineStr">
+        <is>
+          <t>NA - not mentioned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1923" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1923" s="32" t="inlineStr">
+        <is>
+          <t>Cul_nat_government</t>
+        </is>
+      </c>
+      <c r="D1923" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1923" s="32" t="inlineStr">
+        <is>
+          <t>NA - higher authorities named as responsible, not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1924" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1924" s="32" t="inlineStr">
+        <is>
+          <t>Cul_prov_government</t>
+        </is>
+      </c>
+      <c r="D1924" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1924" s="32" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1925" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1925" s="32" t="inlineStr">
+        <is>
+          <t>Cul_loc_government</t>
+        </is>
+      </c>
+      <c r="D1925" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1925" s="32" t="inlineStr">
+        <is>
+          <t>NA - local government portrayed as actor to strengthen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1926" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1926" s="32" t="inlineStr">
+        <is>
+          <t>Cul_students</t>
+        </is>
+      </c>
+      <c r="D1926" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1926" s="32" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1927" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1927" s="32" t="inlineStr">
+        <is>
+          <t>Cul_private_sector</t>
+        </is>
+      </c>
+      <c r="D1927" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1927" s="32" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1928" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1928" s="32" t="inlineStr">
+        <is>
+          <t>Cul_civil_society</t>
+        </is>
+      </c>
+      <c r="D1928" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1928" s="32" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1929" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1929" s="32" t="inlineStr">
+        <is>
+          <t>Cul_science</t>
+        </is>
+      </c>
+      <c r="D1929" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1929" s="32" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1930" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1930" s="32" t="inlineStr">
+        <is>
+          <t>Cul_households</t>
+        </is>
+      </c>
+      <c r="D1930" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1930" s="32" t="inlineStr">
+        <is>
+          <t>NA - community portrayed as solution partner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1931" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1931" s="32" t="inlineStr">
+        <is>
+          <t>Cul_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1931" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1931" s="32" t="inlineStr">
+        <is>
+          <t>NA - schools portrayed as needing to teach, not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1932" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1932" s="32" t="inlineStr">
+        <is>
+          <t>Cul_private_companies</t>
+        </is>
+      </c>
+      <c r="D1932" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1932" s="32" t="inlineStr">
+        <is>
+          <t>NA - not blamed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1933" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1933" s="32" t="inlineStr">
+        <is>
+          <t>Tar_nat_government</t>
+        </is>
+      </c>
+      <c r="D1933" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1933" s="32" t="inlineStr">
+        <is>
+          <t>NA - not named as specific target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1934" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1934" s="32" t="inlineStr">
+        <is>
+          <t>Tar_prov_government</t>
+        </is>
+      </c>
+      <c r="D1934" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1934" s="32" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1935" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1935" s="32" t="inlineStr">
+        <is>
+          <t>Tar_loc_government</t>
+        </is>
+      </c>
+      <c r="D1935" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1935" s="32" t="inlineStr">
+        <is>
+          <t>"Local government has to enforce the regulation"; local government "in charge."</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1936" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1936" s="32" t="inlineStr">
+        <is>
+          <t>Tar_students</t>
+        </is>
+      </c>
+      <c r="D1936" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1936" s="32" t="inlineStr">
+        <is>
+          <t>NA - children as learners, not named as policy target group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1937" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1937" s="32" t="inlineStr">
+        <is>
+          <t>Tar_private_sector</t>
+        </is>
+      </c>
+      <c r="D1937" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1937" s="32" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1938" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1938" s="32" t="inlineStr">
+        <is>
+          <t>Tar_civil_society</t>
+        </is>
+      </c>
+      <c r="D1938" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1938" s="32" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1939" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1939" s="32" t="inlineStr">
+        <is>
+          <t>Tar_science</t>
+        </is>
+      </c>
+      <c r="D1939" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1939" s="32" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1940" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1940" s="32" t="inlineStr">
+        <is>
+          <t>Tar_households</t>
+        </is>
+      </c>
+      <c r="D1940" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1940" s="32" t="inlineStr">
+        <is>
+          <t>Community members as solution actors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1941" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1941" s="32" t="inlineStr">
+        <is>
+          <t>Tar_edu_institutions</t>
+        </is>
+      </c>
+      <c r="D1941" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1941" s="32" t="inlineStr">
+        <is>
+          <t>Children need to be taught; volunteers to share information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1942" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1942" s="32" t="inlineStr">
+        <is>
+          <t>Tar_private_companies</t>
+        </is>
+      </c>
+      <c r="D1942" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1942" s="32" t="inlineStr">
+        <is>
+          <t>NA - not named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1943" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1943" s="32" t="inlineStr">
+        <is>
+          <t>Actor_role</t>
+        </is>
+      </c>
+      <c r="D1943" s="32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E1943" s="32" t="inlineStr">
+        <is>
+          <t>School teacher as street-level educator/awareness actor (role 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1944" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1944" s="32" t="inlineStr">
+        <is>
+          <t>Discretion</t>
+        </is>
+      </c>
+      <c r="D1944" s="32" t="inlineStr">
+        <is>
+          <t>As a school teacher the interviewee is very concerned about plastic pollution and can teach children and mobilise community awareness, but personally must burn plastics monthly because there is no municipal pick-up and plastics cannot be composted (organic waste is composted for an agricultural plot) — cannot enforce regulation, shut production or establish plastic-free zones.</t>
+        </is>
+      </c>
+      <c r="E1944" s="32" t="inlineStr">
+        <is>
+          <t>See Coded_Data Discretion cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1945" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1945" s="32" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D1945" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1945" s="32" t="inlineStr">
+        <is>
+          <t>No waste collection/pick-up forces monthly burning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1946" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1946" s="32" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1946" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1946" s="32" t="inlineStr">
+        <is>
+          <t>NA - Q6 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1947" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1947" s="32" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness</t>
+        </is>
+      </c>
+      <c r="D1947" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1947" s="32" t="inlineStr">
+        <is>
+          <t>NA - Q4 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1948" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1948" s="32" t="inlineStr">
+        <is>
+          <t>Pol_effectiveness_example</t>
+        </is>
+      </c>
+      <c r="D1948" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1948" s="32" t="inlineStr">
+        <is>
+          <t>NA - Q4 not asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1949" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1949" s="32" t="inlineStr">
+        <is>
+          <t>Sol_awareness</t>
+        </is>
+      </c>
+      <c r="D1949" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1949" s="32" t="inlineStr">
+        <is>
+          <t>Community members; volunteers sharing information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1950" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1950" s="32" t="inlineStr">
+        <is>
+          <t>Sol_education</t>
+        </is>
+      </c>
+      <c r="D1950" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1950" s="32" t="inlineStr">
+        <is>
+          <t>Children need to be taught about plastic pollution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1951" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1951" s="32" t="inlineStr">
+        <is>
+          <t>Sol_ban</t>
+        </is>
+      </c>
+      <c r="D1951" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1951" s="32" t="inlineStr">
+        <is>
+          <t>Plastic-free area and shutting down production (seen as impossible).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1952" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1952" s="32" t="inlineStr">
+        <is>
+          <t>Sol_subsitutes</t>
+        </is>
+      </c>
+      <c r="D1952" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1952" s="32" t="inlineStr">
+        <is>
+          <t>Carry around cloth bags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1953" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1953" s="32" t="inlineStr">
+        <is>
+          <t>Sol_enforcement</t>
+        </is>
+      </c>
+      <c r="D1953" s="32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1953" s="32" t="inlineStr">
+        <is>
+          <t>Local government must enforce regulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" s="32" t="inlineStr">
+        <is>
+          <t>NPL_27</t>
+        </is>
+      </c>
+      <c r="B1954" s="32" t="inlineStr">
+        <is>
+          <t>School teacher (unnamed), Nepal (17 February 2026; interviewers: Ram Devi, Marlene Kammerer, Anastasiia; no recording)</t>
+        </is>
+      </c>
+      <c r="C1954" s="32" t="inlineStr">
+        <is>
+          <t>Traditions to build on (free-hand)</t>
+        </is>
+      </c>
+      <c r="D1954" s="32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E1954" s="32" t="inlineStr">
+        <is>
+          <t>NA - Q8 traditions follow-up not asked.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>